<commit_message>
Update dashboards — 2026-09-15
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -1000,7 +1000,7 @@
         <v>97.98</v>
       </c>
       <c r="T2" t="n">
-        <v>3412</v>
+        <v>3413</v>
       </c>
       <c r="U2" s="7" t="n">
         <v>7694.910000000013</v>
@@ -1009,7 +1009,7 @@
         <v>2163</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.39390386869871</v>
+        <v>63.37532962203341</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.01</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/14/2026 18:28</t>
+          <t>09/15/2026 00:25</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/14/2026 18:46</t>
+          <t>09/15/2026 00:44</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/12/2026 00:08</t>
+          <t>09/15/2026 00:10</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/12/2026 00:29</t>
+          <t>09/15/2026 00:32</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5545,7 +5545,7 @@
         <v>647</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-139.26</v>
+        <v>-163.8</v>
       </c>
       <c r="V44" t="n">
         <v>368</v>
@@ -5554,7 +5554,7 @@
         <v>56.87789799072643</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>4.39</v>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5633,22 +5633,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-41.96</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.4413526827319931</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>49</v>
@@ -6020,7 +6011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/12/2026 00:17</t>
+          <t>09/15/2026 00:19</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -8620,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/14/2026 18:50</t>
+          <t>09/15/2026 00:46</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -9320,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/14/2026 18:40</t>
+          <t>09/15/2026 00:37</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -10020,7 +10011,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/14/2026 18:37</t>
+          <t>09/15/2026 00:34</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
@@ -10120,7 +10111,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/14/2026 18:30</t>
+          <t>09/15/2026 00:28</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
@@ -12979,23 +12970,17 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>67.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q119" s="9" t="n">
-        <v>65</v>
-      </c>
-      <c r="R119" s="9" t="n">
-        <v>1.223174978645115</v>
-      </c>
-      <c r="S119" s="9" t="n">
-        <v>0.57</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q119" s="8" t="n"/>
+      <c r="R119" s="8" t="n"/>
+      <c r="S119" s="8" t="n"/>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -14722,7 +14707,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -17446,7 +17431,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/14/2026 18:50</t>
+          <t>09/15/2026 00:46</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-16
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-14 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-16 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/14/2026 22:32</t>
+          <t>09/15/2026 08:41</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>32694.91</v>
+        <v>34401.44</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>49.46</v>
+        <v>57.26</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-20486.36</v>
+        <v>-17611.52</v>
       </c>
       <c r="P2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>65</v>
+        <v>67.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.6235738650269774</v>
+        <v>0.6691129403626142</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>97.98</v>
+        <v>94.02</v>
       </c>
       <c r="T2" t="n">
-        <v>3413</v>
+        <v>3417</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>7694.910000000013</v>
+        <v>16394.02000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>2163</v>
+        <v>2168</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.37532962203341</v>
+        <v>63.44746853965467</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>09/13/2026 19:28</t>
+          <t>09/16/2026 19:57</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>09/12/2026 18:31</t>
+          <t>09/16/2026 10:01</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>09/13/2026 17:21</t>
+          <t>09/16/2026 17:50</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/12/2026 09:02</t>
+          <t>09/15/2026 09:10</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/12/2026 10:45</t>
+          <t>09/15/2026 10:50</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/12/2026 10:47</t>
+          <t>09/15/2026 10:51</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>09/13/2026 21:51</t>
+          <t>09/16/2026 22:08</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>09/12/2026 05:01</t>
+          <t>09/15/2026 05:33</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>09/13/2026 13:06</t>
+          <t>09/16/2026 13:12</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/13/2026 22:15</t>
+          <t>09/16/2026 22:28</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/14/2026 20:22</t>
+          <t>09/16/2026 23:27</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/14/2026 23:54</t>
+          <t>09/16/2026 11:16</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/14/2026 23:00</t>
+          <t>09/15/2026 10:28</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3180,19 +3180,19 @@
         <v>4.5</v>
       </c>
       <c r="T22" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-690.5899999999998</v>
+        <v>-755.73</v>
       </c>
       <c r="V22" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>48.42105263157895</v>
+        <v>48.95833333333333</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="Y22" s="7" t="n">
         <v>6.11</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,14 +3249,14 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/15/2026 00:25</t>
+          <t>09/16/2026 11:58</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19621.51</v>
+        <v>19618.63</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.06</v>
+        <v>-2.07</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.13</v>
@@ -3274,37 +3274,37 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-363.14</v>
+        <v>-380.44</v>
       </c>
       <c r="P23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>25</v>
+        <v>22.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.3064155700288405</v>
+        <v>0.2773482761895716</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
       <c r="T23" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-378.49</v>
+        <v>-381.37</v>
       </c>
       <c r="V23" t="n">
         <v>17</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>30.35714285714285</v>
+        <v>27.86885245901639</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.35</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/14/2026 23:25</t>
+          <t>09/15/2026 11:44</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/14/2026 16:59</t>
+          <t>09/15/2026 10:41</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3616,22 +3616,22 @@
         <v>5.08</v>
       </c>
       <c r="T26" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>-200.05</v>
+        <v>609.1199999999998</v>
       </c>
       <c r="V26" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>42.72727272727273</v>
+        <v>44.24778761061947</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>0.96</v>
+        <v>1.11</v>
       </c>
       <c r="Y26" s="7" t="n">
-        <v>7.4</v>
+        <v>8.99</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/12/2026 08:30</t>
+          <t>09/15/2026 08:36</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/14/2026 23:14</t>
+          <t>09/15/2026 10:55</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3834,19 +3834,19 @@
         <v>3.24</v>
       </c>
       <c r="T28" t="n">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-814.0300000000003</v>
+        <v>-682.1300000000002</v>
       </c>
       <c r="V28" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>42.17687074829932</v>
+        <v>42.10526315789473</v>
       </c>
       <c r="X28" s="7" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="Y28" s="7" t="n">
         <v>7.56</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>09/12/2026 19:14</t>
+          <t>09/16/2026 10:31</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/14/2026 23:28</t>
+          <t>09/15/2026 12:38</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20581.81</v>
+        <v>20581.64</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>2.92</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>1.5</v>
+        <v>1.59</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.74</v>
+        <v>1.72</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,7 +4037,7 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-310.78</v>
+        <v>-282.46</v>
       </c>
       <c r="P30" t="n">
         <v>8</v>
@@ -4046,28 +4046,28 @@
         <v>20</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.1953082519872608</v>
+        <v>0.2334455058619192</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="T30" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>581.8099999999999</v>
+        <v>580.7099999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>25.92592592592592</v>
+        <v>26.4367816091954</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.74</v>
+        <v>1.72</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <v>1.51</v>
+        <v>1.59</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/14/2026 20:32</t>
+          <t>09/16/2026 23:37</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/14/2026 19:45</t>
+          <t>09/16/2026 22:54</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20019.68</v>
+        <v>20383.44</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.11</v>
+        <v>1.93</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
-      <c r="K35" t="n">
-        <v>1</v>
+      <c r="K35" s="7" t="n">
+        <v>1.07</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>19.67999999999977</v>
+        <v>313.7399999999998</v>
       </c>
       <c r="V35" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>49.56521739130435</v>
+        <v>50.84745762711864</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1</v>
+        <v>1.06</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/15/2026 00:44</t>
+          <t>09/16/2026 12:24</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/13/2026 22:23</t>
+          <t>09/16/2026 22:33</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>09/13/2026 14:46</t>
+          <t>09/16/2026 14:54</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>09/12/2026 18:08</t>
+          <t>09/16/2026 09:47</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>09/12/2026 16:57</t>
+          <t>09/16/2026 09:08</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/12/2026 02:49</t>
+          <t>09/15/2026 02:51</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5511,20 +5511,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/14/2026 23:28</t>
+          <t>09/15/2026 12:37</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19836.2</v>
+        <v>19753.78</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-0.78</v>
+        <v>-1.2</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>4.38</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5542,19 +5542,19 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>647</v>
+        <v>660</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-163.8</v>
+        <v>-306.5200000000001</v>
       </c>
       <c r="V44" t="n">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>56.87789799072643</v>
+        <v>56.06060606060606</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>4.39</v>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/14/2026 22:43</t>
+          <t>09/15/2026 09:52</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/14/2026 22:59</t>
+          <t>09/15/2026 10:27</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5742,19 +5742,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-1155.53</v>
+        <v>-120.6399999999999</v>
       </c>
       <c r="V46" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>40.25974025974026</v>
+        <v>44.70588235294118</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.64</v>
+        <v>0.96</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/14/2026 22:47</t>
+          <t>09/15/2026 10:00</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6242,19 +6242,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>88.65999999999947</v>
+        <v>-13.88000000000056</v>
       </c>
       <c r="V51" t="n">
         <v>17</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>30.90909090909091</v>
+        <v>30.35714285714285</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,11 +6311,11 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/14/2026 23:20</t>
+          <t>09/15/2026 11:14</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19557.12</v>
+        <v>19556.36</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>-2.18</v>
@@ -6342,22 +6342,22 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-442.8800000000002</v>
+        <v>-432.7300000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.77551020408163</v>
+        <v>39.6039603960396</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>4.44</v>
+        <v>4.43</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6442,19 +6442,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-160.21</v>
+        <v>-179.67</v>
       </c>
       <c r="V53" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.32608695652174</v>
+        <v>35.62005277044855</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6811,14 +6811,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/14/2026 22:58</t>
+          <t>09/15/2026 10:23</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19707.78</v>
+        <v>19706.78</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.45</v>
+        <v>-1.46</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6842,16 +6842,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>956</v>
+        <v>969</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-291.72</v>
+        <v>-297.37</v>
       </c>
       <c r="V57" t="n">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.93305439330544</v>
+        <v>43.75644994840041</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.8</v>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/14/2026 23:24</t>
+          <t>09/15/2026 11:43</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>09/13/2026 01:02</t>
+          <t>09/16/2026 10:45</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/14/2026 23:15</t>
+          <t>09/15/2026 11:00</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/14/2026 23:51</t>
+          <t>09/16/2026 11:12</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7442,19 +7442,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1158.61</v>
+        <v>-1206.96</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>12.72727272727273</v>
+        <v>12.5</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.51</v>
+        <v>0.5</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7466,7 +7466,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/14/2026 23:51</t>
+          <t>09/16/2026 11:12</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/14/2026 23:24</t>
+          <t>09/15/2026 11:41</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/14/2026 23:47</t>
+          <t>09/16/2026 11:06</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>09/12/2026 22:17</t>
+          <t>09/16/2026 10:42</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>09/13/2026 22:06</t>
+          <t>09/16/2026 22:21</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>09/13/2026 22:06</t>
+          <t>09/16/2026 22:22</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/13/2026 22:06</t>
+          <t>09/16/2026 22:20</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/14/2026 18:58</t>
+          <t>09/16/2026 12:41</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/15/2026 00:46</t>
+          <t>09/16/2026 12:30</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/14/2026 23:21</t>
+          <t>09/15/2026 11:16</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/14/2026 23:57</t>
+          <t>09/16/2026 11:20</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/14/2026 23:56</t>
+          <t>09/16/2026 11:18</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/14/2026 23:49</t>
+          <t>09/16/2026 11:09</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/14/2026 23:21</t>
+          <t>09/15/2026 11:16</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/15/2026 00:37</t>
+          <t>09/16/2026 12:14</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/14/2026 23:54</t>
+          <t>09/16/2026 11:16</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/14/2026 19:04</t>
+          <t>09/15/2026 01:01</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>09/14/2026 19:46</t>
+          <t>09/15/2026 01:40</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9811,14 +9811,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/14/2026 18:53</t>
+          <t>09/16/2026 12:37</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20179.26</v>
+        <v>20182.66</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
@@ -9842,16 +9842,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>179.2600000000001</v>
+        <v>186.62</v>
       </c>
       <c r="V87" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>44.3609022556391</v>
+        <v>45.25547445255474</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>1.1</v>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9911,7 +9911,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>09/13/2026 10:42</t>
+          <t>09/16/2026 11:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10011,20 +10011,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/15/2026 00:34</t>
+          <t>09/16/2026 12:09</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20369.53</v>
+        <v>20371.33</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>1.84</v>
+        <v>1.85</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,19 +10042,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>369.53</v>
+        <v>412.33</v>
       </c>
       <c r="V89" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>84.69387755102041</v>
+        <v>84.76190476190476</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10111,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/15/2026 00:28</t>
+          <t>09/16/2026 12:01</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>24209.48</v>
+        <v>24579.1</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>21.11</v>
+        <v>22.96</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.75</v>
+        <v>1.82</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10142,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>4209.48</v>
+        <v>4559.57</v>
       </c>
       <c r="V90" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>69.79166666666666</v>
+        <v>70.87378640776699</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.75</v>
+        <v>1.78</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/14/2026 22:55</t>
+          <t>09/15/2026 10:18</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>09/13/2026 16:07</t>
+          <t>09/16/2026 16:36</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/14/2026 22:58</t>
+          <t>09/15/2026 10:24</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/14/2026 22:56</t>
+          <t>09/15/2026 10:18</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/14/2026 22:50</t>
+          <t>09/15/2026 10:10</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10711,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/14/2026 22:41</t>
+          <t>09/15/2026 09:49</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10811,7 +10811,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/14/2026 22:50</t>
+          <t>09/15/2026 10:09</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/14/2026 23:11</t>
+          <t>09/15/2026 10:49</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/14/2026 22:43</t>
+          <t>09/15/2026 09:54</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>09/13/2026 16:13</t>
+          <t>09/16/2026 16:42</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/14/2026 19:25</t>
+          <t>09/16/2026 13:22</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11242,19 +11242,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>318.0100000000001</v>
+        <v>679.45</v>
       </c>
       <c r="V101" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>72.72727272727273</v>
+        <v>75</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>1.52</v>
+        <v>2.11</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11266,7 +11266,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11311,20 +11311,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/14/2026 23:25</t>
+          <t>09/15/2026 11:44</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>20246.96</v>
+        <v>20244.86</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="J102" s="7" t="n">
         <v>1.27</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11342,22 +11342,22 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>250.8100000000001</v>
+        <v>-192.9099999999999</v>
       </c>
       <c r="V102" t="n">
         <v>16</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>42.10526315789473</v>
+        <v>36.36363636363637</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>1.71</v>
+        <v>0.76</v>
       </c>
       <c r="Y102" s="7" t="n">
-        <v>1.17</v>
+        <v>2.19</v>
       </c>
       <c r="Z102" t="inlineStr">
         <is>
@@ -11366,7 +11366,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>09/13/2026 21:16</t>
+          <t>09/16/2026 21:38</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11629,20 +11629,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/14/2026 21:20</t>
+          <t>09/15/2026 03:11</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11146.16</v>
+        <v>11032.57</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>11.44</v>
+        <v>10.3</v>
       </c>
       <c r="J105" s="7" t="n">
-        <v>2.38</v>
+        <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.92</v>
+        <v>2.46</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11660,22 +11660,22 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1256.69</v>
+        <v>1408.61</v>
       </c>
       <c r="V105" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>68.29268292682927</v>
+        <v>69.56521739130434</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.59</v>
+        <v>3.35</v>
       </c>
       <c r="Y105" s="7" t="n">
-        <v>1.7</v>
+        <v>2.69</v>
       </c>
       <c r="Z105" t="inlineStr">
         <is>
@@ -11684,7 +11684,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/12/2026 09:02</t>
+          <t>09/15/2026 09:09</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11838,7 +11838,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/14/2026 22:08</t>
+          <t>09/15/2026 07:41</t>
         </is>
       </c>
       <c r="H107" t="n">
@@ -11878,22 +11878,22 @@
         <v>1.61</v>
       </c>
       <c r="T107" t="n">
-        <v>3746</v>
+        <v>3753</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-7158.999999999999</v>
+        <v>-8102.999999999999</v>
       </c>
       <c r="V107" t="n">
-        <v>2298</v>
+        <v>2299</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>61.34543513080619</v>
+        <v>61.25766053823608</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="Y107" s="7" t="n">
-        <v>37.71</v>
+        <v>38.57</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -11902,7 +11902,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 08:16</t>
+          <t>09/15/2026 08:21</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 04:31</t>
+          <t>09/15/2026 04:53</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 19:38</t>
+          <t>09/16/2026 20:07</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12311,7 +12311,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 18:45</t>
+          <t>09/16/2026 10:09</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 09:01</t>
+          <t>09/15/2026 09:08</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12584,7 +12584,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 13:00</t>
+          <t>09/16/2026 13:09</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 04:51</t>
+          <t>09/15/2026 05:19</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12766,7 +12766,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 17:01</t>
+          <t>09/16/2026 17:31</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12948,7 +12948,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/14/2026 23:05</t>
+          <t>09/15/2026 10:40</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13203,7 +13203,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 22:06</t>
+          <t>09/16/2026 22:21</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13288,7 +13288,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 16:23</t>
+          <t>09/16/2026 16:51</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 16:23</t>
+          <t>09/16/2026 16:51</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 16:22</t>
+          <t>09/16/2026 16:51</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 16:32</t>
+          <t>09/16/2026 16:59</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 16:54</t>
+          <t>09/16/2026 17:23</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13713,7 +13713,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>09/13/2026 16:21</t>
+          <t>09/16/2026 16:50</t>
         </is>
       </c>
       <c r="H128" s="9" t="n">
@@ -13798,7 +13798,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 06:22</t>
+          <t>09/15/2026 06:27</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13889,7 +13889,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 05:20</t>
+          <t>09/15/2026 05:58</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14071,7 +14071,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 11:13</t>
+          <t>09/15/2026 11:17</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14246,7 +14246,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/12/2026 08:16</t>
+          <t>09/15/2026 08:21</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/12/2026 04:31</t>
+          <t>09/15/2026 04:53</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>09/13/2026 19:38</t>
+          <t>09/16/2026 20:07</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14410,7 +14410,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>09/12/2026 18:45</t>
+          <t>09/16/2026 10:09</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/12/2026 09:01</t>
+          <t>09/15/2026 09:08</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>09/13/2026 13:00</t>
+          <t>09/16/2026 13:09</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14574,7 +14574,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/12/2026 04:51</t>
+          <t>09/15/2026 05:19</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>09/13/2026 17:01</t>
+          <t>09/16/2026 17:31</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>09/14/2026 23:05</t>
+          <t>09/15/2026 10:40</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/13/2026 22:06</t>
+          <t>09/16/2026 22:21</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14861,7 +14861,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>09/13/2026 16:23</t>
+          <t>09/16/2026 16:51</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14902,7 +14902,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>09/13/2026 16:23</t>
+          <t>09/16/2026 16:51</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>09/13/2026 16:22</t>
+          <t>09/16/2026 16:51</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14984,7 +14984,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>09/13/2026 16:32</t>
+          <t>09/16/2026 16:59</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -15025,7 +15025,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>09/13/2026 16:54</t>
+          <t>09/16/2026 17:23</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>09/13/2026 16:21</t>
+          <t>09/16/2026 16:50</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/12/2026 06:22</t>
+          <t>09/15/2026 06:27</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15148,7 +15148,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/12/2026 05:20</t>
+          <t>09/15/2026 05:58</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15230,7 +15230,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/12/2026 11:13</t>
+          <t>09/15/2026 11:17</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -16971,7 +16971,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09/12/2026 07:28</t>
+          <t>09/15/2026 07:35</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09/13/2026 13:19</t>
+          <t>09/16/2026 13:23</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17017,7 +17017,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/12/2026 07:15</t>
+          <t>09/15/2026 07:26</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/12/2026 04:01</t>
+          <t>09/15/2026 04:14</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17063,7 +17063,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09/13/2026 21:28</t>
+          <t>09/16/2026 21:48</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17086,7 +17086,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09/12/2026 15:56</t>
+          <t>09/16/2026 08:40</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09/12/2026 03:41</t>
+          <t>09/15/2026 03:46</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17132,7 +17132,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09/12/2026 15:58</t>
+          <t>09/16/2026 08:41</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -17155,7 +17155,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09/13/2026 15:39</t>
+          <t>09/16/2026 16:07</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -17178,7 +17178,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/12/2026 08:30</t>
+          <t>09/15/2026 08:36</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09/13/2026 17:36</t>
+          <t>09/16/2026 18:07</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17224,7 +17224,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/12/2026 07:12</t>
+          <t>09/15/2026 07:22</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17270,7 +17270,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09/13/2026 21:38</t>
+          <t>09/16/2026 21:57</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17293,7 +17293,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09/13/2026 21:28</t>
+          <t>09/16/2026 21:49</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/12/2026 09:31</t>
+          <t>09/15/2026 09:35</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17339,7 +17339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/12/2026 03:54</t>
+          <t>09/15/2026 04:05</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -17362,7 +17362,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/14/2026 20:15</t>
+          <t>09/16/2026 23:21</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/12/2026 08:38</t>
+          <t>09/15/2026 08:41</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -17431,7 +17431,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/15/2026 00:46</t>
+          <t>09/16/2026 12:30</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -17477,7 +17477,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09/13/2026 16:41</t>
+          <t>09/16/2026 17:08</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -17500,7 +17500,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09/13/2026 16:41</t>
+          <t>09/16/2026 17:07</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -17569,7 +17569,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09/13/2026 16:30</t>
+          <t>09/16/2026 16:57</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -17592,7 +17592,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>09/13/2026 17:16</t>
+          <t>09/16/2026 17:45</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -17615,7 +17615,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>09/12/2026 15:56</t>
+          <t>09/16/2026 08:40</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -17684,7 +17684,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/12/2026 07:10</t>
+          <t>09/15/2026 07:21</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -17707,7 +17707,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/12/2026 07:56</t>
+          <t>09/15/2026 08:00</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -17730,7 +17730,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/12/2026 11:05</t>
+          <t>09/15/2026 11:09</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -17753,7 +17753,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/14/2026 13:37</t>
+          <t>09/16/2026 13:41</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-17
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-16 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-17 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/15/2026 08:41</t>
+          <t>09/17/2026 22:34</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>34401.44</v>
+        <v>51998.64</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>57.26</v>
+        <v>137.7</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.03</v>
+        <v>1.07</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-17611.52</v>
+        <v>-4669.44</v>
       </c>
       <c r="P2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>67.5</v>
+        <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.6691129403626142</v>
+        <v>0.9021612592580798</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>94.02</v>
+        <v>111.52</v>
       </c>
       <c r="T2" t="n">
-        <v>3417</v>
+        <v>3423</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>16394.02000000001</v>
+        <v>26998.64000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>2168</v>
+        <v>2174</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.44746853965467</v>
+        <v>63.51153958515921</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>09/14/2026 09:18</t>
+          <t>09/17/2026 09:19</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09/14/2026 10:34</t>
+          <t>09/17/2026 10:38</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>09/14/2026 13:18</t>
+          <t>09/17/2026 13:20</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>09/14/2026 06:01</t>
+          <t>09/17/2026 06:04</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09/14/2026 06:01</t>
+          <t>09/17/2026 06:04</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/16/2026 23:27</t>
+          <t>09/17/2026 20:51</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/16/2026 11:16</t>
+          <t>09/17/2026 18:50</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/15/2026 10:28</t>
+          <t>09/17/2026 17:54</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>19309.41</v>
+        <v>19244.27</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-3.44</v>
+        <v>-3.77</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>6.1</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3165,22 +3165,22 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-515.2600000000001</v>
+        <v>-821.1400000000001</v>
       </c>
       <c r="P22" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>45</v>
+        <v>42.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.7992613428288698</v>
+        <v>0.6961565359610139</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>4.5</v>
+        <v>4.88</v>
       </c>
       <c r="T22" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="U22" s="7" t="n">
         <v>-755.73</v>
@@ -3189,7 +3189,7 @@
         <v>47</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>48.95833333333333</v>
+        <v>48.45360824742268</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.86</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/16/2026 11:58</t>
+          <t>09/17/2026 19:16</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19618.63</v>
+        <v>19611.85</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.07</v>
+        <v>-2.1</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2.13</v>
+        <v>2.16</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,25 +3274,25 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-380.44</v>
+        <v>-414.06</v>
       </c>
       <c r="P23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.2773482761895716</v>
+        <v>0.2234870506160569</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>2.14</v>
+        <v>2.17</v>
       </c>
       <c r="T23" t="n">
         <v>61</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-381.37</v>
+        <v>-388.15</v>
       </c>
       <c r="V23" t="n">
         <v>17</v>
@@ -3304,7 +3304,7 @@
         <v>0.35</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>1.97</v>
+        <v>2</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/15/2026 11:44</t>
+          <t>09/17/2026 23:20</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/14/2026 23:00</t>
+          <t>09/17/2026 23:03</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/15/2026 10:41</t>
+          <t>09/17/2026 23:02</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20618.97</v>
+        <v>20668.65</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.4</v>
+        <v>-1.17</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>321.57</v>
+        <v>672.16</v>
       </c>
       <c r="P26" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>52.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.138482408165023</v>
+        <v>1.318788890575201</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5.08</v>
+        <v>5.01</v>
       </c>
       <c r="T26" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>609.1199999999998</v>
+        <v>520.2199999999998</v>
       </c>
       <c r="V26" t="n">
         <v>50</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>44.24778761061947</v>
+        <v>42.73504273504273</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3794,20 +3794,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/15/2026 10:55</t>
+          <t>09/17/2026 23:08</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>19185.97</v>
+        <v>19658.67</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>-4.09</v>
+        <v>-1.73</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="L28" t="n">
         <v>20000</v>
@@ -3819,34 +3819,34 @@
         <v>40</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>-648.6</v>
+        <v>72.99000000000004</v>
       </c>
       <c r="P28" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>0.2784193311527935</v>
+        <v>1.096816553919618</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>3.24</v>
+        <v>2.58</v>
       </c>
       <c r="T28" t="n">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-682.1300000000002</v>
+        <v>-341.3300000000002</v>
       </c>
       <c r="V28" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>42.10526315789473</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X28" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="Y28" s="7" t="n">
         <v>7.56</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/15/2026 12:38</t>
+          <t>09/17/2026 23:22</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20581.64</v>
+        <v>20571.99</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.92</v>
+        <v>2.88</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.59</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.72</v>
+        <v>1.7</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-282.46</v>
+        <v>-240.15</v>
       </c>
       <c r="P30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.2334455058619192</v>
+        <v>0.263975726369989</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>1.5</v>
+        <v>1.24</v>
       </c>
       <c r="T30" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>580.7099999999999</v>
+        <v>571.9899999999999</v>
       </c>
       <c r="V30" t="n">
         <v>23</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>26.4367816091954</v>
+        <v>25.84269662921348</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.72</v>
+        <v>1.7</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.59</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/14/2026 10:37</t>
+          <t>09/17/2026 10:39</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>09/14/2026 11:32</t>
+          <t>09/17/2026 11:34</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/16/2026 23:37</t>
+          <t>09/17/2026 21:00</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/14/2026 00:30</t>
+          <t>09/17/2026 00:32</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/16/2026 22:54</t>
+          <t>09/17/2026 20:25</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20383.44</v>
+        <v>20281.8</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1.93</v>
+        <v>1.42</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>313.7399999999998</v>
+        <v>281.8</v>
       </c>
       <c r="V35" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>50.84745762711864</v>
+        <v>51.2396694214876</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/16/2026 12:24</t>
+          <t>09/17/2026 19:37</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -5333,13 +5333,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5433,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5511,20 +5529,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/15/2026 12:37</t>
+          <t>09/17/2026 23:23</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19753.78</v>
+        <v>19480.16</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.2</v>
+        <v>-2.57</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>4.38</v>
+        <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5533,31 +5551,40 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-353.1</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.1398085215230578</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="T44" t="n">
-        <v>660</v>
+        <v>673</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-306.5200000000001</v>
+        <v>-519.8400000000001</v>
       </c>
       <c r="V44" t="n">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>56.06060606060606</v>
+        <v>56.01783060921248</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.93</v>
+        <v>0.89</v>
       </c>
       <c r="Y44" s="7" t="n">
-        <v>4.39</v>
+        <v>5.13</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -5566,7 +5593,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5576,7 +5603,7 @@
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>Round Numbers MOL | AUDJPY, Round Numbers MOL | AUDUSD, Round Numbers MOL | CADJPY, Round Numbers MOL | EURAUD, Round Numbers MOL | EURJPY, Round Numbers MOL | EURUSD, Round Numbers MOL | GBPCAD, Round Numbers MOL | GBPJPY, Round Numbers MOL | GBPUSD, Round Numbers MOL | NZDJPY, Round Numbers MOL | NZDUSD, Round Numbers MOL | USDCHF, Round Numbers MOL | USDJPY</t>
+          <t>Round Numbers MOL | AUDJPY, Round Numbers MOL | AUDUSD, Round Numbers MOL | CADJPY, Round Numbers MOL | EURAUD, Round Numbers MOL | EURJPY, Round Numbers MOL | EURUSD, Round Numbers MOL | GBPAUD, Round Numbers MOL | GBPCAD, Round Numbers MOL | GBPJPY, Round Numbers MOL | GBPUSD, Round Numbers MOL | NZDJPY, Round Numbers MOL | NZDUSD, Round Numbers MOL | USDCHF, Round Numbers MOL | USDJPY</t>
         </is>
       </c>
     </row>
@@ -5611,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/15/2026 09:52</t>
+          <t>09/17/2026 22:44</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5633,13 +5660,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-41.96</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.4413526827319931</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.28</v>
       </c>
       <c r="T45" t="n">
         <v>49</v>
@@ -5711,20 +5747,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/15/2026 10:27</t>
+          <t>09/17/2026 22:57</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>18844.47</v>
+        <v>19815.81</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-5.75</v>
+        <v>-0.89</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.64</v>
+        <v>0.95</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5742,19 +5778,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-120.6399999999999</v>
+        <v>-184.1899999999999</v>
       </c>
       <c r="V46" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>44.70588235294118</v>
+        <v>45.34883720930232</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5802,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5811,7 +5847,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/14/2026 23:32</t>
+          <t>09/17/2026 23:35</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -6211,20 +6247,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/15/2026 10:00</t>
+          <t>09/17/2026 22:47</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>20088.66</v>
+        <v>19986.12</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>0.46</v>
+        <v>-0.05</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
-      <c r="K51" s="7" t="n">
-        <v>1.02</v>
+      <c r="K51" t="n">
+        <v>1</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6311,20 +6347,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/15/2026 11:14</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="n">
-        <v>19556.36</v>
+          <t>09/17/2026 18:10</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>19645</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-2.18</v>
+        <v>-1.75</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>4.41</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.9</v>
+        <v>0.93</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6342,19 +6378,19 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-432.7300000000002</v>
+        <v>-355.0000000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>39.6039603960396</v>
+        <v>40.19607843137255</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>4.43</v>
@@ -6366,7 +6402,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,20 +6447,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/14/2026 23:46</t>
+          <t>09/17/2026 23:38</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19839.79</v>
+        <v>19779.12</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-0.83</v>
+        <v>-1.14</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.87</v>
+        <v>0.83</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6442,19 +6478,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-179.67</v>
+        <v>-220.8800000000001</v>
       </c>
       <c r="V53" t="n">
         <v>135</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.62005277044855</v>
+        <v>35.06493506493506</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.86</v>
+        <v>0.83</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6502,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6511,7 +6547,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/14/2026 21:12</t>
+          <t>09/17/2026 21:15</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6611,7 +6647,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/14/2026 23:32</t>
+          <t>09/17/2026 23:26</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6811,20 +6847,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/15/2026 10:23</t>
+          <t>09/17/2026 22:57</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19706.78</v>
+        <v>19678.66</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.46</v>
+        <v>-1.6</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6833,28 +6869,37 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-37.61</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.4903103401544925</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T57" t="n">
-        <v>969</v>
+        <v>986</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-297.37</v>
+        <v>-319.58</v>
       </c>
       <c r="V57" t="n">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.75644994840041</v>
+        <v>43.81338742393509</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6866,7 +6911,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,20 +6956,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/15/2026 11:43</t>
+          <t>09/17/2026 23:18</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>16796.02</v>
+        <v>16692.87</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-16.03</v>
+        <v>-16.55</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>16.03</v>
+        <v>16.55</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -7111,20 +7156,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/15/2026 11:00</t>
+          <t>09/17/2026 23:10</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>19908.69</v>
+        <v>19644.84</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-6.41</v>
+        <v>-7.65</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>21100.65</v>
@@ -7211,20 +7256,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/16/2026 11:12</t>
+          <t>09/17/2026 18:48</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>20707.06</v>
+        <v>20449.71</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-3.34</v>
+        <v>-4.54</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>13.96</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L61" s="7" t="n">
         <v>21292.1</v>
@@ -7311,7 +7356,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>09/14/2026 21:03</t>
+          <t>09/17/2026 21:06</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,20 +7456,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/14/2026 23:38</t>
+          <t>09/17/2026 23:30</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18841.39</v>
+        <v>18726.69</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-5.82</v>
+        <v>-6.39</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.51</v>
+        <v>0.49</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7442,19 +7487,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1206.96</v>
+        <v>-1273.31</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>12.5</v>
+        <v>12.28070175438596</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7466,7 +7511,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7511,7 +7556,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/16/2026 11:12</t>
+          <t>09/17/2026 18:48</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,20 +7656,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/14/2026 23:39</t>
+          <t>09/17/2026 23:30</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19346.13</v>
+        <v>19088.95</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-3.32</v>
+        <v>-4.61</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7711,7 +7756,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/15/2026 11:41</t>
+          <t>09/17/2026 23:17</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,7 +7856,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/16/2026 11:06</t>
+          <t>09/17/2026 18:48</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7833,16 +7878,25 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>0</v>
+        <v>-123.7900000000002</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q67" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R67" s="7" t="n">
+        <v>0.9759118434571438</v>
+      </c>
+      <c r="S67" s="7" t="n">
+        <v>12.15</v>
       </c>
       <c r="T67" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="U67" s="7" t="n">
         <v>-442.1100000000005</v>
@@ -7851,7 +7905,7 @@
         <v>21</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>32.8125</v>
+        <v>31.81818181818182</v>
       </c>
       <c r="X67" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -7866,7 +7920,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8311,7 +8365,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/14/2026 23:31</t>
+          <t>09/17/2026 23:28</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8465,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/16/2026 12:41</t>
+          <t>09/17/2026 19:46</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8511,7 +8565,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/14/2026 23:39</t>
+          <t>09/17/2026 23:30</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8611,7 +8665,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/16/2026 12:30</t>
+          <t>09/17/2026 19:40</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8765,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/15/2026 11:16</t>
+          <t>09/17/2026 23:16</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8865,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/16/2026 11:20</t>
+          <t>09/17/2026 18:53</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +8965,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/14/2026 23:43</t>
+          <t>09/17/2026 23:36</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9065,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/16/2026 11:18</t>
+          <t>09/17/2026 18:53</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9165,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/16/2026 11:09</t>
+          <t>09/17/2026 18:46</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9211,7 +9265,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/15/2026 11:16</t>
+          <t>09/17/2026 23:15</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9311,7 +9365,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/16/2026 12:14</t>
+          <t>09/17/2026 19:30</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9411,7 +9465,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/16/2026 11:16</t>
+          <t>09/17/2026 18:52</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9511,7 +9565,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/15/2026 01:01</t>
+          <t>09/17/2026 19:50</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9711,7 +9765,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>09/14/2026 19:29</t>
+          <t>09/17/2026 19:31</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9811,20 +9865,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/16/2026 12:37</t>
+          <t>09/17/2026 19:43</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20182.66</v>
+        <v>20163.9</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>0.9</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9842,19 +9896,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>186.62</v>
+        <v>163.9</v>
       </c>
       <c r="V87" t="n">
         <v>62</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>45.25547445255474</v>
+        <v>44.60431654676259</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>4.52</v>
@@ -9866,7 +9920,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10011,20 +10065,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/16/2026 12:09</t>
+          <t>09/17/2026 19:26</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20371.33</v>
+        <v>20516.53</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>1.85</v>
+        <v>2.57</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.22</v>
+        <v>1.31</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,19 +10096,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>412.33</v>
+        <v>516.53</v>
       </c>
       <c r="V89" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>84.76190476190476</v>
+        <v>85.04672897196261</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.25</v>
+        <v>1.31</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10066,7 +10120,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10165,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/16/2026 12:01</t>
+          <t>09/17/2026 19:19</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>24579.1</v>
+        <v>25092.96</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>22.96</v>
+        <v>25.53</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.82</v>
+        <v>1.87</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10196,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>4559.57</v>
+        <v>5092.96</v>
       </c>
       <c r="V90" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>70.87378640776699</v>
+        <v>71.96261682242991</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.78</v>
+        <v>1.87</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10166,7 +10220,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10265,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/15/2026 10:18</t>
+          <t>09/17/2026 22:54</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10411,7 +10465,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/15/2026 10:24</t>
+          <t>09/17/2026 22:57</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10565,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/15/2026 10:18</t>
+          <t>09/17/2026 22:55</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10665,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/15/2026 10:10</t>
+          <t>09/17/2026 22:51</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10765,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/15/2026 09:49</t>
+          <t>09/17/2026 22:42</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10811,7 +10865,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/15/2026 10:09</t>
+          <t>09/17/2026 22:52</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +10965,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/15/2026 10:49</t>
+          <t>09/17/2026 23:08</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11011,7 +11065,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/15/2026 09:54</t>
+          <t>09/17/2026 22:44</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11211,20 +11265,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/16/2026 13:22</t>
+          <t>09/17/2026 20:08</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>20318.01</v>
+        <v>20793.95</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>1.58</v>
+        <v>3.96</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>1.52</v>
+        <v>2.3</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11242,19 +11296,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>679.45</v>
+        <v>793.95</v>
       </c>
       <c r="V101" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>75</v>
+        <v>76.92307692307693</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>2.11</v>
+        <v>2.3</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11266,7 +11320,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11311,20 +11365,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/15/2026 11:44</t>
+          <t>09/17/2026 23:19</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>20244.86</v>
+        <v>19867.25</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>1.24</v>
+        <v>-0.65</v>
       </c>
       <c r="J102" s="7" t="n">
-        <v>1.27</v>
+        <v>2.2</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>1.69</v>
+        <v>0.83</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11342,22 +11396,22 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>-192.9099999999999</v>
+        <v>-132.7499999999999</v>
       </c>
       <c r="V102" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>36.36363636363637</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>0.76</v>
+        <v>0.83</v>
       </c>
       <c r="Y102" s="7" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="Z102" t="inlineStr">
         <is>
@@ -11366,7 +11420,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11629,20 +11683,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/15/2026 03:11</t>
+          <t>09/17/2026 21:37</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11032.57</v>
+        <v>11298.08</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>10.3</v>
+        <v>12.95</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.46</v>
+        <v>2.83</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11838,20 +11892,20 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/15/2026 07:41</t>
+          <t>09/17/2026 22:17</t>
         </is>
       </c>
       <c r="H107" t="n">
-        <v>27123</v>
+        <v>26275</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-29.37</v>
+        <v>-31.59</v>
       </c>
       <c r="J107" s="7" t="n">
-        <v>37.71</v>
+        <v>38.12</v>
       </c>
       <c r="K107" s="7" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="L107" t="n">
         <v>25000</v>
@@ -11863,37 +11917,37 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-205.3</v>
+        <v>-910.63</v>
       </c>
       <c r="P107" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>77.5</v>
+        <v>30</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.494210396649421</v>
+        <v>0.1235177485177485</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>1.61</v>
+        <v>4.16</v>
       </c>
       <c r="T107" t="n">
-        <v>3753</v>
+        <v>3771</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-8102.999999999999</v>
+        <v>-8007.000000000001</v>
       </c>
       <c r="V107" t="n">
-        <v>2299</v>
+        <v>2311</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>61.25766053823608</v>
+        <v>61.28347918324052</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.78</v>
       </c>
       <c r="Y107" s="7" t="n">
-        <v>38.57</v>
+        <v>38.69</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -11902,7 +11956,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12220,7 +12274,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>09/14/2026 16:44</t>
+          <t>09/17/2026 16:46</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12948,7 +13002,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 10:40</t>
+          <t>09/17/2026 23:03</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12970,17 +13024,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13033,7 +13093,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>09/14/2026 20:47</t>
+          <t>09/17/2026 20:49</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13055,17 +13115,23 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q120" s="8" t="n"/>
-      <c r="R120" s="8" t="n"/>
-      <c r="S120" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q120" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R120" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S120" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13118,7 +13184,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/14/2026 15:10</t>
+          <t>09/17/2026 15:14</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -14369,7 +14435,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09/14/2026 16:44</t>
+          <t>09/17/2026 16:46</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14697,7 +14763,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>09/15/2026 10:40</t>
+          <t>09/17/2026 23:03</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14707,7 +14773,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14738,7 +14804,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>09/14/2026 20:47</t>
+          <t>09/17/2026 20:49</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14748,7 +14814,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -14779,7 +14845,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09/14/2026 15:10</t>
+          <t>09/17/2026 15:14</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -17362,7 +17428,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/16/2026 23:21</t>
+          <t>09/17/2026 20:46</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17431,7 +17497,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/16/2026 12:30</t>
+          <t>09/17/2026 19:39</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -17523,7 +17589,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09/14/2026 22:57</t>
+          <t>09/17/2026 22:58</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -17546,7 +17612,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09/14/2026 23:05</t>
+          <t>09/17/2026 23:08</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-18
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-17 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-18 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/17/2026 22:34</t>
+          <t>09/18/2026 14:17</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>51998.64</v>
+        <v>49141.42</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>137.7</v>
+        <v>124.64</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-4669.44</v>
+        <v>5470.130000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>72.5</v>
+        <v>77.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.9021612592580798</v>
+        <v>1.136651888461734</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>111.52</v>
+        <v>69.98</v>
       </c>
       <c r="T2" t="n">
-        <v>3423</v>
+        <v>3428</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>26998.64000000001</v>
+        <v>22378.89</v>
       </c>
       <c r="V2" t="n">
-        <v>2174</v>
+        <v>2177</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.51153958515921</v>
+        <v>63.50641773628938</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/15/2026 09:10</t>
+          <t>09/18/2026 09:13</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1715,15 +1715,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/15/2026 10:50</t>
+          <t>09/18/2026 10:53</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1824,11 +1824,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/15/2026 10:51</t>
+          <t>09/18/2026 10:54</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>09/15/2026 05:33</t>
+          <t>09/18/2026 05:37</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2591,7 +2591,7 @@
         </is>
       </c>
       <c r="F17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="F18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
         </is>
       </c>
       <c r="F19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -2918,11 +2918,11 @@
         </is>
       </c>
       <c r="F20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/17/2026 20:51</t>
+          <t>09/18/2026 12:11</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3027,11 +3027,11 @@
         </is>
       </c>
       <c r="F21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/17/2026 18:50</t>
+          <t>09/18/2026 15:34</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/17/2026 17:54</t>
+          <t>09/18/2026 14:42</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/17/2026 19:16</t>
+          <t>09/18/2026 00:13</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3289,22 +3289,22 @@
         <v>2.17</v>
       </c>
       <c r="T23" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-388.15</v>
+        <v>-400.4499999999999</v>
       </c>
       <c r="V23" t="n">
         <v>17</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>27.86885245901639</v>
+        <v>27.41935483870968</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>2</v>
+        <v>2.06</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3354,11 +3354,11 @@
         </is>
       </c>
       <c r="F24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/17/2026 23:20</t>
+          <t>09/18/2026 15:04</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="F25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/17/2026 23:02</t>
+          <t>09/18/2026 14:44</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20668.65</v>
+        <v>20679.69</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.17</v>
+        <v>-1.12</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,7 +3601,7 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>672.16</v>
+        <v>680.12</v>
       </c>
       <c r="P26" t="n">
         <v>22</v>
@@ -3610,7 +3610,7 @@
         <v>55.00000000000001</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.318788890575201</v>
+        <v>1.318330743451969</v>
       </c>
       <c r="S26" s="7" t="n">
         <v>5.01</v>
@@ -3619,16 +3619,16 @@
         <v>117</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>520.2199999999998</v>
+        <v>722.6699999999998</v>
       </c>
       <c r="V26" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>42.73504273504273</v>
+        <v>46.15384615384615</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.09</v>
+        <v>1.13</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3681,11 +3681,11 @@
         </is>
       </c>
       <c r="F27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/15/2026 08:36</t>
+          <t>09/18/2026 08:40</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,14 +3794,14 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/17/2026 23:08</t>
+          <t>09/18/2026 14:49</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>19658.67</v>
+        <v>19644.3</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>-1.73</v>
+        <v>-1.8</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>7.56</v>
@@ -3819,34 +3819,34 @@
         <v>40</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>72.99000000000004</v>
+        <v>28.70000000000003</v>
       </c>
       <c r="P28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>25</v>
+        <v>22.5</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>1.096816553919618</v>
+        <v>1.037368331966199</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>2.58</v>
+        <v>2.59</v>
       </c>
       <c r="T28" t="n">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-341.3300000000002</v>
+        <v>-355.7</v>
       </c>
       <c r="V28" t="n">
         <v>66</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>42.03821656050955</v>
       </c>
       <c r="X28" s="7" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="Y28" s="7" t="n">
         <v>7.56</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -3899,7 +3899,7 @@
         </is>
       </c>
       <c r="F29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/17/2026 23:22</t>
+          <t>09/18/2026 15:07</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20571.99</v>
+        <v>20563.28</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.88</v>
+        <v>2.84</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.59</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,7 +4037,7 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-240.15</v>
+        <v>-238.27</v>
       </c>
       <c r="P30" t="n">
         <v>9</v>
@@ -4046,25 +4046,25 @@
         <v>22.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.263975726369989</v>
+        <v>0.2655055487053021</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="T30" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>571.9899999999999</v>
+        <v>563.28</v>
       </c>
       <c r="V30" t="n">
         <v>23</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>25.84269662921348</v>
+        <v>25.27472527472527</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.59</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="F31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -4226,7 +4226,7 @@
         </is>
       </c>
       <c r="F32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4331,15 +4331,15 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/17/2026 21:00</t>
+          <t>09/18/2026 12:36</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Agg V1 Pro XAUUSD May 19</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4440,11 +4440,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -4557,14 +4557,14 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/17/2026 20:25</t>
+          <t>09/18/2026 10:57</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20281.8</v>
+        <v>20282.9</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>281.8</v>
+        <v>282.9</v>
       </c>
       <c r="V35" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>51.2396694214876</v>
+        <v>51.21951219512195</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>1.05</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4653,11 +4653,11 @@
         </is>
       </c>
       <c r="F36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/17/2026 19:37</t>
+          <t>09/18/2026 09:26</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="F37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="F38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -4980,7 +4980,7 @@
         </is>
       </c>
       <c r="F39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -5089,7 +5089,7 @@
         </is>
       </c>
       <c r="F40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -5198,11 +5198,11 @@
         </is>
       </c>
       <c r="F41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/15/2026 00:10</t>
+          <t>09/18/2026 00:14</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5307,11 +5307,11 @@
         </is>
       </c>
       <c r="F42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/15/2026 00:32</t>
+          <t>09/18/2026 00:35</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5333,22 +5333,13 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q42" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R42" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S42" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5416,11 +5407,11 @@
         </is>
       </c>
       <c r="F43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/15/2026 02:51</t>
+          <t>09/18/2026 02:54</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,22 +5433,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5529,20 +5511,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/17/2026 23:23</t>
+          <t>09/18/2026 15:07</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19480.16</v>
+        <v>19701.42</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-2.57</v>
+        <v>-1.46</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5551,37 +5533,28 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-353.1</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.1398085215230578</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>673</v>
+        <v>702</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-519.8400000000001</v>
+        <v>-300.92</v>
       </c>
       <c r="V44" t="n">
-        <v>377</v>
+        <v>393</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>56.01783060921248</v>
+        <v>55.98290598290598</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5593,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5638,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/17/2026 22:44</t>
+          <t>09/18/2026 14:26</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5660,22 +5633,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-41.96</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.4413526827319931</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>49</v>
@@ -5747,7 +5711,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/17/2026 22:57</t>
+          <t>09/18/2026 14:39</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5843,7 +5807,7 @@
         </is>
       </c>
       <c r="F47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -5943,11 +5907,11 @@
         </is>
       </c>
       <c r="F48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09/12/2026 12:43</t>
+          <t>09/18/2026 12:56</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6043,11 +6007,11 @@
         </is>
       </c>
       <c r="F49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/15/2026 00:19</t>
+          <t>09/18/2026 00:23</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6143,11 +6107,11 @@
         </is>
       </c>
       <c r="F50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/14/2026 23:59</t>
+          <t>09/18/2026 00:02</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6247,20 +6211,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/17/2026 22:47</t>
+          <t>09/18/2026 14:29</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19986.12</v>
+        <v>19801.08</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-0.05</v>
+        <v>-0.98</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
-      <c r="K51" t="n">
-        <v>1</v>
+      <c r="K51" s="7" t="n">
+        <v>0.96</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6278,19 +6242,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-13.88000000000056</v>
+        <v>-198.9200000000006</v>
       </c>
       <c r="V51" t="n">
         <v>17</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>30.35714285714285</v>
+        <v>29.82456140350877</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6302,7 +6266,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6347,14 +6311,14 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/17/2026 18:10</t>
-        </is>
-      </c>
-      <c r="H52" t="n">
-        <v>19645</v>
+          <t>09/18/2026 14:59</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="n">
+        <v>19672.74</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-1.75</v>
+        <v>-1.61</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>4.41</v>
@@ -6381,13 +6345,13 @@
         <v>102</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-355.0000000000002</v>
+        <v>-327.2600000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>40.19607843137255</v>
+        <v>41.17647058823529</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.93</v>
@@ -6402,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6447,20 +6411,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/17/2026 23:38</t>
+          <t>09/18/2026 15:21</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19779.12</v>
+        <v>19760.39</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.14</v>
+        <v>-1.23</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6478,16 +6442,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-220.8800000000001</v>
+        <v>-221.28</v>
       </c>
       <c r="V53" t="n">
         <v>135</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.06493506493506</v>
+        <v>34.61538461538461</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>0.83</v>
@@ -6502,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6643,11 +6607,11 @@
         </is>
       </c>
       <c r="F55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/17/2026 23:26</t>
+          <t>09/18/2026 15:10</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6743,7 +6707,7 @@
         </is>
       </c>
       <c r="F56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -6847,14 +6811,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/17/2026 22:57</t>
+          <t>09/18/2026 14:39</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19678.66</v>
+        <v>19685.98</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.6</v>
+        <v>-1.56</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6869,37 +6833,28 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>-37.61</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>0.4903103401544925</v>
-      </c>
-      <c r="S57" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>986</v>
+        <v>993</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-319.58</v>
+        <v>-329.19</v>
       </c>
       <c r="V57" t="n">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.81338742393509</v>
+        <v>43.60523665659618</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6911,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6956,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/17/2026 23:18</t>
+          <t>09/18/2026 15:02</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7052,7 +7007,7 @@
         </is>
       </c>
       <c r="F59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -7152,11 +7107,11 @@
         </is>
       </c>
       <c r="F60" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/17/2026 23:10</t>
+          <t>09/18/2026 14:54</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7252,11 +7207,11 @@
         </is>
       </c>
       <c r="F61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/17/2026 18:48</t>
+          <t>09/18/2026 15:32</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7352,7 +7307,7 @@
         </is>
       </c>
       <c r="F62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -7456,7 +7411,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/17/2026 23:30</t>
+          <t>09/18/2026 15:14</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7552,11 +7507,11 @@
         </is>
       </c>
       <c r="F64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/17/2026 18:48</t>
+          <t>09/18/2026 15:33</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7652,11 +7607,11 @@
         </is>
       </c>
       <c r="F65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/17/2026 23:30</t>
+          <t>09/18/2026 15:14</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7752,11 +7707,11 @@
         </is>
       </c>
       <c r="F66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/17/2026 23:17</t>
+          <t>09/18/2026 15:01</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7856,20 +7811,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/17/2026 18:48</t>
+          <t>09/18/2026 15:33</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>19557.89</v>
+        <v>20450.83</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>-2.19</v>
+        <v>2.27</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.06</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7878,40 +7833,31 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>-123.7900000000002</v>
+        <v>0</v>
       </c>
       <c r="P67" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q67" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R67" s="7" t="n">
-        <v>0.9759118434571438</v>
-      </c>
-      <c r="S67" s="7" t="n">
-        <v>12.15</v>
+        <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>-442.1100000000005</v>
+        <v>928.1599999999994</v>
       </c>
       <c r="V67" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>31.81818181818182</v>
+        <v>32.85714285714285</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.13</v>
       </c>
       <c r="Y67" s="7" t="n">
-        <v>11.38</v>
+        <v>11.37</v>
       </c>
       <c r="Z67" t="inlineStr">
         <is>
@@ -7920,7 +7866,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7961,7 +7907,7 @@
         </is>
       </c>
       <c r="F68" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -8365,7 +8311,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/17/2026 23:28</t>
+          <t>09/18/2026 15:13</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8465,7 +8411,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/17/2026 19:46</t>
+          <t>09/18/2026 09:51</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8565,7 +8511,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/17/2026 23:30</t>
+          <t>09/18/2026 15:14</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8665,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/17/2026 19:40</t>
+          <t>09/18/2026 09:37</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8765,7 +8711,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/17/2026 23:16</t>
+          <t>09/18/2026 15:01</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8865,7 +8811,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/17/2026 18:53</t>
+          <t>09/18/2026 07:39</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8965,7 +8911,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/17/2026 23:36</t>
+          <t>09/18/2026 15:19</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9065,7 +9011,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/17/2026 18:53</t>
+          <t>09/18/2026 07:37</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9165,7 +9111,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/17/2026 18:46</t>
+          <t>09/18/2026 15:29</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9265,7 +9211,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/17/2026 23:15</t>
+          <t>09/18/2026 14:59</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9365,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/17/2026 19:30</t>
+          <t>09/18/2026 08:47</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9465,7 +9411,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/17/2026 18:52</t>
+          <t>09/18/2026 07:37</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9561,11 +9507,11 @@
         </is>
       </c>
       <c r="F84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/17/2026 19:50</t>
+          <t>09/18/2026 09:58</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9661,11 +9607,11 @@
         </is>
       </c>
       <c r="F85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>09/15/2026 01:40</t>
+          <t>09/18/2026 01:42</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9865,7 +9811,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/17/2026 19:43</t>
+          <t>09/18/2026 09:46</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9896,16 +9842,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>163.9</v>
+        <v>160.6</v>
       </c>
       <c r="V87" t="n">
         <v>62</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>44.60431654676259</v>
+        <v>44.28571428571428</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>1.09</v>
@@ -9920,7 +9866,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10065,20 +10011,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/17/2026 19:26</t>
+          <t>09/18/2026 08:40</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20516.53</v>
+        <v>20289.53</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>2.57</v>
+        <v>1.44</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.31</v>
+        <v>1.15</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10096,19 +10042,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>516.53</v>
+        <v>289.53</v>
       </c>
       <c r="V89" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>85.04672897196261</v>
+        <v>83.78378378378379</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.31</v>
+        <v>1.15</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10120,7 +10066,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10165,20 +10111,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/17/2026 19:19</t>
+          <t>09/18/2026 08:17</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>25092.96</v>
+        <v>25418.51</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>25.53</v>
+        <v>27.16</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.87</v>
+        <v>1.93</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10196,19 +10142,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>5092.96</v>
+        <v>5418.51</v>
       </c>
       <c r="V90" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>71.96261682242991</v>
+        <v>71.17117117117117</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.87</v>
+        <v>1.93</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10220,7 +10166,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10265,7 +10211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/17/2026 22:54</t>
+          <t>09/18/2026 14:35</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10465,7 +10411,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/17/2026 22:57</t>
+          <t>09/18/2026 14:38</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10565,7 +10511,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/17/2026 22:55</t>
+          <t>09/18/2026 14:37</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10665,7 +10611,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/17/2026 22:51</t>
+          <t>09/18/2026 14:33</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10765,7 +10711,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/17/2026 22:42</t>
+          <t>09/18/2026 14:25</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10865,7 +10811,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/17/2026 22:52</t>
+          <t>09/18/2026 14:35</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10965,7 +10911,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/17/2026 23:08</t>
+          <t>09/18/2026 14:49</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11065,7 +11011,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/17/2026 22:44</t>
+          <t>09/18/2026 14:26</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11265,20 +11211,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/17/2026 20:08</t>
+          <t>09/18/2026 10:29</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>20793.95</v>
+        <v>20872.45</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>3.96</v>
+        <v>4.35</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>2.3</v>
+        <v>2.43</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11296,19 +11242,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>793.95</v>
+        <v>872.45</v>
       </c>
       <c r="V101" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>76.92307692307693</v>
+        <v>78.57142857142857</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>2.3</v>
+        <v>2.43</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11320,7 +11266,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11365,7 +11311,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/17/2026 23:19</t>
+          <t>09/18/2026 06:08</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11683,20 +11629,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/17/2026 21:37</t>
+          <t>09/18/2026 13:18</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11298.08</v>
+        <v>11477.16</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>12.95</v>
+        <v>14.74</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.83</v>
+        <v>3.08</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11714,19 +11660,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1408.61</v>
+        <v>1587.69</v>
       </c>
       <c r="V105" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>69.56521739130434</v>
+        <v>70.83333333333334</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.35</v>
+        <v>3.65</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11738,7 +11684,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11783,7 +11729,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/15/2026 09:09</t>
+          <t>09/18/2026 09:13</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11892,14 +11838,14 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/17/2026 22:17</t>
-        </is>
-      </c>
-      <c r="H107" t="n">
-        <v>26275</v>
+          <t>09/18/2026 13:59</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="n">
+        <v>26243.88</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-31.59</v>
+        <v>-31.67</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>38.12</v>
@@ -11917,31 +11863,31 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-910.63</v>
+        <v>-547.88</v>
       </c>
       <c r="P107" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.1235177485177485</v>
+        <v>0.2957750099615676</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>4.16</v>
+        <v>2.58</v>
       </c>
       <c r="T107" t="n">
-        <v>3771</v>
+        <v>3778</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-8007.000000000001</v>
+        <v>-8038.12</v>
       </c>
       <c r="V107" t="n">
-        <v>2311</v>
+        <v>2315</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>61.28347918324052</v>
+        <v>61.27580730545262</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.78</v>
@@ -11956,7 +11902,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12001,7 +11947,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 08:21</t>
+          <t>09/18/2026 08:24</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12092,7 +12038,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 04:53</t>
+          <t>09/18/2026 04:57</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12456,7 +12402,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/12/2026 13:02</t>
+          <t>09/18/2026 13:13</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12543,11 +12489,11 @@
         </is>
       </c>
       <c r="F114" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 09:08</t>
+          <t>09/18/2026 09:12</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12634,7 +12580,7 @@
         </is>
       </c>
       <c r="F115" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
@@ -12711,7 +12657,7 @@
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Claude Asian Sweep + NY Killzone</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D116" s="8" t="inlineStr">
@@ -12721,15 +12667,15 @@
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F116" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 05:19</t>
+          <t>09/18/2026 05:22</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12816,7 +12762,7 @@
         </is>
       </c>
       <c r="F117" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
@@ -12911,7 +12857,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/14/2026 23:47</t>
+          <t>09/17/2026 23:50</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13002,7 +12948,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/17/2026 23:03</t>
+          <t>09/18/2026 14:44</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13024,23 +12970,17 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>67.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q119" s="9" t="n">
-        <v>65</v>
-      </c>
-      <c r="R119" s="9" t="n">
-        <v>1.223174978645115</v>
-      </c>
-      <c r="S119" s="9" t="n">
-        <v>0.57</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q119" s="8" t="n"/>
+      <c r="R119" s="8" t="n"/>
+      <c r="S119" s="8" t="n"/>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13115,23 +13055,17 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>-6156.77</v>
+        <v>0</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q120" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="R120" s="9" t="n">
-        <v>0.01160528233794505</v>
-      </c>
-      <c r="S120" s="9" t="n">
-        <v>31.03</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q120" s="8" t="n"/>
+      <c r="R120" s="8" t="n"/>
+      <c r="S120" s="8" t="n"/>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13864,7 +13798,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 06:27</t>
+          <t>09/18/2026 06:29</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13955,7 +13889,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 05:58</t>
+          <t>09/18/2026 06:01</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14137,7 +14071,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/15/2026 11:17</t>
+          <t>09/18/2026 11:20</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14312,7 +14246,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/15/2026 08:21</t>
+          <t>09/18/2026 08:24</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14353,7 +14287,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/15/2026 04:53</t>
+          <t>09/18/2026 04:57</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14517,7 +14451,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09/12/2026 13:02</t>
+          <t>09/18/2026 13:13</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14558,7 +14492,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/15/2026 09:08</t>
+          <t>09/18/2026 09:12</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14625,7 +14559,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Claude Asian Sweep + NY Killzone</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -14635,12 +14569,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/15/2026 05:19</t>
+          <t>09/18/2026 05:22</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14722,7 +14656,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/14/2026 23:47</t>
+          <t>09/17/2026 23:50</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14763,7 +14697,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>09/17/2026 23:03</t>
+          <t>09/18/2026 14:44</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14773,7 +14707,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -14814,7 +14748,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -15173,7 +15107,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/15/2026 06:27</t>
+          <t>09/18/2026 06:29</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15214,7 +15148,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/15/2026 05:58</t>
+          <t>09/18/2026 06:01</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15296,7 +15230,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/15/2026 11:17</t>
+          <t>09/18/2026 11:20</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -15320,7 +15254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -15557,7 +15491,7 @@
         </is>
       </c>
       <c r="D11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -15682,7 +15616,7 @@
         </is>
       </c>
       <c r="D16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -15707,7 +15641,7 @@
         </is>
       </c>
       <c r="D17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -15732,7 +15666,7 @@
         </is>
       </c>
       <c r="D18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -15757,7 +15691,7 @@
         </is>
       </c>
       <c r="D19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -15782,7 +15716,7 @@
         </is>
       </c>
       <c r="D20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -16118,17 +16052,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>56912</t>
+          <t>55966</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>licensed</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Smart Owl FX</t>
+          <t>Range Snap USDJPY</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -16136,39 +16070,39 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>56915</t>
+          <t>56912</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>licensed</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Prop</t>
+          <t>Smart Owl FX</t>
         </is>
       </c>
       <c r="D35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>57677</t>
+          <t>56915</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -16178,7 +16112,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 RCLOCK</t>
+          <t>T&amp;D19L13 L8 Prop</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -16186,24 +16120,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>57681</t>
+          <t>57575</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>licensed</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Demo AuRange Gold Reaper + DC + TALON</t>
+          <t>Gold Snap 1.1</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -16211,14 +16145,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>57685</t>
+          <t>57677</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -16228,36 +16162,36 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gold Talon Vt15 Demo</t>
+          <t>T&amp;D19L13 Meta4 RCLOCK</t>
         </is>
       </c>
       <c r="D38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>57703</t>
+          <t>57681</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>licensed</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Gold Snap Demo 2</t>
+          <t>Demo AuRange Gold Reaper + DC + TALON</t>
         </is>
       </c>
       <c r="D39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -16268,7 +16202,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>57710</t>
+          <t>57685</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -16278,7 +16212,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Donchian H6 5520</t>
+          <t>Gold Talon Vt15 Demo</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -16286,24 +16220,24 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>57825</t>
+          <t>57686</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LIVE Portfolio: Midnight Raven + Gold Reaper + AuRange</t>
+          <t>Talon V2 Stocks</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -16311,14 +16245,14 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>58303</t>
+          <t>57687</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -16328,7 +16262,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Prop</t>
+          <t>Chaos Fractal Alligator</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -16336,14 +16270,14 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>58304</t>
+          <t>57688</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -16353,7 +16287,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 MOL</t>
+          <t>Squeeze Breakout Indices</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -16361,14 +16295,14 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>58305</t>
+          <t>57689</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -16378,7 +16312,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Agg</t>
+          <t>VWAP Mean Reversion</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -16386,14 +16320,14 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>58306</t>
+          <t>57691</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -16403,7 +16337,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Prop</t>
+          <t>Gold Overnight</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -16411,14 +16345,14 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>58307</t>
+          <t>57694</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -16428,7 +16362,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 MOL</t>
+          <t>Dream Talon Book</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -16436,14 +16370,14 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>58308</t>
+          <t>57695</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -16453,7 +16387,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Agg</t>
+          <t>Dual Thrust Strategy</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -16461,14 +16395,14 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>58309</t>
+          <t>57703</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -16478,11 +16412,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DreamCatcher New Sleeves V3</t>
+          <t>Gold Snap Demo 2</t>
         </is>
       </c>
       <c r="D48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -16493,17 +16427,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>58314</t>
+          <t>57710</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>licensed</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LunaAI Pro</t>
+          <t>Donchian H6 5520</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -16511,24 +16445,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>58318</t>
+          <t>57825</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Agg</t>
+          <t>LIVE Portfolio: Midnight Raven + Gold Reaper + AuRange</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -16536,14 +16470,14 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>58319</t>
+          <t>58303</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -16553,7 +16487,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop</t>
+          <t>T&amp;D19L13 L8 Prop</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -16568,7 +16502,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>58320</t>
+          <t>58304</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -16578,7 +16512,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL</t>
+          <t>T&amp;D19L13 L8 MOL</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -16593,7 +16527,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>58321</t>
+          <t>58305</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -16603,7 +16537,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg</t>
+          <t>T&amp;D19L13 L8 Agg</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -16618,7 +16552,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>58322</t>
+          <t>58306</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -16628,7 +16562,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 RCLOCK</t>
+          <t>T&amp;D19L13 L11 Prop</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -16643,7 +16577,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>58323</t>
+          <t>58307</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -16653,7 +16587,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Prop</t>
+          <t>T&amp;D19L13 L11 MOL</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -16668,7 +16602,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>58324</t>
+          <t>58308</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -16678,7 +16612,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop</t>
+          <t>T&amp;D19L13 L11 Agg</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -16693,7 +16627,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>58325</t>
+          <t>58309</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -16703,7 +16637,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Agg</t>
+          <t>DreamCatcher New Sleeves V3</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -16711,14 +16645,14 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>58326</t>
+          <t>58310</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -16728,7 +16662,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Agg Control</t>
+          <t>Donchian H2 Portfolio</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -16736,14 +16670,14 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>58327</t>
+          <t>58311</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -16753,7 +16687,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 MOL</t>
+          <t>Donchian H6 Portfolio</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -16761,14 +16695,14 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>58328</t>
+          <t>58312</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -16778,7 +16712,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 RCLOCK</t>
+          <t>DreamCatcher DCv3</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -16786,14 +16720,14 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>58329</t>
+          <t>58313</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -16803,7 +16737,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 MOL</t>
+          <t>Zfade Portfolio 2</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -16811,24 +16745,24 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>58314</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>licensed</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>LunaAI Pro</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -16836,49 +16770,49 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>58315</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>Gold SuperScalp</t>
         </is>
       </c>
       <c r="D63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>662436</t>
+          <t>58316</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 GBPJPY + XAUUSD</t>
+          <t>3EMA Core5 (DD ERC)</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -16886,24 +16820,24 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>663097</t>
+          <t>58318</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 USDJPY, GBPJPY + XAGUSD</t>
+          <t>T&amp;D19L13 L10 Agg</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -16911,14 +16845,14 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1115443</t>
+          <t>58319</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -16928,22 +16862,22 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta MOL</t>
+          <t>T&amp;D19L13 Meta4 Prop</t>
         </is>
       </c>
       <c r="D66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>600025868</t>
+          <t>58320</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -16953,13 +16887,563 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>FTMO Manual Trading</t>
+          <t>T&amp;D19L13 Meta4 MOL</t>
         </is>
       </c>
       <c r="D67" t="b">
         <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>58321</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta4 Agg</t>
+        </is>
+      </c>
+      <c r="D68" t="b">
+        <v>1</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>58322</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta4 RCLOCK</t>
+        </is>
+      </c>
+      <c r="D69" t="b">
+        <v>1</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>58323</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 Prop</t>
+        </is>
+      </c>
+      <c r="D70" t="b">
+        <v>1</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>58324</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L10 Prop</t>
+        </is>
+      </c>
+      <c r="D71" t="b">
+        <v>1</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>58325</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 Agg</t>
+        </is>
+      </c>
+      <c r="D72" t="b">
+        <v>1</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>58326</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 Agg Control</t>
+        </is>
+      </c>
+      <c r="D73" t="b">
+        <v>1</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>58327</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 MOL</t>
+        </is>
+      </c>
+      <c r="D74" t="b">
+        <v>1</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>58328</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 RCLOCK</t>
+        </is>
+      </c>
+      <c r="D75" t="b">
+        <v>1</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>58329</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L10 MOL</t>
+        </is>
+      </c>
+      <c r="D76" t="b">
+        <v>1</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>58991</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Golden Fractal</t>
+        </is>
+      </c>
+      <c r="D77" t="b">
+        <v>1</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>VPS242</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>58993</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Levels</t>
+        </is>
+      </c>
+      <c r="D78" t="b">
+        <v>1</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>59376</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>For Gold Snap 2HR / Smart Gold Hunter</t>
+        </is>
+      </c>
+      <c r="D79" t="b">
+        <v>1</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>59377</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Gold Snap 2HR</t>
+        </is>
+      </c>
+      <c r="D80" t="b">
+        <v>1</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>662434</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>LIVE Gold Reaper Conservative</t>
+        </is>
+      </c>
+      <c r="D81" t="b">
+        <v>1</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>662435</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Aggv1 Pro Filter 60</t>
+        </is>
+      </c>
+      <c r="D82" t="b">
+        <v>0</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>662436</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>LIVE Talon v2 GBPJPY + XAUUSD</t>
+        </is>
+      </c>
+      <c r="D83" t="b">
+        <v>1</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>663097</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>LIVE Gold Talon V2 USDJPY, GBPJPY + XAGUSD</t>
+        </is>
+      </c>
+      <c r="D84" t="b">
+        <v>1</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1115442</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Gold Snap Internal</t>
+        </is>
+      </c>
+      <c r="D85" t="b">
+        <v>1</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1115443</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta MOL</t>
+        </is>
+      </c>
+      <c r="D86" t="b">
+        <v>0</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1115444</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Gold Snap Demo</t>
+        </is>
+      </c>
+      <c r="D87" t="b">
+        <v>1</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>14189968</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+        </is>
+      </c>
+      <c r="D88" t="b">
+        <v>0</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>600025868</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>FTMO Manual Trading</t>
+        </is>
+      </c>
+      <c r="D89" t="b">
+        <v>1</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -17037,7 +17521,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09/15/2026 07:35</t>
+          <t>09/18/2026 07:39</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17106,7 +17590,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/15/2026 04:14</t>
+          <t>09/18/2026 04:18</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17175,7 +17659,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09/15/2026 03:46</t>
+          <t>09/18/2026 03:49</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17244,7 +17728,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/15/2026 08:36</t>
+          <t>09/18/2026 08:40</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17290,7 +17774,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/15/2026 07:22</t>
+          <t>09/18/2026 07:25</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17382,7 +17866,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/15/2026 09:35</t>
+          <t>09/18/2026 09:37</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17405,7 +17889,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/15/2026 04:05</t>
+          <t>09/18/2026 04:08</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -17428,7 +17912,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/17/2026 20:46</t>
+          <t>09/18/2026 11:48</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17451,7 +17935,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/15/2026 08:41</t>
+          <t>09/18/2026 08:45</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -17497,7 +17981,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/17/2026 19:39</t>
+          <t>09/18/2026 09:33</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -17750,7 +18234,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/15/2026 07:21</t>
+          <t>09/18/2026 07:24</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -17773,7 +18257,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/15/2026 08:00</t>
+          <t>09/18/2026 08:03</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -17796,7 +18280,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/15/2026 11:09</t>
+          <t>09/18/2026 11:12</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -17819,7 +18303,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/16/2026 13:41</t>
+          <t>09/18/2026 13:45</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-22
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-18 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-21 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/18/2026 14:17</t>
+          <t>09/21/2026 20:10</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>49141.42</v>
+        <v>45765.55</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>124.64</v>
+        <v>109.21</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>5470.130000000001</v>
+        <v>630.5900000000009</v>
       </c>
       <c r="P2" t="n">
         <v>31</v>
@@ -994,10 +994,10 @@
         <v>77.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.136651888461734</v>
+        <v>1.014501398995556</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>69.98</v>
+        <v>73.14</v>
       </c>
       <c r="T2" t="n">
         <v>3428</v>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>09/16/2026 19:57</t>
+          <t>09/19/2026 20:01</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>09/17/2026 09:19</t>
+          <t>09/20/2026 09:22</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>09/16/2026 10:01</t>
+          <t>09/19/2026 10:04</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>09/16/2026 17:50</t>
+          <t>09/19/2026 17:53</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/18/2026 09:13</t>
+          <t>09/21/2026 09:17</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/18/2026 10:53</t>
+          <t>09/21/2026 10:56</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/18/2026 10:54</t>
+          <t>09/21/2026 10:57</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>09/16/2026 22:08</t>
+          <t>09/19/2026 22:11</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>09/18/2026 05:37</t>
+          <t>09/21/2026 05:41</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09/17/2026 10:38</t>
+          <t>09/20/2026 10:40</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>09/16/2026 13:12</t>
+          <t>09/19/2026 13:16</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/16/2026 22:28</t>
+          <t>09/19/2026 22:32</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>09/17/2026 06:04</t>
+          <t>09/20/2026 06:07</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09/17/2026 06:04</t>
+          <t>09/20/2026 06:09</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/18/2026 12:11</t>
+          <t>09/21/2026 23:11</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/18/2026 15:34</t>
+          <t>09/19/2026 00:56</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/18/2026 14:42</t>
+          <t>09/21/2026 20:35</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3180,7 +3180,7 @@
         <v>4.88</v>
       </c>
       <c r="T22" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="U22" s="7" t="n">
         <v>-755.73</v>
@@ -3189,7 +3189,7 @@
         <v>47</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>48.45360824742268</v>
+        <v>47</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.86</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/18/2026 00:13</t>
+          <t>09/21/2026 21:46</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19611.85</v>
+        <v>19609.65</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.1</v>
+        <v>-2.11</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2.16</v>
+        <v>2.22</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-414.06</v>
+        <v>-403.99</v>
       </c>
       <c r="P23" t="n">
         <v>8</v>
@@ -3283,25 +3283,25 @@
         <v>20</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.2234870506160569</v>
+        <v>0.2022156835640515</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>2.17</v>
+        <v>2.07</v>
       </c>
       <c r="T23" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-400.4499999999999</v>
+        <v>-390.35</v>
       </c>
       <c r="V23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>27.41935483870968</v>
+        <v>27.69230769230769</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.06</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/18/2026 15:04</t>
+          <t>09/21/2026 20:54</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/17/2026 23:03</t>
+          <t>09/20/2026 23:05</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/18/2026 14:44</t>
+          <t>09/21/2026 20:35</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3619,7 +3619,7 @@
         <v>117</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>722.6699999999998</v>
+        <v>679.6899999999998</v>
       </c>
       <c r="V26" t="n">
         <v>54</v>
@@ -3628,7 +3628,7 @@
         <v>46.15384615384615</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/18/2026 08:40</t>
+          <t>09/21/2026 08:44</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,11 +3794,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/18/2026 14:49</t>
+          <t>09/21/2026 20:40</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>19644.3</v>
+        <v>19644.22</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>-1.8</v>
@@ -3834,16 +3834,16 @@
         <v>2.59</v>
       </c>
       <c r="T28" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-355.7</v>
+        <v>-355.7800000000001</v>
       </c>
       <c r="V28" t="n">
         <v>66</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>42.03821656050955</v>
+        <v>41.77215189873418</v>
       </c>
       <c r="X28" s="7" t="n">
         <v>0.89</v>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>09/16/2026 10:31</t>
+          <t>09/19/2026 10:34</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/18/2026 15:07</t>
+          <t>09/21/2026 20:56</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/17/2026 10:39</t>
+          <t>09/20/2026 10:41</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>09/17/2026 11:34</t>
+          <t>09/20/2026 11:36</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/18/2026 12:36</t>
+          <t>09/21/2026 23:20</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/17/2026 00:32</t>
+          <t>09/20/2026 00:35</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,11 +4557,11 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/18/2026 10:57</t>
+          <t>09/21/2026 22:43</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20282.9</v>
+        <v>20283.78</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>1.43</v>
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>282.9</v>
+        <v>283.78</v>
       </c>
       <c r="V35" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>51.21951219512195</v>
+        <v>51.2</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>1.05</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/18/2026 09:26</t>
+          <t>09/21/2026 21:56</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/16/2026 22:33</t>
+          <t>09/19/2026 22:37</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>09/16/2026 14:54</t>
+          <t>09/19/2026 14:58</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>09/16/2026 09:47</t>
+          <t>09/19/2026 09:50</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>09/16/2026 09:08</t>
+          <t>09/19/2026 09:10</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/18/2026 00:14</t>
+          <t>09/21/2026 00:17</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/18/2026 00:35</t>
+          <t>09/21/2026 00:38</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/18/2026 02:54</t>
+          <t>09/21/2026 02:57</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5511,14 +5511,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/18/2026 15:07</t>
+          <t>09/21/2026 20:56</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19701.42</v>
+        <v>19697.66</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.46</v>
+        <v>-1.48</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5542,16 +5542,16 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-300.92</v>
+        <v>-302.34</v>
       </c>
       <c r="V44" t="n">
-        <v>393</v>
+        <v>407</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.98290598290598</v>
+        <v>57.00280112044818</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/18/2026 14:26</t>
+          <t>09/21/2026 20:17</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/18/2026 14:39</t>
+          <t>09/21/2026 20:30</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/17/2026 23:35</t>
+          <t>09/20/2026 23:37</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09/18/2026 12:56</t>
+          <t>09/21/2026 12:57</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/18/2026 00:23</t>
+          <t>09/21/2026 00:26</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/18/2026 00:02</t>
+          <t>09/21/2026 00:04</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6211,20 +6211,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/18/2026 14:29</t>
+          <t>09/21/2026 20:21</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19801.08</v>
+        <v>19611.45</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-0.98</v>
+        <v>-1.93</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6242,19 +6242,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-198.9200000000006</v>
+        <v>-388.5500000000005</v>
       </c>
       <c r="V51" t="n">
         <v>17</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>29.82456140350877</v>
+        <v>29.3103448275862</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,20 +6311,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/18/2026 14:59</t>
+          <t>09/21/2026 20:48</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19672.74</v>
+        <v>19716.87</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-1.61</v>
+        <v>-1.38</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>4.41</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6342,19 +6342,19 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-327.2600000000002</v>
+        <v>-283.1300000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>41.17647058823529</v>
+        <v>40.18691588785047</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>4.43</v>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,14 +6411,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/18/2026 15:21</t>
+          <t>09/21/2026 21:11</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19760.39</v>
+        <v>19765.4</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.23</v>
+        <v>-1.2</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6442,19 +6442,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-221.28</v>
+        <v>-234.6</v>
       </c>
       <c r="V53" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>34.61538461538461</v>
+        <v>35.18987341772151</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/18/2026 15:10</t>
+          <t>09/21/2026 21:00</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>09/12/2026 17:49</t>
+          <t>09/19/2026 09:40</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6811,20 +6811,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/18/2026 14:39</t>
+          <t>09/21/2026 20:31</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19685.98</v>
+        <v>19694.77</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.56</v>
+        <v>-1.52</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6842,19 +6842,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>993</v>
+        <v>1013</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-329.19</v>
+        <v>-304.76</v>
       </c>
       <c r="V57" t="n">
-        <v>433</v>
+        <v>446</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.60523665659618</v>
+        <v>44.02764067127345</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/18/2026 15:02</t>
+          <t>09/21/2026 16:05</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>09/16/2026 10:45</t>
+          <t>09/19/2026 10:47</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/18/2026 14:54</t>
+          <t>09/21/2026 20:43</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/18/2026 15:32</t>
+          <t>09/21/2026 21:26</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>09/17/2026 21:06</t>
+          <t>09/20/2026 21:08</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/18/2026 15:14</t>
+          <t>09/21/2026 21:05</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/18/2026 15:33</t>
+          <t>09/21/2026 21:24</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/18/2026 15:14</t>
+          <t>09/21/2026 21:03</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/18/2026 15:01</t>
+          <t>09/21/2026 20:52</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,20 +7811,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/18/2026 15:33</t>
+          <t>09/21/2026 21:22</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20450.83</v>
+        <v>21586.55</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>2.27</v>
+        <v>7.96</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.06</v>
+        <v>1.21</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7842,19 +7842,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>928.1599999999994</v>
+        <v>1586.549999999999</v>
       </c>
       <c r="V67" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>32.85714285714285</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.13</v>
+        <v>1.21</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>09/16/2026 10:42</t>
+          <t>09/19/2026 10:45</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>09/16/2026 22:21</t>
+          <t>09/19/2026 22:25</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>09/16/2026 22:22</t>
+          <t>09/19/2026 22:25</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/16/2026 22:20</t>
+          <t>09/19/2026 22:24</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/18/2026 15:13</t>
+          <t>09/21/2026 21:06</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/18/2026 09:51</t>
+          <t>09/21/2026 22:03</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/18/2026 15:14</t>
+          <t>09/21/2026 21:02</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/18/2026 09:37</t>
+          <t>09/20/2026 20:33</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/18/2026 15:01</t>
+          <t>09/20/2026 19:19</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/18/2026 07:39</t>
+          <t>09/20/2026 19:56</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/18/2026 15:19</t>
+          <t>09/20/2026 19:45</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/18/2026 07:37</t>
+          <t>09/20/2026 20:01</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/18/2026 15:29</t>
+          <t>09/20/2026 19:51</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/18/2026 14:59</t>
+          <t>09/20/2026 19:16</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/18/2026 08:47</t>
+          <t>09/20/2026 20:28</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/18/2026 07:37</t>
+          <t>09/20/2026 19:59</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/18/2026 09:58</t>
+          <t>09/21/2026 22:08</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>09/18/2026 01:42</t>
+          <t>09/21/2026 01:46</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>09/17/2026 19:31</t>
+          <t>09/20/2026 19:34</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9811,20 +9811,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/18/2026 09:46</t>
+          <t>09/21/2026 17:16</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20163.9</v>
+        <v>20323.39</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.61</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9842,19 +9842,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>160.6</v>
+        <v>323.3900000000001</v>
       </c>
       <c r="V87" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>44.28571428571428</v>
+        <v>44.29530201342282</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>4.52</v>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9911,7 +9911,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>09/16/2026 11:02</t>
+          <t>09/19/2026 11:04</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10011,20 +10011,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/18/2026 08:40</t>
+          <t>09/21/2026 21:50</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20289.53</v>
+        <v>20341.03</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>1.44</v>
+        <v>1.69</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.15</v>
+        <v>1.18</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,19 +10042,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>289.53</v>
+        <v>341.03</v>
       </c>
       <c r="V89" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>83.78378378378379</v>
+        <v>84.21052631578947</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.15</v>
+        <v>1.18</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10111,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/18/2026 08:17</t>
+          <t>09/21/2026 21:44</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>25418.51</v>
+        <v>25973.21</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>27.16</v>
+        <v>29.93</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.93</v>
+        <v>2.02</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10142,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>5418.51</v>
+        <v>5973.21</v>
       </c>
       <c r="V90" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>71.17117117117117</v>
+        <v>71.30434782608695</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.93</v>
+        <v>2.02</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/18/2026 14:35</t>
+          <t>09/20/2026 18:53</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>09/16/2026 16:36</t>
+          <t>09/19/2026 16:39</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/18/2026 14:38</t>
+          <t>09/20/2026 13:41</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/18/2026 14:37</t>
+          <t>09/20/2026 13:37</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/18/2026 14:33</t>
+          <t>09/20/2026 13:32</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10711,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/18/2026 14:25</t>
+          <t>09/20/2026 23:37</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10811,7 +10811,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/18/2026 14:35</t>
+          <t>09/20/2026 18:52</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/18/2026 14:49</t>
+          <t>09/20/2026 19:08</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/18/2026 14:26</t>
+          <t>09/20/2026 23:39</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>09/16/2026 16:42</t>
+          <t>09/19/2026 16:44</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/18/2026 10:29</t>
+          <t>09/21/2026 22:27</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11311,20 +11311,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/18/2026 06:08</t>
+          <t>09/21/2026 20:52</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>19867.25</v>
+        <v>19887.65</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>-0.65</v>
+        <v>-0.54</v>
       </c>
       <c r="J102" s="7" t="n">
         <v>2.2</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11342,19 +11342,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>-132.7499999999999</v>
+        <v>-112.35</v>
       </c>
       <c r="V102" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>40.42553191489361</v>
+        <v>40</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>2.2</v>
@@ -11366,7 +11366,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11411,7 +11411,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>09/12/2026 17:24</t>
+          <t>09/19/2026 09:26</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>09/16/2026 21:38</t>
+          <t>09/19/2026 21:42</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11629,20 +11629,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/18/2026 13:18</t>
+          <t>09/21/2026 23:58</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11477.16</v>
+        <v>11588.5</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>14.74</v>
+        <v>15.85</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>3.08</v>
+        <v>3.24</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11660,19 +11660,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1587.69</v>
+        <v>1699.03</v>
       </c>
       <c r="V105" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>70.83333333333334</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.65</v>
+        <v>3.84</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11684,7 +11684,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/18/2026 09:13</t>
+          <t>09/21/2026 09:16</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11838,14 +11838,14 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/18/2026 13:59</t>
+          <t>09/21/2026 19:50</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>26243.88</v>
+        <v>26266.46</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-31.67</v>
+        <v>-31.61</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>38.12</v>
@@ -11863,19 +11863,19 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-547.88</v>
+        <v>-478.54</v>
       </c>
       <c r="P107" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>40</v>
+        <v>42.5</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.2957750099615676</v>
+        <v>0.3455684258030989</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>2.58</v>
+        <v>2.39</v>
       </c>
       <c r="T107" t="n">
         <v>3778</v>
@@ -11947,7 +11947,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 08:24</t>
+          <t>09/21/2026 08:27</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 04:57</t>
+          <t>09/21/2026 05:00</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 20:07</t>
+          <t>09/19/2026 20:10</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12220,7 +12220,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>09/17/2026 16:46</t>
+          <t>09/20/2026 16:50</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12311,7 +12311,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 10:09</t>
+          <t>09/19/2026 10:13</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12402,7 +12402,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 13:13</t>
+          <t>09/21/2026 13:15</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 09:12</t>
+          <t>09/21/2026 09:15</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12584,7 +12584,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 13:09</t>
+          <t>09/19/2026 13:11</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 05:22</t>
+          <t>09/21/2026 05:26</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12766,7 +12766,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 17:31</t>
+          <t>09/19/2026 17:35</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12857,7 +12857,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/17/2026 23:50</t>
+          <t>09/20/2026 23:53</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12948,7 +12948,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 14:44</t>
+          <t>09/19/2026 11:02</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13118,7 +13118,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/17/2026 15:14</t>
+          <t>09/20/2026 15:16</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13203,7 +13203,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 22:21</t>
+          <t>09/19/2026 22:25</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13288,7 +13288,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 16:51</t>
+          <t>09/19/2026 16:54</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 16:51</t>
+          <t>09/19/2026 16:54</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 16:51</t>
+          <t>09/19/2026 16:54</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 16:59</t>
+          <t>09/19/2026 17:03</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 17:23</t>
+          <t>09/19/2026 17:26</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13713,7 +13713,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>09/16/2026 16:50</t>
+          <t>09/19/2026 16:52</t>
         </is>
       </c>
       <c r="H128" s="9" t="n">
@@ -13798,7 +13798,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 06:29</t>
+          <t>09/21/2026 06:32</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13889,7 +13889,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 06:01</t>
+          <t>09/21/2026 06:04</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14071,7 +14071,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/18/2026 11:20</t>
+          <t>09/21/2026 11:22</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14246,7 +14246,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/18/2026 08:24</t>
+          <t>09/21/2026 08:27</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/18/2026 04:57</t>
+          <t>09/21/2026 05:00</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>09/16/2026 20:07</t>
+          <t>09/19/2026 20:10</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14369,7 +14369,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09/17/2026 16:46</t>
+          <t>09/20/2026 16:50</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14410,7 +14410,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>09/16/2026 10:09</t>
+          <t>09/19/2026 10:13</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14451,7 +14451,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09/18/2026 13:13</t>
+          <t>09/21/2026 13:15</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/18/2026 09:12</t>
+          <t>09/21/2026 09:15</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>09/16/2026 13:09</t>
+          <t>09/19/2026 13:11</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14574,7 +14574,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/18/2026 05:22</t>
+          <t>09/21/2026 05:26</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>09/16/2026 17:31</t>
+          <t>09/19/2026 17:35</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14656,7 +14656,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/17/2026 23:50</t>
+          <t>09/20/2026 23:53</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>09/18/2026 14:44</t>
+          <t>09/19/2026 11:02</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09/17/2026 15:14</t>
+          <t>09/20/2026 15:16</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/16/2026 22:21</t>
+          <t>09/19/2026 22:25</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14861,7 +14861,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>09/16/2026 16:51</t>
+          <t>09/19/2026 16:54</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14902,7 +14902,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>09/16/2026 16:51</t>
+          <t>09/19/2026 16:54</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>09/16/2026 16:51</t>
+          <t>09/19/2026 16:54</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14984,7 +14984,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>09/16/2026 16:59</t>
+          <t>09/19/2026 17:03</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -15025,7 +15025,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>09/16/2026 17:23</t>
+          <t>09/19/2026 17:26</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>09/16/2026 16:50</t>
+          <t>09/19/2026 16:52</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/18/2026 06:29</t>
+          <t>09/21/2026 06:32</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15148,7 +15148,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/18/2026 06:01</t>
+          <t>09/21/2026 06:04</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15230,7 +15230,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/18/2026 11:20</t>
+          <t>09/21/2026 11:22</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17521,7 +17521,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09/18/2026 07:39</t>
+          <t>09/21/2026 07:42</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09/16/2026 13:23</t>
+          <t>09/19/2026 13:27</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17567,7 +17567,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/15/2026 07:26</t>
+          <t>09/21/2026 07:34</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17590,7 +17590,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/18/2026 04:18</t>
+          <t>09/21/2026 04:21</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17613,7 +17613,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09/16/2026 21:48</t>
+          <t>09/19/2026 21:51</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17636,7 +17636,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09/16/2026 08:40</t>
+          <t>09/19/2026 08:42</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17659,7 +17659,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09/18/2026 03:49</t>
+          <t>09/21/2026 03:52</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17682,7 +17682,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09/16/2026 08:41</t>
+          <t>09/19/2026 08:44</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -17705,7 +17705,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09/16/2026 16:07</t>
+          <t>09/19/2026 16:10</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -17728,7 +17728,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/18/2026 08:40</t>
+          <t>09/21/2026 08:44</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17751,7 +17751,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09/16/2026 18:07</t>
+          <t>09/19/2026 18:10</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17774,7 +17774,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/18/2026 07:25</t>
+          <t>09/21/2026 07:28</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17820,7 +17820,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09/16/2026 21:57</t>
+          <t>09/19/2026 22:01</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17843,7 +17843,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09/16/2026 21:49</t>
+          <t>09/19/2026 21:52</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -17866,7 +17866,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/18/2026 09:37</t>
+          <t>09/21/2026 09:41</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17889,7 +17889,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/18/2026 04:08</t>
+          <t>09/21/2026 04:11</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -17912,7 +17912,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/18/2026 11:48</t>
+          <t>09/21/2026 11:50</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17935,7 +17935,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/18/2026 08:45</t>
+          <t>09/21/2026 08:48</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -17981,7 +17981,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/18/2026 09:33</t>
+          <t>09/21/2026 09:37</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18004,7 +18004,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09/12/2026 14:53</t>
+          <t>09/19/2026 07:50</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09/16/2026 17:08</t>
+          <t>09/19/2026 17:11</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18050,7 +18050,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09/16/2026 17:07</t>
+          <t>09/19/2026 17:11</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18073,7 +18073,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09/17/2026 22:58</t>
+          <t>09/20/2026 23:01</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18096,7 +18096,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09/17/2026 23:08</t>
+          <t>09/20/2026 23:10</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18119,7 +18119,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09/16/2026 16:57</t>
+          <t>09/19/2026 17:00</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18142,7 +18142,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>09/16/2026 17:45</t>
+          <t>09/19/2026 17:48</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18165,7 +18165,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>09/16/2026 08:40</t>
+          <t>09/19/2026 08:42</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18188,7 +18188,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>09/12/2026 16:05</t>
+          <t>09/19/2026 08:47</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -18234,7 +18234,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/18/2026 07:24</t>
+          <t>09/21/2026 07:28</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/18/2026 08:03</t>
+          <t>09/21/2026 08:06</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18303,7 +18303,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/18/2026 13:45</t>
+          <t>09/21/2026 13:53</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-23
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-21 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-23 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/22/2026 00:59</t>
+          <t>09/23/2026 20:40</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>45765.55</v>
+        <v>41968.61</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>109.21</v>
+        <v>91.84999999999999</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>630.5900000000009</v>
+        <v>-4667.879999999999</v>
       </c>
       <c r="P2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>77.5</v>
+        <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.014501398995556</v>
+        <v>0.904524563875895</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>73.14</v>
+        <v>73.11</v>
       </c>
       <c r="T2" t="n">
-        <v>3433</v>
+        <v>3440</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>20765.54999999999</v>
+        <v>16968.60999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2180</v>
+        <v>2185</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.50131080687446</v>
+        <v>63.51744186046512</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>09/19/2026 20:01</t>
+          <t>09/22/2026 23:03</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>09/20/2026 09:22</t>
+          <t>09/23/2026 09:30</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>09/19/2026 10:04</t>
+          <t>09/22/2026 10:07</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>09/19/2026 17:53</t>
+          <t>09/22/2026 19:49</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>09/19/2026 22:11</t>
+          <t>09/23/2026 02:29</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09/20/2026 10:40</t>
+          <t>09/23/2026 10:47</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>09/19/2026 13:16</t>
+          <t>09/22/2026 13:22</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/19/2026 22:32</t>
+          <t>09/23/2026 02:59</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>09/20/2026 06:07</t>
+          <t>09/23/2026 06:10</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09/20/2026 06:09</t>
+          <t>09/23/2026 06:14</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/21/2026 23:11</t>
+          <t>09/22/2026 12:04</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3140,17 +3140,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/21/2026 20:35</t>
+          <t>09/23/2026 21:35</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>19244.27</v>
+        <v>19157.55</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-3.77</v>
+        <v>-4.21</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>6.1</v>
+        <v>7.42</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>0.86</v>
@@ -3165,37 +3165,37 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-821.1400000000001</v>
+        <v>-202.05</v>
       </c>
       <c r="P22" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>42.5</v>
+        <v>47.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.6961565359610139</v>
+        <v>0.9186125668158399</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>4.88</v>
+        <v>6.12</v>
       </c>
       <c r="T22" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-755.73</v>
+        <v>-842.4499999999999</v>
       </c>
       <c r="V22" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>47</v>
+        <v>49.03846153846153</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.86</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>6.11</v>
+        <v>7.43</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,11 +3249,11 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/21/2026 21:46</t>
+          <t>09/23/2026 11:05</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19609.65</v>
+        <v>19609.69</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>-2.11</v>
@@ -3262,7 +3262,7 @@
         <v>2.22</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,31 +3274,31 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-403.99</v>
+        <v>-288.61</v>
       </c>
       <c r="P23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.2022156835640515</v>
+        <v>0.2698593402145315</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>2.07</v>
+        <v>1.49</v>
       </c>
       <c r="T23" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-390.35</v>
+        <v>-400.05</v>
       </c>
       <c r="V23" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>27.69230769230769</v>
+        <v>27.53623188405797</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.36</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/21/2026 20:54</t>
+          <t>09/23/2026 22:18</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/20/2026 23:05</t>
+          <t>09/23/2026 23:09</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/21/2026 20:35</t>
+          <t>09/23/2026 21:37</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20679.69</v>
+        <v>20649.08</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.12</v>
+        <v>-1.27</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>680.12</v>
+        <v>379.93</v>
       </c>
       <c r="P26" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>52.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.318330743451969</v>
+        <v>1.175314817292917</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5.01</v>
+        <v>5.08</v>
       </c>
       <c r="T26" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>679.6899999999998</v>
+        <v>649.0799999999998</v>
       </c>
       <c r="V26" t="n">
         <v>54</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>46.15384615384615</v>
+        <v>45</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3794,11 +3794,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/21/2026 20:40</t>
+          <t>09/23/2026 21:46</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>19644.22</v>
+        <v>19643.7</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>-1.8</v>
@@ -3834,16 +3834,16 @@
         <v>2.59</v>
       </c>
       <c r="T28" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-355.7800000000001</v>
+        <v>-356.3000000000001</v>
       </c>
       <c r="V28" t="n">
         <v>66</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>41.77215189873418</v>
+        <v>40.99378881987577</v>
       </c>
       <c r="X28" s="7" t="n">
         <v>0.89</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>09/19/2026 10:34</t>
+          <t>09/22/2026 11:11</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/21/2026 20:56</t>
+          <t>09/23/2026 22:21</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20563.28</v>
+        <v>20599.16</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.84</v>
+        <v>3.02</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.59</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.68</v>
+        <v>1.72</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-238.27</v>
+        <v>-181.6</v>
       </c>
       <c r="P30" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>22.5</v>
+        <v>27.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.2655055487053021</v>
+        <v>0.4007589506682065</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="T30" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>563.28</v>
+        <v>599.1600000000001</v>
       </c>
       <c r="V30" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>25.27472527472527</v>
+        <v>26.88172043010752</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.68</v>
+        <v>1.72</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.59</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/20/2026 10:41</t>
+          <t>09/23/2026 10:48</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>09/20/2026 11:36</t>
+          <t>09/23/2026 11:42</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/21/2026 23:20</t>
+          <t>09/23/2026 16:05</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/20/2026 00:35</t>
+          <t>09/23/2026 03:41</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/21/2026 22:43</t>
+          <t>09/23/2026 14:10</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20283.78</v>
+        <v>20466.22</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1.43</v>
+        <v>2.34</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.05</v>
+        <v>1.08</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>283.78</v>
+        <v>563.24</v>
       </c>
       <c r="V35" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>51.2</v>
+        <v>52.30769230769231</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.05</v>
+        <v>1.09</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/21/2026 21:56</t>
+          <t>09/23/2026 11:29</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/19/2026 22:37</t>
+          <t>09/23/2026 03:07</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>09/19/2026 14:58</t>
+          <t>09/22/2026 15:40</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>09/19/2026 09:50</t>
+          <t>09/22/2026 09:54</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>09/19/2026 09:10</t>
+          <t>09/22/2026 09:13</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5511,20 +5511,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/21/2026 20:56</t>
+          <t>09/23/2026 22:21</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19697.66</v>
+        <v>19752.71</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.48</v>
+        <v>-1.2</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5542,19 +5542,19 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>714</v>
+        <v>732</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-302.34</v>
+        <v>-247.2900000000001</v>
       </c>
       <c r="V44" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>57.00280112044818</v>
+        <v>56.4207650273224</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/21/2026 20:17</t>
+          <t>09/23/2026 20:54</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5711,20 +5711,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/21/2026 20:30</t>
+          <t>09/23/2026 21:25</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19815.81</v>
+        <v>19695.6</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-0.89</v>
+        <v>-1.49</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.95</v>
+        <v>0.91</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5742,19 +5742,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-184.1899999999999</v>
+        <v>-304.4</v>
       </c>
       <c r="V46" t="n">
         <v>39</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>45.34883720930232</v>
+        <v>44.31818181818182</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/20/2026 23:37</t>
+          <t>09/23/2026 23:43</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -6211,20 +6211,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/21/2026 20:21</t>
+          <t>09/23/2026 21:08</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19611.45</v>
+        <v>19819.05</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-1.93</v>
+        <v>-0.89</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6242,19 +6242,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-388.5500000000005</v>
+        <v>-180.9500000000005</v>
       </c>
       <c r="V51" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>29.3103448275862</v>
+        <v>31.14754098360656</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,20 +6311,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/21/2026 20:48</t>
+          <t>09/23/2026 22:05</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19716.87</v>
+        <v>19515.22</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-1.38</v>
+        <v>-2.39</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>4.41</v>
+        <v>5.23</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6342,22 +6342,22 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-283.1300000000002</v>
+        <v>-484.7800000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>40.18691588785047</v>
+        <v>40</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>4.43</v>
+        <v>5.26</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,20 +6411,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/21/2026 21:11</t>
+          <t>09/23/2026 22:53</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19765.4</v>
+        <v>19768.33</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.2</v>
+        <v>-1.18</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6442,19 +6442,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>395</v>
+        <v>406</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-234.6</v>
+        <v>-231.6700000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.18987341772151</v>
+        <v>35.71428571428572</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/17/2026 21:15</t>
+          <t>09/23/2026 21:23</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/21/2026 21:00</t>
+          <t>09/23/2026 22:30</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>09/19/2026 09:40</t>
+          <t>09/22/2026 09:44</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6811,20 +6811,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/21/2026 20:31</t>
+          <t>09/23/2026 21:24</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19694.77</v>
+        <v>19636.28</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.52</v>
+        <v>-1.81</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6842,19 +6842,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1013</v>
+        <v>1043</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-304.76</v>
+        <v>-363.2500000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>446</v>
+        <v>458</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.02764067127345</v>
+        <v>43.9117929050815</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/21/2026 16:05</t>
+          <t>09/23/2026 08:22</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>09/19/2026 10:47</t>
+          <t>09/22/2026 11:30</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/21/2026 20:43</t>
+          <t>09/23/2026 21:55</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/21/2026 21:26</t>
+          <t>09/23/2026 23:26</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>09/20/2026 21:08</t>
+          <t>09/23/2026 21:14</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,20 +7411,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/21/2026 21:05</t>
+          <t>09/23/2026 22:41</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18726.69</v>
+        <v>18664.19</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.39</v>
+        <v>-6.7</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7442,19 +7442,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1273.31</v>
+        <v>-1335.81</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>12.28070175438596</v>
+        <v>12.06896551724138</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7466,7 +7466,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/21/2026 21:24</t>
+          <t>09/23/2026 23:21</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/21/2026 21:03</t>
+          <t>09/23/2026 22:37</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/21/2026 20:52</t>
+          <t>09/23/2026 22:12</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,20 +7811,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/21/2026 21:22</t>
+          <t>09/23/2026 23:19</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>21586.55</v>
+        <v>22003.75</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>7.96</v>
+        <v>10.05</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.21</v>
+        <v>1.25</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7842,19 +7842,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>1586.549999999999</v>
+        <v>2003.75</v>
       </c>
       <c r="V67" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>34.21052631578947</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.21</v>
+        <v>1.25</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>09/19/2026 10:45</t>
+          <t>09/22/2026 11:30</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>09/19/2026 22:25</t>
+          <t>09/23/2026 02:49</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8033,13 +8033,22 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>0</v>
+        <v>-35.83</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q69" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R69" s="7" t="n">
+        <v>0.5722812462695476</v>
+      </c>
+      <c r="S69" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T69" t="n">
         <v>55</v>
@@ -8111,7 +8120,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>09/19/2026 22:25</t>
+          <t>09/23/2026 02:48</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8220,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/19/2026 22:24</t>
+          <t>09/23/2026 02:47</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8233,13 +8242,22 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O71" s="7" t="n">
-        <v>0</v>
+        <v>19946.4</v>
       </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Q71" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R71" s="7" t="n">
+        <v>278.6503340757238</v>
+      </c>
+      <c r="S71" s="7" t="n">
+        <v>0.17</v>
       </c>
       <c r="T71" t="n">
         <v>7</v>
@@ -8271,7 +8289,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC71" t="inlineStr">
@@ -8311,7 +8329,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/21/2026 21:06</t>
+          <t>09/23/2026 22:41</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8429,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/21/2026 22:03</t>
+          <t>09/23/2026 11:44</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8511,7 +8529,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/21/2026 21:02</t>
+          <t>09/23/2026 22:35</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8711,7 +8729,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/20/2026 19:19</t>
+          <t>09/23/2026 19:25</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8829,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/20/2026 19:56</t>
+          <t>09/23/2026 20:02</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +8929,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/20/2026 19:45</t>
+          <t>09/23/2026 19:48</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9029,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/20/2026 20:01</t>
+          <t>09/23/2026 20:06</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9211,7 +9229,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/20/2026 19:16</t>
+          <t>09/23/2026 19:20</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9233,13 +9251,22 @@
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O81" s="7" t="n">
-        <v>0</v>
+        <v>698.3099999999999</v>
       </c>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="Q81" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="R81" s="7" t="n">
+        <v>4.02390334733469</v>
+      </c>
+      <c r="S81" s="7" t="n">
+        <v>0.64</v>
       </c>
       <c r="T81" t="n">
         <v>2303</v>
@@ -9311,7 +9338,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/20/2026 20:28</t>
+          <t>09/23/2026 20:33</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9411,7 +9438,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/20/2026 19:59</t>
+          <t>09/23/2026 20:02</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9433,13 +9460,22 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>0</v>
+        <v>1042.88</v>
       </c>
       <c r="P83" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q83" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R83" s="7" t="n">
+        <v>1.768473487193091</v>
+      </c>
+      <c r="S83" s="7" t="n">
+        <v>3.89</v>
       </c>
       <c r="T83" t="n">
         <v>67</v>
@@ -9511,7 +9547,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/21/2026 22:08</t>
+          <t>09/23/2026 12:01</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9711,7 +9747,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>09/20/2026 19:34</t>
+          <t>09/23/2026 19:40</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9811,20 +9847,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/21/2026 17:16</t>
+          <t>09/23/2026 11:52</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20323.39</v>
+        <v>20316.59</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>1.61</v>
+        <v>1.58</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9842,19 +9878,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>323.3900000000001</v>
+        <v>310.96</v>
       </c>
       <c r="V87" t="n">
         <v>66</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>44.29530201342282</v>
+        <v>43.13725490196079</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>4.52</v>
@@ -9866,7 +9902,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9911,7 +9947,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>09/19/2026 11:04</t>
+          <t>09/22/2026 11:42</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10011,20 +10047,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/21/2026 21:50</t>
+          <t>09/23/2026 11:17</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20341.03</v>
+        <v>20478.91</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>1.69</v>
+        <v>2.38</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.18</v>
+        <v>1.25</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,19 +10078,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>341.03</v>
+        <v>514.21</v>
       </c>
       <c r="V89" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>84.21052631578947</v>
+        <v>85</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.18</v>
+        <v>1.27</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10066,7 +10102,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10147,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/21/2026 21:44</t>
+          <t>09/23/2026 11:02</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>25973.21</v>
+        <v>25914.47</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>29.93</v>
+        <v>29.64</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>2.02</v>
+        <v>1.93</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10178,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>5973.21</v>
+        <v>5699.240000000001</v>
       </c>
       <c r="V90" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>71.30434782608695</v>
+        <v>69.10569105691057</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>2.02</v>
+        <v>1.87</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10166,7 +10202,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10247,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/20/2026 18:53</t>
+          <t>09/23/2026 18:58</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10311,7 +10347,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>09/19/2026 16:39</t>
+          <t>09/22/2026 18:04</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10411,7 +10447,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/20/2026 13:41</t>
+          <t>09/23/2026 13:49</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10547,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/20/2026 13:37</t>
+          <t>09/23/2026 13:45</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10647,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/20/2026 13:32</t>
+          <t>09/23/2026 13:35</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10747,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/20/2026 23:37</t>
+          <t>09/23/2026 23:39</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10811,7 +10847,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/20/2026 18:52</t>
+          <t>09/23/2026 18:59</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +10947,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/20/2026 19:08</t>
+          <t>09/23/2026 19:11</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11011,7 +11047,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/20/2026 23:39</t>
+          <t>09/23/2026 23:43</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11111,7 +11147,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>09/19/2026 16:44</t>
+          <t>09/22/2026 18:11</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11211,7 +11247,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/21/2026 22:27</t>
+          <t>09/23/2026 13:16</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11242,19 +11278,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>872.45</v>
+        <v>897.2</v>
       </c>
       <c r="V101" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>78.57142857142857</v>
+        <v>80</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>2.43</v>
+        <v>2.47</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11266,7 +11302,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11311,20 +11347,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/21/2026 20:52</t>
+          <t>09/23/2026 22:11</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>19887.65</v>
+        <v>19961.06</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>-0.54</v>
+        <v>-0.17</v>
       </c>
       <c r="J102" s="7" t="n">
         <v>2.2</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>0.86</v>
+        <v>0.95</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11342,19 +11378,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>-112.35</v>
+        <v>-38.93999999999996</v>
       </c>
       <c r="V102" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>40</v>
+        <v>37.93103448275862</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>0.86</v>
+        <v>0.95</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>2.2</v>
@@ -11366,7 +11402,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11411,7 +11447,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>09/19/2026 09:26</t>
+          <t>09/22/2026 09:29</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
@@ -11520,7 +11556,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>09/19/2026 21:42</t>
+          <t>09/23/2026 01:39</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11629,20 +11665,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/21/2026 23:58</t>
+          <t>09/23/2026 18:09</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11588.5</v>
+        <v>11559.62</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>15.85</v>
+        <v>15.56</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>3.24</v>
+        <v>2.89</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11660,19 +11696,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1699.03</v>
+        <v>1670.15</v>
       </c>
       <c r="V105" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>71.42857142857143</v>
+        <v>70.58823529411765</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.84</v>
+        <v>3.34</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11684,7 +11720,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11838,17 +11874,17 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/22/2026 00:39</t>
+          <t>09/23/2026 19:55</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>26266.46</v>
+        <v>25885.08</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-31.61</v>
+        <v>-32.6</v>
       </c>
       <c r="J107" s="7" t="n">
-        <v>38.12</v>
+        <v>38.74</v>
       </c>
       <c r="K107" s="7" t="n">
         <v>0.78</v>
@@ -11863,37 +11899,37 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-478.54</v>
+        <v>-283.51</v>
       </c>
       <c r="P107" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>42.5</v>
+        <v>37.5</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.3455684258030989</v>
+        <v>0.4600220935547768</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>2.39</v>
+        <v>1.69</v>
       </c>
       <c r="T107" t="n">
-        <v>3779</v>
+        <v>3791</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-8015.54</v>
+        <v>-8396.920000000002</v>
       </c>
       <c r="V107" t="n">
         <v>2316</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>61.2860545117756</v>
+        <v>61.09206014244263</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.78</v>
       </c>
       <c r="Y107" s="7" t="n">
-        <v>38.69</v>
+        <v>39.64</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -11902,7 +11938,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12129,7 +12165,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 20:10</t>
+          <t>09/22/2026 23:18</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12220,7 +12256,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>09/20/2026 16:50</t>
+          <t>09/23/2026 16:54</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12311,7 +12347,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 10:13</t>
+          <t>09/22/2026 10:16</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12584,7 +12620,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 13:11</t>
+          <t>09/22/2026 13:18</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12766,7 +12802,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 17:35</t>
+          <t>09/22/2026 19:24</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12948,7 +12984,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 11:02</t>
+          <t>09/22/2026 11:41</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13033,7 +13069,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>09/17/2026 20:49</t>
+          <t>09/23/2026 20:55</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13118,7 +13154,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/20/2026 15:16</t>
+          <t>09/23/2026 15:23</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13140,17 +13176,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13203,7 +13245,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 22:25</t>
+          <t>09/23/2026 02:49</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13288,7 +13330,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 16:54</t>
+          <t>09/22/2026 18:26</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13373,7 +13415,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 16:54</t>
+          <t>09/22/2026 18:26</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13458,7 +13500,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 16:54</t>
+          <t>09/22/2026 18:26</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13543,7 +13585,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 17:03</t>
+          <t>09/22/2026 18:38</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13628,7 +13670,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 17:26</t>
+          <t>09/22/2026 19:12</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13713,7 +13755,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>09/19/2026 16:52</t>
+          <t>09/22/2026 18:24</t>
         </is>
       </c>
       <c r="H128" s="9" t="n">
@@ -14328,7 +14370,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>09/19/2026 20:10</t>
+          <t>09/22/2026 23:18</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14369,7 +14411,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09/20/2026 16:50</t>
+          <t>09/23/2026 16:54</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14410,7 +14452,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>09/19/2026 10:13</t>
+          <t>09/22/2026 10:16</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14533,7 +14575,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>09/19/2026 13:11</t>
+          <t>09/22/2026 13:18</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14615,7 +14657,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>09/19/2026 17:35</t>
+          <t>09/22/2026 19:24</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14697,7 +14739,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>09/19/2026 11:02</t>
+          <t>09/22/2026 11:41</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14738,7 +14780,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>09/17/2026 20:49</t>
+          <t>09/23/2026 20:55</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14779,7 +14821,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09/20/2026 15:16</t>
+          <t>09/23/2026 15:23</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14789,7 +14831,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14820,7 +14862,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/19/2026 22:25</t>
+          <t>09/23/2026 02:49</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14861,7 +14903,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>09/19/2026 16:54</t>
+          <t>09/22/2026 18:26</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14902,7 +14944,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>09/19/2026 16:54</t>
+          <t>09/22/2026 18:26</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14943,7 +14985,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>09/19/2026 16:54</t>
+          <t>09/22/2026 18:26</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14984,7 +15026,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>09/19/2026 17:03</t>
+          <t>09/22/2026 18:38</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -15025,7 +15067,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>09/19/2026 17:26</t>
+          <t>09/22/2026 19:12</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15066,7 +15108,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>09/19/2026 16:52</t>
+          <t>09/22/2026 18:24</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -17544,7 +17586,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09/19/2026 13:27</t>
+          <t>09/22/2026 13:49</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17613,7 +17655,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09/19/2026 21:51</t>
+          <t>09/23/2026 01:56</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17636,7 +17678,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09/19/2026 08:42</t>
+          <t>09/22/2026 08:46</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17682,7 +17724,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09/19/2026 08:44</t>
+          <t>09/22/2026 08:48</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -17705,7 +17747,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09/19/2026 16:10</t>
+          <t>09/22/2026 17:19</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -17751,7 +17793,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09/19/2026 18:10</t>
+          <t>09/22/2026 20:15</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17820,7 +17862,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09/19/2026 22:01</t>
+          <t>09/23/2026 02:12</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17843,7 +17885,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09/19/2026 21:52</t>
+          <t>09/23/2026 01:57</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -18004,7 +18046,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09/19/2026 07:50</t>
+          <t>09/22/2026 07:52</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18027,7 +18069,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09/19/2026 17:11</t>
+          <t>09/22/2026 18:49</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18050,7 +18092,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09/19/2026 17:11</t>
+          <t>09/22/2026 18:49</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18073,7 +18115,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09/20/2026 23:01</t>
+          <t>09/23/2026 23:04</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18096,7 +18138,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09/20/2026 23:10</t>
+          <t>09/23/2026 23:18</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18119,7 +18161,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09/19/2026 17:00</t>
+          <t>09/22/2026 18:34</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18142,7 +18184,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>09/19/2026 17:48</t>
+          <t>09/22/2026 19:45</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18165,7 +18207,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>09/19/2026 08:42</t>
+          <t>09/22/2026 08:46</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18188,7 +18230,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>09/19/2026 08:47</t>
+          <t>09/22/2026 08:51</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -18303,7 +18345,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/21/2026 13:53</t>
+          <t>09/23/2026 13:58</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-25
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-23 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-24 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/23/2026 20:40</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>41968.61</v>
+          <t>09/24/2026 19:47</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>40042</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>91.84999999999999</v>
+        <v>83.04000000000001</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-4667.879999999999</v>
+        <v>-1334.639999999999</v>
       </c>
       <c r="P2" t="n">
         <v>30</v>
@@ -994,22 +994,22 @@
         <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.904524563875895</v>
+        <v>0.9705176248335509</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>73.11</v>
+        <v>50.52</v>
       </c>
       <c r="T2" t="n">
-        <v>3440</v>
+        <v>3443</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>16968.60999999999</v>
+        <v>15041.99999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2185</v>
+        <v>2186</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.51744186046512</v>
+        <v>63.49114144641301</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.03</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/21/2026 09:17</t>
+          <t>09/24/2026 11:34</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/21/2026 10:56</t>
+          <t>09/24/2026 13:18</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/21/2026 10:57</t>
+          <t>09/24/2026 13:19</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>09/21/2026 05:41</t>
+          <t>09/24/2026 06:57</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/23/2026 21:35</t>
+          <t>09/24/2026 20:39</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>19157.55</v>
+        <v>19028.34</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-4.21</v>
+        <v>-4.86</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>7.42</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3165,7 +3165,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-202.05</v>
+        <v>-245.8200000000001</v>
       </c>
       <c r="P22" t="n">
         <v>19</v>
@@ -3174,25 +3174,25 @@
         <v>47.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.9186125668158399</v>
+        <v>0.9026971824853345</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>6.12</v>
+        <v>6.1</v>
       </c>
       <c r="T22" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-842.4499999999999</v>
+        <v>-971.66</v>
       </c>
       <c r="V22" t="n">
         <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>49.03846153846153</v>
+        <v>48.57142857142857</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="Y22" s="7" t="n">
         <v>7.43</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/23/2026 11:05</t>
+          <t>09/24/2026 23:06</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19609.69</v>
+        <v>19582.09</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.11</v>
+        <v>-2.25</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2.22</v>
+        <v>2.31</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,37 +3274,37 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-288.61</v>
+        <v>-298.98</v>
       </c>
       <c r="P23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.2698593402145315</v>
+        <v>0.2170223909912269</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>1.49</v>
       </c>
       <c r="T23" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-400.05</v>
+        <v>-417.91</v>
       </c>
       <c r="V23" t="n">
         <v>19</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>27.53623188405797</v>
+        <v>27.14285714285714</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>2.06</v>
+        <v>2.15</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/23/2026 22:18</t>
+          <t>09/24/2026 21:20</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/23/2026 21:37</t>
+          <t>09/24/2026 20:40</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20649.08</v>
+        <v>20501.48</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.27</v>
+        <v>-1.98</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>379.93</v>
+        <v>539.25</v>
       </c>
       <c r="P26" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>52.5</v>
+        <v>50</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.175314817292917</v>
+        <v>1.291489637725813</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5.08</v>
+        <v>5</v>
       </c>
       <c r="T26" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>649.0799999999998</v>
+        <v>501.4799999999997</v>
       </c>
       <c r="V26" t="n">
         <v>54</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>45</v>
+        <v>44.26229508196721</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/21/2026 08:44</t>
+          <t>09/24/2026 10:47</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3834,19 +3834,19 @@
         <v>2.59</v>
       </c>
       <c r="T28" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-356.3000000000001</v>
+        <v>-353.8100000000002</v>
       </c>
       <c r="V28" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>40.99378881987577</v>
+        <v>41.56626506024097</v>
       </c>
       <c r="X28" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="Y28" s="7" t="n">
         <v>7.56</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/23/2026 22:21</t>
+          <t>09/24/2026 21:22</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20599.16</v>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>3.02</v>
+        <v>20594.26</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.59</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-181.6</v>
+        <v>-219.78</v>
       </c>
       <c r="P30" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>27.5</v>
+        <v>25</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.4007589506682065</v>
+        <v>0.2869610355903059</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="T30" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>599.1600000000001</v>
+        <v>594.2600000000001</v>
       </c>
       <c r="V30" t="n">
         <v>25</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>26.88172043010752</v>
+        <v>26.59574468085106</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.59</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>563.24</v>
+        <v>554.29</v>
       </c>
       <c r="V35" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.30769230769231</v>
+        <v>51.8796992481203</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>1.09</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/21/2026 00:17</t>
+          <t>09/24/2026 00:24</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/21/2026 00:38</t>
+          <t>09/24/2026 00:43</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5333,13 +5333,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5411,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/21/2026 02:57</t>
+          <t>09/24/2026 03:04</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5433,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5511,20 +5529,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/23/2026 22:21</t>
+          <t>09/24/2026 21:23</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19752.71</v>
+        <v>19799.57</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.2</v>
+        <v>-0.96</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5542,19 +5560,19 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>732</v>
+        <v>748</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-247.2900000000001</v>
+        <v>-200.4300000000002</v>
       </c>
       <c r="V44" t="n">
-        <v>413</v>
+        <v>423</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>56.4207650273224</v>
+        <v>56.55080213903744</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5566,7 +5584,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,20 +5629,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/23/2026 20:54</t>
+          <t>09/24/2026 20:00</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19978.19</v>
+        <v>19990.38</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.1</v>
+        <v>-0.04</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.73</v>
+        <v>0.89</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5642,22 +5660,22 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-21.81</v>
+        <v>-9.620000000000005</v>
       </c>
       <c r="V45" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>34.69387755102041</v>
+        <v>35.18518518518518</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.73</v>
+        <v>0.89</v>
       </c>
       <c r="Y45" s="7" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
@@ -5666,7 +5684,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5711,20 +5729,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/23/2026 21:25</t>
+          <t>09/24/2026 20:30</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19695.6</v>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>-1.49</v>
+        <v>19593.88</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-2</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5742,19 +5760,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-304.4</v>
+        <v>-406.12</v>
       </c>
       <c r="V46" t="n">
         <v>39</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>44.31818181818182</v>
+        <v>43.82022471910113</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5784,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5911,7 +5929,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09/21/2026 12:57</t>
+          <t>09/24/2026 15:57</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6011,7 +6029,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/21/2026 00:26</t>
+          <t>09/24/2026 00:33</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6111,7 +6129,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/21/2026 00:04</t>
+          <t>09/24/2026 00:11</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6211,20 +6229,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/23/2026 21:08</t>
+          <t>09/24/2026 20:14</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19819.05</v>
+        <v>19716.33</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-0.89</v>
+        <v>-1.4</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6233,28 +6251,37 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>0</v>
+        <v>332.1600000000001</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R51" s="7" t="n">
+        <v>1.087995464588289</v>
+      </c>
+      <c r="S51" s="7" t="n">
+        <v>6.33</v>
       </c>
       <c r="T51" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-180.9500000000005</v>
+        <v>-283.6700000000005</v>
       </c>
       <c r="V51" t="n">
         <v>19</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>31.14754098360656</v>
+        <v>30.64516129032258</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6266,7 +6293,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,20 +6338,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/23/2026 22:05</t>
+          <t>09/24/2026 21:07</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19515.22</v>
+        <v>19638.54</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-2.39</v>
+        <v>-1.77</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>5.23</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6342,22 +6369,22 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-484.7800000000002</v>
+        <v>-361.4600000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>40</v>
+        <v>40.17857142857143</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>5.26</v>
+        <v>5.25</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6366,7 +6393,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,20 +6438,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/23/2026 22:53</t>
+          <t>09/24/2026 21:55</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19768.33</v>
+        <v>19783.22</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.18</v>
+        <v>-1.11</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6433,28 +6460,37 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>0</v>
+        <v>-52.39</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q53" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R53" s="7" t="n">
+        <v>0.5529482037716529</v>
+      </c>
+      <c r="S53" s="7" t="n">
+        <v>0.48</v>
       </c>
       <c r="T53" t="n">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-231.6700000000001</v>
+        <v>-216.7800000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.71428571428572</v>
+        <v>36.4963503649635</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6502,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6611,7 +6647,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/23/2026 22:30</t>
+          <t>09/24/2026 21:32</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6811,20 +6847,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/23/2026 21:24</t>
+          <t>09/24/2026 20:29</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19636.28</v>
+        <v>19619.34</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.81</v>
+        <v>-1.89</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6833,28 +6869,37 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-66.18000000000001</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.1874769797421731</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.34</v>
       </c>
       <c r="T57" t="n">
-        <v>1043</v>
+        <v>1063</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-363.2500000000001</v>
+        <v>-380.1900000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.9117929050815</v>
+        <v>44.02634054562559</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6866,7 +6911,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6956,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/23/2026 08:22</t>
+          <t>09/24/2026 21:16</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -6933,13 +6978,22 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>0</v>
+        <v>-269.38</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q58" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R58" s="7" t="n">
+        <v>0.1222834055586328</v>
+      </c>
+      <c r="S58" s="7" t="n">
+        <v>1.35</v>
       </c>
       <c r="T58" t="n">
         <v>4426</v>
@@ -7111,7 +7165,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/23/2026 21:55</t>
+          <t>09/24/2026 20:57</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7265,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/23/2026 23:26</t>
+          <t>09/24/2026 22:26</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7411,7 +7465,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/23/2026 22:41</t>
+          <t>09/24/2026 21:43</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7511,7 +7565,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/23/2026 23:21</t>
+          <t>09/24/2026 22:20</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7665,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/23/2026 22:37</t>
+          <t>09/24/2026 21:38</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7711,7 +7765,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/23/2026 22:12</t>
+          <t>09/24/2026 21:14</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,20 +7865,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/23/2026 23:19</t>
+          <t>09/24/2026 22:19</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>22003.75</v>
+        <v>21695.62</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>10.05</v>
+        <v>8.51</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.25</v>
+        <v>1.21</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7833,28 +7887,37 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>0</v>
+        <v>-300.2500000000001</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q67" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R67" s="7" t="n">
+        <v>0.9461566326420819</v>
+      </c>
+      <c r="S67" s="7" t="n">
+        <v>13.51</v>
       </c>
       <c r="T67" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>2003.75</v>
+        <v>1695.62</v>
       </c>
       <c r="V67" t="n">
         <v>26</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>34.21052631578947</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.25</v>
+        <v>1.21</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7866,7 +7929,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8033,22 +8096,13 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>-35.83</v>
+        <v>0</v>
       </c>
       <c r="P69" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q69" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R69" s="7" t="n">
-        <v>0.5722812462695476</v>
-      </c>
-      <c r="S69" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="T69" t="n">
         <v>55</v>
@@ -8242,22 +8296,13 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O71" s="7" t="n">
-        <v>19946.4</v>
+        <v>0</v>
       </c>
       <c r="P71" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q71" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R71" s="7" t="n">
-        <v>278.6503340757238</v>
-      </c>
-      <c r="S71" s="7" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="T71" t="n">
         <v>7</v>
@@ -8289,7 +8334,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC71" t="inlineStr">
@@ -8329,7 +8374,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/23/2026 22:41</t>
+          <t>09/24/2026 21:45</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8429,7 +8474,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/23/2026 11:44</t>
+          <t>09/24/2026 23:35</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8529,7 +8574,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/23/2026 22:35</t>
+          <t>09/24/2026 21:36</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8751,13 +8796,22 @@
         <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O76" s="7" t="n">
-        <v>0</v>
+        <v>-212.9</v>
       </c>
       <c r="P76" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q76" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R76" s="7" t="n">
+        <v>0.5722322684348001</v>
+      </c>
+      <c r="S76" s="7" t="n">
+        <v>1.9</v>
       </c>
       <c r="T76" t="n">
         <v>313</v>
@@ -9251,22 +9305,13 @@
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O81" s="7" t="n">
-        <v>698.3099999999999</v>
+        <v>0</v>
       </c>
       <c r="P81" t="n">
-        <v>30</v>
-      </c>
-      <c r="Q81" s="7" t="n">
-        <v>75</v>
-      </c>
-      <c r="R81" s="7" t="n">
-        <v>4.02390334733469</v>
-      </c>
-      <c r="S81" s="7" t="n">
-        <v>0.64</v>
+        <v>0</v>
       </c>
       <c r="T81" t="n">
         <v>2303</v>
@@ -9460,22 +9505,13 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>1042.88</v>
+        <v>0</v>
       </c>
       <c r="P83" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q83" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R83" s="7" t="n">
-        <v>1.768473487193091</v>
-      </c>
-      <c r="S83" s="7" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="T83" t="n">
         <v>67</v>
@@ -9847,20 +9883,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/23/2026 11:52</t>
+          <t>09/24/2026 23:39</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20316.59</v>
+        <v>20326.04</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>1.58</v>
+        <v>1.63</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9878,19 +9914,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>310.96</v>
+        <v>326.0400000000001</v>
       </c>
       <c r="V87" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>43.13725490196079</v>
+        <v>43.87096774193549</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>4.52</v>
@@ -9902,7 +9938,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10047,20 +10083,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/23/2026 11:17</t>
+          <t>09/24/2026 23:17</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20478.91</v>
+        <v>20513.91</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>2.38</v>
+        <v>2.56</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10078,19 +10114,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>514.21</v>
+        <v>513.9100000000001</v>
       </c>
       <c r="V89" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>85</v>
+        <v>84.55284552845529</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10102,7 +10138,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10147,20 +10183,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/23/2026 11:02</t>
+          <t>09/24/2026 23:03</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>25914.47</v>
+        <v>26043.83</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>29.64</v>
+        <v>30.28</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.93</v>
+        <v>1.88</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10178,19 +10214,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>5699.240000000001</v>
+        <v>6043.83</v>
       </c>
       <c r="V90" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>69.10569105691057</v>
+        <v>69.53125</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.87</v>
+        <v>1.88</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10202,7 +10238,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10369,13 +10405,22 @@
         <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="O92" s="7" t="n">
-        <v>0</v>
+        <v>20269.59</v>
       </c>
       <c r="P92" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="Q92" s="7" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="R92" s="7" t="n">
+        <v>188.9075739315843</v>
+      </c>
+      <c r="S92" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T92" t="n">
         <v>23</v>
@@ -10407,7 +10452,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -10569,13 +10614,22 @@
         <v>0</v>
       </c>
       <c r="N94" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="O94" s="7" t="n">
-        <v>0</v>
+        <v>19959.77</v>
       </c>
       <c r="P94" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="Q94" s="7" t="n">
+        <v>45.45454545454545</v>
+      </c>
+      <c r="R94" s="7" t="n">
+        <v>223.0219132369299</v>
+      </c>
+      <c r="S94" s="7" t="n">
+        <v>0.22</v>
       </c>
       <c r="T94" t="n">
         <v>10</v>
@@ -10607,7 +10661,7 @@
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC94" t="inlineStr">
@@ -11169,13 +11223,22 @@
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>0</v>
+        <v>-304.44</v>
       </c>
       <c r="P100" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q100" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R100" s="7" t="n">
+        <v>0.4682177854635016</v>
+      </c>
+      <c r="S100" s="7" t="n">
+        <v>0.41</v>
       </c>
       <c r="T100" t="n">
         <v>199</v>
@@ -11247,20 +11310,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/23/2026 13:16</t>
+          <t>09/24/2026 01:33</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>20872.45</v>
+        <v>20897.2</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>4.35</v>
+        <v>4.47</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>2.43</v>
+        <v>2.47</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11347,20 +11410,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/23/2026 22:11</t>
+          <t>09/24/2026 21:13</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>19961.06</v>
+        <v>19980.22</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>-0.17</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="J102" s="7" t="n">
         <v>2.2</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11378,19 +11441,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>-38.93999999999996</v>
+        <v>-19.77999999999996</v>
       </c>
       <c r="V102" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>37.93103448275862</v>
+        <v>38.98305084745763</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>2.2</v>
@@ -11402,7 +11465,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11665,20 +11728,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/23/2026 18:09</t>
+          <t>09/24/2026 17:41</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11559.62</v>
+        <v>11481.72</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>15.56</v>
+        <v>14.78</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.89</v>
+        <v>2.57</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11696,19 +11759,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1670.15</v>
+        <v>1592.25</v>
       </c>
       <c r="V105" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>70.58823529411765</v>
+        <v>69.81132075471697</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.34</v>
+        <v>2.91</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11720,7 +11783,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11765,7 +11828,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/21/2026 09:16</t>
+          <t>09/24/2026 11:32</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11874,20 +11937,20 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/23/2026 19:55</t>
+          <t>09/24/2026 19:07</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>25885.08</v>
+        <v>25533.19</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-32.6</v>
+        <v>-33.52</v>
       </c>
       <c r="J107" s="7" t="n">
-        <v>38.74</v>
+        <v>39.57</v>
       </c>
       <c r="K107" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="L107" t="n">
         <v>25000</v>
@@ -11899,37 +11962,37 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-283.51</v>
+        <v>-798.5599999999999</v>
       </c>
       <c r="P107" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>37.5</v>
+        <v>12.5</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.4600220935547768</v>
+        <v>0.1347462401941663</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>1.69</v>
+        <v>3.29</v>
       </c>
       <c r="T107" t="n">
-        <v>3791</v>
+        <v>3838</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-8396.920000000002</v>
+        <v>-8748.810000000001</v>
       </c>
       <c r="V107" t="n">
         <v>2316</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>61.09206014244263</v>
+        <v>60.34392912975508</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="Y107" s="7" t="n">
-        <v>39.64</v>
+        <v>40.92</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -11938,7 +12001,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -11983,7 +12046,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 08:27</t>
+          <t>09/24/2026 10:23</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12074,7 +12137,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 05:00</t>
+          <t>09/24/2026 05:52</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12438,7 +12501,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 13:15</t>
+          <t>09/24/2026 16:02</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12529,7 +12592,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 09:15</t>
+          <t>09/24/2026 11:31</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12711,7 +12774,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 05:26</t>
+          <t>09/24/2026 06:33</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12893,7 +12956,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/20/2026 23:53</t>
+          <t>09/23/2026 23:57</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13176,23 +13239,17 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>3326.65</v>
+        <v>0</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>31</v>
-      </c>
-      <c r="Q121" s="9" t="n">
-        <v>77.5</v>
-      </c>
-      <c r="R121" s="9" t="n">
-        <v>8.896717069812709</v>
-      </c>
-      <c r="S121" s="9" t="n">
-        <v>1.04</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q121" s="8" t="n"/>
+      <c r="R121" s="8" t="n"/>
+      <c r="S121" s="8" t="n"/>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13267,17 +13324,23 @@
         <v>0</v>
       </c>
       <c r="N122" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O122" s="9" t="n">
-        <v>0</v>
+        <v>-58.49</v>
       </c>
       <c r="P122" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q122" s="8" t="n"/>
-      <c r="R122" s="8" t="n"/>
-      <c r="S122" s="8" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="Q122" s="9" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R122" s="9" t="n">
+        <v>0.2666750250752257</v>
+      </c>
+      <c r="S122" s="9" t="n">
+        <v>0.32</v>
+      </c>
       <c r="T122" s="8" t="n">
         <v>0</v>
       </c>
@@ -13840,7 +13903,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 06:32</t>
+          <t>09/24/2026 08:06</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13931,7 +13994,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 06:04</t>
+          <t>09/24/2026 07:36</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14113,7 +14176,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/21/2026 11:22</t>
+          <t>09/24/2026 13:48</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14288,7 +14351,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/21/2026 08:27</t>
+          <t>09/24/2026 10:23</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14329,7 +14392,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/21/2026 05:00</t>
+          <t>09/24/2026 05:52</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14493,7 +14556,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09/21/2026 13:15</t>
+          <t>09/24/2026 16:02</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14534,7 +14597,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/21/2026 09:15</t>
+          <t>09/24/2026 11:31</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14616,7 +14679,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/21/2026 05:26</t>
+          <t>09/24/2026 06:33</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14698,7 +14761,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/20/2026 23:53</t>
+          <t>09/23/2026 23:57</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14831,7 +14894,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -14872,7 +14935,7 @@
         <v>-0.16</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20">
@@ -15149,7 +15212,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/21/2026 06:32</t>
+          <t>09/24/2026 08:06</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15190,7 +15253,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/21/2026 06:04</t>
+          <t>09/24/2026 07:36</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15272,7 +15335,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/21/2026 11:22</t>
+          <t>09/24/2026 13:48</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17563,7 +17626,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09/21/2026 07:42</t>
+          <t>09/24/2026 09:47</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17609,7 +17672,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/21/2026 07:34</t>
+          <t>09/24/2026 09:32</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17632,7 +17695,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/21/2026 04:21</t>
+          <t>09/24/2026 04:47</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17770,7 +17833,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/21/2026 08:44</t>
+          <t>09/24/2026 10:48</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17816,7 +17879,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/21/2026 07:28</t>
+          <t>09/24/2026 09:24</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17908,7 +17971,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/21/2026 09:41</t>
+          <t>09/24/2026 12:10</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17931,7 +17994,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/21/2026 04:11</t>
+          <t>09/24/2026 04:32</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -17977,7 +18040,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/21/2026 08:48</t>
+          <t>09/24/2026 10:52</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18023,7 +18086,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/21/2026 09:37</t>
+          <t>09/24/2026 12:03</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18276,7 +18339,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/21/2026 07:28</t>
+          <t>09/24/2026 09:26</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18299,7 +18362,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/21/2026 08:06</t>
+          <t>09/24/2026 10:08</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18322,7 +18385,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/18/2026 11:12</t>
+          <t>09/24/2026 13:43</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18345,7 +18408,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/23/2026 13:58</t>
+          <t>09/24/2026 14:00</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-29
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-24 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-28 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/24/2026 19:47</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>40042</v>
+          <t>09/28/2026 17:10</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>44943.22</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>83.04000000000001</v>
+        <v>105.45</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-1334.639999999999</v>
+        <v>14114</v>
       </c>
       <c r="P2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.9705176248335509</v>
+        <v>1.416240639820315</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>50.52</v>
+        <v>26.33</v>
       </c>
       <c r="T2" t="n">
-        <v>3443</v>
+        <v>3452</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>15041.99999999999</v>
+        <v>21641.98999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2186</v>
+        <v>2194</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.49114144641301</v>
+        <v>63.55735805330244</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>09/22/2026 23:03</t>
+          <t>09/28/2026 23:13</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>09/23/2026 09:30</t>
+          <t>09/26/2026 09:34</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>09/22/2026 10:07</t>
+          <t>09/28/2026 10:40</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>09/22/2026 19:49</t>
+          <t>09/28/2026 20:00</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/24/2026 11:34</t>
+          <t>09/27/2026 11:41</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/24/2026 13:18</t>
+          <t>09/27/2026 13:20</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/24/2026 13:19</t>
+          <t>09/27/2026 13:22</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>09/23/2026 02:29</t>
+          <t>09/26/2026 02:36</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09/23/2026 10:47</t>
+          <t>09/26/2026 10:55</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>09/22/2026 13:22</t>
+          <t>09/28/2026 13:31</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/23/2026 02:59</t>
+          <t>09/26/2026 03:05</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>09/17/2026 13:20</t>
+          <t>09/26/2026 13:38</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>09/23/2026 06:10</t>
+          <t>09/26/2026 06:15</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09/23/2026 06:14</t>
+          <t>09/26/2026 06:19</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/22/2026 12:04</t>
+          <t>09/28/2026 23:22</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/22/2026 00:57</t>
+          <t>09/28/2026 01:07</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/24/2026 20:39</t>
+          <t>09/28/2026 18:01</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>19028.34</v>
+        <v>18897.99</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-4.86</v>
+        <v>-5.51</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>7.42</v>
+        <v>7.74</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3165,37 +3165,37 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-245.8200000000001</v>
+        <v>-602.99</v>
       </c>
       <c r="P22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>47.5</v>
+        <v>45</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.9026971824853345</v>
+        <v>0.7730295969797002</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>6.1</v>
+        <v>6.48</v>
       </c>
       <c r="T22" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-971.66</v>
+        <v>-1102.01</v>
       </c>
       <c r="V22" t="n">
         <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>48.57142857142857</v>
+        <v>48.11320754716981</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>7.43</v>
+        <v>7.74</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/24/2026 23:06</t>
+          <t>09/28/2026 20:28</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19582.09</v>
+        <v>19529.11</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.25</v>
+        <v>-2.51</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2.31</v>
+        <v>2.57</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-298.98</v>
+        <v>-336.93</v>
       </c>
       <c r="P23" t="n">
         <v>8</v>
@@ -3283,28 +3283,28 @@
         <v>20</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.2170223909912269</v>
+        <v>0.1974035254883278</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>1.49</v>
+        <v>1.68</v>
       </c>
       <c r="T23" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-417.91</v>
+        <v>-470.89</v>
       </c>
       <c r="V23" t="n">
         <v>19</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>27.14285714285714</v>
+        <v>26.38888888888889</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>2.15</v>
+        <v>2.41</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/24/2026 21:20</t>
+          <t>09/28/2026 18:36</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/23/2026 23:09</t>
+          <t>09/26/2026 23:15</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/24/2026 20:40</t>
+          <t>09/28/2026 17:56</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20501.48</v>
+        <v>20547.65</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.98</v>
+        <v>-1.76</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>539.25</v>
+        <v>422.29</v>
       </c>
       <c r="P26" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>50</v>
+        <v>47.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.291489637725813</v>
+        <v>1.248921295859662</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5</v>
+        <v>5.04</v>
       </c>
       <c r="T26" t="n">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>501.4799999999997</v>
+        <v>486.9000000000003</v>
       </c>
       <c r="V26" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>44.26229508196721</v>
+        <v>44.27480916030535</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/24/2026 10:47</t>
+          <t>09/27/2026 10:55</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,20 +3794,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/23/2026 21:46</t>
+          <t>09/28/2026 18:09</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>19643.7</v>
-      </c>
-      <c r="I28" s="7" t="n">
-        <v>-1.8</v>
+        <v>19605.3</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-2</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="L28" t="n">
         <v>20000</v>
@@ -3819,19 +3819,19 @@
         <v>40</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>28.70000000000003</v>
+        <v>68.60000000000004</v>
       </c>
       <c r="P28" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>22.5</v>
+        <v>27.5</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>1.037368331966199</v>
+        <v>1.110284069900166</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>2.59</v>
+        <v>1.78</v>
       </c>
       <c r="T28" t="n">
         <v>166</v>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>09/22/2026 11:11</t>
+          <t>09/28/2026 11:20</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/24/2026 21:22</t>
+          <t>09/28/2026 18:44</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20594.26</v>
-      </c>
-      <c r="I30" t="n">
-        <v>3</v>
+        <v>20585.06</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>2.96</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.59</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.71</v>
+        <v>1.7</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-219.78</v>
+        <v>-230.39</v>
       </c>
       <c r="P30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>25</v>
+        <v>22.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.2869610355903059</v>
+        <v>0.2739963446146089</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="T30" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>594.2600000000001</v>
+        <v>585.0599999999999</v>
       </c>
       <c r="V30" t="n">
         <v>25</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>26.59574468085106</v>
+        <v>26.04166666666667</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.71</v>
+        <v>1.7</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.59</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>09/23/2026 11:42</t>
+          <t>09/26/2026 11:47</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/23/2026 16:05</t>
+          <t>09/26/2026 16:11</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/23/2026 03:41</t>
+          <t>09/26/2026 03:48</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/25/2026 00:56</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="n">
-        <v>20659.44</v>
+          <t>09/28/2026 22:20</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>20556</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>3.31</v>
+        <v>2.79</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>554.29</v>
+        <v>556</v>
       </c>
       <c r="V35" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>51.8796992481203</v>
+        <v>52.23880597014925</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>1.09</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/23/2026 11:29</t>
+          <t>09/26/2026 11:36</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/23/2026 03:07</t>
+          <t>09/26/2026 03:15</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>09/22/2026 15:40</t>
+          <t>09/28/2026 15:58</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>09/22/2026 09:54</t>
+          <t>09/28/2026 10:22</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>09/22/2026 09:13</t>
+          <t>09/28/2026 09:32</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/24/2026 00:24</t>
+          <t>09/27/2026 00:29</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/24/2026 00:43</t>
+          <t>09/27/2026 00:47</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/24/2026 03:04</t>
+          <t>09/27/2026 03:10</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,20 +5529,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/24/2026 21:23</t>
+          <t>09/28/2026 18:45</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19799.57</v>
+        <v>19959.09</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-0.96</v>
+        <v>-0.17</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5554,34 +5554,34 @@
         <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>71.42999999999998</v>
+        <v>199.18</v>
       </c>
       <c r="P44" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="Q44" s="7" t="n">
-        <v>52.5</v>
+        <v>80</v>
       </c>
       <c r="R44" s="7" t="n">
-        <v>1.429499128134207</v>
+        <v>3.483231517267173</v>
       </c>
       <c r="S44" s="7" t="n">
-        <v>0.53</v>
+        <v>0.34</v>
       </c>
       <c r="T44" t="n">
-        <v>748</v>
+        <v>772</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-200.4300000000002</v>
+        <v>-40.90999999999994</v>
       </c>
       <c r="V44" t="n">
-        <v>423</v>
+        <v>445</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>56.55080213903744</v>
+        <v>57.64248704663213</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5593,7 +5593,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/24/2026 20:00</t>
+          <t>09/28/2026 17:20</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5660,22 +5660,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-26.6</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.6475887652358241</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>54</v>
@@ -5747,7 +5738,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/24/2026 20:30</t>
+          <t>09/28/2026 17:50</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5769,13 +5760,22 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>598.1899999999999</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>1.424850852272727</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>2.39</v>
       </c>
       <c r="T46" t="n">
         <v>89</v>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/23/2026 23:43</t>
+          <t>09/26/2026 23:49</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5869,22 +5869,13 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>504.68</v>
+        <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q47" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R47" s="7" t="n">
-        <v>2.47982641332395</v>
-      </c>
-      <c r="S47" s="7" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5956,7 +5947,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09/24/2026 15:57</t>
+          <t>09/27/2026 15:59</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6056,7 +6047,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/24/2026 00:33</t>
+          <t>09/27/2026 00:38</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6156,7 +6147,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/24/2026 00:11</t>
+          <t>09/27/2026 00:16</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6256,20 +6247,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/24/2026 20:14</t>
+          <t>09/28/2026 17:33</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19716.33</v>
+        <v>19861.05</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-1.4</v>
+        <v>-0.67</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6287,19 +6278,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-283.6700000000005</v>
+        <v>-138.9500000000005</v>
       </c>
       <c r="V51" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>30.64516129032258</v>
+        <v>32.35294117647059</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6311,7 +6302,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6356,20 +6347,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/24/2026 21:07</t>
+          <t>09/28/2026 18:27</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19638.54</v>
+        <v>19374.9</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-1.77</v>
+        <v>-3.1</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>5.23</v>
+        <v>5.3</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.93</v>
+        <v>0.89</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6387,22 +6378,22 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-361.4600000000002</v>
+        <v>-625.1000000000001</v>
       </c>
       <c r="V52" t="n">
         <v>45</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>40.17857142857143</v>
+        <v>39.47368421052632</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.93</v>
+        <v>0.89</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6411,7 +6402,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6456,20 +6447,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/24/2026 21:55</t>
+          <t>09/28/2026 19:14</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19783.22</v>
+        <v>19737.68</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.11</v>
+        <v>-1.35</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6487,19 +6478,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-216.7800000000001</v>
+        <v>-262.32</v>
       </c>
       <c r="V53" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.4963503649635</v>
+        <v>35.78199052132701</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6511,7 +6502,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6556,7 +6547,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/23/2026 21:23</t>
+          <t>09/26/2026 21:30</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6656,7 +6647,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/24/2026 21:32</t>
+          <t>09/28/2026 18:46</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6756,7 +6747,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>09/22/2026 09:44</t>
+          <t>09/28/2026 10:09</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6856,17 +6847,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/24/2026 20:29</t>
+          <t>09/28/2026 17:45</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19619.34</v>
+        <v>19611.9</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.89</v>
+        <v>-1.93</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>1.95</v>
+        <v>2.01</v>
       </c>
       <c r="K57" s="7" t="n">
         <v>0.77</v>
@@ -6881,37 +6872,37 @@
         <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>-66.18000000000001</v>
+        <v>-45.43</v>
       </c>
       <c r="P57" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q57" s="7" t="n">
-        <v>45</v>
+        <v>37.5</v>
       </c>
       <c r="R57" s="7" t="n">
-        <v>0.1874769797421731</v>
+        <v>0.3725138121546961</v>
       </c>
       <c r="S57" s="7" t="n">
-        <v>0.34</v>
+        <v>0.31</v>
       </c>
       <c r="T57" t="n">
-        <v>1063</v>
+        <v>1078</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-380.1900000000001</v>
+        <v>-387.6300000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.02634054562559</v>
+        <v>43.69202226345084</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.77</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>1.95</v>
+        <v>2.02</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6920,7 +6911,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6965,7 +6956,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/24/2026 21:16</t>
+          <t>09/28/2026 18:34</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7065,7 +7056,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>09/22/2026 11:30</t>
+          <t>09/28/2026 11:43</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7165,20 +7156,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/24/2026 20:57</t>
+          <t>09/28/2026 18:15</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>19644.84</v>
+        <v>19177.85</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-7.65</v>
+        <v>-9.84</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>21100.65</v>
@@ -7265,20 +7256,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/24/2026 22:26</t>
+          <t>09/28/2026 19:48</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>20449.71</v>
+        <v>20219.74</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-4.54</v>
+        <v>-5.61</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>13.96</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L61" s="7" t="n">
         <v>21292.1</v>
@@ -7365,7 +7356,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>09/23/2026 21:14</t>
+          <t>09/26/2026 21:21</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7465,7 +7456,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/24/2026 21:43</t>
+          <t>09/28/2026 10:17</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7496,19 +7487,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1335.81</v>
+        <v>-1375.76</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>12.06896551724138</v>
+        <v>11.86440677966102</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7520,7 +7511,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7565,7 +7556,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/24/2026 22:20</t>
+          <t>09/28/2026 19:40</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7587,13 +7578,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-90.82000000000002</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.7198297137216189</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>0.96</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7665,20 +7665,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/24/2026 21:38</t>
+          <t>09/28/2026 18:54</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19088.95</v>
+        <v>18429.16</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-4.61</v>
+        <v>-7.9</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>11.64</v>
+        <v>11.66</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.93</v>
+        <v>0.89</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/24/2026 21:14</t>
+          <t>09/28/2026 18:33</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7865,20 +7865,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/24/2026 22:19</t>
+          <t>09/28/2026 19:41</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>21695.62</v>
+        <v>21526.55</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>8.51</v>
+        <v>7.67</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.21</v>
+        <v>1.17</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7896,19 +7896,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>1695.62</v>
+        <v>1526.55</v>
       </c>
       <c r="V67" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>34.11764705882353</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.21</v>
+        <v>1.17</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>09/22/2026 11:30</t>
+          <t>09/28/2026 11:43</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>09/23/2026 02:49</t>
+          <t>09/26/2026 02:56</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8165,7 +8165,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>09/23/2026 02:48</t>
+          <t>09/26/2026 02:55</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/23/2026 02:47</t>
+          <t>09/26/2026 02:54</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/24/2026 21:45</t>
+          <t>09/28/2026 19:00</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/24/2026 23:35</t>
+          <t>09/28/2026 20:57</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/24/2026 21:36</t>
+          <t>09/28/2026 18:53</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8587,22 +8587,13 @@
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>-53.91</v>
+        <v>0</v>
       </c>
       <c r="P74" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q74" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R74" s="7" t="n">
-        <v>0.8335391835978508</v>
-      </c>
-      <c r="S74" s="7" t="n">
-        <v>0.73</v>
+        <v>0</v>
       </c>
       <c r="T74" t="n">
         <v>329</v>
@@ -8696,22 +8687,13 @@
         <v>0</v>
       </c>
       <c r="N75" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O75" s="7" t="n">
-        <v>-204.85</v>
+        <v>0</v>
       </c>
       <c r="P75" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q75" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R75" s="7" t="n">
-        <v>0.7749840725850743</v>
-      </c>
-      <c r="S75" s="7" t="n">
-        <v>2.41</v>
+        <v>0</v>
       </c>
       <c r="T75" t="n">
         <v>101</v>
@@ -8783,7 +8765,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/23/2026 19:25</t>
+          <t>09/26/2026 19:29</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8983,7 +8965,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/23/2026 19:48</t>
+          <t>09/26/2026 19:52</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9083,7 +9065,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/23/2026 20:06</t>
+          <t>09/26/2026 20:11</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9183,7 +9165,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/20/2026 19:51</t>
+          <t>09/26/2026 20:01</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9283,7 +9265,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/23/2026 19:20</t>
+          <t>09/26/2026 19:24</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9383,7 +9365,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/23/2026 20:33</t>
+          <t>09/26/2026 20:36</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9483,7 +9465,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/23/2026 20:02</t>
+          <t>09/26/2026 20:06</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9583,7 +9565,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/23/2026 12:01</t>
+          <t>09/26/2026 12:05</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9683,7 +9665,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>09/21/2026 01:46</t>
+          <t>09/27/2026 01:53</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9783,7 +9765,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>09/23/2026 19:40</t>
+          <t>09/26/2026 19:47</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9805,13 +9787,22 @@
         <v>0</v>
       </c>
       <c r="N86" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>0</v>
+        <v>3093.07</v>
       </c>
       <c r="P86" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q86" s="7" t="n">
+        <v>51.51515151515152</v>
+      </c>
+      <c r="R86" s="7" t="n">
+        <v>12.34780056499248</v>
+      </c>
+      <c r="S86" s="7" t="n">
+        <v>2.89</v>
       </c>
       <c r="T86" t="n">
         <v>32</v>
@@ -9843,7 +9834,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC86" t="inlineStr">
@@ -9883,20 +9874,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/24/2026 23:39</t>
+          <t>09/28/2026 21:04</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20326.04</v>
+        <v>19979.53</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>1.63</v>
+        <v>-0.11</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>1.17</v>
+        <v>0.99</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9914,19 +9905,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>326.0400000000001</v>
+        <v>-20.47000000000003</v>
       </c>
       <c r="V87" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>43.87096774193549</v>
+        <v>43.63636363636363</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>1.17</v>
+        <v>0.99</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>4.52</v>
@@ -9938,7 +9929,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9983,7 +9974,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>09/22/2026 11:42</t>
+          <t>09/28/2026 12:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10083,20 +10074,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/24/2026 23:17</t>
+          <t>09/28/2026 20:36</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20513.91</v>
+        <v>20588.81</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>2.56</v>
+        <v>2.94</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.26</v>
+        <v>1.29</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10114,19 +10105,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>513.9100000000001</v>
+        <v>588.8099999999999</v>
       </c>
       <c r="V89" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>84.55284552845529</v>
+        <v>85.38461538461539</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.26</v>
+        <v>1.29</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10138,7 +10129,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10183,20 +10174,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/24/2026 23:03</t>
+          <t>09/28/2026 20:23</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>26043.83</v>
+        <v>27282.84</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>30.28</v>
+        <v>36.47</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.88</v>
+        <v>2.02</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10214,19 +10205,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>6043.83</v>
+        <v>7282.840000000001</v>
       </c>
       <c r="V90" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>69.53125</v>
+        <v>70.58823529411765</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.88</v>
+        <v>2.02</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10238,7 +10229,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10283,7 +10274,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/23/2026 18:58</t>
+          <t>09/26/2026 19:03</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10383,7 +10374,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>09/22/2026 18:04</t>
+          <t>09/28/2026 18:14</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10483,7 +10474,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/23/2026 13:49</t>
+          <t>09/26/2026 13:55</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10583,7 +10574,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/23/2026 13:45</t>
+          <t>09/26/2026 13:50</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10683,7 +10674,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/23/2026 13:35</t>
+          <t>09/26/2026 13:42</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10783,7 +10774,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/23/2026 23:39</t>
+          <t>09/26/2026 23:45</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10883,7 +10874,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/23/2026 18:59</t>
+          <t>09/26/2026 19:03</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10983,7 +10974,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/23/2026 19:11</t>
+          <t>09/26/2026 19:15</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11005,22 +10996,13 @@
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>-812.92</v>
+        <v>0</v>
       </c>
       <c r="P98" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q98" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R98" s="7" t="n">
-        <v>0.1283107079285423</v>
-      </c>
-      <c r="S98" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="T98" t="n">
         <v>448</v>
@@ -11092,7 +11074,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/23/2026 23:43</t>
+          <t>09/26/2026 23:49</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11192,7 +11174,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>09/22/2026 18:11</t>
+          <t>09/28/2026 18:21</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11292,20 +11274,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/25/2026 00:29</t>
+          <t>09/28/2026 21:55</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>20897.2</v>
-      </c>
-      <c r="I101" s="7" t="n">
-        <v>4.47</v>
+        <v>21403.45</v>
+      </c>
+      <c r="I101" t="n">
+        <v>7</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>2.47</v>
+        <v>3.3</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11323,19 +11305,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>897.2</v>
+        <v>1403.45</v>
       </c>
       <c r="V101" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>80</v>
+        <v>81.25</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>2.47</v>
+        <v>3.3</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11347,7 +11329,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11392,7 +11374,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/24/2026 21:13</t>
+          <t>09/28/2026 18:30</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11492,7 +11474,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>09/22/2026 09:29</t>
+          <t>09/28/2026 09:53</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
@@ -11601,7 +11583,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>09/23/2026 01:39</t>
+          <t>09/26/2026 01:46</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11710,20 +11692,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/24/2026 17:41</t>
+          <t>09/29/2026 01:10</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11481.72</v>
+        <v>11777.01</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>14.78</v>
+        <v>17.73</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.57</v>
+        <v>2.89</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11741,19 +11723,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1592.25</v>
+        <v>2004.2</v>
       </c>
       <c r="V105" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>69.81132075471697</v>
+        <v>73.21428571428571</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>2.91</v>
+        <v>3.8</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11765,7 +11747,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11810,7 +11792,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/24/2026 11:32</t>
+          <t>09/27/2026 11:40</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11919,20 +11901,20 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/24/2026 19:07</t>
+          <t>09/28/2026 16:44</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>25533.19</v>
+        <v>25876.64</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-33.52</v>
+        <v>-32.63</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>39.57</v>
       </c>
       <c r="K107" s="7" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="L107" t="n">
         <v>25000</v>
@@ -11944,34 +11926,34 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-798.5599999999999</v>
+        <v>-139.01</v>
       </c>
       <c r="P107" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>12.5</v>
+        <v>65</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.1347462401941663</v>
+        <v>0.7079130946377543</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>3.29</v>
+        <v>1.9</v>
       </c>
       <c r="T107" t="n">
-        <v>3838</v>
+        <v>3876</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-8748.810000000001</v>
+        <v>-8405.359999999999</v>
       </c>
       <c r="V107" t="n">
-        <v>2316</v>
+        <v>2342</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>60.34392912975508</v>
+        <v>60.42311661506707</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="Y107" s="7" t="n">
         <v>40.92</v>
@@ -11983,7 +11965,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12028,7 +12010,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 10:23</t>
+          <t>09/27/2026 10:30</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12119,7 +12101,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 05:52</t>
+          <t>09/27/2026 06:00</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12210,7 +12192,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 23:18</t>
+          <t>09/28/2026 23:29</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12301,7 +12283,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>09/23/2026 16:54</t>
+          <t>09/26/2026 16:59</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12392,7 +12374,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 10:16</t>
+          <t>09/28/2026 10:48</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12483,7 +12465,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 16:02</t>
+          <t>09/27/2026 16:05</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12574,7 +12556,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 11:31</t>
+          <t>09/27/2026 11:39</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12665,7 +12647,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 13:18</t>
+          <t>09/28/2026 13:27</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12756,7 +12738,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 06:33</t>
+          <t>09/27/2026 06:41</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12847,7 +12829,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 19:24</t>
+          <t>09/28/2026 19:34</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12938,7 +12920,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/23/2026 23:57</t>
+          <t>09/27/2026 00:03</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13029,7 +13011,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 11:41</t>
+          <t>09/28/2026 12:00</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13051,23 +13033,17 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>67.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q119" s="9" t="n">
-        <v>65</v>
-      </c>
-      <c r="R119" s="9" t="n">
-        <v>1.223174978645115</v>
-      </c>
-      <c r="S119" s="9" t="n">
-        <v>0.57</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q119" s="8" t="n"/>
+      <c r="R119" s="8" t="n"/>
+      <c r="S119" s="8" t="n"/>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13120,7 +13096,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>09/23/2026 20:55</t>
+          <t>09/26/2026 20:59</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13142,23 +13118,17 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>-6156.77</v>
+        <v>0</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q120" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="R120" s="9" t="n">
-        <v>0.01160528233794505</v>
-      </c>
-      <c r="S120" s="9" t="n">
-        <v>31.03</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q120" s="8" t="n"/>
+      <c r="R120" s="8" t="n"/>
+      <c r="S120" s="8" t="n"/>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13211,7 +13181,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/23/2026 15:23</t>
+          <t>09/26/2026 15:30</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13233,23 +13203,17 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>3326.65</v>
+        <v>0</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>31</v>
-      </c>
-      <c r="Q121" s="9" t="n">
-        <v>77.5</v>
-      </c>
-      <c r="R121" s="9" t="n">
-        <v>8.896717069812709</v>
-      </c>
-      <c r="S121" s="9" t="n">
-        <v>1.04</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q121" s="8" t="n"/>
+      <c r="R121" s="8" t="n"/>
+      <c r="S121" s="8" t="n"/>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13302,7 +13266,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/23/2026 02:49</t>
+          <t>09/26/2026 02:56</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13387,7 +13351,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 18:26</t>
+          <t>09/28/2026 18:35</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13472,7 +13436,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 18:26</t>
+          <t>09/28/2026 18:36</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13557,7 +13521,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 18:26</t>
+          <t>09/28/2026 18:37</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13642,7 +13606,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 18:38</t>
+          <t>09/28/2026 18:49</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13727,7 +13691,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 19:12</t>
+          <t>09/28/2026 19:24</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13812,7 +13776,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>09/22/2026 18:24</t>
+          <t>09/28/2026 18:33</t>
         </is>
       </c>
       <c r="H128" s="9" t="n">
@@ -13897,7 +13861,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 08:06</t>
+          <t>09/27/2026 08:14</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13988,7 +13952,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 07:36</t>
+          <t>09/27/2026 07:46</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14170,7 +14134,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/24/2026 13:48</t>
+          <t>09/27/2026 13:51</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14345,7 +14309,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/24/2026 10:23</t>
+          <t>09/27/2026 10:30</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14386,7 +14350,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/24/2026 05:52</t>
+          <t>09/27/2026 06:00</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14427,7 +14391,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>09/22/2026 23:18</t>
+          <t>09/28/2026 23:29</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14468,7 +14432,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09/23/2026 16:54</t>
+          <t>09/26/2026 16:59</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14509,7 +14473,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>09/22/2026 10:16</t>
+          <t>09/28/2026 10:48</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14550,7 +14514,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09/24/2026 16:02</t>
+          <t>09/27/2026 16:05</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14591,7 +14555,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/24/2026 11:31</t>
+          <t>09/27/2026 11:39</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14632,7 +14596,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>09/22/2026 13:18</t>
+          <t>09/28/2026 13:27</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14673,7 +14637,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/24/2026 06:33</t>
+          <t>09/27/2026 06:41</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14714,7 +14678,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>09/22/2026 19:24</t>
+          <t>09/28/2026 19:34</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14755,7 +14719,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/23/2026 23:57</t>
+          <t>09/27/2026 00:03</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14796,7 +14760,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>09/22/2026 11:41</t>
+          <t>09/28/2026 12:00</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14806,7 +14770,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -14837,7 +14801,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>09/23/2026 20:55</t>
+          <t>09/26/2026 20:59</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14847,7 +14811,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -14878,7 +14842,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09/23/2026 15:23</t>
+          <t>09/26/2026 15:30</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14888,7 +14852,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -14919,7 +14883,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/23/2026 02:49</t>
+          <t>09/26/2026 02:56</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14960,7 +14924,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>09/22/2026 18:26</t>
+          <t>09/28/2026 18:35</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -15001,7 +14965,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>09/22/2026 18:26</t>
+          <t>09/28/2026 18:36</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -15042,7 +15006,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>09/22/2026 18:26</t>
+          <t>09/28/2026 18:37</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -15083,7 +15047,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>09/22/2026 18:38</t>
+          <t>09/28/2026 18:49</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -15124,7 +15088,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>09/22/2026 19:12</t>
+          <t>09/28/2026 19:24</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15165,7 +15129,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>09/22/2026 18:24</t>
+          <t>09/28/2026 18:33</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -15206,7 +15170,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/24/2026 08:06</t>
+          <t>09/27/2026 08:14</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15247,7 +15211,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/24/2026 07:36</t>
+          <t>09/27/2026 07:46</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15329,7 +15293,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/24/2026 13:48</t>
+          <t>09/27/2026 13:51</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17643,7 +17607,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09/22/2026 13:49</t>
+          <t>09/28/2026 13:58</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17666,7 +17630,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/24/2026 09:32</t>
+          <t>09/27/2026 09:39</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17689,7 +17653,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/24/2026 04:47</t>
+          <t>09/27/2026 04:54</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17712,7 +17676,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09/23/2026 01:56</t>
+          <t>09/26/2026 02:03</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17735,7 +17699,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09/22/2026 08:46</t>
+          <t>09/28/2026 08:58</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17758,7 +17722,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09/21/2026 03:52</t>
+          <t>09/27/2026 04:07</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17781,7 +17745,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09/22/2026 08:48</t>
+          <t>09/28/2026 09:01</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -17804,7 +17768,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09/22/2026 17:19</t>
+          <t>09/28/2026 17:30</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -17827,7 +17791,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/24/2026 10:48</t>
+          <t>09/27/2026 10:55</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17850,7 +17814,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09/22/2026 20:15</t>
+          <t>09/28/2026 20:26</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17873,7 +17837,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/24/2026 09:24</t>
+          <t>09/27/2026 09:31</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17919,7 +17883,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09/23/2026 02:12</t>
+          <t>09/26/2026 02:20</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17942,7 +17906,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09/23/2026 01:57</t>
+          <t>09/26/2026 02:04</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -17965,7 +17929,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/24/2026 12:10</t>
+          <t>09/27/2026 12:12</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17988,7 +17952,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/24/2026 04:32</t>
+          <t>09/27/2026 04:39</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -18011,7 +17975,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/21/2026 11:50</t>
+          <t>09/27/2026 14:30</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -18034,7 +17998,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/24/2026 10:52</t>
+          <t>09/27/2026 11:00</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18080,7 +18044,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/24/2026 12:03</t>
+          <t>09/27/2026 12:08</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18103,7 +18067,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09/22/2026 07:52</t>
+          <t>09/28/2026 08:01</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18126,7 +18090,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09/22/2026 18:49</t>
+          <t>09/28/2026 19:00</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18149,7 +18113,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09/22/2026 18:49</t>
+          <t>09/28/2026 19:01</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18172,7 +18136,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09/23/2026 23:04</t>
+          <t>09/26/2026 23:10</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18195,7 +18159,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09/23/2026 23:18</t>
+          <t>09/26/2026 23:24</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18218,7 +18182,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09/22/2026 18:34</t>
+          <t>09/28/2026 18:44</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18241,7 +18205,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>09/22/2026 19:45</t>
+          <t>09/28/2026 19:56</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18264,7 +18228,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>09/22/2026 08:46</t>
+          <t>09/28/2026 08:58</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18287,7 +18251,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>09/22/2026 08:51</t>
+          <t>09/28/2026 09:05</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -18333,7 +18297,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/24/2026 09:26</t>
+          <t>09/27/2026 09:33</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18356,7 +18320,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/24/2026 10:08</t>
+          <t>09/27/2026 10:15</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18379,7 +18343,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/24/2026 13:43</t>
+          <t>09/27/2026 13:46</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18402,7 +18366,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/24/2026 14:00</t>
+          <t>09/28/2026 14:15</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-01
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-28 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-30 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/28/2026 17:10</t>
+          <t>10/01/2026 00:20</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>44943.22</v>
+        <v>43453.4</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>105.45</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>14114</v>
+        <v>5215.67</v>
       </c>
       <c r="P2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.416240639820315</v>
+        <v>1.128948557741754</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>26.33</v>
+        <v>31.3</v>
       </c>
       <c r="T2" t="n">
-        <v>3452</v>
+        <v>3456</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>21641.98999999999</v>
+        <v>18453.4</v>
       </c>
       <c r="V2" t="n">
-        <v>2194</v>
+        <v>2196</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.55735805330244</v>
+        <v>63.54166666666666</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>09/26/2026 09:34</t>
+          <t>09/29/2026 09:37</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/27/2026 11:41</t>
+          <t>09/30/2026 11:45</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/27/2026 13:20</t>
+          <t>09/30/2026 13:23</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/27/2026 13:22</t>
+          <t>09/30/2026 13:25</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>09/26/2026 02:36</t>
+          <t>09/29/2026 02:39</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>09/24/2026 06:57</t>
+          <t>09/30/2026 07:09</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09/26/2026 10:55</t>
+          <t>09/29/2026 10:56</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/26/2026 03:05</t>
+          <t>09/29/2026 03:09</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>09/26/2026 13:38</t>
+          <t>09/29/2026 13:41</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>09/26/2026 06:15</t>
+          <t>09/29/2026 06:17</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09/26/2026 06:19</t>
+          <t>09/29/2026 06:22</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09/28/2026 23:22</t>
+          <t>09/30/2026 22:21</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/28/2026 18:01</t>
+          <t>09/30/2026 19:35</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/28/2026 20:28</t>
+          <t>09/30/2026 20:47</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19529.11</v>
+        <v>19494.84</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.51</v>
+        <v>-2.68</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2.57</v>
+        <v>2.74</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-336.93</v>
+        <v>-367.24</v>
       </c>
       <c r="P23" t="n">
         <v>8</v>
@@ -3283,28 +3283,28 @@
         <v>20</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.1974035254883278</v>
+        <v>0.1841105507542601</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>1.68</v>
+        <v>1.84</v>
       </c>
       <c r="T23" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-470.89</v>
+        <v>-505.1600000000001</v>
       </c>
       <c r="V23" t="n">
         <v>19</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>26.38888888888889</v>
+        <v>26.02739726027397</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>2.41</v>
+        <v>2.58</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/28/2026 18:36</t>
+          <t>09/30/2026 19:52</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/26/2026 23:15</t>
+          <t>09/29/2026 23:18</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/28/2026 17:56</t>
+          <t>09/30/2026 19:33</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20547.65</v>
+        <v>20383.8</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.76</v>
+        <v>-2.55</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>422.29</v>
+        <v>-121.94</v>
       </c>
       <c r="P26" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>47.5</v>
+        <v>37.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.248921295859662</v>
+        <v>0.9350612694845482</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5.04</v>
+        <v>5.14</v>
       </c>
       <c r="T26" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>486.9000000000003</v>
+        <v>383.8000000000004</v>
       </c>
       <c r="V26" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>44.27480916030535</v>
+        <v>43.38235294117647</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/27/2026 10:55</t>
+          <t>09/30/2026 10:59</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,20 +3794,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/28/2026 18:09</t>
+          <t>09/30/2026 19:39</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>19605.3</v>
-      </c>
-      <c r="I28" t="n">
-        <v>-2</v>
+        <v>19569.8</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>-2.18</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="L28" t="n">
         <v>20000</v>
@@ -3819,7 +3819,7 @@
         <v>40</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>68.60000000000004</v>
+        <v>54.18000000000004</v>
       </c>
       <c r="P28" t="n">
         <v>11</v>
@@ -3828,10 +3828,10 @@
         <v>27.5</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>1.110284069900166</v>
+        <v>1.085128446853641</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>1.78</v>
+        <v>1.67</v>
       </c>
       <c r="T28" t="n">
         <v>166</v>
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/28/2026 18:44</t>
-        </is>
-      </c>
-      <c r="H30" s="7" t="n">
-        <v>20585.06</v>
+          <t>09/30/2026 19:56</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>20515</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.96</v>
+        <v>2.61</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>1.59</v>
+        <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.7</v>
+        <v>1.57</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,7 +4037,7 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-230.39</v>
+        <v>-205.59</v>
       </c>
       <c r="P30" t="n">
         <v>9</v>
@@ -4046,28 +4046,28 @@
         <v>22.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.2739963446146089</v>
+        <v>0.2972243112053052</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>1.25</v>
+        <v>1.13</v>
       </c>
       <c r="T30" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>585.0599999999999</v>
+        <v>514.9999999999999</v>
       </c>
       <c r="V30" t="n">
         <v>25</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>26.04166666666667</v>
+        <v>25</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.7</v>
+        <v>1.57</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <v>1.59</v>
+        <v>1.83</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/23/2026 10:48</t>
+          <t>09/29/2026 10:58</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>09/26/2026 11:47</t>
+          <t>09/29/2026 11:50</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/26/2026 16:11</t>
+          <t>09/29/2026 16:14</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/26/2026 03:48</t>
+          <t>09/29/2026 03:52</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09/28/2026 22:20</t>
-        </is>
-      </c>
-      <c r="H35" t="n">
-        <v>20556</v>
+          <t>09/30/2026 21:50</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>20555.28</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>2.79</v>
+        <v>2.78</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>556</v>
+        <v>555.2800000000002</v>
       </c>
       <c r="V35" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.23880597014925</v>
+        <v>51.79856115107913</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/26/2026 11:36</t>
+          <t>09/29/2026 11:40</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/26/2026 03:15</t>
+          <t>09/29/2026 03:18</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/27/2026 00:29</t>
+          <t>09/30/2026 00:32</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/27/2026 00:47</t>
+          <t>09/30/2026 00:50</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5333,22 +5333,13 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q42" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R42" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S42" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5420,7 +5411,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/27/2026 03:10</t>
+          <t>09/30/2026 03:12</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,22 +5433,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5529,20 +5511,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/28/2026 18:45</t>
+          <t>09/30/2026 19:57</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19959.09</v>
+        <v>19884.77</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-0.17</v>
+        <v>-0.55</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5551,37 +5533,28 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>199.18</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>3.483231517267173</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>772</v>
+        <v>789</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-40.90999999999994</v>
+        <v>-115.2300000000001</v>
       </c>
       <c r="V44" t="n">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>57.64248704663213</v>
+        <v>56.90747782002536</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5593,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5638,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/28/2026 17:20</t>
+          <t>10/01/2026 00:27</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5738,20 +5711,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/28/2026 17:50</t>
+          <t>10/01/2026 00:43</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19593.88</v>
-      </c>
-      <c r="I46" t="n">
-        <v>-2</v>
+        <v>19386.26</v>
+      </c>
+      <c r="I46" s="7" t="n">
+        <v>-3.04</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5760,37 +5733,28 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="n">
+        <v>93</v>
+      </c>
+      <c r="U46" s="7" t="n">
+        <v>-613.74</v>
+      </c>
+      <c r="V46" t="n">
         <v>40</v>
       </c>
-      <c r="O46" s="7" t="n">
-        <v>598.1899999999999</v>
-      </c>
-      <c r="P46" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="R46" s="7" t="n">
-        <v>1.424850852272727</v>
-      </c>
-      <c r="S46" s="7" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="T46" t="n">
-        <v>89</v>
-      </c>
-      <c r="U46" s="7" t="n">
-        <v>-406.12</v>
-      </c>
-      <c r="V46" t="n">
-        <v>39</v>
-      </c>
       <c r="W46" s="7" t="n">
-        <v>43.82022471910113</v>
+        <v>43.01075268817204</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5802,7 +5766,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5847,7 +5811,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/26/2026 23:49</t>
+          <t>09/29/2026 23:51</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5947,7 +5911,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09/27/2026 15:59</t>
+          <t>09/30/2026 16:03</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6047,7 +6011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/27/2026 00:38</t>
+          <t>09/30/2026 00:41</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6147,7 +6111,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/27/2026 00:16</t>
+          <t>09/30/2026 00:19</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6247,7 +6211,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/28/2026 17:33</t>
+          <t>10/01/2026 00:36</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6347,20 +6311,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/28/2026 18:27</t>
+          <t>09/30/2026 19:47</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19374.9</v>
+        <v>19276.9</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.1</v>
+        <v>-3.59</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>5.3</v>
+        <v>5.79</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6381,7 +6345,7 @@
         <v>114</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-625.1000000000001</v>
+        <v>-723.1000000000001</v>
       </c>
       <c r="V52" t="n">
         <v>45</v>
@@ -6390,10 +6354,10 @@
         <v>39.47368421052632</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>5.33</v>
+        <v>5.81</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6402,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6447,20 +6411,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/28/2026 19:14</t>
+          <t>09/30/2026 20:11</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19737.68</v>
+        <v>19711.51</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.35</v>
+        <v>-1.48</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6478,19 +6442,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>422</v>
+        <v>433</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-262.32</v>
+        <v>-288.49</v>
       </c>
       <c r="V53" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.78199052132701</v>
+        <v>35.56581986143187</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6502,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6547,7 +6511,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/26/2026 21:30</t>
+          <t>09/29/2026 21:33</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6647,7 +6611,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/28/2026 18:46</t>
+          <t>09/30/2026 20:00</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6847,20 +6811,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/28/2026 17:45</t>
+          <t>10/01/2026 00:40</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19611.9</v>
+        <v>19586.64</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.93</v>
+        <v>-2.06</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>2.01</v>
+        <v>2.06</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6869,40 +6833,31 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>-45.43</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>0.3725138121546961</v>
-      </c>
-      <c r="S57" s="7" t="n">
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1078</v>
+        <v>1102</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-387.6300000000001</v>
+        <v>-409.3699999999999</v>
       </c>
       <c r="V57" t="n">
-        <v>471</v>
+        <v>482</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.69202226345084</v>
+        <v>43.73865698729583</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>2.02</v>
+        <v>2.07</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6911,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6956,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/28/2026 18:34</t>
+          <t>09/30/2026 19:52</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7156,20 +7111,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/28/2026 18:15</t>
+          <t>09/30/2026 19:41</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>19177.85</v>
+        <v>19155.27</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-9.84</v>
+        <v>-9.949999999999999</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>21100.65</v>
@@ -7256,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/28/2026 19:48</t>
+          <t>09/30/2026 20:31</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7356,7 +7311,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>09/26/2026 21:21</t>
+          <t>09/29/2026 21:24</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7456,20 +7411,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/28/2026 10:17</t>
+          <t>09/30/2026 20:05</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18664.19</v>
+        <v>18584.3</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.7</v>
+        <v>-7.1</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7487,19 +7442,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1375.76</v>
+        <v>-1415.7</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>11.86440677966102</v>
+        <v>11.66666666666667</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7511,7 +7466,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7556,7 +7511,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/28/2026 19:40</t>
+          <t>09/30/2026 20:24</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7578,22 +7533,13 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>-90.82000000000002</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q64" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R64" s="7" t="n">
-        <v>0.7198297137216189</v>
-      </c>
-      <c r="S64" s="7" t="n">
-        <v>0.96</v>
+        <v>0</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7665,7 +7611,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/28/2026 18:54</t>
+          <t>09/30/2026 20:06</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7675,7 +7621,7 @@
         <v>-7.9</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>11.66</v>
+        <v>12.22</v>
       </c>
       <c r="K65" s="7" t="n">
         <v>0.89</v>
@@ -7765,7 +7711,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/28/2026 18:33</t>
+          <t>09/30/2026 19:51</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7865,20 +7811,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/28/2026 19:41</t>
+          <t>09/30/2026 20:24</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>21526.55</v>
+        <v>20792.48</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>7.67</v>
+        <v>3.99</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.17</v>
+        <v>1.08</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7896,19 +7842,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>1526.55</v>
+        <v>792.4799999999999</v>
       </c>
       <c r="V67" t="n">
         <v>29</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>34.11764705882353</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.17</v>
+        <v>1.08</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7920,7 +7866,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8065,7 +8011,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>09/26/2026 02:56</t>
+          <t>09/29/2026 02:58</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8165,7 +8111,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>09/26/2026 02:55</t>
+          <t>09/29/2026 02:58</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8265,7 +8211,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/26/2026 02:54</t>
+          <t>09/29/2026 02:57</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8365,7 +8311,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/28/2026 19:00</t>
+          <t>09/30/2026 20:05</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8465,7 +8411,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/28/2026 20:57</t>
+          <t>09/30/2026 21:04</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8565,7 +8511,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/28/2026 18:53</t>
+          <t>09/30/2026 20:01</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8665,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/20/2026 20:33</t>
+          <t>09/29/2026 20:45</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8765,7 +8711,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/26/2026 19:29</t>
+          <t>09/29/2026 19:31</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8865,7 +8811,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/23/2026 20:02</t>
+          <t>09/29/2026 20:08</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8965,7 +8911,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/26/2026 19:52</t>
+          <t>09/29/2026 19:55</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9065,7 +9011,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/26/2026 20:11</t>
+          <t>09/29/2026 20:13</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9165,7 +9111,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/26/2026 20:01</t>
+          <t>09/29/2026 20:04</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9265,7 +9211,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/26/2026 19:24</t>
+          <t>09/29/2026 19:26</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9365,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/26/2026 20:36</t>
+          <t>09/29/2026 20:38</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9465,7 +9411,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/26/2026 20:06</t>
+          <t>09/29/2026 20:09</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9565,7 +9511,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/26/2026 12:05</t>
+          <t>09/29/2026 12:08</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9665,7 +9611,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>09/27/2026 01:53</t>
+          <t>09/30/2026 01:56</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9787,22 +9733,13 @@
         <v>0</v>
       </c>
       <c r="N86" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>3093.07</v>
+        <v>0</v>
       </c>
       <c r="P86" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q86" s="7" t="n">
-        <v>51.51515151515152</v>
-      </c>
-      <c r="R86" s="7" t="n">
-        <v>12.34780056499248</v>
-      </c>
-      <c r="S86" s="7" t="n">
-        <v>2.89</v>
+        <v>0</v>
       </c>
       <c r="T86" t="n">
         <v>32</v>
@@ -9834,7 +9771,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC86" t="inlineStr">
@@ -9874,14 +9811,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/28/2026 21:04</t>
+          <t>09/30/2026 21:10</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19979.53</v>
+        <v>19974.49</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.54</v>
@@ -9905,16 +9842,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-20.47000000000003</v>
+        <v>-25.50999999999999</v>
       </c>
       <c r="V87" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>43.63636363636363</v>
+        <v>43.19526627218935</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>0.99</v>
@@ -9929,7 +9866,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10074,20 +10011,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/28/2026 20:36</t>
+          <t>09/30/2026 20:52</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20588.81</v>
+        <v>20366.81</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>2.94</v>
+        <v>1.82</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.29</v>
+        <v>1.16</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10105,19 +10042,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>588.8099999999999</v>
+        <v>366.8099999999999</v>
       </c>
       <c r="V89" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>85.38461538461539</v>
+        <v>83.94160583941606</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.29</v>
+        <v>1.16</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10129,7 +10066,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10174,20 +10111,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/28/2026 20:23</t>
+          <t>09/30/2026 20:45</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27282.84</v>
+        <v>27231.46</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>36.47</v>
+        <v>36.21</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>2.02</v>
+        <v>1.94</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10205,19 +10142,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7282.840000000001</v>
+        <v>7231.460000000001</v>
       </c>
       <c r="V90" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>70.58823529411765</v>
+        <v>70</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>2.02</v>
+        <v>1.94</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10229,7 +10166,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10274,7 +10211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/26/2026 19:03</t>
+          <t>09/29/2026 19:06</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10474,7 +10411,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/26/2026 13:55</t>
+          <t>09/29/2026 13:57</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10574,7 +10511,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/26/2026 13:50</t>
+          <t>09/29/2026 13:53</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10674,7 +10611,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/26/2026 13:42</t>
+          <t>09/29/2026 13:44</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10774,7 +10711,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/26/2026 23:45</t>
+          <t>09/29/2026 23:47</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10874,7 +10811,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/26/2026 19:03</t>
+          <t>09/29/2026 19:06</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10974,7 +10911,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/26/2026 19:15</t>
+          <t>09/29/2026 19:17</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11074,7 +11011,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/26/2026 23:49</t>
+          <t>09/29/2026 23:51</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11274,7 +11211,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>09/28/2026 21:55</t>
+          <t>09/30/2026 21:36</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11374,20 +11311,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/28/2026 18:30</t>
+          <t>09/30/2026 19:51</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>19980.22</v>
+        <v>19736.73</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-1.3</v>
       </c>
       <c r="J102" s="7" t="n">
-        <v>2.2</v>
+        <v>4.35</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>0.98</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11405,22 +11342,22 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>-19.77999999999996</v>
+        <v>-263.2700000000001</v>
       </c>
       <c r="V102" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>38.98305084745763</v>
+        <v>38.80597014925373</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>0.98</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y102" s="7" t="n">
-        <v>2.2</v>
+        <v>4.04</v>
       </c>
       <c r="Z102" t="inlineStr">
         <is>
@@ -11429,7 +11366,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11583,7 +11520,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>09/26/2026 01:46</t>
+          <t>09/29/2026 01:49</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11692,20 +11629,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>09/29/2026 01:10</t>
+          <t>09/30/2026 23:19</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11777.01</v>
+        <v>11734.89</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>17.73</v>
+        <v>17.31</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.89</v>
+        <v>2.47</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11723,19 +11660,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>2004.2</v>
+        <v>1962.079999999999</v>
       </c>
       <c r="V105" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>73.21428571428571</v>
+        <v>72.1311475409836</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.8</v>
+        <v>3.06</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11747,7 +11684,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11792,7 +11729,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/27/2026 11:40</t>
+          <t>09/30/2026 11:43</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11901,20 +11838,20 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>09/28/2026 16:44</t>
+          <t>10/01/2026 00:04</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>25876.64</v>
+        <v>24995.02</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-32.63</v>
+        <v>-34.93</v>
       </c>
       <c r="J107" s="7" t="n">
-        <v>39.57</v>
+        <v>40.85</v>
       </c>
       <c r="K107" s="7" t="n">
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
       <c r="L107" t="n">
         <v>25000</v>
@@ -11926,37 +11863,37 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-139.01</v>
+        <v>-904.96</v>
       </c>
       <c r="P107" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.7079130946377543</v>
+        <v>0.0467482672172246</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>1.9</v>
+        <v>3.79</v>
       </c>
       <c r="T107" t="n">
-        <v>3876</v>
+        <v>3917</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-8405.359999999999</v>
+        <v>-9286.980000000001</v>
       </c>
       <c r="V107" t="n">
         <v>2342</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>60.42311661506707</v>
+        <v>59.79065611437324</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
       <c r="Y107" s="7" t="n">
-        <v>40.92</v>
+        <v>42.87</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -11965,7 +11902,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12010,7 +11947,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 10:30</t>
+          <t>09/30/2026 10:34</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12101,7 +12038,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 06:00</t>
+          <t>09/30/2026 06:03</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12283,7 +12220,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>09/26/2026 16:59</t>
+          <t>09/29/2026 17:01</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12465,7 +12402,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 16:05</t>
+          <t>09/30/2026 16:08</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12556,7 +12493,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 11:39</t>
+          <t>09/30/2026 11:42</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12738,7 +12675,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 06:41</t>
+          <t>09/30/2026 06:44</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12920,7 +12857,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 00:03</t>
+          <t>09/30/2026 00:05</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13096,7 +13033,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>09/26/2026 20:59</t>
+          <t>09/29/2026 21:01</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13181,7 +13118,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/26/2026 15:30</t>
+          <t>09/29/2026 15:31</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13266,7 +13203,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/26/2026 02:56</t>
+          <t>09/29/2026 02:58</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13861,7 +13798,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 08:14</t>
+          <t>09/30/2026 08:17</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13952,7 +13889,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 07:46</t>
+          <t>09/30/2026 07:49</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14134,7 +14071,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/27/2026 13:51</t>
+          <t>09/30/2026 13:55</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14309,7 +14246,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/27/2026 10:30</t>
+          <t>09/30/2026 10:34</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14350,7 +14287,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/27/2026 06:00</t>
+          <t>09/30/2026 06:03</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14432,7 +14369,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09/26/2026 16:59</t>
+          <t>09/29/2026 17:01</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14514,7 +14451,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09/27/2026 16:05</t>
+          <t>09/30/2026 16:08</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14555,7 +14492,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/27/2026 11:39</t>
+          <t>09/30/2026 11:42</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14637,7 +14574,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/27/2026 06:41</t>
+          <t>09/30/2026 06:44</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14719,7 +14656,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/27/2026 00:03</t>
+          <t>09/30/2026 00:05</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14801,7 +14738,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>09/26/2026 20:59</t>
+          <t>09/29/2026 21:01</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14842,7 +14779,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09/26/2026 15:30</t>
+          <t>09/29/2026 15:31</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14883,7 +14820,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/26/2026 02:56</t>
+          <t>09/29/2026 02:58</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -15170,7 +15107,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/27/2026 08:14</t>
+          <t>09/30/2026 08:17</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15211,7 +15148,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/27/2026 07:46</t>
+          <t>09/30/2026 07:49</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15293,7 +15230,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/27/2026 13:51</t>
+          <t>09/30/2026 13:55</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17584,7 +17521,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09/24/2026 09:47</t>
+          <t>09/30/2026 09:58</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17630,7 +17567,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/27/2026 09:39</t>
+          <t>09/30/2026 09:41</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17653,7 +17590,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/27/2026 04:54</t>
+          <t>09/30/2026 04:57</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17676,7 +17613,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09/26/2026 02:03</t>
+          <t>09/29/2026 02:06</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17722,7 +17659,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09/27/2026 04:07</t>
+          <t>09/30/2026 04:10</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17791,7 +17728,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/27/2026 10:55</t>
+          <t>09/30/2026 10:58</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17837,7 +17774,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/27/2026 09:31</t>
+          <t>09/30/2026 09:34</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17883,7 +17820,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09/26/2026 02:20</t>
+          <t>09/29/2026 02:23</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17906,7 +17843,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09/26/2026 02:04</t>
+          <t>09/29/2026 02:08</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -17929,7 +17866,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/27/2026 12:12</t>
+          <t>09/30/2026 12:17</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17952,7 +17889,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/27/2026 04:39</t>
+          <t>09/30/2026 04:44</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -17975,7 +17912,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/27/2026 14:30</t>
+          <t>09/30/2026 14:34</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17998,7 +17935,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/27/2026 11:00</t>
+          <t>09/30/2026 11:03</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18044,7 +17981,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/27/2026 12:08</t>
+          <t>09/30/2026 12:11</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18136,7 +18073,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09/26/2026 23:10</t>
+          <t>09/29/2026 23:13</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18159,7 +18096,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09/26/2026 23:24</t>
+          <t>09/29/2026 23:27</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18297,7 +18234,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/27/2026 09:33</t>
+          <t>09/30/2026 09:36</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18320,7 +18257,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/27/2026 10:15</t>
+          <t>09/30/2026 10:18</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18343,7 +18280,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/27/2026 13:46</t>
+          <t>09/30/2026 13:49</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18366,7 +18303,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>09/28/2026 14:15</t>
+          <t>09/30/2026 14:20</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-30
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/28/2026 01:07</t>
+          <t>10/01/2026 01:09</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/30/2026 19:35</t>
+          <t>10/01/2026 00:48</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/30/2026 20:47</t>
+          <t>10/01/2026 02:00</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09/30/2026 19:52</t>
+          <t>10/01/2026 01:05</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>09/30/2026 19:33</t>
+          <t>10/01/2026 00:46</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>09/30/2026 19:39</t>
+          <t>10/01/2026 00:52</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09/30/2026 19:56</t>
+          <t>10/01/2026 01:09</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -5333,13 +5333,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5433,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5511,11 +5529,11 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/30/2026 19:57</t>
+          <t>10/01/2026 01:10</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19884.77</v>
+        <v>19884.01</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>-0.55</v>
@@ -5533,13 +5551,22 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>13.00999999999999</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>1.075714368852936</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>0.71</v>
       </c>
       <c r="T44" t="n">
         <v>789</v>
@@ -5633,13 +5660,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-26.6</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.6475887652358241</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T45" t="n">
         <v>54</v>
@@ -5733,13 +5769,22 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>368.6999999999999</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>1.243665490304929</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>3.06</v>
       </c>
       <c r="T46" t="n">
         <v>93</v>
@@ -5833,13 +5878,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5933,13 +5987,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6033,13 +6096,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T49" t="n">
         <v>1161</v>
@@ -6133,13 +6205,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>-52.41999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>0.8051952878219183</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>1.3</v>
       </c>
       <c r="T50" t="n">
         <v>1978</v>
@@ -6233,13 +6314,22 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>0</v>
+        <v>963.6800000000001</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R51" s="7" t="n">
+        <v>1.279444173800079</v>
+      </c>
+      <c r="S51" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="T51" t="n">
         <v>68</v>
@@ -6311,7 +6401,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/30/2026 19:47</t>
+          <t>10/01/2026 01:00</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6333,13 +6423,22 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>-1018.16</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>0.5725967592981278</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>5.77</v>
       </c>
       <c r="T52" t="n">
         <v>114</v>
@@ -6411,7 +6510,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/30/2026 20:11</t>
+          <t>10/01/2026 01:24</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
@@ -6433,13 +6532,22 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>0</v>
+        <v>-53.3</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q53" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R53" s="7" t="n">
+        <v>0.5529273611810099</v>
+      </c>
+      <c r="S53" s="7" t="n">
+        <v>0.42</v>
       </c>
       <c r="T53" t="n">
         <v>433</v>
@@ -6533,13 +6641,22 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>0</v>
+        <v>-149.77</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q54" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R54" s="7" t="n">
+        <v>0.4112351599968551</v>
+      </c>
+      <c r="S54" s="7" t="n">
+        <v>0.83</v>
       </c>
       <c r="T54" t="n">
         <v>229</v>
@@ -6611,7 +6728,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/30/2026 20:00</t>
+          <t>10/01/2026 01:13</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6633,13 +6750,22 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>0</v>
+        <v>-104.34</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q55" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R55" s="7" t="n">
+        <v>0.347793474184273</v>
+      </c>
+      <c r="S55" s="7" t="n">
+        <v>0.52</v>
       </c>
       <c r="T55" t="n">
         <v>1920</v>
@@ -6733,13 +6859,22 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>0</v>
+        <v>4.35</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q56" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R56" s="7" t="n">
+        <v>1.066564651874522</v>
+      </c>
+      <c r="S56" s="7" t="n">
+        <v>0.16</v>
       </c>
       <c r="T56" t="n">
         <v>1272</v>
@@ -6833,25 +6968,34 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-36.6</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.4392523364485982</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.18</v>
       </c>
       <c r="T57" t="n">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-409.3699999999999</v>
+        <v>-411.49</v>
       </c>
       <c r="V57" t="n">
         <v>482</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.73865698729583</v>
+        <v>43.61990950226244</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.76</v>
@@ -6866,7 +7010,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +7055,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/30/2026 19:52</t>
+          <t>10/01/2026 01:07</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -6933,13 +7077,22 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>0</v>
+        <v>-269.38</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q58" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R58" s="7" t="n">
+        <v>0.1222834055586328</v>
+      </c>
+      <c r="S58" s="7" t="n">
+        <v>1.35</v>
       </c>
       <c r="T58" t="n">
         <v>4426</v>
@@ -7033,13 +7186,22 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>0</v>
+        <v>-80.78999999999999</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="Q59" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R59" s="7" t="n">
+        <v>0.32387647501883</v>
+      </c>
+      <c r="S59" s="7" t="n">
+        <v>0.43</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7111,7 +7273,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/30/2026 19:41</t>
+          <t>10/01/2026 00:54</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7133,13 +7295,22 @@
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>0</v>
+        <v>-1105.06</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q60" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R60" s="7" t="n">
+        <v>0.2343571374133069</v>
+      </c>
+      <c r="S60" s="7" t="n">
+        <v>6.68</v>
       </c>
       <c r="T60" t="n">
         <v>7019</v>
@@ -7211,7 +7382,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/30/2026 20:31</t>
+          <t>10/01/2026 01:44</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7233,13 +7404,22 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>0</v>
+        <v>-448.41</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q61" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R61" s="7" t="n">
+        <v>0.480495858193825</v>
+      </c>
+      <c r="S61" s="7" t="n">
+        <v>3.68</v>
       </c>
       <c r="T61" t="n">
         <v>3982</v>
@@ -7411,7 +7591,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/30/2026 20:05</t>
+          <t>10/01/2026 01:18</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7433,13 +7613,22 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>0</v>
+        <v>-190.42</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Q63" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="R63" s="7" t="n">
+        <v>0.8552643580310725</v>
+      </c>
+      <c r="S63" s="7" t="n">
+        <v>2.54</v>
       </c>
       <c r="T63" t="n">
         <v>60</v>
@@ -7511,7 +7700,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/30/2026 20:24</t>
+          <t>10/01/2026 01:38</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7533,13 +7722,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-90.82000000000002</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.7198297137216189</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>0.96</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7611,7 +7809,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/30/2026 20:06</t>
+          <t>10/01/2026 01:20</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7633,13 +7831,22 @@
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O65" s="7" t="n">
-        <v>0</v>
+        <v>-1009.4</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q65" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R65" s="7" t="n">
+        <v>0.4962168852688107</v>
+      </c>
+      <c r="S65" s="7" t="n">
+        <v>7.37</v>
       </c>
       <c r="T65" t="n">
         <v>3298</v>
@@ -7711,7 +7918,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/30/2026 19:51</t>
+          <t>10/01/2026 01:04</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,7 +8018,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>09/30/2026 20:24</t>
+          <t>10/01/2026 01:38</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -8311,7 +8518,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>09/30/2026 20:05</t>
+          <t>10/01/2026 01:18</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8333,13 +8540,22 @@
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O72" s="7" t="n">
-        <v>0</v>
+        <v>-19.59</v>
       </c>
       <c r="P72" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q72" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R72" s="7" t="n">
+        <v>0.8233543733092877</v>
+      </c>
+      <c r="S72" s="7" t="n">
+        <v>0.23</v>
       </c>
       <c r="T72" t="n">
         <v>326</v>
@@ -8433,13 +8649,22 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>0</v>
+        <v>-39.43999999999999</v>
       </c>
       <c r="P73" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q73" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R73" s="7" t="n">
+        <v>0.8172212438594866</v>
+      </c>
+      <c r="S73" s="7" t="n">
+        <v>0.49</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -8511,7 +8736,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>09/30/2026 20:01</t>
+          <t>10/01/2026 01:13</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8533,13 +8758,22 @@
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>0</v>
+        <v>-53.91</v>
       </c>
       <c r="P74" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q74" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R74" s="7" t="n">
+        <v>0.8335391835978508</v>
+      </c>
+      <c r="S74" s="7" t="n">
+        <v>0.73</v>
       </c>
       <c r="T74" t="n">
         <v>329</v>
@@ -9033,13 +9267,22 @@
         <v>0</v>
       </c>
       <c r="N79" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O79" s="7" t="n">
-        <v>0</v>
+        <v>-124.11</v>
       </c>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q79" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R79" s="7" t="n">
+        <v>0.8885296257376122</v>
+      </c>
+      <c r="S79" s="7" t="n">
+        <v>3.16</v>
       </c>
       <c r="T79" t="n">
         <v>94</v>
@@ -9233,13 +9476,22 @@
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O81" s="7" t="n">
-        <v>0</v>
+        <v>698.3099999999999</v>
       </c>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="Q81" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="R81" s="7" t="n">
+        <v>4.02390334733469</v>
+      </c>
+      <c r="S81" s="7" t="n">
+        <v>0.64</v>
       </c>
       <c r="T81" t="n">
         <v>2303</v>
@@ -9333,13 +9585,22 @@
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>0</v>
+        <v>-308.22</v>
       </c>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q82" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R82" s="7" t="n">
+        <v>0.412903102916246</v>
+      </c>
+      <c r="S82" s="7" t="n">
+        <v>1.62</v>
       </c>
       <c r="T82" t="n">
         <v>1156</v>
@@ -9533,13 +9794,22 @@
         <v>0</v>
       </c>
       <c r="N84" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O84" s="7" t="n">
-        <v>0</v>
+        <v>20136.49</v>
       </c>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="Q84" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="R84" s="7" t="n">
+        <v>408.2914644012945</v>
+      </c>
+      <c r="S84" s="7" t="n">
+        <v>0.12</v>
       </c>
       <c r="T84" t="n">
         <v>3</v>
@@ -9571,7 +9841,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC84" t="inlineStr">
@@ -9707,7 +9977,7 @@
         </is>
       </c>
       <c r="F86" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -9933,13 +10203,22 @@
         <v>0</v>
       </c>
       <c r="N88" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O88" s="7" t="n">
-        <v>0</v>
+        <v>20470.4</v>
       </c>
       <c r="P88" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q88" s="7" t="n">
+        <v>83.33333333333334</v>
+      </c>
+      <c r="R88" s="7" t="n">
+        <v>191.0687093779016</v>
+      </c>
+      <c r="S88" s="7" t="n">
+        <v>0.17</v>
       </c>
       <c r="T88" t="n">
         <v>17</v>
@@ -9971,7 +10250,7 @@
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC88" t="inlineStr">
@@ -10011,14 +10290,14 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>09/30/2026 20:52</t>
+          <t>10/01/2026 02:04</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20366.81</v>
+        <v>20379.51</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>1.82</v>
+        <v>1.88</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
@@ -10033,13 +10312,22 @@
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O89" s="7" t="n">
-        <v>0</v>
+        <v>9.98</v>
       </c>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>33</v>
+      </c>
+      <c r="Q89" s="7" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="R89" s="7" t="n">
+        <v>1.013021920668058</v>
+      </c>
+      <c r="S89" s="7" t="n">
+        <v>1.4</v>
       </c>
       <c r="T89" t="n">
         <v>137</v>
@@ -10111,7 +10399,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/30/2026 20:45</t>
+          <t>10/01/2026 01:58</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
@@ -11311,7 +11599,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>09/30/2026 19:51</t>
+          <t>10/01/2026 01:03</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11878,7 +12166,7 @@
         <v>3.79</v>
       </c>
       <c r="T107" t="n">
-        <v>3917</v>
+        <v>3918</v>
       </c>
       <c r="U107" s="7" t="n">
         <v>-9286.980000000001</v>
@@ -11887,7 +12175,7 @@
         <v>2342</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>59.79065611437324</v>
+        <v>59.7753956100051</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.76</v>
@@ -12970,17 +13258,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13055,17 +13349,23 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q120" s="8" t="n"/>
-      <c r="R120" s="8" t="n"/>
-      <c r="S120" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q120" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R120" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S120" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13140,17 +13440,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13310,17 +13616,23 @@
         <v>0</v>
       </c>
       <c r="N123" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O123" s="9" t="n">
-        <v>0</v>
+        <v>-413.36</v>
       </c>
       <c r="P123" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q123" s="8" t="n"/>
-      <c r="R123" s="8" t="n"/>
-      <c r="S123" s="8" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="Q123" s="9" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R123" s="9" t="n">
+        <v>0.2523107533689066</v>
+      </c>
+      <c r="S123" s="9" t="n">
+        <v>0.83</v>
+      </c>
       <c r="T123" s="8" t="n">
         <v>0</v>
       </c>
@@ -13735,17 +14047,23 @@
         <v>0</v>
       </c>
       <c r="N128" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O128" s="9" t="n">
-        <v>0</v>
+        <v>-1038.15</v>
       </c>
       <c r="P128" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q128" s="8" t="n"/>
-      <c r="R128" s="8" t="n"/>
-      <c r="S128" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q128" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R128" s="9" t="n">
+        <v>0.2354119561935203</v>
+      </c>
+      <c r="S128" s="9" t="n">
+        <v>1.16</v>
+      </c>
       <c r="T128" s="8" t="n">
         <v>0</v>
       </c>
@@ -14707,7 +15025,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14748,7 +15066,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -14789,7 +15107,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14871,7 +15189,7 @@
         <v>-1.27</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21">
@@ -15076,7 +15394,7 @@
         <v>-3.92</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26">
@@ -15254,7 +15572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -15477,7 +15795,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>47370</t>
+          <t>47369</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -15487,7 +15805,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Donchain Mean Reversion ML</t>
+          <t>Donchain Breakout ML</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -15495,14 +15813,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>47771</t>
+          <t>47370</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -15516,18 +15834,18 @@
         </is>
       </c>
       <c r="D12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>47774</t>
+          <t>47771</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -15537,7 +15855,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Adaptive Regime Trader</t>
+          <t>Donchain Mean Reversion ML</t>
         </is>
       </c>
       <c r="D13" t="b">
@@ -15545,14 +15863,14 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>47777</t>
+          <t>47774</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -15562,7 +15880,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Automation Tester</t>
+          <t>Adaptive Regime Trader</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -15570,14 +15888,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>49058</t>
+          <t>47777</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -15587,7 +15905,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Momentum Master ML 2</t>
+          <t>Automation Tester</t>
         </is>
       </c>
       <c r="D15" t="b">
@@ -15602,7 +15920,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>49059</t>
+          <t>49058</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -15612,22 +15930,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Orbgasmatron PropBots</t>
+          <t>Momentum Master ML 2</t>
         </is>
       </c>
       <c r="D16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>49060</t>
+          <t>49059</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -15637,7 +15955,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TapDancer</t>
+          <t>Orbgasmatron PropBots</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -15652,7 +15970,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>49061</t>
+          <t>49060</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -15662,7 +15980,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Orbgasmatron MOL Bots</t>
+          <t>TapDancer</t>
         </is>
       </c>
       <c r="D18" t="b">
@@ -15677,7 +15995,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>49063</t>
+          <t>49061</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -15687,7 +16005,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ML Trader</t>
+          <t>Orbgasmatron MOL Bots</t>
         </is>
       </c>
       <c r="D19" t="b">
@@ -15702,7 +16020,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>53896</t>
+          <t>49063</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -15712,7 +16030,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Codex AggressiveV2_DemoScout</t>
+          <t>ML Trader</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -15720,24 +16038,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>54284</t>
+          <t>53896</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sweep suite</t>
+          <t>Codex AggressiveV2_DemoScout</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -15745,14 +16063,14 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>54285</t>
+          <t>54284</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -15762,7 +16080,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NY Killzone</t>
+          <t>Sweep suite</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -15777,17 +16095,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>55123</t>
+          <t>54285</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>T&amp;D19L9 MOL</t>
+          <t>NY Killzone</t>
         </is>
       </c>
       <c r="D23" t="b">
@@ -15795,14 +16113,14 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>55209</t>
+          <t>55123</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -15812,7 +16130,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>T&amp;D19L8 V2 MOL</t>
+          <t>T&amp;D19L9 MOL</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -15827,7 +16145,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>55384</t>
+          <t>55209</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -15837,7 +16155,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>T&amp;D19L10 V2 MOL</t>
+          <t>T&amp;D19L8 V2 MOL</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -15852,7 +16170,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>55388</t>
+          <t>55384</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -15862,7 +16180,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>T&amp;D19L10 V2 Agg</t>
+          <t>T&amp;D19L10 V2 MOL</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -15877,7 +16195,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>55389</t>
+          <t>55388</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -15887,7 +16205,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>T&amp;D19L10 V2 Prop</t>
+          <t>T&amp;D19L10 V2 Agg</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -15902,7 +16220,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>55390</t>
+          <t>55389</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -15912,7 +16230,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>T&amp;D19L10 V2 RClock</t>
+          <t>T&amp;D19L10 V2 Prop</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -15927,7 +16245,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>55391</t>
+          <t>55390</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -15937,7 +16255,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>T&amp;D19L9 V2 Agg</t>
+          <t>T&amp;D19L10 V2 RClock</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -15952,7 +16270,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>55392</t>
+          <t>55391</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -15962,7 +16280,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>T&amp;D19L9 V2 Prop</t>
+          <t>T&amp;D19L9 V2 Agg</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -15977,7 +16295,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>55393</t>
+          <t>55392</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -15987,7 +16305,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>T&amp;D19L9 V2 RClock</t>
+          <t>T&amp;D19L9 V2 Prop</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -16002,32 +16320,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>55955</t>
+          <t>55393</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LIVE Dream Catcher Gold</t>
+          <t>T&amp;D19L9 V2 RClock</t>
         </is>
       </c>
       <c r="D32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>55956</t>
+          <t>55955</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -16037,11 +16355,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LIVE Time and Day Cells</t>
+          <t>LIVE Dream Catcher Gold</t>
         </is>
       </c>
       <c r="D33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -16052,42 +16370,42 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>55966</t>
+          <t>55956</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Range Snap USDJPY</t>
+          <t>LIVE Time and Day Cells</t>
         </is>
       </c>
       <c r="D34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>56912</t>
+          <t>55966</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>licensed</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Smart Owl FX</t>
+          <t>Range Snap USDJPY</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -16095,39 +16413,39 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>56915</t>
+          <t>56912</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>licensed</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Prop</t>
+          <t>Smart Owl FX</t>
         </is>
       </c>
       <c r="D36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>57575</t>
+          <t>56915</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -16137,11 +16455,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Gold Snap 1.1</t>
+          <t>T&amp;D19L13 L8 Prop</t>
         </is>
       </c>
       <c r="D37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -16152,7 +16470,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>57677</t>
+          <t>57575</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -16162,57 +16480,57 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 RCLOCK</t>
+          <t>Gold Snap 1.1</t>
         </is>
       </c>
       <c r="D38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>57681</t>
+          <t>57677</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>licensed</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Demo AuRange Gold Reaper + DC + TALON</t>
+          <t>T&amp;D19L13 Meta4 RCLOCK</t>
         </is>
       </c>
       <c r="D39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>57685</t>
+          <t>57681</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>licensed</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Gold Talon Vt15 Demo</t>
+          <t>Demo AuRange Gold Reaper + DC + TALON</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -16227,7 +16545,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>57686</t>
+          <t>57685</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -16237,7 +16555,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Talon V2 Stocks</t>
+          <t>Gold Talon Vt15 Demo</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -16252,7 +16570,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>57687</t>
+          <t>57686</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -16262,7 +16580,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Chaos Fractal Alligator</t>
+          <t>Talon V2 Stocks</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -16277,7 +16595,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>57688</t>
+          <t>57687</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -16287,7 +16605,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Squeeze Breakout Indices</t>
+          <t>Chaos Fractal Alligator</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -16302,7 +16620,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>57689</t>
+          <t>57688</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -16312,7 +16630,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>VWAP Mean Reversion</t>
+          <t>Squeeze Breakout Indices</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -16327,7 +16645,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>57691</t>
+          <t>57689</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -16337,7 +16655,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Gold Overnight</t>
+          <t>VWAP Mean Reversion</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -16352,7 +16670,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>57694</t>
+          <t>57691</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -16362,7 +16680,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dream Talon Book</t>
+          <t>Gold Overnight</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -16377,7 +16695,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>57695</t>
+          <t>57694</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -16387,7 +16705,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dual Thrust Strategy</t>
+          <t>Dream Talon Book</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -16402,7 +16720,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>57703</t>
+          <t>57695</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -16412,11 +16730,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Gold Snap Demo 2</t>
+          <t>Dual Thrust Strategy</t>
         </is>
       </c>
       <c r="D48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -16427,7 +16745,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>57710</t>
+          <t>57703</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -16437,32 +16755,32 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Donchian H6 5520</t>
+          <t>Gold Snap Demo 2</t>
         </is>
       </c>
       <c r="D49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>57825</t>
+          <t>57706</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>LIVE Portfolio: Midnight Raven + Gold Reaper + AuRange</t>
+          <t>Donchian H2 Portfolio (VPS92)</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -16470,14 +16788,14 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>58303</t>
+          <t>57710</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -16487,7 +16805,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Prop</t>
+          <t>Donchian H6 Portfolio (VPS92)</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -16495,24 +16813,24 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>58304</t>
+          <t>57825</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 MOL</t>
+          <t>LIVE Portfolio: Midnight Raven + Gold Reaper + AuRange</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -16520,14 +16838,14 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>58305</t>
+          <t>58303</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -16537,7 +16855,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Agg</t>
+          <t>T&amp;D19L13 L8 Prop</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -16552,7 +16870,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>58306</t>
+          <t>58304</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -16562,7 +16880,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Prop</t>
+          <t>T&amp;D19L13 L8 MOL</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -16577,7 +16895,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>58307</t>
+          <t>58305</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -16587,7 +16905,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 MOL</t>
+          <t>T&amp;D19L13 L8 Agg</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -16602,7 +16920,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>58308</t>
+          <t>58306</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -16612,7 +16930,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Agg</t>
+          <t>T&amp;D19L13 L11 Prop</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -16627,7 +16945,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>58309</t>
+          <t>58307</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -16637,7 +16955,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DreamCatcher New Sleeves V3</t>
+          <t>T&amp;D19L13 L11 MOL</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -16645,14 +16963,14 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>58310</t>
+          <t>58308</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -16662,7 +16980,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Donchian H2 Portfolio</t>
+          <t>T&amp;D19L13 L11 Agg</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -16670,14 +16988,14 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>58311</t>
+          <t>58309</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -16687,7 +17005,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Donchian H6 Portfolio</t>
+          <t>DreamCatcher New Sleeves V3</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -16695,14 +17013,14 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>58312</t>
+          <t>58310</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -16712,7 +17030,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>DreamCatcher DCv3</t>
+          <t>Donchian H2 Portfolio</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -16727,7 +17045,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>58313</t>
+          <t>58311</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -16737,7 +17055,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Zfade Portfolio 2</t>
+          <t>Donchian H6 Portfolio</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -16752,17 +17070,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>58314</t>
+          <t>58312</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>licensed</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LunaAI Pro</t>
+          <t>DreamCatcher DCv3</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -16770,14 +17088,14 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>58315</t>
+          <t>58313</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -16787,7 +17105,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Gold SuperScalp</t>
+          <t>Zfade Portfolio 2</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -16795,24 +17113,24 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>58316</t>
+          <t>58314</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>licensed</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>3EMA Core5 (DD ERC)</t>
+          <t>LunaAI Pro</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -16820,14 +17138,14 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>58318</t>
+          <t>58315</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -16837,7 +17155,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Agg</t>
+          <t>Gold SuperScalp</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -16845,14 +17163,14 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>58319</t>
+          <t>58316</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -16862,7 +17180,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop</t>
+          <t>3EMA Core5 (DD ERC)</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -16870,14 +17188,14 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>58320</t>
+          <t>58318</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -16887,7 +17205,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL</t>
+          <t>T&amp;D19L13 L10 Agg</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -16902,7 +17220,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>58321</t>
+          <t>58319</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -16912,7 +17230,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg</t>
+          <t>T&amp;D19L13 Meta4 Prop</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -16927,7 +17245,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>58322</t>
+          <t>58320</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -16937,7 +17255,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 RCLOCK</t>
+          <t>T&amp;D19L13 Meta4 MOL</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -16952,7 +17270,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>58323</t>
+          <t>58321</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -16962,7 +17280,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Prop</t>
+          <t>T&amp;D19L13 Meta4 Agg</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -16977,7 +17295,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>58324</t>
+          <t>58322</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -16987,7 +17305,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop</t>
+          <t>T&amp;D19L13 Meta4 RCLOCK</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -17002,7 +17320,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>58325</t>
+          <t>58323</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -17012,7 +17330,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Agg</t>
+          <t>T&amp;D19L13 L9 Prop</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -17027,7 +17345,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>58326</t>
+          <t>58324</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -17037,7 +17355,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Agg Control</t>
+          <t>T&amp;D19L13 L10 Prop</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -17052,7 +17370,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>58327</t>
+          <t>58325</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -17062,7 +17380,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 MOL</t>
+          <t>T&amp;D19L13 L9 Agg</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -17077,7 +17395,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>58328</t>
+          <t>58326</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -17087,7 +17405,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 RCLOCK</t>
+          <t>T&amp;D19L13 L9 Agg Control</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -17102,7 +17420,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>58329</t>
+          <t>58327</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -17112,7 +17430,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 MOL</t>
+          <t>T&amp;D19L13 L9 MOL</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -17127,7 +17445,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>58991</t>
+          <t>58328</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -17137,7 +17455,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Golden Fractal</t>
+          <t>T&amp;D19L13 L9 RCLOCK</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -17145,14 +17463,14 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>58993</t>
+          <t>58329</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -17162,7 +17480,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Levels</t>
+          <t>T&amp;D19L13 L10 MOL</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -17170,24 +17488,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>59376</t>
+          <t>58992</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>For Gold Snap 2HR / Smart Gold Hunter</t>
+          <t>Golden Fractal</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -17195,24 +17513,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>59377</t>
+          <t>58993</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Gold Snap 2HR</t>
+          <t>Levels</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -17220,14 +17538,14 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>59376</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -17237,7 +17555,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>For Gold Snap 2HR / Smart Gold Hunter</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -17245,14 +17563,14 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS153t2</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>59377</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -17262,11 +17580,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>Gold Snap 2HR</t>
         </is>
       </c>
       <c r="D82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -17277,7 +17595,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>662436</t>
+          <t>662434</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -17287,7 +17605,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 GBPJPY + XAUUSD</t>
+          <t>LIVE Gold Reaper Conservative</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -17302,7 +17620,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>663097</t>
+          <t>662435</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -17312,32 +17630,32 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 USDJPY, GBPJPY + XAGUSD</t>
+          <t>Aggv1 Pro Filter 60</t>
         </is>
       </c>
       <c r="D84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1115442</t>
+          <t>662436</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Gold Snap Internal</t>
+          <t>LIVE Talon v2 GBPJPY + XAUUSD</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -17345,39 +17663,39 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1115443</t>
+          <t>663097</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta MOL</t>
+          <t>LIVE Gold Talon V2 USDJPY, GBPJPY + XAGUSD</t>
         </is>
       </c>
       <c r="D86" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1115444</t>
+          <t>1115442</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -17387,7 +17705,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Gold Snap Demo</t>
+          <t>Gold Snap Internal</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -17402,7 +17720,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>14189968</t>
+          <t>1115443</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -17412,7 +17730,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+          <t>T&amp;D19L13 Meta MOL</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -17420,14 +17738,14 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>600025868</t>
+          <t>1115444</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -17437,13 +17755,63 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>FTMO Manual Trading</t>
+          <t>Gold Snap Demo</t>
         </is>
       </c>
       <c r="D89" t="b">
         <v>1</v>
       </c>
       <c r="E89" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>14189968</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+        </is>
+      </c>
+      <c r="D90" t="b">
+        <v>0</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>600025868</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>FTMO Manual Trading</t>
+        </is>
+      </c>
+      <c r="D91" t="b">
+        <v>1</v>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>

</xml_diff>

<commit_message>
Update dashboards — 2026-10-02
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-01 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-02 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/01/2026 21:28</t>
+          <t>10/02/2026 11:38</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
@@ -1000,16 +1000,16 @@
         <v>50.73</v>
       </c>
       <c r="T2" t="n">
-        <v>3456</v>
+        <v>3467</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>18453.4</v>
+        <v>19027.37</v>
       </c>
       <c r="V2" t="n">
-        <v>2196</v>
+        <v>2205</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.54166666666666</v>
+        <v>63.59965387943467</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.03</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>09/29/2026 09:37</t>
+          <t>10/02/2026 09:40</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>09/29/2026 02:39</t>
+          <t>10/02/2026 02:42</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09/29/2026 10:56</t>
+          <t>10/02/2026 10:58</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/29/2026 03:09</t>
+          <t>10/02/2026 03:11</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>09/29/2026 13:41</t>
+          <t>10/02/2026 13:44</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>09/29/2026 06:17</t>
+          <t>10/02/2026 06:20</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09/29/2026 06:22</t>
+          <t>10/02/2026 06:25</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/01/2026 17:30</t>
+          <t>10/02/2026 09:29</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/01/2026 22:19</t>
+          <t>10/02/2026 12:08</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/02/2026 00:55</t>
+          <t>10/02/2026 13:41</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19494.84</v>
+        <v>19515.33</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.68</v>
+        <v>-2.58</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.74</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-367.24</v>
+        <v>-272.96</v>
       </c>
       <c r="P23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q23" s="7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="R23" s="7" t="n">
+        <v>0.2928680604129427</v>
+      </c>
+      <c r="S23" s="7" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="T23" t="n">
+        <v>77</v>
+      </c>
+      <c r="U23" s="7" t="n">
+        <v>-484.6700000000001</v>
+      </c>
+      <c r="V23" t="n">
         <v>20</v>
       </c>
-      <c r="R23" s="7" t="n">
-        <v>0.1841105507542601</v>
-      </c>
-      <c r="S23" s="7" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="T23" t="n">
-        <v>74</v>
-      </c>
-      <c r="U23" s="7" t="n">
-        <v>-505.1600000000001</v>
-      </c>
-      <c r="V23" t="n">
-        <v>19</v>
-      </c>
       <c r="W23" s="7" t="n">
-        <v>25.67567567567567</v>
+        <v>25.97402597402597</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.58</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/01/2026 22:58</t>
+          <t>10/02/2026 12:28</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/29/2026 23:18</t>
+          <t>10/02/2026 23:37</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/01/2026 22:17</t>
+          <t>10/02/2026 12:07</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3619,13 +3619,13 @@
         <v>139</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>231.8300000000003</v>
+        <v>256.6400000000003</v>
       </c>
       <c r="V26" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>43.16546762589928</v>
+        <v>43.88489208633094</v>
       </c>
       <c r="X26" s="7" t="n">
         <v>1.04</v>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/01/2026 22:29</t>
+          <t>10/02/2026 12:14</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/01/2026 23:08</t>
+          <t>10/02/2026 12:34</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20533.84</v>
+        <v>20560.31</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.7</v>
+        <v>2.83</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.59</v>
+        <v>1.61</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-180.73</v>
+        <v>-181.24</v>
       </c>
       <c r="P30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>25</v>
+        <v>22.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.3683419544247169</v>
+        <v>0.3687216997561825</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>1.13</v>
       </c>
       <c r="T30" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>533.8399999999999</v>
+        <v>560.3099999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>25.74257425742574</v>
+        <v>26.21359223300971</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.59</v>
+        <v>1.61</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/29/2026 10:58</t>
+          <t>10/02/2026 11:01</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>09/29/2026 11:50</t>
+          <t>10/02/2026 11:52</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09/29/2026 16:14</t>
+          <t>10/02/2026 16:49</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/29/2026 03:52</t>
+          <t>10/02/2026 03:54</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/01/2026 16:41</t>
+          <t>10/02/2026 14:59</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20867.74</v>
+        <v>20642.02</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>4.34</v>
+        <v>3.21</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.13</v>
+        <v>1.09</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>752.0600000000002</v>
+        <v>642.0199999999999</v>
       </c>
       <c r="V35" t="n">
         <v>75</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.8169014084507</v>
+        <v>52.08333333333334</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/29/2026 11:40</t>
+          <t>10/02/2026 11:41</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/29/2026 03:18</t>
+          <t>10/02/2026 03:22</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -5511,14 +5511,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/01/2026 23:10</t>
+          <t>10/02/2026 12:35</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19715.18</v>
+        <v>19713.72</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.4</v>
+        <v>-1.41</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5542,16 +5542,16 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>808</v>
+        <v>815</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-284.8200000000001</v>
+        <v>-292.7100000000001</v>
       </c>
       <c r="V44" t="n">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.81683168316832</v>
+        <v>55.58282208588957</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/01/2026 21:45</t>
+          <t>10/02/2026 11:47</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/01/2026 22:10</t>
+          <t>10/02/2026 12:04</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/29/2026 23:51</t>
+          <t>10/03/2026 00:03</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/30/2026 00:19</t>
+          <t>10/03/2026 00:30</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/01/2026 21:54</t>
+          <t>10/02/2026 11:53</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6242,19 +6242,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-239.6900000000005</v>
+        <v>-417.8300000000005</v>
       </c>
       <c r="V51" t="n">
         <v>22</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>31.88405797101449</v>
+        <v>31.42857142857143</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/01/2026 22:50</t>
+          <t>10/02/2026 12:24</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6342,16 +6342,16 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-695.89</v>
+        <v>-697.2500000000001</v>
       </c>
       <c r="V52" t="n">
         <v>46</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.98305084745763</v>
+        <v>38.01652892561984</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.88</v>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/01/2026 23:41</t>
+          <t>10/02/2026 07:13</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
@@ -6442,19 +6442,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-293.28</v>
+        <v>-325.24</v>
       </c>
       <c r="V53" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.13636363636364</v>
+        <v>35.87443946188341</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/29/2026 21:33</t>
+          <t>10/02/2026 21:41</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10/01/2026 23:17</t>
+          <t>10/02/2026 12:39</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6811,20 +6811,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/01/2026 22:03</t>
+          <t>10/02/2026 12:00</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19556.2</v>
+        <v>19532.61</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.21</v>
+        <v>-2.33</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6842,22 +6842,22 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1123</v>
+        <v>1140</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-443.3299999999999</v>
+        <v>-469.23</v>
       </c>
       <c r="V57" t="n">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.27693677649155</v>
+        <v>43.24561403508772</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>2.33</v>
+        <v>2.35</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/01/2026 23:02</t>
+          <t>10/02/2026 12:30</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/01/2026 22:33</t>
+          <t>10/02/2026 12:16</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/02/2026 00:24</t>
+          <t>10/02/2026 13:22</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>09/29/2026 21:24</t>
+          <t>10/02/2026 21:32</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/01/2026 23:29</t>
+          <t>10/02/2026 12:47</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7442,22 +7442,22 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1522.85</v>
+        <v>-1563.64</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>11.29032258064516</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.44</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>7.61</v>
+        <v>7.82</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7466,7 +7466,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>10/02/2026 00:09</t>
+          <t>10/02/2026 13:09</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/01/2026 23:33</t>
+          <t>10/02/2026 12:48</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>10/01/2026 22:56</t>
+          <t>10/02/2026 12:27</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/02/2026 00:13</t>
+          <t>10/02/2026 13:14</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7842,19 +7842,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>225.7399999999999</v>
+        <v>77.28999999999991</v>
       </c>
       <c r="V67" t="n">
         <v>29</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>31.86813186813187</v>
+        <v>31.18279569892473</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>09/29/2026 02:58</t>
+          <t>10/02/2026 03:01</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>09/29/2026 02:58</t>
+          <t>10/02/2026 03:01</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/29/2026 02:57</t>
+          <t>10/02/2026 03:01</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>10/01/2026 23:28</t>
+          <t>10/02/2026 12:45</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>10/01/2026 15:03</t>
+          <t>10/02/2026 14:02</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>10/01/2026 23:15</t>
+          <t>10/02/2026 12:38</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/29/2026 20:45</t>
+          <t>10/02/2026 20:53</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/29/2026 19:31</t>
+          <t>10/02/2026 19:40</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/29/2026 20:08</t>
+          <t>10/02/2026 20:16</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/29/2026 19:55</t>
+          <t>10/02/2026 20:05</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/29/2026 20:13</t>
+          <t>10/02/2026 20:24</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/29/2026 20:04</t>
+          <t>10/02/2026 20:09</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>09/29/2026 19:26</t>
+          <t>10/02/2026 19:33</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/29/2026 20:38</t>
+          <t>10/02/2026 20:46</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09/29/2026 20:09</t>
+          <t>10/02/2026 20:16</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>09/29/2026 12:08</t>
+          <t>10/02/2026 12:10</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9811,14 +9811,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/01/2026 15:15</t>
+          <t>10/02/2026 14:11</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19933.88</v>
+        <v>19939.88</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.33</v>
+        <v>-0.3</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.7</v>
@@ -9842,19 +9842,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-66.12</v>
+        <v>-58.37</v>
       </c>
       <c r="V87" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>42.69005847953216</v>
+        <v>43.10344827586206</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>4.69</v>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10011,20 +10011,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/02/2026 01:05</t>
+          <t>10/02/2026 13:48</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20399.21</v>
+        <v>20441.71</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>1.98</v>
+        <v>2.19</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.17</v>
+        <v>1.19</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,19 +10042,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>399.2099999999999</v>
+        <v>441.71</v>
       </c>
       <c r="V89" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>84.28571428571429</v>
+        <v>84.72222222222221</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.17</v>
+        <v>1.19</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3</v>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10111,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/02/2026 00:51</t>
+          <t>10/02/2026 13:41</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27549.45</v>
+        <v>27977.18</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>37.8</v>
+        <v>39.94</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
-      <c r="K90" s="7" t="n">
-        <v>1.98</v>
+      <c r="K90" t="n">
+        <v>2</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10142,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7549.450000000001</v>
+        <v>7977.72</v>
       </c>
       <c r="V90" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>69.93006993006993</v>
+        <v>69.79865771812081</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/29/2026 19:06</t>
+          <t>10/02/2026 19:16</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>09/29/2026 13:57</t>
+          <t>10/02/2026 14:01</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>09/29/2026 13:53</t>
+          <t>10/02/2026 13:56</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>09/29/2026 13:44</t>
+          <t>10/02/2026 13:47</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10711,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/29/2026 23:47</t>
+          <t>10/02/2026 23:56</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10733,13 +10733,22 @@
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>0</v>
+        <v>-225.16</v>
       </c>
       <c r="P96" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q96" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R96" s="7" t="n">
+        <v>0.1289411582653101</v>
+      </c>
+      <c r="S96" s="7" t="n">
+        <v>0.23</v>
       </c>
       <c r="T96" t="n">
         <v>393</v>
@@ -10811,7 +10820,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/29/2026 19:06</t>
+          <t>10/02/2026 19:16</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +10920,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>09/29/2026 19:17</t>
+          <t>10/02/2026 19:26</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11011,7 +11020,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/29/2026 23:51</t>
+          <t>10/03/2026 00:03</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11211,20 +11220,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/01/2026 16:10</t>
+          <t>10/02/2026 14:42</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>21403.45</v>
-      </c>
-      <c r="I101" t="n">
-        <v>7</v>
+        <v>21381.61</v>
+      </c>
+      <c r="I101" s="7" t="n">
+        <v>6.89</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>3.3</v>
+        <v>3.13</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11242,19 +11251,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>1403.45</v>
+        <v>1381.61</v>
       </c>
       <c r="V101" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>81.25</v>
+        <v>77.77777777777779</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>3.3</v>
+        <v>3.13</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11266,7 +11275,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11311,20 +11320,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/01/2026 22:53</t>
+          <t>10/02/2026 12:27</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>20734.08</v>
+        <v>20675.95</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>3.69</v>
+        <v>3.4</v>
       </c>
       <c r="J102" s="7" t="n">
         <v>4.35</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>1.46</v>
+        <v>1.4</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11342,19 +11351,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>734.0799999999999</v>
+        <v>675.9499999999999</v>
       </c>
       <c r="V102" t="n">
         <v>30</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>41.0958904109589</v>
+        <v>40.54054054054054</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>1.46</v>
+        <v>1.4</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>4.04</v>
@@ -11366,7 +11375,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11520,7 +11529,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>09/29/2026 01:49</t>
+          <t>10/02/2026 01:52</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11629,20 +11638,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/01/2026 19:27</t>
+          <t>10/02/2026 22:09</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>11731.38</v>
+        <v>12555.84</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>17.27</v>
+        <v>25.51</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.33</v>
+        <v>2.96</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11660,19 +11669,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>1958.57</v>
+        <v>2728.04</v>
       </c>
       <c r="V105" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>71.875</v>
+        <v>72.05882352941177</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>2.82</v>
+        <v>3.53</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11684,7 +11693,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11838,14 +11847,14 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>10/01/2026 20:58</t>
+          <t>10/02/2026 11:21</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>24136.66</v>
+        <v>24147.86</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-37.16</v>
+        <v>-37.13</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>42.89</v>
@@ -11863,37 +11872,37 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-1112.13</v>
+        <v>-1041.01</v>
       </c>
       <c r="P107" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.01925111996895834</v>
+        <v>0.03068084472419829</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>4.45</v>
+        <v>4.21</v>
       </c>
       <c r="T107" t="n">
-        <v>3918</v>
+        <v>3946</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-9286.980000000001</v>
+        <v>-9694.07</v>
       </c>
       <c r="V107" t="n">
-        <v>2342</v>
+        <v>2368</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>59.7753956100051</v>
+        <v>60.01013684744044</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="Y107" s="7" t="n">
-        <v>42.87</v>
+        <v>45.99</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -11902,7 +11911,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12220,7 +12229,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>09/29/2026 17:01</t>
+          <t>10/02/2026 17:30</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12857,7 +12866,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 00:05</t>
+          <t>10/03/2026 00:17</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13033,7 +13042,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>09/29/2026 21:01</t>
+          <t>10/02/2026 21:09</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13118,7 +13127,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/29/2026 15:31</t>
+          <t>10/02/2026 15:35</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13650,17 +13659,23 @@
         <v>0</v>
       </c>
       <c r="N127" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O127" s="9" t="n">
-        <v>0</v>
+        <v>-4944.48</v>
       </c>
       <c r="P127" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q127" s="8" t="n"/>
-      <c r="R127" s="8" t="n"/>
-      <c r="S127" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q127" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R127" s="9" t="n">
+        <v>0.2385997385250534</v>
+      </c>
+      <c r="S127" s="9" t="n">
+        <v>5.42</v>
+      </c>
       <c r="T127" s="8" t="n">
         <v>0</v>
       </c>
@@ -14369,7 +14384,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09/29/2026 17:01</t>
+          <t>10/02/2026 17:30</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14656,7 +14671,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/30/2026 00:05</t>
+          <t>10/03/2026 00:17</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14738,7 +14753,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>09/29/2026 21:01</t>
+          <t>10/02/2026 21:09</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14779,7 +14794,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09/29/2026 15:31</t>
+          <t>10/02/2026 15:35</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -15035,7 +15050,7 @@
         <v>-20.23</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25">
@@ -16037,7 +16052,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LIVE Dream Catcher Gold</t>
+          <t>LIVE Dream Catcher multi-market (indices + FX + gold)</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -17237,7 +17252,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>For Gold Snap 2HR / Smart Gold Hunter</t>
+          <t>LIVE XAUUSD: YuHeng Gift EA + fundedtoday copy feed</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -17262,11 +17277,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Gold Snap 2HR</t>
+          <t>UNFUNDED, never traded (earmarked Gold Snap 2HR)</t>
         </is>
       </c>
       <c r="D82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -17337,7 +17352,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 GBPJPY + XAUUSD</t>
+          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -17362,7 +17377,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 USDJPY, GBPJPY + XAGUSD</t>
+          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -17663,7 +17678,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09/29/2026 02:06</t>
+          <t>10/02/2026 02:09</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17870,7 +17885,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09/29/2026 02:23</t>
+          <t>10/02/2026 02:26</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17893,7 +17908,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09/29/2026 02:08</t>
+          <t>10/02/2026 02:10</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -18123,7 +18138,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09/29/2026 23:13</t>
+          <t>10/02/2026 23:37</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18146,7 +18161,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09/29/2026 23:27</t>
+          <t>10/02/2026 23:38</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18353,7 +18368,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/01/2026 14:22</t>
+          <t>10/02/2026 14:24</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-03
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-02 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-03 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>09/30/2026 07:09</t>
+          <t>10/03/2026 08:29</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>09/30/2026 00:32</t>
+          <t>10/03/2026 00:43</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/30/2026 00:50</t>
+          <t>10/03/2026 01:01</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/30/2026 03:12</t>
+          <t>10/03/2026 03:20</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/30/2026 00:41</t>
+          <t>10/03/2026 00:55</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>09/30/2026 01:56</t>
+          <t>10/03/2026 02:07</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -10733,22 +10733,13 @@
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>-225.16</v>
+        <v>0</v>
       </c>
       <c r="P96" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q96" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R96" s="7" t="n">
-        <v>0.1289411582653101</v>
-      </c>
-      <c r="S96" s="7" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="T96" t="n">
         <v>393</v>
@@ -11847,20 +11838,20 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>10/02/2026 11:21</t>
+          <t>10/03/2026 03:11</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>24147.86</v>
+        <v>24587.93</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-37.13</v>
+        <v>-35.98</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>42.89</v>
       </c>
       <c r="K107" s="7" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="L107" t="n">
         <v>25000</v>
@@ -11872,19 +11863,19 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>-1041.01</v>
+        <v>189.6600000000001</v>
       </c>
       <c r="P107" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>7.5</v>
+        <v>65</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>0.03068084472419829</v>
+        <v>1.705842947525121</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>4.21</v>
+        <v>0.99</v>
       </c>
       <c r="T107" t="n">
         <v>3946</v>
@@ -12047,7 +12038,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 06:03</t>
+          <t>10/03/2026 06:56</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12684,7 +12675,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 06:44</t>
+          <t>10/03/2026 07:54</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -13659,23 +13650,17 @@
         <v>0</v>
       </c>
       <c r="N127" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O127" s="9" t="n">
-        <v>-4944.48</v>
+        <v>0</v>
       </c>
       <c r="P127" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q127" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R127" s="9" t="n">
-        <v>0.2385997385250534</v>
-      </c>
-      <c r="S127" s="9" t="n">
-        <v>5.42</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q127" s="8" t="n"/>
+      <c r="R127" s="8" t="n"/>
+      <c r="S127" s="8" t="n"/>
       <c r="T127" s="8" t="n">
         <v>0</v>
       </c>
@@ -13813,7 +13798,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 08:17</t>
+          <t>10/03/2026 10:00</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13904,7 +13889,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 07:49</t>
+          <t>10/03/2026 09:25</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14302,7 +14287,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>09/30/2026 06:03</t>
+          <t>10/03/2026 06:56</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14589,7 +14574,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>09/30/2026 06:44</t>
+          <t>10/03/2026 07:54</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -15050,7 +15035,7 @@
         <v>-20.23</v>
       </c>
       <c r="I24" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -15122,7 +15107,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>09/30/2026 08:17</t>
+          <t>10/03/2026 10:00</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15163,7 +15148,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>09/30/2026 07:49</t>
+          <t>10/03/2026 09:25</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -17586,7 +17571,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09/30/2026 09:58</t>
+          <t>10/03/2026 12:17</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17632,7 +17617,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/30/2026 09:41</t>
+          <t>10/03/2026 11:56</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17655,7 +17640,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09/30/2026 04:57</t>
+          <t>10/03/2026 05:26</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17724,7 +17709,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09/30/2026 04:10</t>
+          <t>10/03/2026 04:23</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17839,7 +17824,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09/30/2026 09:34</t>
+          <t>10/03/2026 11:46</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17954,7 +17939,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09/30/2026 04:44</t>
+          <t>10/03/2026 05:13</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -18299,7 +18284,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09/30/2026 09:36</t>
+          <t>10/03/2026 11:49</t>
         </is>
       </c>
       <c r="E35" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-05
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-03 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-05 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/02/2026 11:38</t>
+          <t>10/03/2026 22:24</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>46297.07</v>
+        <v>44027.37</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>111.65</v>
+        <v>101.27</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-6050.400000000001</v>
+        <v>-1505.490000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>72.5</v>
+        <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.8677914214323251</v>
+        <v>0.9655534085877947</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>50.73</v>
+        <v>38.45</v>
       </c>
       <c r="T2" t="n">
-        <v>3467</v>
+        <v>3469</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>19027.37</v>
+        <v>22465.37</v>
       </c>
       <c r="V2" t="n">
-        <v>2205</v>
+        <v>2207</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.59965387943467</v>
+        <v>63.6206399538772</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/01/2026 23:16</t>
+          <t>10/05/2026 15:13</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/02/2026 09:40</t>
+          <t>10/05/2026 18:12</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/01/2026 10:43</t>
+          <t>10/04/2026 12:03</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/01/2026 20:02</t>
+          <t>10/05/2026 09:43</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>09/30/2026 11:45</t>
+          <t>10/03/2026 14:46</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>09/30/2026 13:23</t>
+          <t>10/03/2026 17:19</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09/30/2026 13:25</t>
+          <t>10/03/2026 17:22</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/02/2026 02:42</t>
+          <t>10/05/2026 16:55</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/02/2026 10:58</t>
+          <t>10/05/2026 18:21</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/01/2026 13:33</t>
+          <t>10/04/2026 16:12</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/02/2026 03:11</t>
+          <t>10/05/2026 17:11</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/02/2026 13:44</t>
+          <t>10/05/2026 18:53</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/02/2026 06:20</t>
+          <t>10/05/2026 17:54</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/02/2026 06:25</t>
+          <t>10/05/2026 17:54</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/02/2026 09:29</t>
+          <t>10/05/2026 18:10</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/01/2026 01:09</t>
+          <t>10/04/2026 01:17</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/02/2026 12:08</t>
+          <t>10/03/2026 23:44</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/02/2026 13:41</t>
+          <t>10/04/2026 03:25</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3289,16 +3289,16 @@
         <v>1.55</v>
       </c>
       <c r="T23" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-484.6700000000001</v>
+        <v>-487.2900000000001</v>
       </c>
       <c r="V23" t="n">
         <v>20</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>25.97402597402597</v>
+        <v>25.64102564102564</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.34</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/02/2026 12:28</t>
+          <t>10/04/2026 00:39</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3576,14 +3576,14 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/02/2026 12:07</t>
+          <t>10/03/2026 23:40</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20231.83</v>
+        <v>20256.64</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-3.28</v>
+        <v>-3.16</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
@@ -3601,19 +3601,19 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-339.19</v>
+        <v>-209.19</v>
       </c>
       <c r="P26" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>0.833201378883026</v>
+        <v>0.8915180932823049</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5.46</v>
+        <v>4.94</v>
       </c>
       <c r="T26" t="n">
         <v>139</v>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/30/2026 10:59</t>
+          <t>10/03/2026 13:40</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/02/2026 12:14</t>
+          <t>10/03/2026 23:58</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/01/2026 11:24</t>
+          <t>10/04/2026 13:19</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/02/2026 12:34</t>
+          <t>10/04/2026 00:53</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4052,19 +4052,19 @@
         <v>1.13</v>
       </c>
       <c r="T30" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>560.3099999999999</v>
+        <v>661.2099999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>26.21359223300971</v>
+        <v>28.30188679245283</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.61</v>
+        <v>1.73</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/02/2026 11:01</t>
+          <t>10/05/2026 18:21</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/02/2026 11:52</t>
+          <t>10/05/2026 18:28</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/02/2026 16:49</t>
+          <t>10/05/2026 19:42</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>10/02/2026 03:54</t>
+          <t>10/05/2026 17:33</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/02/2026 14:59</t>
+          <t>10/04/2026 06:42</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>642.0199999999999</v>
+        <v>632.37</v>
       </c>
       <c r="V35" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.08333333333334</v>
+        <v>52.38095238095239</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>1.09</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>10/02/2026 11:41</t>
+          <t>10/05/2026 18:26</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>10/02/2026 03:22</t>
+          <t>10/05/2026 17:15</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>10/01/2026 16:02</t>
+          <t>10/04/2026 22:24</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10/01/2026 10:25</t>
+          <t>10/04/2026 11:45</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10/01/2026 09:36</t>
+          <t>10/04/2026 10:14</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5333,13 +5333,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5433,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5511,14 +5529,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/02/2026 12:35</t>
+          <t>10/04/2026 00:58</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19713.72</v>
+        <v>19707.29</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.41</v>
+        <v>-1.44</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5533,25 +5551,34 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-272.93</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.05354232409751361</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>1.36</v>
       </c>
       <c r="T44" t="n">
-        <v>815</v>
+        <v>828</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-292.7100000000001</v>
+        <v>-311.6700000000001</v>
       </c>
       <c r="V44" t="n">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.58282208588957</v>
+        <v>55.91787439613527</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -5566,7 +5593,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/02/2026 11:47</t>
+          <t>10/03/2026 22:48</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5633,13 +5660,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-23.72</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.684112398455187</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T45" t="n">
         <v>57</v>
@@ -5711,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/02/2026 12:04</t>
+          <t>10/03/2026 23:32</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5833,13 +5869,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5911,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09/30/2026 16:03</t>
+          <t>10/03/2026 20:52</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5933,13 +5978,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6033,13 +6087,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T49" t="n">
         <v>1161</v>
@@ -6133,13 +6196,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>-52.41999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>0.8051952878219183</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>1.3</v>
       </c>
       <c r="T50" t="n">
         <v>1978</v>
@@ -6211,20 +6283,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/02/2026 11:53</t>
+          <t>10/03/2026 23:07</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19760.31</v>
+        <v>19582.17</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-1.17</v>
+        <v>-2.06</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6233,13 +6305,22 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>0</v>
+        <v>998.4000000000001</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R51" s="7" t="n">
+        <v>1.292456588475148</v>
+      </c>
+      <c r="S51" s="7" t="n">
+        <v>5.92</v>
       </c>
       <c r="T51" t="n">
         <v>70</v>
@@ -6311,11 +6392,11 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/02/2026 12:24</t>
+          <t>10/04/2026 00:27</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19304.11</v>
+        <v>19302.75</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>-3.45</v>
@@ -6333,25 +6414,34 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>-986.53</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>0.5861402088323762</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>5.77</v>
       </c>
       <c r="T52" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-697.2500000000001</v>
+        <v>-675.53</v>
       </c>
       <c r="V52" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.01652892561984</v>
+        <v>38.21138211382114</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.88</v>
@@ -6366,7 +6456,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,20 +6501,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/02/2026 07:13</t>
+          <t>10/04/2026 01:41</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19706.72</v>
+        <v>19674.76</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.51</v>
+        <v>-1.67</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6442,19 +6532,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-325.24</v>
+        <v>-338.0900000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.87443946188341</v>
+        <v>36.06194690265487</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6556,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6611,7 +6701,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10/02/2026 12:39</t>
+          <t>10/05/2026 18:35</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6711,7 +6801,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10/01/2026 10:13</t>
+          <t>10/04/2026 11:11</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6811,17 +6901,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/02/2026 12:00</t>
+          <t>10/03/2026 23:20</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19532.61</v>
+        <v>19530.3</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.33</v>
+        <v>-2.34</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="K57" s="7" t="n">
         <v>0.74</v>
@@ -6833,31 +6923,40 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-69.06</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.2955217790472304</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.35</v>
       </c>
       <c r="T57" t="n">
-        <v>1140</v>
+        <v>1156</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-469.23</v>
+        <v>-491.08</v>
       </c>
       <c r="V57" t="n">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.24561403508772</v>
+        <v>43.0795847750865</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>2.35</v>
+        <v>2.46</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6866,7 +6965,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +7010,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/02/2026 12:30</t>
+          <t>10/04/2026 00:42</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7011,7 +7110,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>10/01/2026 11:46</t>
+          <t>10/04/2026 14:02</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7111,7 +7210,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/02/2026 12:16</t>
+          <t>10/04/2026 00:10</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7310,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/02/2026 13:22</t>
+          <t>10/04/2026 02:39</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7311,7 +7410,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>10/02/2026 21:32</t>
+          <t>10/05/2026 21:34</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,17 +7510,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/02/2026 12:47</t>
+          <t>10/04/2026 01:25</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18477.15</v>
+        <v>18436.36</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-7.64</v>
+        <v>-7.84</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>7.64</v>
+        <v>7.84</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>0.44</v>
@@ -7433,31 +7532,40 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>0</v>
+        <v>-218.04</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Q63" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="R63" s="7" t="n">
+        <v>0.8376784836889359</v>
+      </c>
+      <c r="S63" s="7" t="n">
+        <v>3.12</v>
       </c>
       <c r="T63" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1563.64</v>
+        <v>-1606.49</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>11.11111111111111</v>
+        <v>10.9375</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>7.82</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7466,7 +7574,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7511,7 +7619,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>10/02/2026 13:09</t>
+          <t>10/05/2026 18:43</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7719,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/02/2026 12:48</t>
+          <t>10/04/2026 01:27</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7711,7 +7819,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>10/02/2026 12:27</t>
+          <t>10/05/2026 18:34</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7733,13 +7841,22 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>0</v>
+        <v>-114.21</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q66" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R66" s="7" t="n">
+        <v>0.3210272873194221</v>
+      </c>
+      <c r="S66" s="7" t="n">
+        <v>0.67</v>
       </c>
       <c r="T66" t="n">
         <v>262</v>
@@ -7811,20 +7928,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/02/2026 13:14</t>
+          <t>10/04/2026 02:24</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20225.74</v>
+        <v>20077.29</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>1.16</v>
+        <v>0.42</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7842,16 +7959,16 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>77.28999999999991</v>
+        <v>75.32999999999991</v>
       </c>
       <c r="V67" t="n">
         <v>29</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>31.18279569892473</v>
+        <v>30.85106382978723</v>
       </c>
       <c r="X67" s="7" t="n">
         <v>1.01</v>
@@ -7866,7 +7983,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7911,7 +8028,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>10/01/2026 11:46</t>
+          <t>10/04/2026 14:02</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8011,7 +8128,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>10/02/2026 03:01</t>
+          <t>10/05/2026 17:05</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8111,7 +8228,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>10/02/2026 03:01</t>
+          <t>10/05/2026 17:05</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8328,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>10/02/2026 03:01</t>
+          <t>10/05/2026 17:04</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8311,7 +8428,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>10/02/2026 12:45</t>
+          <t>10/05/2026 18:38</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8528,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>10/02/2026 14:02</t>
+          <t>10/05/2026 18:59</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8433,13 +8550,22 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>0</v>
+        <v>-39.43999999999999</v>
       </c>
       <c r="P73" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q73" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R73" s="7" t="n">
+        <v>0.8172212438594866</v>
+      </c>
+      <c r="S73" s="7" t="n">
+        <v>0.49</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -8511,7 +8637,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>10/02/2026 12:38</t>
+          <t>10/05/2026 18:35</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8611,7 +8737,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>10/02/2026 20:53</t>
+          <t>10/05/2026 20:55</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8837,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>10/02/2026 19:40</t>
+          <t>10/05/2026 20:20</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8937,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>10/02/2026 20:16</t>
+          <t>10/05/2026 20:32</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +9037,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>10/02/2026 20:05</t>
+          <t>10/05/2026 20:28</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9137,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>10/02/2026 20:24</t>
+          <t>10/05/2026 20:35</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9237,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>10/02/2026 20:09</t>
+          <t>10/05/2026 20:30</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9211,7 +9337,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>10/02/2026 19:33</t>
+          <t>10/05/2026 20:18</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9311,7 +9437,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>10/02/2026 20:46</t>
+          <t>10/05/2026 20:48</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9333,13 +9459,22 @@
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>0</v>
+        <v>-308.22</v>
       </c>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q82" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R82" s="7" t="n">
+        <v>0.412903102916246</v>
+      </c>
+      <c r="S82" s="7" t="n">
+        <v>1.62</v>
       </c>
       <c r="T82" t="n">
         <v>1156</v>
@@ -9411,7 +9546,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>10/02/2026 20:16</t>
+          <t>10/05/2026 20:32</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9711,7 +9846,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>09/26/2026 19:47</t>
+          <t>10/05/2026 20:32</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9811,20 +9946,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/02/2026 14:11</t>
+          <t>10/04/2026 04:35</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19939.88</v>
+        <v>19941.63</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.3</v>
+        <v>-0.29</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>4.7</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9833,31 +9968,40 @@
         <v>0</v>
       </c>
       <c r="N87" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O87" s="7" t="n">
-        <v>0</v>
+        <v>-264.31</v>
       </c>
       <c r="P87" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q87" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R87" s="7" t="n">
+        <v>0.5617549037489016</v>
+      </c>
+      <c r="S87" s="7" t="n">
+        <v>2.03</v>
       </c>
       <c r="T87" t="n">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-58.37</v>
+        <v>-179.7799999999997</v>
       </c>
       <c r="V87" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>43.10344827586206</v>
+        <v>43.33333333333334</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="Y87" s="7" t="n">
-        <v>4.69</v>
+        <v>5.36</v>
       </c>
       <c r="Z87" t="inlineStr">
         <is>
@@ -9866,7 +10010,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9911,7 +10055,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>10/01/2026 12:04</t>
+          <t>10/04/2026 14:54</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10011,7 +10155,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/02/2026 13:48</t>
+          <t>10/04/2026 03:41</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
@@ -10033,31 +10177,40 @@
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O89" s="7" t="n">
-        <v>0</v>
+        <v>58.18</v>
       </c>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="Q89" s="7" t="n">
+        <v>85</v>
+      </c>
+      <c r="R89" s="7" t="n">
+        <v>1.087318024913703</v>
+      </c>
+      <c r="S89" s="7" t="n">
+        <v>1.4</v>
       </c>
       <c r="T89" t="n">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>441.71</v>
+        <v>-7.20999999999998</v>
       </c>
       <c r="V89" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>84.72222222222221</v>
+        <v>82.5503355704698</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.19</v>
+        <v>1</v>
       </c>
       <c r="Y89" s="7" t="n">
-        <v>3</v>
+        <v>3.63</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10066,7 +10219,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,11 +10264,11 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/02/2026 13:41</t>
+          <t>10/04/2026 03:23</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27977.18</v>
+        <v>27977.72</v>
       </c>
       <c r="I90" s="7" t="n">
         <v>39.94</v>
@@ -10142,19 +10295,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7977.72</v>
+        <v>7274.49</v>
       </c>
       <c r="V90" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>69.79865771812081</v>
+        <v>68.62745098039215</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>2</v>
+        <v>1.83</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10166,7 +10319,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10364,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>10/02/2026 19:16</t>
+          <t>10/05/2026 20:13</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10311,7 +10464,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>10/01/2026 18:17</t>
+          <t>10/05/2026 04:31</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10411,7 +10564,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>10/02/2026 14:01</t>
+          <t>10/05/2026 18:59</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10664,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>10/02/2026 13:56</t>
+          <t>10/05/2026 18:57</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10764,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>10/02/2026 13:47</t>
+          <t>10/05/2026 18:55</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10811,7 +10964,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>10/02/2026 19:16</t>
+          <t>10/05/2026 20:12</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +11064,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>10/02/2026 19:26</t>
+          <t>10/05/2026 20:15</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -10933,13 +11086,22 @@
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>0</v>
+        <v>-812.92</v>
       </c>
       <c r="P98" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q98" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R98" s="7" t="n">
+        <v>0.1283107079285423</v>
+      </c>
+      <c r="S98" s="7" t="n">
+        <v>0.8100000000000001</v>
       </c>
       <c r="T98" t="n">
         <v>448</v>
@@ -11111,7 +11273,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>10/01/2026 18:24</t>
+          <t>10/05/2026 04:55</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11133,13 +11295,22 @@
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>0</v>
+        <v>-304.44</v>
       </c>
       <c r="P100" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q100" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R100" s="7" t="n">
+        <v>0.4682177854635016</v>
+      </c>
+      <c r="S100" s="7" t="n">
+        <v>0.41</v>
       </c>
       <c r="T100" t="n">
         <v>199</v>
@@ -11211,7 +11382,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/02/2026 14:42</t>
+          <t>10/04/2026 06:00</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11311,7 +11482,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/02/2026 12:27</t>
+          <t>10/04/2026 00:34</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11342,19 +11513,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>675.9499999999999</v>
+        <v>1219.26</v>
       </c>
       <c r="V102" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>40.54054054054054</v>
+        <v>40.50632911392405</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>4.04</v>
@@ -11366,7 +11537,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11411,7 +11582,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>10/01/2026 09:56</t>
+          <t>10/04/2026 10:45</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
@@ -11520,7 +11691,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>10/02/2026 01:52</t>
+          <t>10/05/2026 16:31</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -11629,20 +11800,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/02/2026 22:09</t>
+          <t>10/05/2026 21:01</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>12555.84</v>
+        <v>12728.89</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>25.51</v>
+        <v>27.24</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.96</v>
+        <v>3.1</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11660,19 +11831,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>2728.04</v>
+        <v>2901.09</v>
       </c>
       <c r="V105" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>72.05882352941177</v>
+        <v>73.23943661971832</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.53</v>
+        <v>3.69</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.69</v>
@@ -11684,7 +11855,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11729,7 +11900,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>09/30/2026 11:43</t>
+          <t>10/03/2026 14:44</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -11838,14 +12009,14 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>10/03/2026 03:11</t>
+          <t>10/05/2026 21:47</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>24587.93</v>
+        <v>24475.57</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-35.98</v>
+        <v>-36.27</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>42.89</v>
@@ -11863,7 +12034,7 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>189.6600000000001</v>
+        <v>132.79</v>
       </c>
       <c r="P107" t="n">
         <v>26</v>
@@ -11872,22 +12043,22 @@
         <v>65</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>1.705842947525121</v>
+        <v>1.407143952169247</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>0.99</v>
+        <v>0.77</v>
       </c>
       <c r="T107" t="n">
-        <v>3946</v>
+        <v>3951</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-9694.07</v>
+        <v>-9806.43</v>
       </c>
       <c r="V107" t="n">
-        <v>2368</v>
+        <v>2369</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>60.01013684744044</v>
+        <v>59.95950392305745</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.75</v>
@@ -11902,7 +12073,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -11947,7 +12118,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 10:34</t>
+          <t>10/03/2026 13:07</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12129,7 +12300,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 23:32</t>
+          <t>10/05/2026 15:20</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12220,7 +12391,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>10/02/2026 17:30</t>
+          <t>10/05/2026 19:50</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12311,7 +12482,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 10:51</t>
+          <t>10/04/2026 12:17</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12402,7 +12573,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 16:08</t>
+          <t>10/03/2026 21:01</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12493,7 +12664,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 11:42</t>
+          <t>10/03/2026 14:42</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12584,7 +12755,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 13:29</t>
+          <t>10/04/2026 16:10</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12766,7 +12937,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 19:37</t>
+          <t>10/05/2026 08:30</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12948,7 +13119,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 12:03</t>
+          <t>10/04/2026 14:52</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12970,17 +13141,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13033,7 +13210,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>10/02/2026 21:09</t>
+          <t>10/05/2026 21:11</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13055,17 +13232,23 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q120" s="8" t="n"/>
-      <c r="R120" s="8" t="n"/>
-      <c r="S120" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q120" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R120" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S120" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13118,7 +13301,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>10/02/2026 15:35</t>
+          <t>10/05/2026 19:23</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13140,17 +13323,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13203,7 +13392,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/29/2026 02:58</t>
+          <t>10/05/2026 17:06</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13288,7 +13477,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 18:39</t>
+          <t>10/05/2026 05:36</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13373,7 +13562,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 18:39</t>
+          <t>10/05/2026 05:37</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13458,7 +13647,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 18:40</t>
+          <t>10/05/2026 05:38</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13480,17 +13669,23 @@
         <v>0</v>
       </c>
       <c r="N125" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O125" s="9" t="n">
-        <v>0</v>
+        <v>-1180.45</v>
       </c>
       <c r="P125" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q125" s="8" t="n"/>
-      <c r="R125" s="8" t="n"/>
-      <c r="S125" s="8" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="Q125" s="9" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R125" s="9" t="n">
+        <v>0.2676972896517925</v>
+      </c>
+      <c r="S125" s="9" t="n">
+        <v>1.18</v>
+      </c>
       <c r="T125" s="8" t="n">
         <v>0</v>
       </c>
@@ -13543,7 +13738,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 18:51</t>
+          <t>10/05/2026 06:15</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13628,7 +13823,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 19:27</t>
+          <t>10/05/2026 07:54</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13650,17 +13845,23 @@
         <v>0</v>
       </c>
       <c r="N127" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O127" s="9" t="n">
-        <v>0</v>
+        <v>-4944.48</v>
       </c>
       <c r="P127" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q127" s="8" t="n"/>
-      <c r="R127" s="8" t="n"/>
-      <c r="S127" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q127" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R127" s="9" t="n">
+        <v>0.2385997385250534</v>
+      </c>
+      <c r="S127" s="9" t="n">
+        <v>5.42</v>
+      </c>
       <c r="T127" s="8" t="n">
         <v>0</v>
       </c>
@@ -13713,7 +13914,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>10/01/2026 18:36</t>
+          <t>10/05/2026 05:26</t>
         </is>
       </c>
       <c r="H128" s="9" t="n">
@@ -14071,7 +14272,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>09/30/2026 13:55</t>
+          <t>10/03/2026 18:08</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14246,7 +14447,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09/30/2026 10:34</t>
+          <t>10/03/2026 13:07</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14328,7 +14529,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10/01/2026 23:32</t>
+          <t>10/05/2026 15:20</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14369,7 +14570,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10/02/2026 17:30</t>
+          <t>10/05/2026 19:50</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14410,7 +14611,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10/01/2026 10:51</t>
+          <t>10/04/2026 12:17</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14451,7 +14652,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09/30/2026 16:08</t>
+          <t>10/03/2026 21:01</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14492,7 +14693,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>09/30/2026 11:42</t>
+          <t>10/03/2026 14:42</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14533,7 +14734,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10/01/2026 13:29</t>
+          <t>10/04/2026 16:10</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14615,7 +14816,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10/01/2026 19:37</t>
+          <t>10/05/2026 08:30</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14697,7 +14898,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>10/01/2026 12:03</t>
+          <t>10/04/2026 14:52</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14707,7 +14908,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14738,7 +14939,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>10/02/2026 21:09</t>
+          <t>10/05/2026 21:11</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14748,7 +14949,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -14779,7 +14980,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>10/02/2026 15:35</t>
+          <t>10/05/2026 19:23</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14789,7 +14990,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14820,7 +15021,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/29/2026 02:58</t>
+          <t>10/05/2026 17:06</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14861,7 +15062,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10/01/2026 18:39</t>
+          <t>10/05/2026 05:36</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14902,7 +15103,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10/01/2026 18:39</t>
+          <t>10/05/2026 05:37</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14943,7 +15144,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>10/01/2026 18:40</t>
+          <t>10/05/2026 05:38</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14953,7 +15154,7 @@
         <v>-2.31</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -14984,7 +15185,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10/01/2026 18:51</t>
+          <t>10/05/2026 06:15</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -15025,7 +15226,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10/01/2026 19:27</t>
+          <t>10/05/2026 07:54</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15035,7 +15236,7 @@
         <v>-20.23</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25">
@@ -15066,7 +15267,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>10/01/2026 18:36</t>
+          <t>10/05/2026 05:26</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -15230,7 +15431,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>09/30/2026 13:55</t>
+          <t>10/03/2026 18:08</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17594,7 +17795,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10/01/2026 14:00</t>
+          <t>10/04/2026 16:24</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17663,7 +17864,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10/02/2026 02:09</t>
+          <t>10/05/2026 16:40</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17686,7 +17887,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10/01/2026 09:01</t>
+          <t>10/04/2026 09:23</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17732,7 +17933,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10/01/2026 09:03</t>
+          <t>10/04/2026 09:27</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -17755,7 +17956,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10/01/2026 17:33</t>
+          <t>10/05/2026 02:26</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -17778,7 +17979,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09/30/2026 10:58</t>
+          <t>10/03/2026 13:40</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17801,7 +18002,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10/01/2026 20:30</t>
+          <t>10/05/2026 11:04</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17870,7 +18071,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10/02/2026 02:26</t>
+          <t>10/05/2026 16:47</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17893,7 +18094,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10/02/2026 02:10</t>
+          <t>10/05/2026 16:40</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -17916,7 +18117,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09/30/2026 12:17</t>
+          <t>10/03/2026 15:41</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17962,7 +18163,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09/30/2026 14:34</t>
+          <t>10/03/2026 19:03</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17985,7 +18186,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09/30/2026 11:03</t>
+          <t>10/03/2026 13:47</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18031,7 +18232,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09/30/2026 12:11</t>
+          <t>10/03/2026 15:27</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18054,7 +18255,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10/01/2026 08:05</t>
+          <t>10/04/2026 08:16</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18077,7 +18278,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10/01/2026 19:03</t>
+          <t>10/05/2026 06:44</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18100,7 +18301,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10/01/2026 19:04</t>
+          <t>10/05/2026 06:47</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18169,7 +18370,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10/01/2026 18:47</t>
+          <t>10/05/2026 06:03</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18192,7 +18393,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10/01/2026 19:59</t>
+          <t>10/05/2026 09:30</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18215,7 +18416,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10/01/2026 09:00</t>
+          <t>10/04/2026 09:22</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18238,7 +18439,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10/01/2026 09:08</t>
+          <t>10/04/2026 09:33</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -18307,7 +18508,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09/30/2026 10:18</t>
+          <t>10/03/2026 12:46</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18330,7 +18531,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/30/2026 13:49</t>
+          <t>10/03/2026 17:57</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18353,7 +18554,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/02/2026 14:24</t>
+          <t>10/05/2026 14:31</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-06
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-05 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-06 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/03/2026 22:24</t>
+          <t>10/06/2026 20:34</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>44027.37</v>
+        <v>50028.39</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>101.27</v>
+        <v>128.71</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-1505.490000000001</v>
+        <v>166.0299999999987</v>
       </c>
       <c r="P2" t="n">
         <v>30</v>
@@ -994,22 +994,22 @@
         <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.9655534085877947</v>
+        <v>1.003798874500773</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>38.45</v>
+        <v>44.62</v>
       </c>
       <c r="T2" t="n">
-        <v>3469</v>
+        <v>3471</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>22465.37</v>
+        <v>25395.21</v>
       </c>
       <c r="V2" t="n">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.6206399538772</v>
+        <v>63.67041198501872</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.04</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/03/2026 14:46</t>
+          <t>10/06/2026 14:50</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/03/2026 17:19</t>
+          <t>10/06/2026 17:22</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/03/2026 17:22</t>
+          <t>10/06/2026 17:25</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/03/2026 08:29</t>
+          <t>10/06/2026 08:32</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/03/2026 23:44</t>
+          <t>10/06/2026 21:11</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/04/2026 03:25</t>
+          <t>10/06/2026 22:41</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19515.33</v>
+        <v>19533.88</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.58</v>
+        <v>-2.48</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.74</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-272.96</v>
+        <v>-233.79</v>
       </c>
       <c r="P23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.2928680604129427</v>
+        <v>0.3402099678275103</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>1.55</v>
       </c>
       <c r="T23" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-487.2900000000001</v>
+        <v>-466.1200000000001</v>
       </c>
       <c r="V23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>25.64102564102564</v>
+        <v>25.92592592592592</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.34</v>
+        <v>0.37</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.58</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/04/2026 00:39</t>
+          <t>10/06/2026 21:38</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/02/2026 23:37</t>
+          <t>10/05/2026 23:39</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/03/2026 23:40</t>
+          <t>10/06/2026 21:16</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/03/2026 13:40</t>
+          <t>10/06/2026 13:43</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/03/2026 23:58</t>
+          <t>10/06/2026 21:19</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/04/2026 00:53</t>
+          <t>10/06/2026 21:46</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20560.31</v>
+        <v>20678.71</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.83</v>
+        <v>3.42</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.61</v>
+        <v>1.74</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-181.24</v>
+        <v>-0.159999999999998</v>
       </c>
       <c r="P30" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>22.5</v>
+        <v>30</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.3687216997561825</v>
+        <v>0.999279344203225</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>1.13</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="T30" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>661.2099999999999</v>
+        <v>678.7099999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>28.30188679245283</v>
+        <v>28.97196261682243</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/04/2026 06:42</t>
+          <t>10/06/2026 23:46</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20642.02</v>
+        <v>20217.96</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>3.21</v>
+        <v>1.09</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.09</v>
+        <v>1.03</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4579,28 +4579,37 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>0</v>
+        <v>255.36</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q35" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R35" s="7" t="n">
+        <v>1.138761492816311</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>3.19</v>
       </c>
       <c r="T35" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>632.37</v>
+        <v>217.9599999999999</v>
       </c>
       <c r="V35" t="n">
         <v>77</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.38095238095239</v>
+        <v>50.99337748344372</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.09</v>
+        <v>1.03</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4621,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -5202,7 +5211,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10/03/2026 00:43</t>
+          <t>10/06/2026 00:44</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5320,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>10/03/2026 01:01</t>
+          <t>10/06/2026 01:05</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5429,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>10/03/2026 03:20</t>
+          <t>10/06/2026 03:23</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,14 +5538,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/04/2026 00:58</t>
+          <t>10/06/2026 21:48</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19707.29</v>
+        <v>19672.79</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.44</v>
+        <v>-1.61</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5554,31 +5563,31 @@
         <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-272.93</v>
+        <v>-185.9</v>
       </c>
       <c r="P44" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="Q44" s="7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="R44" s="7" t="n">
-        <v>0.05354232409751361</v>
+        <v>0.1371547922951961</v>
       </c>
       <c r="S44" s="7" t="n">
-        <v>1.36</v>
+        <v>0.93</v>
       </c>
       <c r="T44" t="n">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-311.6700000000001</v>
+        <v>-327.2100000000001</v>
       </c>
       <c r="V44" t="n">
         <v>463</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.91787439613527</v>
+        <v>55.78313253012048</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -5593,7 +5602,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5638,7 +5647,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/03/2026 22:48</t>
+          <t>10/06/2026 20:45</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5747,20 +5756,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/03/2026 23:32</t>
+          <t>10/06/2026 21:08</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19386.26</v>
+        <v>19294.33</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-3.04</v>
+        <v>-3.5</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5778,19 +5787,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-613.74</v>
+        <v>-705.6700000000001</v>
       </c>
       <c r="V46" t="n">
         <v>40</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>43.01075268817204</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5802,7 +5811,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5847,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>10/03/2026 00:03</t>
+          <t>10/06/2026 00:05</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5956,7 +5965,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>10/03/2026 20:52</t>
+          <t>10/06/2026 20:55</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5978,22 +5987,13 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>698.46</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q48" s="7" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="R48" s="7" t="n">
-        <v>7.636199524940618</v>
-      </c>
-      <c r="S48" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>10/03/2026 00:55</t>
+          <t>10/06/2026 00:57</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6087,22 +6087,13 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>13.93999999999999</v>
+        <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q49" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R49" s="7" t="n">
-        <v>1.066618876941458</v>
-      </c>
-      <c r="S49" s="7" t="n">
-        <v>0.89</v>
+        <v>0</v>
       </c>
       <c r="T49" t="n">
         <v>1161</v>
@@ -6174,7 +6165,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>10/03/2026 00:30</t>
+          <t>10/06/2026 00:32</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6196,22 +6187,13 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>-52.41999999999999</v>
+        <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q50" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R50" s="7" t="n">
-        <v>0.8051952878219183</v>
-      </c>
-      <c r="S50" s="7" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="T50" t="n">
         <v>1978</v>
@@ -6283,7 +6265,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/03/2026 23:07</t>
+          <t>10/06/2026 20:56</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6305,22 +6287,13 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>998.4000000000001</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q51" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="R51" s="7" t="n">
-        <v>1.292456588475148</v>
-      </c>
-      <c r="S51" s="7" t="n">
-        <v>5.92</v>
+        <v>0</v>
       </c>
       <c r="T51" t="n">
         <v>70</v>
@@ -6392,20 +6365,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/04/2026 00:27</t>
+          <t>10/06/2026 21:31</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19302.75</v>
+        <v>19368.38</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.45</v>
+        <v>-3.12</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>5.79</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6414,37 +6387,28 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>-986.53</v>
+        <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q52" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R52" s="7" t="n">
-        <v>0.5861402088323762</v>
-      </c>
-      <c r="S52" s="7" t="n">
-        <v>5.77</v>
+        <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-675.53</v>
+        <v>-631.62</v>
       </c>
       <c r="V52" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.21138211382114</v>
+        <v>38.4</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>5.81</v>
@@ -6456,7 +6420,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6501,14 +6465,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/04/2026 01:41</t>
+          <t>10/06/2026 22:05</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19674.76</v>
+        <v>19678.78</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.67</v>
+        <v>-1.64</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6532,19 +6496,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-338.0900000000001</v>
+        <v>-321.2200000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.06194690265487</v>
+        <v>36.54266958424508</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6556,7 +6520,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6901,20 +6865,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/03/2026 23:20</t>
+          <t>10/06/2026 21:03</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19530.3</v>
+        <v>19489.74</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.34</v>
+        <v>-2.54</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>2.35</v>
+        <v>2.54</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6923,40 +6887,31 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>-69.06</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>0.2955217790472304</v>
-      </c>
-      <c r="S57" s="7" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1156</v>
+        <v>1174</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-491.08</v>
+        <v>-509.7900000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.0795847750865</v>
+        <v>42.84497444633731</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.73</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>2.46</v>
+        <v>2.55</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6965,7 +6920,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -7010,7 +6965,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/04/2026 00:42</t>
+          <t>10/06/2026 21:42</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7210,7 +7165,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/04/2026 00:10</t>
+          <t>10/06/2026 21:24</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7232,13 +7187,22 @@
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>0</v>
+        <v>-1105.06</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q60" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R60" s="7" t="n">
+        <v>0.2343571374133069</v>
+      </c>
+      <c r="S60" s="7" t="n">
+        <v>6.68</v>
       </c>
       <c r="T60" t="n">
         <v>7019</v>
@@ -7310,7 +7274,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/04/2026 02:39</t>
+          <t>10/06/2026 22:27</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7510,20 +7474,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/04/2026 01:25</t>
+          <t>10/06/2026 21:59</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18436.36</v>
+        <v>18393.51</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-7.84</v>
+        <v>-8.050000000000001</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>7.84</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7532,22 +7496,13 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>-218.04</v>
+        <v>0</v>
       </c>
       <c r="P63" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q63" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="R63" s="7" t="n">
-        <v>0.8376784836889359</v>
-      </c>
-      <c r="S63" s="7" t="n">
-        <v>3.12</v>
+        <v>0</v>
       </c>
       <c r="T63" t="n">
         <v>64</v>
@@ -7719,7 +7674,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/04/2026 01:27</t>
+          <t>10/06/2026 21:59</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7841,22 +7796,13 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>-114.21</v>
+        <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q66" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R66" s="7" t="n">
-        <v>0.3210272873194221</v>
-      </c>
-      <c r="S66" s="7" t="n">
-        <v>0.67</v>
+        <v>0</v>
       </c>
       <c r="T66" t="n">
         <v>262</v>
@@ -7928,20 +7874,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/04/2026 02:24</t>
+          <t>10/06/2026 22:19</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20077.29</v>
+        <v>20718.18</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>0.42</v>
+        <v>3.64</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.01</v>
+        <v>1.07</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7959,19 +7905,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>75.32999999999991</v>
+        <v>718.1799999999998</v>
       </c>
       <c r="V67" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>30.85106382978723</v>
+        <v>31.57894736842105</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.01</v>
+        <v>1.07</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -8450,13 +8396,22 @@
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O72" s="7" t="n">
-        <v>0</v>
+        <v>-19.59</v>
       </c>
       <c r="P72" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q72" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R72" s="7" t="n">
+        <v>0.8233543733092877</v>
+      </c>
+      <c r="S72" s="7" t="n">
+        <v>0.23</v>
       </c>
       <c r="T72" t="n">
         <v>326</v>
@@ -8550,22 +8505,13 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>-39.43999999999999</v>
+        <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q73" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R73" s="7" t="n">
-        <v>0.8172212438594866</v>
-      </c>
-      <c r="S73" s="7" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -9459,22 +9405,13 @@
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>-308.22</v>
+        <v>0</v>
       </c>
       <c r="P82" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q82" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R82" s="7" t="n">
-        <v>0.412903102916246</v>
-      </c>
-      <c r="S82" s="7" t="n">
-        <v>1.62</v>
+        <v>0</v>
       </c>
       <c r="T82" t="n">
         <v>1156</v>
@@ -9746,7 +9683,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>10/03/2026 02:07</t>
+          <t>10/06/2026 02:09</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9946,20 +9883,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/04/2026 04:35</t>
+          <t>10/06/2026 23:04</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19941.63</v>
+        <v>19804.32</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.29</v>
+        <v>-0.98</v>
       </c>
       <c r="J87" s="7" t="n">
-        <v>4.7</v>
+        <v>5.37</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>0.98</v>
+        <v>0.92</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9968,37 +9905,28 @@
         <v>0</v>
       </c>
       <c r="N87" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O87" s="7" t="n">
-        <v>-264.31</v>
+        <v>0</v>
       </c>
       <c r="P87" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q87" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="R87" s="7" t="n">
-        <v>0.5617549037489016</v>
-      </c>
-      <c r="S87" s="7" t="n">
-        <v>2.03</v>
+        <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-179.7799999999997</v>
+        <v>-195.6799999999997</v>
       </c>
       <c r="V87" t="n">
         <v>78</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>43.33333333333334</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>5.36</v>
@@ -10010,7 +9938,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10155,20 +10083,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/04/2026 03:41</t>
+          <t>10/06/2026 22:45</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20441.71</v>
+        <v>20033.47</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>2.19</v>
+        <v>0.16</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>2.99</v>
+        <v>3.63</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.19</v>
+        <v>1.01</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10177,37 +10105,28 @@
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O89" s="7" t="n">
-        <v>58.18</v>
+        <v>0</v>
       </c>
       <c r="P89" t="n">
-        <v>34</v>
-      </c>
-      <c r="Q89" s="7" t="n">
-        <v>85</v>
-      </c>
-      <c r="R89" s="7" t="n">
-        <v>1.087318024913703</v>
-      </c>
-      <c r="S89" s="7" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>-7.20999999999998</v>
+        <v>33.47</v>
       </c>
       <c r="V89" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>82.5503355704698</v>
+        <v>82.89473684210526</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3.63</v>
@@ -10219,7 +10138,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10264,20 +10183,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/04/2026 03:23</t>
+          <t>10/06/2026 22:42</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27977.72</v>
+        <v>27747.08</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>39.94</v>
+        <v>38.79</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
-      <c r="K90" t="n">
-        <v>2</v>
+      <c r="K90" s="7" t="n">
+        <v>1.88</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10295,19 +10214,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7274.49</v>
+        <v>7747.08</v>
       </c>
       <c r="V90" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>68.62745098039215</v>
+        <v>69.03225806451613</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.83</v>
+        <v>1.88</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10319,7 +10238,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10786,13 +10705,22 @@
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O95" s="7" t="n">
-        <v>0</v>
+        <v>19948.18</v>
       </c>
       <c r="P95" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Q95" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R95" s="7" t="n">
+        <v>109.8042980255264</v>
+      </c>
+      <c r="S95" s="7" t="n">
+        <v>0.45</v>
       </c>
       <c r="T95" t="n">
         <v>11</v>
@@ -10824,7 +10752,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC95" t="inlineStr">
@@ -10864,7 +10792,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>10/02/2026 23:56</t>
+          <t>10/05/2026 23:58</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -11086,22 +11014,13 @@
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>-812.92</v>
+        <v>0</v>
       </c>
       <c r="P98" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q98" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R98" s="7" t="n">
-        <v>0.1283107079285423</v>
-      </c>
-      <c r="S98" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="T98" t="n">
         <v>448</v>
@@ -11173,7 +11092,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>10/03/2026 00:03</t>
+          <t>10/06/2026 00:05</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11295,22 +11214,13 @@
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>-304.44</v>
+        <v>0</v>
       </c>
       <c r="P100" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q100" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R100" s="7" t="n">
-        <v>0.4682177854635016</v>
-      </c>
-      <c r="S100" s="7" t="n">
-        <v>0.41</v>
+        <v>0</v>
       </c>
       <c r="T100" t="n">
         <v>199</v>
@@ -11382,20 +11292,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/04/2026 06:00</t>
+          <t>10/06/2026 23:30</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>21381.61</v>
+        <v>21162.64</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>6.89</v>
+        <v>5.8</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>3.13</v>
+        <v>2.34</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11413,19 +11323,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>1381.61</v>
+        <v>1162.64</v>
       </c>
       <c r="V101" t="n">
         <v>14</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>77.77777777777779</v>
+        <v>73.68421052631578</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>3.13</v>
+        <v>2.34</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11437,7 +11347,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11482,20 +11392,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/04/2026 00:34</t>
+          <t>10/06/2026 21:36</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>20675.95</v>
+        <v>21207.19</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>3.4</v>
+        <v>6.06</v>
       </c>
       <c r="J102" s="7" t="n">
-        <v>4.35</v>
+        <v>6.68</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>1.4</v>
+        <v>1.68</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11513,19 +11423,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>1219.26</v>
+        <v>1207.19</v>
       </c>
       <c r="V102" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>40.50632911392405</v>
+        <v>41.25</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>4.04</v>
@@ -11537,7 +11447,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11800,20 +11710,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/05/2026 21:01</t>
+          <t>10/06/2026 18:52</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>12728.89</v>
+        <v>12345.14</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>27.24</v>
+        <v>23.4</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>3.1</v>
+        <v>2.39</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11831,22 +11741,22 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>2901.09</v>
+        <v>2556.29</v>
       </c>
       <c r="V105" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>73.23943661971832</v>
+        <v>70.66666666666667</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>3.69</v>
+        <v>2.75</v>
       </c>
       <c r="Y105" s="7" t="n">
-        <v>2.69</v>
+        <v>2.97</v>
       </c>
       <c r="Z105" t="inlineStr">
         <is>
@@ -11855,7 +11765,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11900,7 +11810,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/03/2026 14:44</t>
+          <t>10/06/2026 14:47</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
@@ -12009,14 +11919,14 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>10/05/2026 21:47</t>
+          <t>10/06/2026 20:02</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>24475.57</v>
+        <v>24546.14</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-36.27</v>
+        <v>-36.08</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>42.89</v>
@@ -12034,31 +11944,31 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>132.79</v>
+        <v>392.8800000000001</v>
       </c>
       <c r="P107" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>1.407143952169247</v>
+        <v>3.915188840246347</v>
       </c>
       <c r="S107" s="7" t="n">
-        <v>0.77</v>
+        <v>0.53</v>
       </c>
       <c r="T107" t="n">
-        <v>3951</v>
+        <v>3962</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-9806.43</v>
+        <v>-9771.25</v>
       </c>
       <c r="V107" t="n">
-        <v>2369</v>
+        <v>2379</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>59.95950392305745</v>
+        <v>60.04543160020192</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.75</v>
@@ -12073,7 +11983,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12118,7 +12028,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 13:07</t>
+          <t>10/06/2026 13:09</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12209,7 +12119,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 06:56</t>
+          <t>10/06/2026 07:00</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
@@ -12573,7 +12483,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 21:01</t>
+          <t>10/06/2026 21:04</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12664,7 +12574,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 14:42</t>
+          <t>10/06/2026 14:45</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12846,7 +12756,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 07:54</t>
+          <t>10/06/2026 07:57</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -13028,7 +12938,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 00:17</t>
+          <t>10/06/2026 00:19</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13669,23 +13579,17 @@
         <v>0</v>
       </c>
       <c r="N125" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O125" s="9" t="n">
-        <v>-1180.45</v>
+        <v>0</v>
       </c>
       <c r="P125" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q125" s="9" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R125" s="9" t="n">
-        <v>0.2676972896517925</v>
-      </c>
-      <c r="S125" s="9" t="n">
-        <v>1.18</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q125" s="8" t="n"/>
+      <c r="R125" s="8" t="n"/>
+      <c r="S125" s="8" t="n"/>
       <c r="T125" s="8" t="n">
         <v>0</v>
       </c>
@@ -13760,17 +13664,23 @@
         <v>0</v>
       </c>
       <c r="N126" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O126" s="9" t="n">
-        <v>0</v>
+        <v>-3715.63</v>
       </c>
       <c r="P126" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q126" s="8" t="n"/>
-      <c r="R126" s="8" t="n"/>
-      <c r="S126" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q126" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R126" s="9" t="n">
+        <v>0.2438039067238144</v>
+      </c>
+      <c r="S126" s="9" t="n">
+        <v>3.72</v>
+      </c>
       <c r="T126" s="8" t="n">
         <v>0</v>
       </c>
@@ -13845,23 +13755,17 @@
         <v>0</v>
       </c>
       <c r="N127" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O127" s="9" t="n">
-        <v>-4944.48</v>
+        <v>0</v>
       </c>
       <c r="P127" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q127" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R127" s="9" t="n">
-        <v>0.2385997385250534</v>
-      </c>
-      <c r="S127" s="9" t="n">
-        <v>5.42</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q127" s="8" t="n"/>
+      <c r="R127" s="8" t="n"/>
+      <c r="S127" s="8" t="n"/>
       <c r="T127" s="8" t="n">
         <v>0</v>
       </c>
@@ -13999,7 +13903,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 10:00</t>
+          <t>10/06/2026 10:03</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -14090,7 +13994,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 09:25</t>
+          <t>10/06/2026 09:27</t>
         </is>
       </c>
       <c r="H130" s="8" t="n">
@@ -14272,7 +14176,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>10/03/2026 18:08</t>
+          <t>10/06/2026 18:12</t>
         </is>
       </c>
       <c r="H132" s="9" t="n">
@@ -14447,7 +14351,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10/03/2026 13:07</t>
+          <t>10/06/2026 13:09</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14488,7 +14392,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/03/2026 06:56</t>
+          <t>10/06/2026 07:00</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14652,7 +14556,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10/03/2026 21:01</t>
+          <t>10/06/2026 21:04</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14693,7 +14597,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10/03/2026 14:42</t>
+          <t>10/06/2026 14:45</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14775,7 +14679,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10/03/2026 07:54</t>
+          <t>10/06/2026 07:57</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14857,7 +14761,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10/03/2026 00:17</t>
+          <t>10/06/2026 00:19</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -15154,7 +15058,7 @@
         <v>-2.31</v>
       </c>
       <c r="I22" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -15195,7 +15099,7 @@
         <v>-6.66</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -15236,7 +15140,7 @@
         <v>-20.23</v>
       </c>
       <c r="I24" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -15308,7 +15212,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>10/03/2026 10:00</t>
+          <t>10/06/2026 10:03</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15349,7 +15253,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10/03/2026 09:25</t>
+          <t>10/06/2026 09:27</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15431,7 +15335,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>10/03/2026 18:08</t>
+          <t>10/06/2026 18:12</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17772,7 +17676,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/03/2026 12:17</t>
+          <t>10/06/2026 12:20</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17818,7 +17722,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10/03/2026 11:56</t>
+          <t>10/06/2026 11:58</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17841,7 +17745,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10/03/2026 05:26</t>
+          <t>10/06/2026 05:29</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17910,7 +17814,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10/03/2026 04:23</t>
+          <t>10/06/2026 04:26</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17979,7 +17883,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10/03/2026 13:40</t>
+          <t>10/06/2026 13:42</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -18025,7 +17929,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10/03/2026 11:46</t>
+          <t>10/06/2026 11:48</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -18117,7 +18021,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10/03/2026 15:41</t>
+          <t>10/06/2026 15:44</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -18140,7 +18044,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10/03/2026 05:13</t>
+          <t>10/06/2026 05:16</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -18163,7 +18067,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10/03/2026 19:03</t>
+          <t>10/06/2026 19:06</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -18186,7 +18090,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10/03/2026 13:47</t>
+          <t>10/06/2026 13:50</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18232,7 +18136,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10/03/2026 15:27</t>
+          <t>10/06/2026 15:30</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18324,7 +18228,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10/02/2026 23:37</t>
+          <t>10/05/2026 23:39</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18347,7 +18251,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10/02/2026 23:38</t>
+          <t>10/05/2026 23:40</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18485,7 +18389,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10/03/2026 11:49</t>
+          <t>10/06/2026 11:53</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18508,7 +18412,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10/03/2026 12:46</t>
+          <t>10/06/2026 12:49</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18531,7 +18435,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10/03/2026 17:57</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18554,7 +18458,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/05/2026 14:31</t>
+          <t>10/06/2026 19:17</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-07
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-06 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-07 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/06/2026 20:34</t>
+          <t>10/07/2026 20:37</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>50028.39</v>
+        <v>36279.84</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>128.71</v>
+        <v>65.86</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.06</v>
+        <v>1.03</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>166.0299999999987</v>
+        <v>-6242.860000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>75</v>
+        <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.003798874500773</v>
+        <v>0.8704616197370869</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>44.62</v>
+        <v>47.96</v>
       </c>
       <c r="T2" t="n">
-        <v>3471</v>
+        <v>3477</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>25395.21</v>
+        <v>12149.04999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2210</v>
+        <v>2212</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.67041198501872</v>
+        <v>63.6180615473109</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/04/2026 12:03</t>
+          <t>10/07/2026 12:06</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/04/2026 16:12</t>
+          <t>10/07/2026 16:15</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/04/2026 01:17</t>
+          <t>10/07/2026 01:20</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/06/2026 21:11</t>
+          <t>10/07/2026 21:02</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/06/2026 22:41</t>
+          <t>10/07/2026 22:19</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19533.88</v>
+        <v>19510.04</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.48</v>
+        <v>-2.6</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.74</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,37 +3274,37 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-233.79</v>
+        <v>-294.83</v>
       </c>
       <c r="P23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.3402099678275103</v>
+        <v>0.2203976942196837</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>1.55</v>
       </c>
       <c r="T23" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-466.1200000000001</v>
+        <v>-567.4900000000001</v>
       </c>
       <c r="V23" t="n">
         <v>21</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>25.92592592592592</v>
+        <v>25.60975609756098</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>2.58</v>
+        <v>2.9</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/06/2026 21:38</t>
+          <t>10/07/2026 21:20</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/06/2026 21:16</t>
+          <t>10/07/2026 21:05</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/06/2026 21:19</t>
+          <t>10/07/2026 21:07</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/04/2026 13:19</t>
+          <t>10/07/2026 13:20</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/06/2026 21:46</t>
+          <t>10/07/2026 21:28</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20678.71</v>
+        <v>20676.34</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.74</v>
+        <v>1.73</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-0.159999999999998</v>
+        <v>39.77</v>
       </c>
       <c r="P30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>30</v>
+        <v>32.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.999279344203225</v>
+        <v>1.209381910076866</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="T30" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>678.7099999999999</v>
+        <v>676.3399999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>28.97196261682243</v>
+        <v>29.35779816513762</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.74</v>
+        <v>1.73</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/06/2026 23:46</t>
+          <t>10/07/2026 23:34</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4579,37 +4579,28 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>255.36</v>
+        <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q35" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R35" s="7" t="n">
-        <v>1.138761492816311</v>
-      </c>
-      <c r="S35" s="7" t="n">
-        <v>3.19</v>
+        <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>217.9599999999999</v>
+        <v>125.1799999999998</v>
       </c>
       <c r="V35" t="n">
         <v>77</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>50.99337748344372</v>
+        <v>50.6578947368421</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4621,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4884,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>10/04/2026 22:24</t>
+          <t>10/07/2026 22:27</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4993,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10/04/2026 11:45</t>
+          <t>10/07/2026 11:47</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5102,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10/04/2026 10:14</t>
+          <t>10/07/2026 10:17</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5538,20 +5529,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/06/2026 21:48</t>
+          <t>10/07/2026 21:31</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19672.79</v>
+        <v>19637.57</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.61</v>
+        <v>-1.78</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5563,34 +5554,34 @@
         <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-185.9</v>
+        <v>-78.93000000000001</v>
       </c>
       <c r="P44" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q44" s="7" t="n">
-        <v>35</v>
+        <v>42.5</v>
       </c>
       <c r="R44" s="7" t="n">
-        <v>0.1371547922951961</v>
+        <v>0.3050713153724247</v>
       </c>
       <c r="S44" s="7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="T44" t="n">
+        <v>848</v>
+      </c>
+      <c r="U44" s="7" t="n">
+        <v>-363.0900000000001</v>
+      </c>
+      <c r="V44" t="n">
+        <v>467</v>
+      </c>
+      <c r="W44" s="7" t="n">
+        <v>55.07075471698113</v>
+      </c>
+      <c r="X44" s="7" t="n">
         <v>0.93</v>
-      </c>
-      <c r="T44" t="n">
-        <v>830</v>
-      </c>
-      <c r="U44" s="7" t="n">
-        <v>-327.2100000000001</v>
-      </c>
-      <c r="V44" t="n">
-        <v>463</v>
-      </c>
-      <c r="W44" s="7" t="n">
-        <v>55.78313253012048</v>
-      </c>
-      <c r="X44" s="7" t="n">
-        <v>0.9399999999999999</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5602,7 +5593,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5647,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/06/2026 20:45</t>
+          <t>10/07/2026 20:42</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5756,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/06/2026 21:08</t>
+          <t>10/07/2026 15:02</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5987,13 +5978,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6087,13 +6087,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T49" t="n">
         <v>1161</v>
@@ -6187,13 +6196,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>-52.41999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>0.8051952878219183</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>1.3</v>
       </c>
       <c r="T50" t="n">
         <v>1978</v>
@@ -6265,20 +6283,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/06/2026 20:56</t>
+          <t>10/07/2026 20:53</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19582.17</v>
+        <v>19781.85</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-2.06</v>
+        <v>-1.06</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6287,28 +6305,37 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>0</v>
+        <v>1248.12</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R51" s="7" t="n">
+        <v>1.376252547298356</v>
+      </c>
+      <c r="S51" s="7" t="n">
+        <v>5.9</v>
       </c>
       <c r="T51" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-417.8300000000005</v>
+        <v>-218.1500000000001</v>
       </c>
       <c r="V51" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>31.42857142857143</v>
+        <v>32.87671232876712</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6320,7 +6347,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6365,20 +6392,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/06/2026 21:31</t>
+          <t>10/07/2026 21:16</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19368.38</v>
+        <v>19202.71</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.12</v>
+        <v>-3.95</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>5.79</v>
+        <v>6.13</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6396,22 +6423,22 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-631.62</v>
+        <v>-797.29</v>
       </c>
       <c r="V52" t="n">
         <v>48</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.4</v>
+        <v>37.79527559055118</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>5.81</v>
+        <v>6.17</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6420,7 +6447,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6465,14 +6492,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/06/2026 22:05</t>
+          <t>10/07/2026 21:42</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19678.78</v>
+        <v>19674.98</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.64</v>
+        <v>-1.66</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6496,16 +6523,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-321.2200000000001</v>
+        <v>-325.02</v>
       </c>
       <c r="V53" t="n">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.54266958424508</v>
+        <v>36.79653679653679</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>0.79</v>
@@ -6520,7 +6547,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6687,13 +6714,22 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>0</v>
+        <v>-104.34</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q55" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R55" s="7" t="n">
+        <v>0.347793474184273</v>
+      </c>
+      <c r="S55" s="7" t="n">
+        <v>0.52</v>
       </c>
       <c r="T55" t="n">
         <v>1920</v>
@@ -6765,7 +6801,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10/04/2026 11:11</t>
+          <t>10/07/2026 11:15</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6865,20 +6901,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/06/2026 21:03</t>
+          <t>10/07/2026 20:57</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19489.74</v>
+        <v>19509.32</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.54</v>
+        <v>-2.45</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>2.54</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6887,28 +6923,37 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-30.19</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.5627805937726286</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T57" t="n">
-        <v>1174</v>
+        <v>1189</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-509.7900000000001</v>
+        <v>-490.72</v>
       </c>
       <c r="V57" t="n">
-        <v>503</v>
+        <v>511</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>42.84497444633731</v>
+        <v>42.97729184188393</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>2.55</v>
@@ -6920,7 +6965,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6965,7 +7010,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/06/2026 21:42</t>
+          <t>10/07/2026 21:24</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7065,7 +7110,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>10/04/2026 14:02</t>
+          <t>10/07/2026 14:04</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7087,13 +7132,22 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>0</v>
+        <v>-80.78999999999999</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="Q59" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R59" s="7" t="n">
+        <v>0.32387647501883</v>
+      </c>
+      <c r="S59" s="7" t="n">
+        <v>0.43</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7165,7 +7219,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/06/2026 21:24</t>
+          <t>10/07/2026 21:11</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7274,7 +7328,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/06/2026 22:27</t>
+          <t>10/07/2026 22:04</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7474,7 +7528,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/06/2026 21:59</t>
+          <t>10/07/2026 21:37</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7596,13 +7650,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-90.82000000000002</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.7198297137216189</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>0.96</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7674,7 +7737,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/06/2026 21:59</t>
+          <t>10/07/2026 21:38</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7684,7 +7747,7 @@
         <v>-7.9</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>12.22</v>
+        <v>12.41</v>
       </c>
       <c r="K65" s="7" t="n">
         <v>0.89</v>
@@ -7874,20 +7937,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/06/2026 22:19</t>
+          <t>10/07/2026 21:55</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20718.18</v>
+        <v>20646.21</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>3.64</v>
+        <v>3.28</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7905,19 +7968,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>718.1799999999998</v>
+        <v>579.8199999999993</v>
       </c>
       <c r="V67" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>31.57894736842105</v>
+        <v>32.6530612244898</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7929,7 +7992,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7974,7 +8037,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>10/04/2026 14:02</t>
+          <t>10/07/2026 14:05</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8396,22 +8459,13 @@
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O72" s="7" t="n">
-        <v>-19.59</v>
+        <v>0</v>
       </c>
       <c r="P72" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q72" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R72" s="7" t="n">
-        <v>0.8233543733092877</v>
-      </c>
-      <c r="S72" s="7" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="T72" t="n">
         <v>326</v>
@@ -8505,13 +8559,22 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>0</v>
+        <v>-39.43999999999999</v>
       </c>
       <c r="P73" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q73" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R73" s="7" t="n">
+        <v>0.8172212438594866</v>
+      </c>
+      <c r="S73" s="7" t="n">
+        <v>0.49</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -8805,13 +8868,22 @@
         <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O76" s="7" t="n">
-        <v>0</v>
+        <v>-212.9</v>
       </c>
       <c r="P76" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q76" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R76" s="7" t="n">
+        <v>0.5722322684348001</v>
+      </c>
+      <c r="S76" s="7" t="n">
+        <v>1.9</v>
       </c>
       <c r="T76" t="n">
         <v>313</v>
@@ -9883,14 +9955,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/06/2026 23:04</t>
+          <t>10/07/2026 22:47</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19804.32</v>
-      </c>
-      <c r="I87" s="7" t="n">
-        <v>-0.98</v>
+        <v>19800.55</v>
+      </c>
+      <c r="I87" t="n">
+        <v>-1</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>5.37</v>
@@ -9914,16 +9986,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-195.6799999999997</v>
+        <v>-199.4499999999999</v>
       </c>
       <c r="V87" t="n">
         <v>78</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>42.39130434782609</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>0.92</v>
@@ -9938,7 +10010,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9983,7 +10055,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>10/04/2026 14:54</t>
+          <t>10/07/2026 14:58</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10083,14 +10155,14 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/06/2026 22:45</t>
+          <t>10/07/2026 22:23</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20033.47</v>
+        <v>20041.37</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>3.63</v>
@@ -10114,16 +10186,16 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>33.47</v>
+        <v>41.37</v>
       </c>
       <c r="V89" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>82.89473684210526</v>
+        <v>83.00653594771242</v>
       </c>
       <c r="X89" s="7" t="n">
         <v>1.01</v>
@@ -10138,7 +10210,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10183,20 +10255,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/06/2026 22:42</t>
+          <t>10/07/2026 22:21</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27747.08</v>
+        <v>27700.59</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>38.79</v>
+        <v>38.56</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.88</v>
+        <v>1.86</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10214,19 +10286,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7747.08</v>
+        <v>7700.59</v>
       </c>
       <c r="V90" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>69.03225806451613</v>
+        <v>68.98734177215189</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.88</v>
+        <v>1.86</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>3.32</v>
@@ -10238,7 +10310,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10405,13 +10477,22 @@
         <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="O92" s="7" t="n">
-        <v>0</v>
+        <v>20269.59</v>
       </c>
       <c r="P92" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="Q92" s="7" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="R92" s="7" t="n">
+        <v>188.9075739315843</v>
+      </c>
+      <c r="S92" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T92" t="n">
         <v>23</v>
@@ -10443,7 +10524,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -10705,22 +10786,13 @@
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O95" s="7" t="n">
-        <v>19948.18</v>
+        <v>0</v>
       </c>
       <c r="P95" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q95" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R95" s="7" t="n">
-        <v>109.8042980255264</v>
-      </c>
-      <c r="S95" s="7" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="T95" t="n">
         <v>11</v>
@@ -10752,7 +10824,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC95" t="inlineStr">
@@ -11292,20 +11364,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/06/2026 23:30</t>
+          <t>10/07/2026 23:16</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>21162.64</v>
+        <v>21470.74</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>5.8</v>
+        <v>7.34</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>2.34</v>
+        <v>2.69</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11314,28 +11386,37 @@
         <v>0</v>
       </c>
       <c r="N101" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="O101" s="7" t="n">
-        <v>0</v>
+        <v>21470.74</v>
       </c>
       <c r="P101" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q101" s="7" t="n">
+        <v>76.19047619047619</v>
+      </c>
+      <c r="R101" s="7" t="n">
+        <v>25.72135035866024</v>
+      </c>
+      <c r="S101" s="7" t="n">
+        <v>1.01</v>
       </c>
       <c r="T101" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>1162.64</v>
+        <v>1470.74</v>
       </c>
       <c r="V101" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>73.68421052631578</v>
+        <v>75</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>2.34</v>
+        <v>2.69</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11347,12 +11428,12 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC101" t="inlineStr">
@@ -11392,20 +11473,20 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/06/2026 21:36</t>
+          <t>10/07/2026 21:22</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
-        <v>21207.19</v>
+        <v>21187.19</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>6.06</v>
+        <v>5.96</v>
       </c>
       <c r="J102" s="7" t="n">
         <v>6.68</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>1.68</v>
+        <v>1.66</v>
       </c>
       <c r="L102" t="n">
         <v>20000</v>
@@ -11423,19 +11504,19 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="U102" s="7" t="n">
-        <v>1207.19</v>
+        <v>1187.19</v>
       </c>
       <c r="V102" t="n">
         <v>33</v>
       </c>
       <c r="W102" s="7" t="n">
-        <v>41.25</v>
+        <v>40.74074074074074</v>
       </c>
       <c r="X102" s="7" t="n">
-        <v>1.68</v>
+        <v>1.66</v>
       </c>
       <c r="Y102" s="7" t="n">
         <v>4.04</v>
@@ -11447,7 +11528,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -11492,7 +11573,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>10/04/2026 10:45</t>
+          <t>10/07/2026 10:47</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
@@ -11710,20 +11791,20 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/06/2026 18:52</t>
+          <t>10/07/2026 19:23</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
-        <v>12345.14</v>
+        <v>12445.59</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>23.4</v>
+        <v>24.4</v>
       </c>
       <c r="J105" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K105" s="7" t="n">
-        <v>2.39</v>
+        <v>2.45</v>
       </c>
       <c r="L105" t="n">
         <v>10000</v>
@@ -11741,19 +11822,19 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="U105" s="7" t="n">
-        <v>2556.29</v>
+        <v>2613.28</v>
       </c>
       <c r="V105" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>70.66666666666667</v>
+        <v>70.12987012987013</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>2.75</v>
+        <v>2.79</v>
       </c>
       <c r="Y105" s="7" t="n">
         <v>2.97</v>
@@ -11765,7 +11846,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -11919,14 +12000,14 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>10/06/2026 20:02</t>
+          <t>10/07/2026 20:13</t>
         </is>
       </c>
       <c r="H107" s="7" t="n">
-        <v>24546.14</v>
+        <v>24564.71</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>-36.08</v>
+        <v>-36.03</v>
       </c>
       <c r="J107" s="7" t="n">
         <v>42.89</v>
@@ -11944,31 +12025,31 @@
         <v>40</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>392.8800000000001</v>
+        <v>379.7500000000001</v>
       </c>
       <c r="P107" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q107" s="7" t="n">
-        <v>90</v>
+        <v>87.5</v>
       </c>
       <c r="R107" s="7" t="n">
-        <v>3.915188840246347</v>
+        <v>3.199154505443595</v>
       </c>
       <c r="S107" s="7" t="n">
         <v>0.53</v>
       </c>
       <c r="T107" t="n">
-        <v>3962</v>
+        <v>3968</v>
       </c>
       <c r="U107" s="7" t="n">
-        <v>-9771.25</v>
+        <v>-9750.250000000002</v>
       </c>
       <c r="V107" t="n">
-        <v>2379</v>
+        <v>2383</v>
       </c>
       <c r="W107" s="7" t="n">
-        <v>60.04543160020192</v>
+        <v>60.0554435483871</v>
       </c>
       <c r="X107" s="7" t="n">
         <v>0.75</v>
@@ -11983,7 +12064,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -12392,7 +12473,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>10/04/2026 12:17</t>
+          <t>10/07/2026 12:20</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12665,7 +12746,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>10/04/2026 16:10</t>
+          <t>10/07/2026 16:13</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -13029,7 +13110,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>10/04/2026 14:52</t>
+          <t>10/07/2026 14:55</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13664,23 +13745,17 @@
         <v>0</v>
       </c>
       <c r="N126" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O126" s="9" t="n">
-        <v>-3715.63</v>
+        <v>0</v>
       </c>
       <c r="P126" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q126" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R126" s="9" t="n">
-        <v>0.2438039067238144</v>
-      </c>
-      <c r="S126" s="9" t="n">
-        <v>3.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q126" s="8" t="n"/>
+      <c r="R126" s="8" t="n"/>
+      <c r="S126" s="8" t="n"/>
       <c r="T126" s="8" t="n">
         <v>0</v>
       </c>
@@ -14515,7 +14590,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10/04/2026 12:17</t>
+          <t>10/07/2026 12:20</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14638,7 +14713,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10/04/2026 16:10</t>
+          <t>10/07/2026 16:13</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14802,7 +14877,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>10/04/2026 14:52</t>
+          <t>10/07/2026 14:55</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -15099,7 +15174,7 @@
         <v>-6.66</v>
       </c>
       <c r="I23" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -17699,7 +17774,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10/04/2026 16:24</t>
+          <t>10/07/2026 16:27</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17791,7 +17866,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10/04/2026 09:23</t>
+          <t>10/07/2026 09:26</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17837,7 +17912,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10/04/2026 09:27</t>
+          <t>10/07/2026 09:30</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -18159,7 +18234,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10/04/2026 08:16</t>
+          <t>10/07/2026 08:18</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18320,7 +18395,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10/04/2026 09:22</t>
+          <t>10/07/2026 09:24</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18343,7 +18418,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10/04/2026 09:33</t>
+          <t>10/07/2026 09:35</t>
         </is>
       </c>
       <c r="E33" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-13
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-09 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-13 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/09/2026 19:13</t>
+          <t>10/13/2026 20:27</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>29396.94</v>
+        <v>35164.19</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>34.39</v>
+        <v>60.75</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-13327.63</v>
+        <v>-13567.74</v>
       </c>
       <c r="P2" t="n">
         <v>29</v>
@@ -994,25 +994,25 @@
         <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.7540055497947712</v>
+        <v>0.7495737245236033</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>87.23999999999999</v>
+        <v>106.82</v>
       </c>
       <c r="T2" t="n">
-        <v>3484</v>
+        <v>3489</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>4396.939999999999</v>
+        <v>10164.19</v>
       </c>
       <c r="V2" t="n">
-        <v>2217</v>
+        <v>2221</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.6337543053961</v>
+        <v>63.65720836916022</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/08/2026 15:18</t>
+          <t>10/11/2026 15:26</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/08/2026 18:17</t>
+          <t>10/11/2026 18:36</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/07/2026 12:06</t>
+          <t>10/13/2026 12:11</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/08/2026 09:45</t>
+          <t>10/11/2026 09:49</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/09/2026 14:52</t>
+          <t>10/12/2026 14:55</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/09/2026 17:26</t>
+          <t>10/12/2026 17:31</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/09/2026 17:28</t>
+          <t>10/12/2026 17:33</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/08/2026 17:03</t>
+          <t>10/11/2026 17:17</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/09/2026 08:35</t>
+          <t>10/12/2026 08:38</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/08/2026 18:27</t>
+          <t>10/11/2026 18:47</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/07/2026 16:15</t>
+          <t>10/13/2026 16:21</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/08/2026 17:18</t>
+          <t>10/11/2026 17:32</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/08/2026 18:59</t>
+          <t>10/11/2026 19:22</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/08/2026 18:00</t>
+          <t>10/11/2026 18:18</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/08/2026 18:01</t>
+          <t>10/11/2026 18:19</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/08/2026 18:16</t>
+          <t>10/11/2026 18:35</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/07/2026 01:20</t>
+          <t>10/13/2026 01:24</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/09/2026 19:48</t>
+          <t>10/13/2026 20:55</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>18897.99</v>
-      </c>
-      <c r="I22" s="7" t="n">
-        <v>-5.51</v>
+        <v>18800.01</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-6</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>7.74</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3165,37 +3165,37 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-602.99</v>
+        <v>-689.0500000000001</v>
       </c>
       <c r="P22" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>45</v>
+        <v>42.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.7730295969797002</v>
+        <v>0.7369927745057999</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>6.48</v>
+        <v>6.96</v>
       </c>
       <c r="T22" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-1102.01</v>
+        <v>-1199.99</v>
       </c>
       <c r="V22" t="n">
         <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>47.22222222222222</v>
+        <v>46.78899082568807</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>7.74</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/09/2026 21:33</t>
+          <t>10/13/2026 22:11</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19415.81</v>
+        <v>19442.14</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-3.07</v>
+        <v>-2.94</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.13</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-335.7</v>
+        <v>-235.99</v>
       </c>
       <c r="P23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>17.5</v>
+        <v>22.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.1989022789643241</v>
+        <v>0.3172968438105707</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>1.68</v>
+        <v>1.31</v>
       </c>
       <c r="T23" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-584.1900000000002</v>
+        <v>-557.86</v>
       </c>
       <c r="V23" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>24.70588235294118</v>
+        <v>25.55555555555555</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.98</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/08/2026 09:23</t>
+          <t>10/11/2026 09:26</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/08/2026 23:42</t>
+          <t>10/11/2026 23:46</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,14 +3576,14 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/09/2026 19:50</t>
+          <t>10/13/2026 14:51</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20256.64</v>
+        <v>20252.01</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-3.16</v>
+        <v>-3.18</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
@@ -3601,7 +3601,7 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-209.19</v>
+        <v>-197.47</v>
       </c>
       <c r="P26" t="n">
         <v>15</v>
@@ -3610,22 +3610,22 @@
         <v>37.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>0.8915180932823049</v>
+        <v>0.8969696653483736</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>4.94</v>
+        <v>4.86</v>
       </c>
       <c r="T26" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>256.6400000000003</v>
+        <v>252.0099999999999</v>
       </c>
       <c r="V26" t="n">
         <v>61</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>43.88489208633094</v>
+        <v>42.36111111111111</v>
       </c>
       <c r="X26" s="7" t="n">
         <v>1.04</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/09/2026 13:47</t>
+          <t>10/12/2026 13:50</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/09/2026 19:53</t>
+          <t>10/13/2026 20:54</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/07/2026 13:20</t>
+          <t>10/13/2026 13:26</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/09/2026 20:21</t>
+          <t>10/13/2026 21:18</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20667.49</v>
+        <v>20649.89</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>3.37</v>
+        <v>3.28</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.72</v>
+        <v>1.68</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,7 +4037,7 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>47.17</v>
+        <v>36.84</v>
       </c>
       <c r="P30" t="n">
         <v>13</v>
@@ -4046,25 +4046,25 @@
         <v>32.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>1.258409115810233</v>
+        <v>1.191009488256338</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.51</v>
+        <v>0.47</v>
       </c>
       <c r="T30" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>667.4899999999999</v>
+        <v>649.8899999999999</v>
       </c>
       <c r="V30" t="n">
         <v>32</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>28.82882882882883</v>
+        <v>28.31858407079646</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.72</v>
+        <v>1.68</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/08/2026 18:27</t>
+          <t>10/11/2026 18:47</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/08/2026 18:33</t>
+          <t>10/11/2026 18:54</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/08/2026 19:45</t>
+          <t>10/11/2026 19:59</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>10/08/2026 17:40</t>
+          <t>10/11/2026 17:56</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/09/2026 22:58</t>
+          <t>10/13/2026 23:26</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20327.86</v>
+        <v>20633.14</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1.64</v>
+        <v>3.17</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.04</v>
+        <v>1.08</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>327.8599999999998</v>
+        <v>633.1399999999999</v>
       </c>
       <c r="V35" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>51.2987012987013</v>
+        <v>51.89873417721519</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.04</v>
+        <v>1.08</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>10/08/2026 18:32</t>
+          <t>10/11/2026 18:53</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>10/08/2026 17:22</t>
+          <t>10/11/2026 17:37</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>10/07/2026 22:27</t>
+          <t>10/13/2026 22:34</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10/07/2026 11:47</t>
+          <t>10/13/2026 11:51</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10/07/2026 10:17</t>
+          <t>10/13/2026 10:23</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10/09/2026 00:47</t>
+          <t>10/12/2026 00:51</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>10/09/2026 01:08</t>
+          <t>10/12/2026 01:11</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>10/09/2026 03:25</t>
+          <t>10/12/2026 03:30</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5511,14 +5511,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/09/2026 20:26</t>
+          <t>10/13/2026 21:21</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19638.49</v>
+        <v>19633.29</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.78</v>
+        <v>-1.81</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5542,16 +5542,16 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-361.5100000000001</v>
+        <v>-366.71</v>
       </c>
       <c r="V44" t="n">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.04694835680751</v>
+        <v>55.0233644859813</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.93</v>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,20 +5611,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/09/2026 19:18</t>
+          <t>10/13/2026 20:32</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19983.51</v>
+        <v>19978.73</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.09</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>0.26</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5642,19 +5642,19 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-16.49</v>
+        <v>-21.27</v>
       </c>
       <c r="V45" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>35.08771929824561</v>
+        <v>34.42622950819672</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>0.27</v>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5711,20 +5711,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/09/2026 19:49</t>
+          <t>10/13/2026 20:53</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19329.32</v>
+        <v>19229.81</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-3.33</v>
+        <v>-3.83</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5742,19 +5742,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-670.6800000000001</v>
+        <v>-770.1900000000001</v>
       </c>
       <c r="V46" t="n">
         <v>41</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>42.70833333333333</v>
+        <v>42.2680412371134</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>10/09/2026 00:08</t>
+          <t>10/12/2026 00:11</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>10/09/2026 20:57</t>
+          <t>10/12/2026 21:01</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>10/09/2026 01:00</t>
+          <t>10/12/2026 01:03</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>10/09/2026 00:35</t>
+          <t>10/12/2026 00:38</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/09/2026 19:34</t>
+          <t>10/13/2026 20:41</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/09/2026 20:04</t>
+          <t>10/13/2026 21:04</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6342,16 +6342,16 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-891.12</v>
+        <v>-891.1200000000001</v>
       </c>
       <c r="V52" t="n">
         <v>48</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>37.79527559055118</v>
+        <v>37.5</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.85</v>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,14 +6411,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/09/2026 20:40</t>
+          <t>10/13/2026 21:36</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19644.4</v>
+        <v>19640.11</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.81</v>
+        <v>-1.84</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6442,16 +6442,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>473</v>
+        <v>483</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-355.6</v>
+        <v>-359.8899999999999</v>
       </c>
       <c r="V53" t="n">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.36363636363637</v>
+        <v>36.43892339544513</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>0.78</v>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>10/08/2026 21:47</t>
+          <t>10/11/2026 21:49</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10/08/2026 18:40</t>
+          <t>10/11/2026 19:03</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10/07/2026 11:15</t>
+          <t>10/13/2026 11:22</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6811,14 +6811,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/09/2026 19:39</t>
+          <t>10/13/2026 20:50</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19498.97</v>
+        <v>19496.12</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.51</v>
+        <v>-2.53</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>2.54</v>
@@ -6842,16 +6842,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1218</v>
+        <v>1243</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-500.5599999999999</v>
+        <v>-503.63</v>
       </c>
       <c r="V57" t="n">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.02134646962233</v>
+        <v>43.04102976669348</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.74</v>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/09/2026 20:16</t>
+          <t>10/13/2026 21:12</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>10/07/2026 14:04</t>
+          <t>10/13/2026 14:10</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/09/2026 20:03</t>
+          <t>10/13/2026 21:06</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/09/2026 21:11</t>
+          <t>10/13/2026 21:53</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>10/08/2026 21:37</t>
+          <t>10/11/2026 21:39</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/09/2026 20:33</t>
+          <t>10/13/2026 21:31</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>10/08/2026 18:49</t>
+          <t>10/11/2026 19:11</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/09/2026 20:34</t>
+          <t>10/13/2026 21:27</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>10/08/2026 18:39</t>
+          <t>10/11/2026 19:00</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/09/2026 12:20</t>
+          <t>10/13/2026 21:49</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>10/07/2026 14:05</t>
+          <t>10/13/2026 14:12</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>10/08/2026 17:12</t>
+          <t>10/11/2026 17:26</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>10/08/2026 17:12</t>
+          <t>10/11/2026 17:26</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>10/08/2026 17:11</t>
+          <t>10/11/2026 17:26</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>10/08/2026 18:43</t>
+          <t>10/11/2026 19:05</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>10/08/2026 19:05</t>
+          <t>10/11/2026 19:28</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>10/08/2026 18:40</t>
+          <t>10/11/2026 19:01</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>10/08/2026 20:57</t>
+          <t>10/11/2026 21:01</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>10/08/2026 20:23</t>
+          <t>10/11/2026 20:27</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>10/08/2026 20:35</t>
+          <t>10/11/2026 20:38</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>10/08/2026 20:32</t>
+          <t>10/11/2026 20:36</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>10/08/2026 20:38</t>
+          <t>10/11/2026 20:41</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>10/08/2026 20:33</t>
+          <t>10/11/2026 20:36</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>10/08/2026 20:51</t>
+          <t>10/11/2026 20:54</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>10/08/2026 20:35</t>
+          <t>10/11/2026 20:39</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>10/08/2026 18:38</t>
+          <t>10/11/2026 18:59</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>10/09/2026 02:12</t>
+          <t>10/12/2026 02:15</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>10/08/2026 20:35</t>
+          <t>10/11/2026 20:39</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9811,20 +9811,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/09/2026 22:13</t>
+          <t>10/13/2026 22:39</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19800.01</v>
+        <v>19896.06</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-1.01</v>
+        <v>-0.54</v>
       </c>
       <c r="J87" s="7" t="n">
-        <v>5.37</v>
+        <v>5.56</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9842,22 +9842,22 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-199.9899999999999</v>
+        <v>-103.9399999999999</v>
       </c>
       <c r="V87" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>43.14720812182741</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="Y87" s="7" t="n">
-        <v>5.36</v>
+        <v>5.55</v>
       </c>
       <c r="Z87" t="inlineStr">
         <is>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9911,7 +9911,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>10/07/2026 14:58</t>
+          <t>10/13/2026 15:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10011,20 +10011,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/09/2026 21:43</t>
+          <t>10/13/2026 22:17</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>20097.07</v>
+        <v>19929.86</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>0.48</v>
+        <v>-0.35</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>3.63</v>
+        <v>3.94</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,22 +10042,22 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>97.07000000000001</v>
+        <v>-70.14000000000004</v>
       </c>
       <c r="V89" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>83.43949044585987</v>
+        <v>82.82208588957054</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="Y89" s="7" t="n">
-        <v>3.63</v>
+        <v>3.96</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10111,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/09/2026 21:34</t>
+          <t>10/13/2026 22:11</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27281.27</v>
+        <v>27786.09</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>36.47</v>
+        <v>38.99</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>4.12</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.72</v>
+        <v>1.74</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10142,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7281.27</v>
+        <v>7786.09</v>
       </c>
       <c r="V90" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>68.45238095238095</v>
+        <v>68.36158192090396</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.72</v>
+        <v>1.74</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>4.12</v>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>10/08/2026 20:16</t>
+          <t>10/11/2026 20:24</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>10/08/2026 04:34</t>
+          <t>10/11/2026 04:36</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>10/08/2026 19:05</t>
+          <t>10/11/2026 19:29</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>10/08/2026 19:03</t>
+          <t>10/11/2026 19:26</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>10/08/2026 19:01</t>
+          <t>10/11/2026 19:24</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10711,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>10/09/2026 00:01</t>
+          <t>10/12/2026 00:04</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>10/08/2026 20:18</t>
+          <t>10/11/2026 20:25</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>10/09/2026 00:08</t>
+          <t>10/12/2026 00:11</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>10/08/2026 04:57</t>
+          <t>10/11/2026 05:01</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11211,20 +11211,20 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/09/2026 22:41</t>
+          <t>10/13/2026 23:10</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
-        <v>21478.57</v>
+        <v>21499.09</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>7.38</v>
+        <v>7.48</v>
       </c>
       <c r="J101" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>2.7</v>
+        <v>2.73</v>
       </c>
       <c r="L101" t="n">
         <v>20000</v>
@@ -11242,19 +11242,19 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>1478.57</v>
+        <v>1499.09</v>
       </c>
       <c r="V101" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>76.19047619047619</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>2.7</v>
+        <v>2.73</v>
       </c>
       <c r="Y101" s="7" t="n">
         <v>2</v>
@@ -11266,7 +11266,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/07/2026 10:47</t>
+          <t>10/13/2026 10:54</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11420,7 +11420,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>10/08/2026 16:38</t>
+          <t>10/11/2026 16:51</t>
         </is>
       </c>
       <c r="H103" t="n">
@@ -11529,20 +11529,20 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>10/10/2026 00:42</t>
+          <t>10/13/2026 19:09</t>
         </is>
       </c>
       <c r="H104" s="7" t="n">
-        <v>12622.71</v>
+        <v>12684.45</v>
       </c>
       <c r="I104" s="7" t="n">
-        <v>26.17</v>
+        <v>26.79</v>
       </c>
       <c r="J104" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K104" s="7" t="n">
-        <v>2.56</v>
+        <v>2.48</v>
       </c>
       <c r="L104" t="n">
         <v>10000</v>
@@ -11560,19 +11560,19 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="U104" s="7" t="n">
-        <v>2730.54</v>
+        <v>2792.28</v>
       </c>
       <c r="V104" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="W104" s="7" t="n">
-        <v>70.88607594936708</v>
+        <v>71.08433734939759</v>
       </c>
       <c r="X104" s="7" t="n">
-        <v>2.87</v>
+        <v>2.75</v>
       </c>
       <c r="Y104" s="7" t="n">
         <v>2.97</v>
@@ -11584,7 +11584,7 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AB104" t="inlineStr">
@@ -11629,7 +11629,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/09/2026 14:51</t>
+          <t>10/12/2026 14:54</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
@@ -11738,14 +11738,14 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/09/2026 18:37</t>
+          <t>10/13/2026 20:03</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
-        <v>24573.42</v>
+        <v>24684.64</v>
       </c>
       <c r="I106" s="7" t="n">
-        <v>-36.01</v>
+        <v>-35.72</v>
       </c>
       <c r="J106" s="7" t="n">
         <v>42.89</v>
@@ -11763,31 +11763,31 @@
         <v>40</v>
       </c>
       <c r="O106" s="7" t="n">
-        <v>258.5700000000001</v>
+        <v>190.67</v>
       </c>
       <c r="P106" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q106" s="7" t="n">
-        <v>85</v>
+        <v>87.5</v>
       </c>
       <c r="R106" s="7" t="n">
-        <v>2.257391558062634</v>
+        <v>2.217327459618209</v>
       </c>
       <c r="S106" s="7" t="n">
-        <v>0.53</v>
+        <v>0.15</v>
       </c>
       <c r="T106" t="n">
-        <v>3978</v>
+        <v>3996</v>
       </c>
       <c r="U106" s="7" t="n">
-        <v>-9708.580000000002</v>
+        <v>-9597.360000000001</v>
       </c>
       <c r="V106" t="n">
-        <v>2385</v>
+        <v>2405</v>
       </c>
       <c r="W106" s="7" t="n">
-        <v>59.95475113122172</v>
+        <v>60.18518518518518</v>
       </c>
       <c r="X106" s="7" t="n">
         <v>0.76</v>
@@ -11802,7 +11802,7 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB106" t="inlineStr">
@@ -11847,7 +11847,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 13:12</t>
+          <t>10/12/2026 13:14</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 07:03</t>
+          <t>10/12/2026 07:07</t>
         </is>
       </c>
       <c r="H108" s="8" t="n">
@@ -12029,7 +12029,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 15:25</t>
+          <t>10/11/2026 15:34</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12120,7 +12120,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 19:53</t>
+          <t>10/11/2026 20:06</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>10/07/2026 12:20</t>
+          <t>10/13/2026 12:25</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12302,7 +12302,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 21:07</t>
+          <t>10/12/2026 21:10</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>10/06/2026 14:45</t>
+          <t>10/12/2026 14:54</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12484,7 +12484,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>10/07/2026 16:13</t>
+          <t>10/13/2026 16:18</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 08:00</t>
+          <t>10/12/2026 08:03</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12666,7 +12666,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>10/05/2026 08:30</t>
+          <t>10/11/2026 08:35</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 00:22</t>
+          <t>10/12/2026 00:23</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>10/07/2026 14:55</t>
+          <t>10/13/2026 15:02</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12933,7 +12933,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 21:16</t>
+          <t>10/11/2026 21:19</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 19:26</t>
+          <t>10/11/2026 19:50</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13103,7 +13103,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 17:12</t>
+          <t>10/11/2026 17:26</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13188,7 +13188,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 05:38</t>
+          <t>10/11/2026 05:41</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 05:40</t>
+          <t>10/11/2026 05:43</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13358,7 +13358,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 05:40</t>
+          <t>10/11/2026 05:43</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 06:17</t>
+          <t>10/11/2026 06:20</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13528,7 +13528,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 07:56</t>
+          <t>10/11/2026 08:00</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13698,7 +13698,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 10:08</t>
+          <t>10/12/2026 10:12</t>
         </is>
       </c>
       <c r="H128" s="8" t="n">
@@ -13789,7 +13789,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 09:30</t>
+          <t>10/12/2026 09:33</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>10/09/2026 18:15</t>
+          <t>10/12/2026 18:18</t>
         </is>
       </c>
       <c r="H131" s="9" t="n">
@@ -14146,7 +14146,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10/09/2026 13:12</t>
+          <t>10/12/2026 13:14</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14187,7 +14187,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/09/2026 07:03</t>
+          <t>10/12/2026 07:07</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14228,7 +14228,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10/08/2026 15:25</t>
+          <t>10/11/2026 15:34</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14269,7 +14269,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10/08/2026 19:53</t>
+          <t>10/11/2026 20:06</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14310,7 +14310,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10/07/2026 12:20</t>
+          <t>10/13/2026 12:25</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14351,7 +14351,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10/09/2026 21:07</t>
+          <t>10/12/2026 21:10</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14392,7 +14392,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10/06/2026 14:45</t>
+          <t>10/12/2026 14:54</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14433,7 +14433,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10/07/2026 16:13</t>
+          <t>10/13/2026 16:18</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10/09/2026 08:00</t>
+          <t>10/12/2026 08:03</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14515,7 +14515,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10/05/2026 08:30</t>
+          <t>10/11/2026 08:35</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10/09/2026 00:22</t>
+          <t>10/12/2026 00:23</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14597,7 +14597,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>10/07/2026 14:55</t>
+          <t>10/13/2026 15:02</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>10/08/2026 21:16</t>
+          <t>10/11/2026 21:19</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14679,7 +14679,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>10/08/2026 19:26</t>
+          <t>10/11/2026 19:50</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>10/08/2026 17:12</t>
+          <t>10/11/2026 17:26</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14761,7 +14761,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10/08/2026 05:38</t>
+          <t>10/11/2026 05:41</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14802,7 +14802,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10/08/2026 05:40</t>
+          <t>10/11/2026 05:43</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14843,7 +14843,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>10/08/2026 05:40</t>
+          <t>10/11/2026 05:43</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14884,7 +14884,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10/08/2026 06:17</t>
+          <t>10/11/2026 06:20</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14925,7 +14925,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10/08/2026 07:56</t>
+          <t>10/11/2026 08:00</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15007,7 +15007,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>10/09/2026 10:08</t>
+          <t>10/12/2026 10:12</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15048,7 +15048,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10/09/2026 09:30</t>
+          <t>10/12/2026 09:33</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15130,7 +15130,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>10/09/2026 18:15</t>
+          <t>10/12/2026 18:18</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/09/2026 12:23</t>
+          <t>10/12/2026 12:27</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17519,7 +17519,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10/07/2026 16:27</t>
+          <t>10/13/2026 16:32</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10/06/2026 11:58</t>
+          <t>10/12/2026 12:07</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10/09/2026 05:32</t>
+          <t>10/12/2026 05:36</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17588,7 +17588,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10/08/2026 16:47</t>
+          <t>10/11/2026 17:00</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10/07/2026 09:26</t>
+          <t>10/10/2026 09:29</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17634,7 +17634,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10/09/2026 04:29</t>
+          <t>10/12/2026 04:33</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17657,7 +17657,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10/07/2026 09:30</t>
+          <t>10/13/2026 09:35</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -17703,7 +17703,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10/09/2026 13:45</t>
+          <t>10/12/2026 13:50</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10/08/2026 11:08</t>
+          <t>10/11/2026 11:11</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17749,7 +17749,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10/09/2026 11:50</t>
+          <t>10/12/2026 11:55</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17795,7 +17795,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10/08/2026 16:56</t>
+          <t>10/11/2026 17:10</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17818,7 +17818,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10/08/2026 16:47</t>
+          <t>10/11/2026 17:00</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -17841,7 +17841,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10/09/2026 15:47</t>
+          <t>10/12/2026 15:51</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17864,7 +17864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10/09/2026 05:18</t>
+          <t>10/12/2026 05:22</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -17887,7 +17887,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10/09/2026 19:09</t>
+          <t>10/12/2026 19:13</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -17910,7 +17910,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10/09/2026 13:52</t>
+          <t>10/12/2026 13:56</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10/09/2026 15:32</t>
+          <t>10/12/2026 15:36</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10/07/2026 08:18</t>
+          <t>10/13/2026 08:23</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18002,7 +18002,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10/08/2026 06:46</t>
+          <t>10/11/2026 06:50</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18025,7 +18025,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10/08/2026 06:50</t>
+          <t>10/11/2026 06:53</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18048,7 +18048,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10/08/2026 23:42</t>
+          <t>10/11/2026 23:44</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18071,7 +18071,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10/08/2026 23:42</t>
+          <t>10/11/2026 23:44</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18094,7 +18094,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10/08/2026 06:06</t>
+          <t>10/11/2026 06:09</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18117,7 +18117,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10/08/2026 09:33</t>
+          <t>10/11/2026 09:36</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18140,7 +18140,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10/07/2026 09:24</t>
+          <t>10/13/2026 09:30</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18163,7 +18163,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10/07/2026 09:35</t>
+          <t>10/13/2026 09:41</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -18209,7 +18209,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10/09/2026 11:55</t>
+          <t>10/12/2026 11:59</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18232,7 +18232,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10/09/2026 12:53</t>
+          <t>10/12/2026 12:56</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18255,7 +18255,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10/09/2026 18:03</t>
+          <t>10/12/2026 18:06</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18278,7 +18278,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/06/2026 19:17</t>
+          <t>10/13/2026 01:20</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-14
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-13 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-14 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/13/2026 20:27</t>
+          <t>10/14/2026 22:01</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>35164.19</v>
+        <v>28785.11</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>60.75</v>
+        <v>31.58</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-13567.74</v>
+        <v>-14289.32</v>
       </c>
       <c r="P2" t="n">
         <v>29</v>
@@ -994,25 +994,25 @@
         <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.7495737245236033</v>
+        <v>0.7332933160945639</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>106.82</v>
+        <v>88.06999999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>3489</v>
+        <v>3494</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>10164.19</v>
+        <v>3785.110000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.65720836916022</v>
+        <v>63.6519748139668</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/11/2026 15:26</t>
+          <t>10/14/2026 15:31</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/11/2026 18:36</t>
+          <t>10/14/2026 18:46</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/11/2026 09:49</t>
+          <t>10/14/2026 09:51</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/11/2026 17:17</t>
+          <t>10/14/2026 17:28</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/11/2026 18:47</t>
+          <t>10/14/2026 18:57</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/11/2026 17:32</t>
+          <t>10/14/2026 17:42</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/11/2026 19:22</t>
+          <t>10/14/2026 19:32</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/11/2026 18:18</t>
+          <t>10/14/2026 18:28</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/11/2026 18:19</t>
+          <t>10/14/2026 18:29</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/11/2026 18:35</t>
+          <t>10/14/2026 18:45</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/13/2026 20:55</t>
+          <t>10/14/2026 22:30</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>18800.01</v>
-      </c>
-      <c r="I22" t="n">
-        <v>-6</v>
+        <v>18729.76</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>-6.35</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>8.210000000000001</v>
+        <v>8.56</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3165,37 +3165,37 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-689.0500000000001</v>
+        <v>-773.6600000000001</v>
       </c>
       <c r="P22" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>42.5</v>
+        <v>40</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.7369927745057999</v>
+        <v>0.7128914222944639</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>6.96</v>
+        <v>7.32</v>
       </c>
       <c r="T22" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-1199.99</v>
+        <v>-1270.24</v>
       </c>
       <c r="V22" t="n">
         <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>46.78899082568807</v>
+        <v>46.36363636363636</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>8.210000000000001</v>
+        <v>8.56</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/13/2026 22:11</t>
+          <t>10/14/2026 23:47</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19442.14</v>
+        <v>19446.11</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.94</v>
+        <v>-2.92</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.13</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-235.99</v>
+        <v>-206</v>
       </c>
       <c r="P23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>22.5</v>
+        <v>25</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.3172968438105707</v>
+        <v>0.3555451274831847</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>1.31</v>
+        <v>1.18</v>
       </c>
       <c r="T23" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-557.86</v>
+        <v>-553.8900000000001</v>
       </c>
       <c r="V23" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>25.55555555555555</v>
+        <v>26.37362637362638</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.98</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/11/2026 09:26</t>
+          <t>10/14/2026 09:29</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/11/2026 23:46</t>
+          <t>10/14/2026 23:48</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,14 +3576,14 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/13/2026 14:51</t>
+          <t>10/14/2026 22:31</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20252.01</v>
+        <v>20242.28</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-3.18</v>
+        <v>-3.23</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
@@ -3601,31 +3601,31 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-197.47</v>
+        <v>-38.04000000000001</v>
       </c>
       <c r="P26" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>0.8969696653483736</v>
+        <v>0.9794816472936162</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>4.86</v>
+        <v>4.02</v>
       </c>
       <c r="T26" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>252.0099999999999</v>
+        <v>237.1899999999999</v>
       </c>
       <c r="V26" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>42.36111111111111</v>
+        <v>42.75862068965517</v>
       </c>
       <c r="X26" s="7" t="n">
         <v>1.04</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/13/2026 20:54</t>
+          <t>10/14/2026 22:29</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/13/2026 21:18</t>
+          <t>10/14/2026 22:54</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/11/2026 18:47</t>
+          <t>10/14/2026 18:57</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/11/2026 18:54</t>
+          <t>10/14/2026 19:04</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/11/2026 19:59</t>
+          <t>10/14/2026 20:08</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>10/11/2026 17:56</t>
+          <t>10/14/2026 18:07</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/13/2026 23:26</t>
+          <t>10/14/2026 12:24</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20633.14</v>
+        <v>20733.46</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>3.17</v>
+        <v>3.67</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4588,19 +4588,19 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>633.1399999999999</v>
+        <v>733.4599999999998</v>
       </c>
       <c r="V35" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>51.89873417721519</v>
+        <v>52.20125786163522</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>10/11/2026 18:53</t>
+          <t>10/14/2026 19:03</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>10/11/2026 17:37</t>
+          <t>10/14/2026 17:48</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -5333,13 +5333,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5433,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5511,20 +5529,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/13/2026 21:21</t>
+          <t>10/14/2026 22:57</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19633.29</v>
+        <v>19657.64</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.81</v>
+        <v>-1.69</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5533,28 +5551,37 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-75.73999999999999</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.4087431693989071</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>0.51</v>
       </c>
       <c r="T44" t="n">
-        <v>856</v>
+        <v>864</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-366.71</v>
+        <v>-342.36</v>
       </c>
       <c r="V44" t="n">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.0233644859813</v>
+        <v>54.97685185185185</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5566,7 +5593,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/13/2026 20:32</t>
+          <t>10/14/2026 22:07</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5633,13 +5660,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-18.29</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.7507834854884862</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.16</v>
       </c>
       <c r="T45" t="n">
         <v>61</v>
@@ -5711,20 +5747,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/13/2026 20:53</t>
+          <t>10/14/2026 22:28</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19229.81</v>
+        <v>19131.29</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-3.83</v>
+        <v>-4.32</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5742,19 +5778,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-770.1900000000001</v>
+        <v>-868.71</v>
       </c>
       <c r="V46" t="n">
         <v>41</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>42.2680412371134</v>
+        <v>41.83673469387755</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5802,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5833,13 +5869,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5933,13 +5978,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6211,20 +6265,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/13/2026 20:41</t>
+          <t>10/14/2026 22:16</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19781.85</v>
+        <v>19644.06</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-1.06</v>
+        <v>-1.75</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6242,19 +6296,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-218.1500000000001</v>
+        <v>-355.9400000000001</v>
       </c>
       <c r="V51" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>32.43243243243244</v>
+        <v>32.89473684210527</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6266,7 +6320,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,20 +6365,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/13/2026 21:04</t>
+          <t>10/14/2026 22:38</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19108.88</v>
+        <v>19267.22</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-4.42</v>
+        <v>-3.64</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>6.6</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6345,19 +6399,19 @@
         <v>128</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-891.1200000000001</v>
+        <v>-732.7800000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>37.5</v>
+        <v>39.0625</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>6.63</v>
+        <v>6.62</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6366,7 +6420,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,20 +6465,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/13/2026 21:36</t>
+          <t>10/14/2026 10:25</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19640.11</v>
+        <v>19637.15</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.84</v>
+        <v>-1.85</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6442,19 +6496,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-359.8899999999999</v>
+        <v>-372.74</v>
       </c>
       <c r="V53" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.43892339544513</v>
+        <v>36.19631901840491</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6466,7 +6520,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6511,7 +6565,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>10/11/2026 21:49</t>
+          <t>10/14/2026 21:51</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6611,7 +6665,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10/11/2026 19:03</t>
+          <t>10/14/2026 19:13</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6811,17 +6865,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/13/2026 20:50</t>
+          <t>10/14/2026 22:24</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19496.12</v>
+        <v>19488.43</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.53</v>
+        <v>-2.56</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
       <c r="K57" s="7" t="n">
         <v>0.74</v>
@@ -6842,22 +6896,22 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1243</v>
+        <v>1262</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-503.63</v>
+        <v>-511.48</v>
       </c>
       <c r="V57" t="n">
-        <v>535</v>
+        <v>544</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.04102976669348</v>
+        <v>43.10618066561015</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.74</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>2.55</v>
+        <v>2.56</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6866,7 +6920,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +6965,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/13/2026 21:12</t>
+          <t>10/14/2026 22:47</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7111,7 +7165,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/13/2026 21:06</t>
+          <t>10/14/2026 22:42</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7211,7 +7265,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/13/2026 21:53</t>
+          <t>10/14/2026 23:28</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7233,13 +7287,22 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>0</v>
+        <v>-448.41</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q61" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R61" s="7" t="n">
+        <v>0.480495858193825</v>
+      </c>
+      <c r="S61" s="7" t="n">
+        <v>3.68</v>
       </c>
       <c r="T61" t="n">
         <v>3982</v>
@@ -7311,7 +7374,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>10/11/2026 21:39</t>
+          <t>10/14/2026 21:40</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7411,20 +7474,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/13/2026 21:31</t>
+          <t>10/14/2026 23:06</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18361.24</v>
+        <v>18332.37</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-8.210000000000001</v>
+        <v>-8.35</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>8.210000000000001</v>
+        <v>8.35</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7442,22 +7505,22 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1638.76</v>
+        <v>-1667.63</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.76923076923077</v>
+        <v>10.60606060606061</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>8.19</v>
+        <v>8.34</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7466,7 +7529,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7511,7 +7574,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>10/11/2026 19:11</t>
+          <t>10/14/2026 19:22</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7611,7 +7674,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/13/2026 21:27</t>
+          <t>10/14/2026 23:02</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7621,7 +7684,7 @@
         <v>-7.9</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>12.41</v>
+        <v>13.65</v>
       </c>
       <c r="K65" s="7" t="n">
         <v>0.89</v>
@@ -7711,7 +7774,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>10/11/2026 19:00</t>
+          <t>10/14/2026 19:10</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7811,20 +7874,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/13/2026 21:49</t>
+          <t>10/14/2026 23:25</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20579.38</v>
+        <v>20398.62</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>2.95</v>
+        <v>2.04</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7842,19 +7905,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>579.3799999999992</v>
+        <v>398.6199999999992</v>
       </c>
       <c r="V67" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>32</v>
+        <v>32.35294117647059</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7866,7 +7929,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8011,7 +8074,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>10/11/2026 17:26</t>
+          <t>10/14/2026 17:36</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8033,13 +8096,22 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>0</v>
+        <v>-35.83</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q69" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R69" s="7" t="n">
+        <v>0.5722812462695476</v>
+      </c>
+      <c r="S69" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T69" t="n">
         <v>55</v>
@@ -8111,7 +8183,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>10/11/2026 17:26</t>
+          <t>10/14/2026 17:37</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8211,7 +8283,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>10/11/2026 17:26</t>
+          <t>10/14/2026 17:36</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8311,7 +8383,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>10/11/2026 19:05</t>
+          <t>10/14/2026 19:15</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8411,7 +8483,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>10/11/2026 19:28</t>
+          <t>10/14/2026 19:38</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8511,7 +8583,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>10/11/2026 19:01</t>
+          <t>10/14/2026 19:12</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8611,7 +8683,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>10/11/2026 21:01</t>
+          <t>10/14/2026 21:02</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8711,7 +8783,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>10/11/2026 20:27</t>
+          <t>10/14/2026 20:35</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8811,7 +8883,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>10/11/2026 20:38</t>
+          <t>10/14/2026 20:41</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8911,7 +8983,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>10/11/2026 20:36</t>
+          <t>10/14/2026 20:40</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9011,7 +9083,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>10/11/2026 20:41</t>
+          <t>10/14/2026 20:45</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9111,7 +9183,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>10/11/2026 20:36</t>
+          <t>10/14/2026 20:40</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9211,7 +9283,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>10/08/2026 20:20</t>
+          <t>10/14/2026 20:36</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9311,7 +9383,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>10/11/2026 20:54</t>
+          <t>10/14/2026 20:57</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9333,13 +9405,22 @@
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>0</v>
+        <v>-308.22</v>
       </c>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q82" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R82" s="7" t="n">
+        <v>0.412903102916246</v>
+      </c>
+      <c r="S82" s="7" t="n">
+        <v>1.62</v>
       </c>
       <c r="T82" t="n">
         <v>1156</v>
@@ -9711,7 +9792,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>10/11/2026 20:39</t>
+          <t>10/14/2026 20:42</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9811,7 +9892,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/13/2026 22:39</t>
+          <t>10/14/2026 11:35</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9842,16 +9923,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-103.9399999999999</v>
+        <v>-110.2699999999999</v>
       </c>
       <c r="V87" t="n">
         <v>85</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>43.14720812182741</v>
+        <v>42.71356783919598</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>0.96</v>
@@ -9866,7 +9947,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10011,20 +10092,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/13/2026 22:17</t>
+          <t>10/14/2026 23:52</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>19929.86</v>
+        <v>19858.4</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>-0.35</v>
+        <v>-0.7</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>3.94</v>
+        <v>4.25</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10042,22 +10123,22 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>-70.14000000000004</v>
+        <v>-141.6</v>
       </c>
       <c r="V89" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>82.82208588957054</v>
+        <v>82.53012048192771</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="Y89" s="7" t="n">
-        <v>3.96</v>
+        <v>4.27</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10066,7 +10147,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10111,20 +10192,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/13/2026 22:11</t>
+          <t>10/14/2026 23:47</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27786.09</v>
+        <v>27221.69</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>38.99</v>
+        <v>36.17</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>4.12</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.74</v>
+        <v>1.65</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,19 +10223,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7786.09</v>
+        <v>7221.690000000001</v>
       </c>
       <c r="V90" t="n">
         <v>121</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>68.36158192090396</v>
+        <v>67.22222222222223</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.74</v>
+        <v>1.65</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>4.12</v>
@@ -10166,7 +10247,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10211,7 +10292,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>10/11/2026 20:24</t>
+          <t>10/14/2026 20:33</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10311,7 +10392,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>10/11/2026 04:36</t>
+          <t>10/14/2026 04:39</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10411,7 +10492,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>10/11/2026 19:29</t>
+          <t>10/14/2026 19:38</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10511,7 +10592,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>10/11/2026 19:26</t>
+          <t>10/14/2026 19:36</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10611,7 +10692,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>10/11/2026 19:24</t>
+          <t>10/14/2026 19:34</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10711,7 +10792,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>10/12/2026 00:04</t>
+          <t>10/15/2026 00:06</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10733,13 +10814,22 @@
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>0</v>
+        <v>-225.16</v>
       </c>
       <c r="P96" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q96" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R96" s="7" t="n">
+        <v>0.1289411582653101</v>
+      </c>
+      <c r="S96" s="7" t="n">
+        <v>0.23</v>
       </c>
       <c r="T96" t="n">
         <v>393</v>
@@ -10811,7 +10901,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>10/08/2026 20:14</t>
+          <t>10/14/2026 20:33</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10911,7 +11001,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>10/11/2026 20:25</t>
+          <t>10/14/2026 20:33</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11111,7 +11201,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>10/11/2026 05:01</t>
+          <t>10/14/2026 05:03</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11211,7 +11301,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/13/2026 23:10</t>
+          <t>10/14/2026 12:08</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11420,7 +11510,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>10/11/2026 16:51</t>
+          <t>10/14/2026 17:00</t>
         </is>
       </c>
       <c r="H103" t="n">
@@ -11529,20 +11619,20 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>10/13/2026 19:09</t>
+          <t>10/14/2026 14:33</t>
         </is>
       </c>
       <c r="H104" s="7" t="n">
-        <v>12684.45</v>
+        <v>12555.51</v>
       </c>
       <c r="I104" s="7" t="n">
-        <v>26.79</v>
+        <v>25.5</v>
       </c>
       <c r="J104" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K104" s="7" t="n">
-        <v>2.48</v>
+        <v>2.32</v>
       </c>
       <c r="L104" t="n">
         <v>10000</v>
@@ -11560,19 +11650,19 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="U104" s="7" t="n">
-        <v>2792.28</v>
+        <v>2663.34</v>
       </c>
       <c r="V104" t="n">
         <v>59</v>
       </c>
       <c r="W104" s="7" t="n">
-        <v>71.08433734939759</v>
+        <v>70.23809523809523</v>
       </c>
       <c r="X104" s="7" t="n">
-        <v>2.75</v>
+        <v>2.55</v>
       </c>
       <c r="Y104" s="7" t="n">
         <v>2.97</v>
@@ -11584,7 +11674,7 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="AB104" t="inlineStr">
@@ -11738,20 +11828,20 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/13/2026 20:03</t>
+          <t>10/14/2026 21:36</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
-        <v>24684.64</v>
+        <v>24236.45</v>
       </c>
       <c r="I106" s="7" t="n">
-        <v>-35.72</v>
+        <v>-36.88</v>
       </c>
       <c r="J106" s="7" t="n">
         <v>42.89</v>
       </c>
       <c r="K106" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="L106" t="n">
         <v>25000</v>
@@ -11763,34 +11853,34 @@
         <v>40</v>
       </c>
       <c r="O106" s="7" t="n">
-        <v>190.67</v>
+        <v>-533.48</v>
       </c>
       <c r="P106" t="n">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="Q106" s="7" t="n">
-        <v>87.5</v>
+        <v>60</v>
       </c>
       <c r="R106" s="7" t="n">
-        <v>2.217327459618209</v>
+        <v>0.2862379920259024</v>
       </c>
       <c r="S106" s="7" t="n">
-        <v>0.15</v>
+        <v>2.5</v>
       </c>
       <c r="T106" t="n">
-        <v>3996</v>
+        <v>4013</v>
       </c>
       <c r="U106" s="7" t="n">
-        <v>-9597.360000000001</v>
+        <v>-10045.55</v>
       </c>
       <c r="V106" t="n">
-        <v>2405</v>
+        <v>2428</v>
       </c>
       <c r="W106" s="7" t="n">
-        <v>60.18518518518518</v>
+        <v>60.50336406678296</v>
       </c>
       <c r="X106" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="Y106" s="7" t="n">
         <v>45.99</v>
@@ -11802,7 +11892,7 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB106" t="inlineStr">
@@ -12029,7 +12119,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 15:34</t>
+          <t>10/14/2026 15:40</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12120,7 +12210,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 20:06</t>
+          <t>10/14/2026 20:15</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12666,7 +12756,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 08:35</t>
+          <t>10/14/2026 08:37</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12870,17 +12960,23 @@
         <v>0</v>
       </c>
       <c r="N118" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O118" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P118" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q118" s="8" t="n"/>
-      <c r="R118" s="8" t="n"/>
-      <c r="S118" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q118" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R118" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S118" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T118" s="8" t="n">
         <v>0</v>
       </c>
@@ -12933,7 +13029,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 21:19</t>
+          <t>10/14/2026 21:22</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12955,17 +13051,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13018,7 +13120,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 19:50</t>
+          <t>10/14/2026 19:59</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13040,17 +13142,23 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q120" s="8" t="n"/>
-      <c r="R120" s="8" t="n"/>
-      <c r="S120" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q120" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R120" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S120" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13103,7 +13211,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 17:26</t>
+          <t>10/14/2026 17:37</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13188,7 +13296,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 05:41</t>
+          <t>10/14/2026 05:44</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13273,7 +13381,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 05:43</t>
+          <t>10/14/2026 05:47</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13358,7 +13466,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 05:43</t>
+          <t>10/14/2026 05:47</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13443,7 +13551,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 06:20</t>
+          <t>10/14/2026 06:23</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13465,17 +13573,23 @@
         <v>0</v>
       </c>
       <c r="N125" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O125" s="9" t="n">
-        <v>0</v>
+        <v>-3715.63</v>
       </c>
       <c r="P125" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q125" s="8" t="n"/>
-      <c r="R125" s="8" t="n"/>
-      <c r="S125" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q125" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R125" s="9" t="n">
+        <v>0.2438039067238144</v>
+      </c>
+      <c r="S125" s="9" t="n">
+        <v>3.72</v>
+      </c>
       <c r="T125" s="8" t="n">
         <v>0</v>
       </c>
@@ -13528,7 +13642,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>10/11/2026 08:00</t>
+          <t>10/14/2026 08:03</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13613,7 +13727,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>10/08/2026 05:29</t>
+          <t>10/14/2026 05:35</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -14228,7 +14342,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10/11/2026 15:34</t>
+          <t>10/14/2026 15:40</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14269,7 +14383,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10/11/2026 20:06</t>
+          <t>10/14/2026 20:15</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14515,7 +14629,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10/11/2026 08:35</t>
+          <t>10/14/2026 08:37</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14607,7 +14721,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14638,7 +14752,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>10/11/2026 21:19</t>
+          <t>10/14/2026 21:22</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14648,7 +14762,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -14679,7 +14793,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>10/11/2026 19:50</t>
+          <t>10/14/2026 19:59</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14689,7 +14803,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14720,7 +14834,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>10/11/2026 17:26</t>
+          <t>10/14/2026 17:37</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14761,7 +14875,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10/11/2026 05:41</t>
+          <t>10/14/2026 05:44</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14802,7 +14916,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10/11/2026 05:43</t>
+          <t>10/14/2026 05:47</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14843,7 +14957,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>10/11/2026 05:43</t>
+          <t>10/14/2026 05:47</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14884,7 +14998,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10/11/2026 06:20</t>
+          <t>10/14/2026 06:23</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14894,7 +15008,7 @@
         <v>-6.66</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -14925,7 +15039,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10/11/2026 08:00</t>
+          <t>10/14/2026 08:03</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14966,7 +15080,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>10/08/2026 05:29</t>
+          <t>10/14/2026 05:35</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -17588,7 +17702,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10/11/2026 17:00</t>
+          <t>10/14/2026 17:10</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -17680,7 +17794,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10/08/2026 02:30</t>
+          <t>10/14/2026 02:37</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -17726,7 +17840,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10/11/2026 11:11</t>
+          <t>10/14/2026 11:13</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -17795,7 +17909,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10/11/2026 17:10</t>
+          <t>10/14/2026 17:20</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -17818,7 +17932,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10/11/2026 17:00</t>
+          <t>10/14/2026 17:10</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -18002,7 +18116,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10/11/2026 06:50</t>
+          <t>10/14/2026 06:52</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18025,7 +18139,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10/11/2026 06:53</t>
+          <t>10/14/2026 06:55</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18048,7 +18162,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10/11/2026 23:44</t>
+          <t>10/14/2026 23:45</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18071,7 +18185,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10/11/2026 23:44</t>
+          <t>10/14/2026 23:45</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18094,7 +18208,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10/11/2026 06:09</t>
+          <t>10/14/2026 06:13</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18117,7 +18231,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10/11/2026 09:36</t>
+          <t>10/14/2026 09:40</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18278,7 +18392,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/13/2026 01:20</t>
+          <t>10/14/2026 01:22</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-15
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-14 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-15 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/14/2026 22:01</t>
+          <t>10/15/2026 13:41</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>28785.11</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>31.58</v>
+        <v>31939.44</v>
+      </c>
+      <c r="I2" t="n">
+        <v>46</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-14289.32</v>
+        <v>-11722.96</v>
       </c>
       <c r="P2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>72.5</v>
+        <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.7332933160945639</v>
+        <v>0.7762981307482064</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>88.06999999999999</v>
+        <v>89.45</v>
       </c>
       <c r="T2" t="n">
-        <v>3494</v>
+        <v>3496</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>3785.110000000002</v>
+        <v>6939.440000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>2224</v>
+        <v>2226</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.6519748139668</v>
+        <v>63.67276887871854</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.01</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/12/2026 14:55</t>
+          <t>10/15/2026 14:58</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/12/2026 17:31</t>
+          <t>10/15/2026 17:33</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/12/2026 17:33</t>
+          <t>10/15/2026 17:37</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/12/2026 08:38</t>
+          <t>10/15/2026 08:41</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/14/2026 22:30</t>
+          <t>10/15/2026 14:27</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3180,7 +3180,7 @@
         <v>7.32</v>
       </c>
       <c r="T22" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="U22" s="7" t="n">
         <v>-1270.24</v>
@@ -3189,7 +3189,7 @@
         <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>46.36363636363636</v>
+        <v>45.53571428571428</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.8</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/14/2026 23:47</t>
+          <t>10/15/2026 16:23</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19446.11</v>
+        <v>19450.32</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.92</v>
+        <v>-2.9</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.13</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-206</v>
+        <v>-171.79</v>
       </c>
       <c r="P23" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.3555451274831847</v>
+        <v>0.4006768071448507</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>1.18</v>
+        <v>1.07</v>
       </c>
       <c r="T23" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-553.8900000000001</v>
+        <v>-530.6</v>
       </c>
       <c r="V23" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>26.37362637362638</v>
+        <v>28.8659793814433</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.36</v>
+        <v>0.39</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.98</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/14/2026 22:31</t>
+          <t>10/15/2026 14:27</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20242.28</v>
+        <v>20370.36</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-3.23</v>
+        <v>-2.62</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-38.04000000000001</v>
+        <v>319.37</v>
       </c>
       <c r="P26" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>40</v>
+        <v>42.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>0.9794816472936162</v>
+        <v>1.196317924760266</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>4.02</v>
+        <v>2.86</v>
       </c>
       <c r="T26" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>237.1899999999999</v>
+        <v>370.3599999999999</v>
       </c>
       <c r="V26" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>42.75862068965517</v>
+        <v>43.24324324324324</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.04</v>
+        <v>1.06</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/12/2026 13:50</t>
+          <t>10/15/2026 13:53</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/14/2026 22:29</t>
+          <t>10/15/2026 14:28</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/14/2026 22:54</t>
+          <t>10/15/2026 15:06</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20649.89</v>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>3.28</v>
+        <v>20592.99</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.68</v>
+        <v>1.59</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,7 +4037,7 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>36.84</v>
+        <v>-17.43</v>
       </c>
       <c r="P30" t="n">
         <v>13</v>
@@ -4046,25 +4046,25 @@
         <v>32.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>1.191009488256338</v>
+        <v>0.929473173100267</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="T30" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>649.8899999999999</v>
+        <v>592.9899999999998</v>
       </c>
       <c r="V30" t="n">
         <v>32</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>28.31858407079646</v>
+        <v>27.82608695652174</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.68</v>
+        <v>1.59</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/14/2026 12:24</t>
+          <t>10/15/2026 18:12</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20733.46</v>
+        <v>20634.7</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>3.67</v>
+        <v>3.18</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4591,7 +4591,7 @@
         <v>159</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>733.4599999999998</v>
+        <v>634.6999999999998</v>
       </c>
       <c r="V35" t="n">
         <v>83</v>
@@ -4600,7 +4600,7 @@
         <v>52.20125786163522</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10/12/2026 00:51</t>
+          <t>10/15/2026 00:55</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>10/12/2026 01:11</t>
+          <t>10/15/2026 01:15</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5333,22 +5333,13 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q42" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R42" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S42" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5420,7 +5411,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>10/12/2026 03:30</t>
+          <t>10/15/2026 03:33</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,22 +5433,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5529,14 +5511,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/14/2026 22:57</t>
+          <t>10/15/2026 15:09</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19657.64</v>
+        <v>19662.88</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.69</v>
+        <v>-1.66</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5551,34 +5533,25 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-75.73999999999999</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.4087431693989071</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>864</v>
+        <v>872</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-342.36</v>
+        <v>-314.52</v>
       </c>
       <c r="V44" t="n">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>54.97685185185185</v>
+        <v>55.04587155963303</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -5593,7 +5566,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5638,7 +5611,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/14/2026 22:07</t>
+          <t>10/15/2026 13:52</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5660,22 +5633,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-18.29</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.7507834854884862</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>61</v>
@@ -5747,20 +5711,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/14/2026 22:28</t>
+          <t>10/15/2026 14:23</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19131.29</v>
+        <v>19033.57</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-4.32</v>
+        <v>-4.81</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5778,19 +5742,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-868.71</v>
+        <v>-974.4400000000001</v>
       </c>
       <c r="V46" t="n">
         <v>41</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>41.83673469387755</v>
+        <v>41</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5802,7 +5766,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5847,7 +5811,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>10/12/2026 00:11</t>
+          <t>10/15/2026 00:14</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5869,22 +5833,13 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>504.68</v>
+        <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q47" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R47" s="7" t="n">
-        <v>2.47982641332395</v>
-      </c>
-      <c r="S47" s="7" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5956,7 +5911,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>10/12/2026 21:01</t>
+          <t>10/15/2026 21:04</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5978,22 +5933,13 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>698.46</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q48" s="7" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="R48" s="7" t="n">
-        <v>7.636199524940618</v>
-      </c>
-      <c r="S48" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6065,7 +6011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>10/12/2026 01:03</t>
+          <t>10/15/2026 01:07</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6165,7 +6111,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>10/12/2026 00:38</t>
+          <t>10/15/2026 00:42</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6265,7 +6211,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/14/2026 22:16</t>
+          <t>10/15/2026 14:05</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6365,7 +6311,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/14/2026 22:38</t>
+          <t>10/15/2026 14:40</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6396,16 +6342,16 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-732.7800000000002</v>
+        <v>-733.4600000000003</v>
       </c>
       <c r="V52" t="n">
         <v>50</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>39.0625</v>
+        <v>38.46153846153847</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.88</v>
@@ -6420,7 +6366,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6465,20 +6411,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/14/2026 10:25</t>
+          <t>10/15/2026 15:30</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19637.15</v>
+        <v>19594.73</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.85</v>
+        <v>-2.06</v>
       </c>
       <c r="J53" s="7" t="n">
-        <v>1.9</v>
+        <v>2.06</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6496,22 +6442,22 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-372.74</v>
+        <v>-405.27</v>
       </c>
       <c r="V53" t="n">
         <v>177</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.19631901840491</v>
+        <v>35.75757575757576</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="Y53" s="7" t="n">
-        <v>1.89</v>
+        <v>2.03</v>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
@@ -6520,7 +6466,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6865,20 +6811,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/14/2026 22:24</t>
+          <t>10/15/2026 14:20</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19488.43</v>
+        <v>19466.18</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.56</v>
+        <v>-2.67</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>2.56</v>
+        <v>2.72</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6896,22 +6842,22 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1262</v>
+        <v>1291</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-511.48</v>
+        <v>-535.46</v>
       </c>
       <c r="V57" t="n">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.10618066561015</v>
+        <v>43.14484895429899</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>2.56</v>
+        <v>2.71</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -6965,7 +6911,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/14/2026 22:47</t>
+          <t>10/15/2026 14:53</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7165,7 +7111,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/14/2026 22:42</t>
+          <t>10/15/2026 14:46</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7265,7 +7211,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/14/2026 23:28</t>
+          <t>10/15/2026 15:56</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7287,22 +7233,13 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>-448.41</v>
+        <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q61" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R61" s="7" t="n">
-        <v>0.480495858193825</v>
-      </c>
-      <c r="S61" s="7" t="n">
-        <v>3.68</v>
+        <v>0</v>
       </c>
       <c r="T61" t="n">
         <v>3982</v>
@@ -7474,17 +7411,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/14/2026 23:06</t>
+          <t>10/15/2026 15:22</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18332.37</v>
+        <v>18288.49</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-8.35</v>
+        <v>-8.57</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>8.35</v>
+        <v>8.57</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>0.42</v>
@@ -7496,31 +7433,40 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>0</v>
+        <v>-784.0600000000001</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Q63" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="R63" s="7" t="n">
+        <v>0.44620709139709</v>
+      </c>
+      <c r="S63" s="7" t="n">
+        <v>3.92</v>
       </c>
       <c r="T63" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1667.63</v>
+        <v>-1711.51</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.60606060606061</v>
+        <v>10.44776119402985</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.42</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>8.34</v>
+        <v>8.56</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7529,7 +7475,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7674,7 +7620,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/14/2026 23:02</t>
+          <t>10/15/2026 15:16</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7874,11 +7820,11 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/14/2026 23:25</t>
+          <t>10/15/2026 15:54</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20398.62</v>
+        <v>20398.18</v>
       </c>
       <c r="I67" s="7" t="n">
         <v>2.04</v>
@@ -7905,16 +7851,16 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>398.6199999999992</v>
+        <v>398.1799999999992</v>
       </c>
       <c r="V67" t="n">
         <v>33</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>32.35294117647059</v>
+        <v>32.03883495145632</v>
       </c>
       <c r="X67" s="7" t="n">
         <v>1.04</v>
@@ -7929,7 +7875,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8096,22 +8042,13 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>-35.83</v>
+        <v>0</v>
       </c>
       <c r="P69" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q69" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R69" s="7" t="n">
-        <v>0.5722812462695476</v>
-      </c>
-      <c r="S69" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="T69" t="n">
         <v>55</v>
@@ -9405,22 +9342,13 @@
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>-308.22</v>
+        <v>0</v>
       </c>
       <c r="P82" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q82" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R82" s="7" t="n">
-        <v>0.412903102916246</v>
-      </c>
-      <c r="S82" s="7" t="n">
-        <v>1.62</v>
+        <v>0</v>
       </c>
       <c r="T82" t="n">
         <v>1156</v>
@@ -9692,7 +9620,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>10/12/2026 02:15</t>
+          <t>10/15/2026 02:16</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9892,14 +9820,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/14/2026 11:35</t>
+          <t>10/15/2026 17:07</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19896.06</v>
+        <v>19887.17</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.54</v>
+        <v>-0.58</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>5.56</v>
@@ -9923,16 +9851,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-110.2699999999999</v>
+        <v>-112.8299999999998</v>
       </c>
       <c r="V87" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>42.71356783919598</v>
+        <v>42.78606965174129</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>0.96</v>
@@ -9947,7 +9875,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10092,20 +10020,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/14/2026 23:52</t>
+          <t>10/15/2026 16:31</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>19858.4</v>
+        <v>19875.23</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>-0.7</v>
+        <v>-0.62</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>4.25</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10123,19 +10051,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>-141.6</v>
+        <v>-111.6000000000001</v>
       </c>
       <c r="V89" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>82.53012048192771</v>
+        <v>82.24852071005917</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>4.27</v>
@@ -10147,7 +10075,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10192,20 +10120,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/14/2026 23:47</t>
+          <t>10/15/2026 16:23</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>27221.69</v>
+        <v>26806.23</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>36.17</v>
+        <v>34.09</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>4.12</v>
+        <v>4.18</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.65</v>
+        <v>1.59</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10223,22 +10151,22 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>7221.690000000001</v>
+        <v>6810.01</v>
       </c>
       <c r="V90" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>67.22222222222223</v>
+        <v>66.84782608695652</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.65</v>
+        <v>1.59</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>4.12</v>
+        <v>4.19</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10247,7 +10175,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10814,22 +10742,13 @@
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>-225.16</v>
+        <v>0</v>
       </c>
       <c r="P96" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q96" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R96" s="7" t="n">
-        <v>0.1289411582653101</v>
-      </c>
-      <c r="S96" s="7" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="T96" t="n">
         <v>393</v>
@@ -11101,7 +11020,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>10/12/2026 00:11</t>
+          <t>10/15/2026 00:14</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11301,7 +11220,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/14/2026 12:08</t>
+          <t>10/15/2026 17:50</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11619,20 +11538,20 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>10/14/2026 14:33</t>
+          <t>10/15/2026 20:51</t>
         </is>
       </c>
       <c r="H104" s="7" t="n">
-        <v>12555.51</v>
+        <v>12556.74</v>
       </c>
       <c r="I104" s="7" t="n">
-        <v>25.5</v>
+        <v>25.51</v>
       </c>
       <c r="J104" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K104" s="7" t="n">
-        <v>2.32</v>
+        <v>2.24</v>
       </c>
       <c r="L104" t="n">
         <v>10000</v>
@@ -11650,19 +11569,19 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="U104" s="7" t="n">
-        <v>2663.34</v>
+        <v>2787.57</v>
       </c>
       <c r="V104" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="W104" s="7" t="n">
-        <v>70.23809523809523</v>
+        <v>70.11494252873564</v>
       </c>
       <c r="X104" s="7" t="n">
-        <v>2.55</v>
+        <v>2.62</v>
       </c>
       <c r="Y104" s="7" t="n">
         <v>2.97</v>
@@ -11674,7 +11593,7 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="AB104" t="inlineStr">
@@ -11719,7 +11638,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/12/2026 14:54</t>
+          <t>10/15/2026 14:58</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
@@ -11828,14 +11747,14 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/14/2026 21:36</t>
+          <t>10/15/2026 13:04</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
-        <v>24236.45</v>
+        <v>24240.53</v>
       </c>
       <c r="I106" s="7" t="n">
-        <v>-36.88</v>
+        <v>-36.87</v>
       </c>
       <c r="J106" s="7" t="n">
         <v>42.89</v>
@@ -11853,37 +11772,37 @@
         <v>40</v>
       </c>
       <c r="O106" s="7" t="n">
-        <v>-533.48</v>
+        <v>-460.85</v>
       </c>
       <c r="P106" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q106" s="7" t="n">
-        <v>60</v>
+        <v>62.5</v>
       </c>
       <c r="R106" s="7" t="n">
-        <v>0.2862379920259024</v>
+        <v>0.3397942811300212</v>
       </c>
       <c r="S106" s="7" t="n">
         <v>2.5</v>
       </c>
       <c r="T106" t="n">
-        <v>4013</v>
+        <v>4025</v>
       </c>
       <c r="U106" s="7" t="n">
-        <v>-10045.55</v>
+        <v>-10157.35</v>
       </c>
       <c r="V106" t="n">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="W106" s="7" t="n">
-        <v>60.50336406678296</v>
+        <v>60.3975155279503</v>
       </c>
       <c r="X106" s="7" t="n">
         <v>0.75</v>
       </c>
       <c r="Y106" s="7" t="n">
-        <v>45.99</v>
+        <v>46.04</v>
       </c>
       <c r="Z106" t="inlineStr">
         <is>
@@ -11892,7 +11811,7 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB106" t="inlineStr">
@@ -11937,7 +11856,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 13:14</t>
+          <t>10/15/2026 13:18</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -12028,7 +11947,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 07:07</t>
+          <t>10/15/2026 07:11</t>
         </is>
       </c>
       <c r="H108" s="8" t="n">
@@ -12392,7 +12311,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 21:10</t>
+          <t>10/15/2026 21:13</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12483,7 +12402,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 14:54</t>
+          <t>10/15/2026 14:58</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12665,7 +12584,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 08:03</t>
+          <t>10/15/2026 08:07</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12847,7 +12766,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 00:23</t>
+          <t>10/15/2026 00:27</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12960,23 +12879,17 @@
         <v>0</v>
       </c>
       <c r="N118" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O118" s="9" t="n">
-        <v>67.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="P118" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q118" s="9" t="n">
-        <v>65</v>
-      </c>
-      <c r="R118" s="9" t="n">
-        <v>1.223174978645115</v>
-      </c>
-      <c r="S118" s="9" t="n">
-        <v>0.57</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q118" s="8" t="n"/>
+      <c r="R118" s="8" t="n"/>
+      <c r="S118" s="8" t="n"/>
       <c r="T118" s="8" t="n">
         <v>0</v>
       </c>
@@ -13051,23 +12964,17 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>-6156.77</v>
+        <v>0</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q119" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="R119" s="9" t="n">
-        <v>0.01160528233794505</v>
-      </c>
-      <c r="S119" s="9" t="n">
-        <v>31.03</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q119" s="8" t="n"/>
+      <c r="R119" s="8" t="n"/>
+      <c r="S119" s="8" t="n"/>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13573,23 +13480,17 @@
         <v>0</v>
       </c>
       <c r="N125" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O125" s="9" t="n">
-        <v>-3715.63</v>
+        <v>0</v>
       </c>
       <c r="P125" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q125" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R125" s="9" t="n">
-        <v>0.2438039067238144</v>
-      </c>
-      <c r="S125" s="9" t="n">
-        <v>3.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q125" s="8" t="n"/>
+      <c r="R125" s="8" t="n"/>
+      <c r="S125" s="8" t="n"/>
       <c r="T125" s="8" t="n">
         <v>0</v>
       </c>
@@ -13812,7 +13713,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 10:12</t>
+          <t>10/15/2026 10:16</t>
         </is>
       </c>
       <c r="H128" s="8" t="n">
@@ -13903,7 +13804,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 09:33</t>
+          <t>10/15/2026 09:37</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -14085,7 +13986,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>10/12/2026 18:18</t>
+          <t>10/15/2026 18:20</t>
         </is>
       </c>
       <c r="H131" s="9" t="n">
@@ -14260,7 +14161,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10/12/2026 13:14</t>
+          <t>10/15/2026 13:18</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14301,7 +14202,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/12/2026 07:07</t>
+          <t>10/15/2026 07:11</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14465,7 +14366,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10/12/2026 21:10</t>
+          <t>10/15/2026 21:13</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14506,7 +14407,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10/12/2026 14:54</t>
+          <t>10/15/2026 14:58</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14588,7 +14489,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10/12/2026 08:03</t>
+          <t>10/15/2026 08:07</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14670,7 +14571,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10/12/2026 00:23</t>
+          <t>10/15/2026 00:27</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14721,7 +14622,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -14762,7 +14663,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -15008,7 +14909,7 @@
         <v>-6.66</v>
       </c>
       <c r="I23" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -15121,7 +15022,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>10/12/2026 10:12</t>
+          <t>10/15/2026 10:16</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15162,7 +15063,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10/12/2026 09:33</t>
+          <t>10/15/2026 09:37</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15244,7 +15145,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>10/12/2026 18:18</t>
+          <t>10/15/2026 18:20</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -15268,7 +15169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -17216,7 +17117,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>58992</t>
+          <t>58980</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -17226,7 +17127,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Golden Fractal</t>
+          <t>Tokio Trigger</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -17234,14 +17135,14 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>58993</t>
+          <t>58981</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -17251,7 +17152,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Levels</t>
+          <t>LinLit EURAUD</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -17259,24 +17160,24 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>59376</t>
+          <t>58982</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LIVE XAUUSD: YuHeng Gift EA + fundedtoday copy feed</t>
+          <t>Session RSI Scalper EURUSD</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -17284,49 +17185,49 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>VPS153t2</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>59377</t>
+          <t>58984</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>UNFUNDED, never traded (earmarked Gold Snap 2HR)</t>
+          <t>Best Forex 15TF EURUSD</t>
         </is>
       </c>
       <c r="D83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>58985</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>Channel Scalper EURUSD</t>
         </is>
       </c>
       <c r="D84" t="b">
@@ -17334,49 +17235,49 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>58986</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>AiriumBot EURUSD H1</t>
         </is>
       </c>
       <c r="D85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>662436</t>
+          <t>58987</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+          <t>Forex Diamond EURUSD M1</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -17384,24 +17285,24 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>663097</t>
+          <t>58988</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+          <t>Long Haul</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -17409,14 +17310,14 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>1115442</t>
+          <t>58989</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -17426,7 +17327,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Gold Snap Internal</t>
+          <t>TSma4f AUDCAD</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -17434,14 +17335,14 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1115443</t>
+          <t>58992</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -17451,22 +17352,22 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta MOL</t>
+          <t>Golden Fractal</t>
         </is>
       </c>
       <c r="D89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1115444</t>
+          <t>58993</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -17476,7 +17377,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Gold Snap Demo</t>
+          <t>Levels</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -17484,55 +17385,280 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>14189968</t>
+          <t>59376</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+          <t>LIVE XAUUSD: YuHeng Gift EA + fundedtoday copy feed</t>
         </is>
       </c>
       <c r="D91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153t2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>59377</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>UNFUNDED, never traded (earmarked Gold Snap 2HR)</t>
+        </is>
+      </c>
+      <c r="D92" t="b">
+        <v>0</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>662434</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>LIVE Gold Reaper Conservative</t>
+        </is>
+      </c>
+      <c r="D93" t="b">
+        <v>1</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>662435</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Aggv1 Pro Filter 60</t>
+        </is>
+      </c>
+      <c r="D94" t="b">
+        <v>0</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>662436</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+        </is>
+      </c>
+      <c r="D95" t="b">
+        <v>1</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>663097</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+        </is>
+      </c>
+      <c r="D96" t="b">
+        <v>1</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1115442</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Gold Snap Internal</t>
+        </is>
+      </c>
+      <c r="D97" t="b">
+        <v>1</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1115443</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta MOL</t>
+        </is>
+      </c>
+      <c r="D98" t="b">
+        <v>0</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1115444</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Gold Snap Demo</t>
+        </is>
+      </c>
+      <c r="D99" t="b">
+        <v>1</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>14189968</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+        </is>
+      </c>
+      <c r="D100" t="b">
+        <v>0</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
           <t>600025868</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
         <is>
           <t>FTMO Manual Trading</t>
         </is>
       </c>
-      <c r="D92" t="b">
+      <c r="D101" t="b">
         <v>1</v>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -17610,7 +17736,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/12/2026 12:27</t>
+          <t>10/15/2026 12:30</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17656,7 +17782,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10/12/2026 12:07</t>
+          <t>10/15/2026 12:11</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -17679,7 +17805,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10/12/2026 05:36</t>
+          <t>10/15/2026 05:40</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -17748,7 +17874,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10/12/2026 04:33</t>
+          <t>10/15/2026 04:35</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -17817,7 +17943,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10/12/2026 13:50</t>
+          <t>10/15/2026 13:53</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -17863,7 +17989,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10/12/2026 11:55</t>
+          <t>10/15/2026 11:57</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -17955,7 +18081,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10/12/2026 15:51</t>
+          <t>10/15/2026 15:54</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -17978,7 +18104,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10/12/2026 05:22</t>
+          <t>10/15/2026 05:24</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -18001,7 +18127,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10/12/2026 19:13</t>
+          <t>10/15/2026 19:17</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -18024,7 +18150,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10/12/2026 13:56</t>
+          <t>10/15/2026 13:58</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18070,7 +18196,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10/12/2026 15:36</t>
+          <t>10/15/2026 15:39</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18323,7 +18449,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10/12/2026 11:59</t>
+          <t>10/15/2026 12:02</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18346,7 +18472,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10/12/2026 12:56</t>
+          <t>10/15/2026 12:59</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18369,7 +18495,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10/12/2026 18:06</t>
+          <t>10/15/2026 18:09</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18392,7 +18518,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/14/2026 01:22</t>
+          <t>10/15/2026 01:36</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-16
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-15 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-16 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/15/2026 13:41</t>
+          <t>10/16/2026 10:36</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>31939.44</v>
-      </c>
-      <c r="I2" t="n">
-        <v>46</v>
+        <v>28205.46</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>28.94</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-11722.96</v>
+        <v>-11651.55</v>
       </c>
       <c r="P2" t="n">
         <v>30</v>
@@ -994,22 +994,22 @@
         <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.7762981307482064</v>
+        <v>0.7762421947240511</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>89.45</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="T2" t="n">
-        <v>3496</v>
+        <v>3498</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>6939.440000000001</v>
+        <v>3205.459999999997</v>
       </c>
       <c r="V2" t="n">
-        <v>2226</v>
+        <v>2228</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.67276887871854</v>
+        <v>63.69353916523728</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.01</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/13/2026 12:11</t>
+          <t>10/16/2026 12:14</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/13/2026 01:24</t>
+          <t>10/16/2026 01:27</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,17 +3140,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/15/2026 14:27</t>
+          <t>10/16/2026 11:24</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>18729.76</v>
+        <v>18719.87</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-6.35</v>
+        <v>-6.4</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>8.56</v>
+        <v>8.6</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>0.8</v>
@@ -3165,37 +3165,37 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-773.6600000000001</v>
+        <v>-865.48</v>
       </c>
       <c r="P22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.7128914222944639</v>
+        <v>0.6799331375783082</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>7.32</v>
+        <v>7.4</v>
       </c>
       <c r="T22" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-1270.24</v>
+        <v>-1280.13</v>
       </c>
       <c r="V22" t="n">
         <v>51</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>45.53571428571428</v>
+        <v>45.13274336283185</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>8.56</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/15/2026 16:23</t>
+          <t>10/16/2026 12:51</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19450.32</v>
+        <v>19469.4</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.9</v>
+        <v>-2.8</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.13</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-171.79</v>
+        <v>-159.8</v>
       </c>
       <c r="P23" t="n">
         <v>12</v>
@@ -3283,13 +3283,13 @@
         <v>30</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.4006768071448507</v>
+        <v>0.4425062796539213</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>1.07</v>
       </c>
       <c r="T23" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="U23" s="7" t="n">
         <v>-530.6</v>
@@ -3298,7 +3298,7 @@
         <v>28</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>28.8659793814433</v>
+        <v>28.28282828282828</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.39</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/15/2026 14:27</t>
+          <t>10/16/2026 11:24</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20370.36</v>
+        <v>20502.09</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-2.62</v>
+        <v>-1.99</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,7 +3601,7 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>319.37</v>
+        <v>489.35</v>
       </c>
       <c r="P26" t="n">
         <v>17</v>
@@ -3610,25 +3610,25 @@
         <v>42.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.196317924760266</v>
+        <v>1.338713808116395</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>2.86</v>
+        <v>2.67</v>
       </c>
       <c r="T26" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>370.3599999999999</v>
+        <v>502.0899999999999</v>
       </c>
       <c r="V26" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>43.24324324324324</v>
+        <v>43.6241610738255</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/15/2026 14:28</t>
+          <t>10/16/2026 11:24</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/15/2026 15:06</t>
+          <t>10/16/2026 11:53</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20592.99</v>
-      </c>
-      <c r="I30" t="n">
-        <v>3</v>
+        <v>20555.01</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>2.81</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.59</v>
+        <v>1.53</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-17.43</v>
+        <v>-45.64</v>
       </c>
       <c r="P30" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.929473173100267</v>
+        <v>0.8297332587203879</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.45</v>
+        <v>0.64</v>
       </c>
       <c r="T30" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>592.9899999999998</v>
+        <v>555.0099999999998</v>
       </c>
       <c r="V30" t="n">
         <v>32</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>27.82608695652174</v>
+        <v>26.89075630252101</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.59</v>
+        <v>1.53</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/15/2026 18:12</t>
+          <t>10/16/2026 06:59</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20634.7</v>
+        <v>20735.74</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>3.18</v>
+        <v>3.69</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4579,28 +4579,37 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>0</v>
+        <v>343.53</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q35" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R35" s="7" t="n">
+        <v>1.187614688919958</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>3.68</v>
       </c>
       <c r="T35" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>634.6999999999998</v>
+        <v>836.2999999999998</v>
       </c>
       <c r="V35" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.20125786163522</v>
+        <v>52.79503105590062</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4621,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4984,7 +4993,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10/13/2026 11:51</t>
+          <t>10/16/2026 11:55</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5102,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10/13/2026 10:23</t>
+          <t>10/16/2026 10:26</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5333,13 +5342,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T42" t="n">
         <v>4278</v>
@@ -5433,13 +5451,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T43" t="n">
         <v>57</v>
@@ -5511,14 +5538,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/15/2026 15:09</t>
+          <t>10/16/2026 11:56</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19662.88</v>
+        <v>19685.32</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.66</v>
+        <v>-1.55</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
@@ -5533,25 +5560,34 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>12.92</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>1.161762864655064</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T44" t="n">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-314.52</v>
+        <v>-314.68</v>
       </c>
       <c r="V44" t="n">
         <v>480</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>55.04587155963303</v>
+        <v>54.91990846681922</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -5566,7 +5602,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5611,7 +5647,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/15/2026 13:52</t>
+          <t>10/16/2026 10:55</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5633,13 +5669,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-18.29</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.7507834854884862</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.16</v>
       </c>
       <c r="T45" t="n">
         <v>61</v>
@@ -5711,20 +5756,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/15/2026 14:23</t>
+          <t>10/16/2026 11:21</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19033.57</v>
+        <v>18927.2</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-4.81</v>
+        <v>-5.34</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5733,28 +5778,37 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>-272.7500000000001</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>0.8497228619599114</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>4.97</v>
       </c>
       <c r="T46" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-974.4400000000001</v>
+        <v>-1076.24</v>
       </c>
       <c r="V46" t="n">
         <v>41</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>41</v>
+        <v>40.19607843137255</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5766,7 +5820,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5833,13 +5887,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5933,13 +5996,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6033,13 +6105,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T49" t="n">
         <v>1161</v>
@@ -6133,13 +6214,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>-52.41999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>0.8051952878219183</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>1.3</v>
       </c>
       <c r="T50" t="n">
         <v>1978</v>
@@ -6211,7 +6301,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/15/2026 14:05</t>
+          <t>10/16/2026 11:06</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6242,7 +6332,7 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="U51" s="7" t="n">
         <v>-355.9400000000001</v>
@@ -6251,7 +6341,7 @@
         <v>25</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>32.89473684210527</v>
+        <v>32.46753246753246</v>
       </c>
       <c r="X51" s="7" t="n">
         <v>0.95</v>
@@ -6266,7 +6356,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6311,14 +6401,14 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/15/2026 14:40</t>
+          <t>10/16/2026 11:34</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19267.22</v>
+        <v>19250.93</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.64</v>
+        <v>-3.72</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>6.6</v>
@@ -6333,25 +6423,34 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>-1032.84</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>0.5568845833726607</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>5.79</v>
       </c>
       <c r="T52" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-733.4600000000003</v>
+        <v>-749.6700000000003</v>
       </c>
       <c r="V52" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.46153846153847</v>
+        <v>38.63636363636363</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.88</v>
@@ -6366,7 +6465,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6411,20 +6510,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/15/2026 15:30</t>
+          <t>10/16/2026 12:14</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19594.73</v>
+        <v>19574.66</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-2.06</v>
+        <v>-2.16</v>
       </c>
       <c r="J53" s="7" t="n">
-        <v>2.06</v>
+        <v>2.16</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6433,31 +6532,40 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>0</v>
+        <v>-102.03</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q53" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R53" s="7" t="n">
+        <v>0.201830556207463</v>
+      </c>
+      <c r="S53" s="7" t="n">
+        <v>0.52</v>
       </c>
       <c r="T53" t="n">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-405.27</v>
+        <v>-425.34</v>
       </c>
       <c r="V53" t="n">
         <v>177</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.75757575757576</v>
+        <v>35.32934131736527</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="Y53" s="7" t="n">
-        <v>2.03</v>
+        <v>2.13</v>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
@@ -6466,7 +6574,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6711,7 +6819,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10/13/2026 11:22</t>
+          <t>10/16/2026 11:23</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6811,20 +6919,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/15/2026 14:20</t>
+          <t>10/16/2026 04:44</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19466.18</v>
+        <v>19469.35</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-2.67</v>
+        <v>-2.65</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>2.72</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6833,28 +6941,37 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-41.46</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.466889546097467</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T57" t="n">
-        <v>1291</v>
+        <v>1302</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-535.46</v>
+        <v>-526.5600000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.14484895429899</v>
+        <v>43.08755760368664</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>2.71</v>
@@ -6866,7 +6983,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6911,7 +7028,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/15/2026 14:53</t>
+          <t>10/16/2026 11:45</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7111,7 +7228,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/15/2026 14:46</t>
+          <t>10/16/2026 11:40</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7133,13 +7250,22 @@
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>0</v>
+        <v>-1105.06</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q60" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R60" s="7" t="n">
+        <v>0.2343571374133069</v>
+      </c>
+      <c r="S60" s="7" t="n">
+        <v>6.68</v>
       </c>
       <c r="T60" t="n">
         <v>7019</v>
@@ -7211,7 +7337,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/15/2026 15:56</t>
+          <t>10/16/2026 12:35</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7233,13 +7359,22 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>0</v>
+        <v>-448.41</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q61" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R61" s="7" t="n">
+        <v>0.480495858193825</v>
+      </c>
+      <c r="S61" s="7" t="n">
+        <v>3.68</v>
       </c>
       <c r="T61" t="n">
         <v>3982</v>
@@ -7411,20 +7546,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/15/2026 15:22</t>
+          <t>10/16/2026 12:06</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18288.49</v>
+        <v>18253.94</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-8.57</v>
+        <v>-8.74</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>8.57</v>
+        <v>8.74</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7433,40 +7568,31 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>-784.0600000000001</v>
+        <v>0</v>
       </c>
       <c r="P63" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q63" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="R63" s="7" t="n">
-        <v>0.44620709139709</v>
-      </c>
-      <c r="S63" s="7" t="n">
-        <v>3.92</v>
+        <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1711.51</v>
+        <v>-1746.06</v>
       </c>
       <c r="V63" t="n">
         <v>7</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.44776119402985</v>
+        <v>10.29411764705882</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>8.56</v>
+        <v>8.73</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7475,7 +7601,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7542,13 +7668,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-90.82000000000002</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.7198297137216189</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>0.96</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7620,7 +7755,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/15/2026 15:16</t>
+          <t>10/16/2026 05:17</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7642,13 +7777,22 @@
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O65" s="7" t="n">
-        <v>0</v>
+        <v>-1009.4</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q65" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R65" s="7" t="n">
+        <v>0.4962168852688107</v>
+      </c>
+      <c r="S65" s="7" t="n">
+        <v>7.37</v>
       </c>
       <c r="T65" t="n">
         <v>3298</v>
@@ -7742,13 +7886,22 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>0</v>
+        <v>-114.21</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q66" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R66" s="7" t="n">
+        <v>0.3210272873194221</v>
+      </c>
+      <c r="S66" s="7" t="n">
+        <v>0.67</v>
       </c>
       <c r="T66" t="n">
         <v>262</v>
@@ -7820,7 +7973,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/15/2026 15:54</t>
+          <t>10/16/2026 12:36</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7842,25 +7995,34 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>0</v>
+        <v>210.35</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q67" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R67" s="7" t="n">
+        <v>1.04640312369019</v>
+      </c>
+      <c r="S67" s="7" t="n">
+        <v>9.81</v>
       </c>
       <c r="T67" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>398.1799999999992</v>
+        <v>398.1799999999989</v>
       </c>
       <c r="V67" t="n">
         <v>33</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>32.03883495145632</v>
+        <v>31.73076923076923</v>
       </c>
       <c r="X67" s="7" t="n">
         <v>1.04</v>
@@ -7875,7 +8037,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7942,13 +8104,22 @@
         <v>0</v>
       </c>
       <c r="N68" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O68" s="7" t="n">
-        <v>0</v>
+        <v>-51.36999999999998</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q68" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R68" s="7" t="n">
+        <v>0.9115149427267248</v>
+      </c>
+      <c r="S68" s="7" t="n">
+        <v>2.12</v>
       </c>
       <c r="T68" t="n">
         <v>215</v>
@@ -9042,13 +9213,22 @@
         <v>0</v>
       </c>
       <c r="N79" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O79" s="7" t="n">
-        <v>0</v>
+        <v>-124.11</v>
       </c>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q79" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R79" s="7" t="n">
+        <v>0.8885296257376122</v>
+      </c>
+      <c r="S79" s="7" t="n">
+        <v>3.16</v>
       </c>
       <c r="T79" t="n">
         <v>94</v>
@@ -9142,13 +9322,22 @@
         <v>0</v>
       </c>
       <c r="N80" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O80" s="7" t="n">
-        <v>0</v>
+        <v>-879.54</v>
       </c>
       <c r="P80" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q80" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R80" s="7" t="n">
+        <v>0.5714327479681135</v>
+      </c>
+      <c r="S80" s="7" t="n">
+        <v>7.73</v>
       </c>
       <c r="T80" t="n">
         <v>318</v>
@@ -9242,13 +9431,22 @@
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O81" s="7" t="n">
-        <v>0</v>
+        <v>698.3099999999999</v>
       </c>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="Q81" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="R81" s="7" t="n">
+        <v>4.02390334733469</v>
+      </c>
+      <c r="S81" s="7" t="n">
+        <v>0.64</v>
       </c>
       <c r="T81" t="n">
         <v>2303</v>
@@ -9342,13 +9540,22 @@
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>0</v>
+        <v>-308.22</v>
       </c>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q82" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R82" s="7" t="n">
+        <v>0.412903102916246</v>
+      </c>
+      <c r="S82" s="7" t="n">
+        <v>1.62</v>
       </c>
       <c r="T82" t="n">
         <v>1156</v>
@@ -9442,13 +9649,22 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>0</v>
+        <v>1042.88</v>
       </c>
       <c r="P83" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q83" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R83" s="7" t="n">
+        <v>1.768473487193091</v>
+      </c>
+      <c r="S83" s="7" t="n">
+        <v>3.89</v>
       </c>
       <c r="T83" t="n">
         <v>67</v>
@@ -9542,13 +9758,22 @@
         <v>0</v>
       </c>
       <c r="N84" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O84" s="7" t="n">
-        <v>0</v>
+        <v>20136.49</v>
       </c>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="Q84" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="R84" s="7" t="n">
+        <v>408.2914644012945</v>
+      </c>
+      <c r="S84" s="7" t="n">
+        <v>0.12</v>
       </c>
       <c r="T84" t="n">
         <v>3</v>
@@ -9580,7 +9805,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC84" t="inlineStr">
@@ -9642,13 +9867,22 @@
         <v>0</v>
       </c>
       <c r="N85" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O85" s="7" t="n">
-        <v>0</v>
+        <v>20105.63</v>
       </c>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="Q85" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R85" s="7" t="n">
+        <v>210.761398017736</v>
+      </c>
+      <c r="S85" s="7" t="n">
+        <v>0.12</v>
       </c>
       <c r="T85" t="n">
         <v>4</v>
@@ -9680,7 +9914,7 @@
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC85" t="inlineStr">
@@ -9820,14 +10054,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/15/2026 17:07</t>
+          <t>10/16/2026 13:24</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19887.17</v>
+        <v>19885.27</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.58</v>
+        <v>-0.59</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>5.56</v>
@@ -9851,16 +10085,16 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-112.8299999999998</v>
+        <v>-114.7299999999998</v>
       </c>
       <c r="V87" t="n">
         <v>86</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>42.78606965174129</v>
+        <v>42.57425742574257</v>
       </c>
       <c r="X87" s="7" t="n">
         <v>0.96</v>
@@ -9875,7 +10109,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -10020,20 +10254,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/15/2026 16:31</t>
+          <t>10/16/2026 12:59</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>19875.23</v>
+        <v>19918.01</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>-0.62</v>
+        <v>-0.4</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>4.25</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10051,19 +10285,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>-111.6000000000001</v>
+        <v>-81.99000000000007</v>
       </c>
       <c r="V89" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>82.24852071005917</v>
+        <v>82.45614035087719</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>4.27</v>
@@ -10075,7 +10309,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10120,20 +10354,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/15/2026 16:23</t>
+          <t>10/16/2026 12:54</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>26806.23</v>
+        <v>26510.23</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>34.09</v>
+        <v>32.61</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>4.18</v>
+        <v>5.24</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.59</v>
+        <v>1.55</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10151,22 +10385,22 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>6810.01</v>
+        <v>6510.23</v>
       </c>
       <c r="V90" t="n">
         <v>123</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>66.84782608695652</v>
+        <v>66.12903225806451</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.59</v>
+        <v>1.55</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>4.19</v>
+        <v>5.25</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10175,7 +10409,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10242,13 +10476,22 @@
         <v>0</v>
       </c>
       <c r="N91" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="O91" s="7" t="n">
-        <v>0</v>
+        <v>19746</v>
       </c>
       <c r="P91" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q91" s="7" t="n">
+        <v>72.72727272727273</v>
+      </c>
+      <c r="R91" s="7" t="n">
+        <v>39.6388541014402</v>
+      </c>
+      <c r="S91" s="7" t="n">
+        <v>1.03</v>
       </c>
       <c r="T91" t="n">
         <v>32</v>
@@ -10280,7 +10523,7 @@
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC91" t="inlineStr">
@@ -10842,13 +11085,22 @@
         <v>0</v>
       </c>
       <c r="N97" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O97" s="7" t="n">
-        <v>0</v>
+        <v>-574.2</v>
       </c>
       <c r="P97" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q97" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R97" s="7" t="n">
+        <v>0.1321433429560328</v>
+      </c>
+      <c r="S97" s="7" t="n">
+        <v>0.57</v>
       </c>
       <c r="T97" t="n">
         <v>448</v>
@@ -11142,13 +11394,22 @@
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>0</v>
+        <v>-304.44</v>
       </c>
       <c r="P100" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q100" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R100" s="7" t="n">
+        <v>0.4682177854635016</v>
+      </c>
+      <c r="S100" s="7" t="n">
+        <v>0.41</v>
       </c>
       <c r="T100" t="n">
         <v>199</v>
@@ -11220,7 +11481,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/15/2026 17:50</t>
+          <t>10/16/2026 06:45</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11320,7 +11581,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/13/2026 10:54</t>
+          <t>10/16/2026 10:56</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11538,20 +11799,20 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>10/15/2026 20:51</t>
+          <t>10/16/2026 08:45</t>
         </is>
       </c>
       <c r="H104" s="7" t="n">
-        <v>12556.74</v>
+        <v>12645.71</v>
       </c>
       <c r="I104" s="7" t="n">
-        <v>25.51</v>
+        <v>26.4</v>
       </c>
       <c r="J104" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K104" s="7" t="n">
-        <v>2.24</v>
+        <v>2.28</v>
       </c>
       <c r="L104" t="n">
         <v>10000</v>
@@ -11560,28 +11821,37 @@
         <v>0</v>
       </c>
       <c r="N104" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O104" s="7" t="n">
-        <v>0</v>
+        <v>945.14</v>
       </c>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>29</v>
+      </c>
+      <c r="Q104" s="7" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="R104" s="7" t="n">
+        <v>1.679458239277652</v>
+      </c>
+      <c r="S104" s="7" t="n">
+        <v>3.54</v>
       </c>
       <c r="T104" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="U104" s="7" t="n">
-        <v>2787.57</v>
+        <v>2876.54</v>
       </c>
       <c r="V104" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W104" s="7" t="n">
-        <v>70.11494252873564</v>
+        <v>70.45454545454545</v>
       </c>
       <c r="X104" s="7" t="n">
-        <v>2.62</v>
+        <v>2.67</v>
       </c>
       <c r="Y104" s="7" t="n">
         <v>2.97</v>
@@ -11593,7 +11863,7 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="AB104" t="inlineStr">
@@ -11747,17 +12017,17 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/15/2026 13:04</t>
+          <t>10/16/2026 10:05</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
-        <v>24240.53</v>
+        <v>24081.8</v>
       </c>
       <c r="I106" s="7" t="n">
-        <v>-36.87</v>
-      </c>
-      <c r="J106" s="7" t="n">
-        <v>42.89</v>
+        <v>-37.28</v>
+      </c>
+      <c r="J106" t="n">
+        <v>43</v>
       </c>
       <c r="K106" s="7" t="n">
         <v>0.75</v>
@@ -11772,37 +12042,37 @@
         <v>40</v>
       </c>
       <c r="O106" s="7" t="n">
-        <v>-460.85</v>
+        <v>-794.13</v>
       </c>
       <c r="P106" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="Q106" s="7" t="n">
-        <v>62.5</v>
+        <v>40</v>
       </c>
       <c r="R106" s="7" t="n">
-        <v>0.3397942811300212</v>
+        <v>0.1336984149494377</v>
       </c>
       <c r="S106" s="7" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="T106" t="n">
-        <v>4025</v>
+        <v>4034</v>
       </c>
       <c r="U106" s="7" t="n">
-        <v>-10157.35</v>
+        <v>-10241.92</v>
       </c>
       <c r="V106" t="n">
-        <v>2431</v>
+        <v>2442</v>
       </c>
       <c r="W106" s="7" t="n">
-        <v>60.3975155279503</v>
+        <v>60.53544868616758</v>
       </c>
       <c r="X106" s="7" t="n">
         <v>0.75</v>
       </c>
       <c r="Y106" s="7" t="n">
-        <v>46.04</v>
+        <v>46.43</v>
       </c>
       <c r="Z106" t="inlineStr">
         <is>
@@ -12220,7 +12490,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>10/13/2026 12:25</t>
+          <t>10/16/2026 12:27</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12879,17 +13149,23 @@
         <v>0</v>
       </c>
       <c r="N118" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O118" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P118" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q118" s="8" t="n"/>
-      <c r="R118" s="8" t="n"/>
-      <c r="S118" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q118" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R118" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S118" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T118" s="8" t="n">
         <v>0</v>
       </c>
@@ -12964,17 +13240,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -14325,7 +14607,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10/13/2026 12:25</t>
+          <t>10/16/2026 12:27</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14622,7 +14904,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14663,7 +14945,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -15169,7 +15451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -17442,17 +17724,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>60490</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>KC_A52_DEMO_T1_20k</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -17460,49 +17742,49 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>60491</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>KC_A52_DEMO_T2_20k</t>
         </is>
       </c>
       <c r="D94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>662436</t>
+          <t>60492</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+          <t>KC_A52_DEMO_T2_1k</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -17510,24 +17792,24 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>663097</t>
+          <t>60569</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+          <t>Demo Dream Catcher Portfolio</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -17535,14 +17817,14 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1115442</t>
+          <t>60570</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -17552,7 +17834,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Gold Snap Internal</t>
+          <t>EURO Overnight</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -17560,14 +17842,14 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>1115443</t>
+          <t>60572</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -17577,22 +17859,22 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta MOL</t>
+          <t>Portfolio DC FT Luna</t>
         </is>
       </c>
       <c r="D98" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>1115444</t>
+          <t>60575</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -17602,7 +17884,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Gold Snap Demo</t>
+          <t>ML_POC</t>
         </is>
       </c>
       <c r="D99" t="b">
@@ -17610,55 +17892,230 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>14189968</t>
+          <t>662434</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+          <t>LIVE Gold Reaper Conservative</t>
         </is>
       </c>
       <c r="D100" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
+          <t>662435</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Aggv1 Pro Filter 60</t>
+        </is>
+      </c>
+      <c r="D101" t="b">
+        <v>0</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>662436</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+        </is>
+      </c>
+      <c r="D102" t="b">
+        <v>1</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>663097</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+        </is>
+      </c>
+      <c r="D103" t="b">
+        <v>1</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1115442</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Gold Snap Internal</t>
+        </is>
+      </c>
+      <c r="D104" t="b">
+        <v>1</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1115443</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta MOL</t>
+        </is>
+      </c>
+      <c r="D105" t="b">
+        <v>0</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1115444</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Gold Snap Demo</t>
+        </is>
+      </c>
+      <c r="D106" t="b">
+        <v>1</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>14189968</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+        </is>
+      </c>
+      <c r="D107" t="b">
+        <v>0</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
           <t>600025868</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
         <is>
           <t>FTMO Manual Trading</t>
         </is>
       </c>
-      <c r="D101" t="b">
+      <c r="D108" t="b">
         <v>1</v>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E108" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -17851,7 +18308,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10/10/2026 09:29</t>
+          <t>10/16/2026 09:35</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -17897,7 +18354,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10/13/2026 09:35</t>
+          <t>10/16/2026 09:39</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -18219,7 +18676,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10/13/2026 08:23</t>
+          <t>10/16/2026 08:26</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18380,7 +18837,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10/13/2026 09:30</t>
+          <t>10/16/2026 09:32</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18403,7 +18860,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10/13/2026 09:41</t>
+          <t>10/16/2026 09:44</t>
         </is>
       </c>
       <c r="E33" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-19
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-16 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-19 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/16/2026 10:36</t>
+          <t>10/19/2026 21:27</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>28205.46</v>
+        <v>31172.48</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>28.94</v>
+        <v>42.51</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-11651.55</v>
+        <v>-14464.5</v>
       </c>
       <c r="P2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>75</v>
+        <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.7762421947240511</v>
+        <v>0.7329309464615589</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>79.93000000000001</v>
+        <v>95.28</v>
       </c>
       <c r="T2" t="n">
-        <v>3498</v>
+        <v>3502</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>2745.919999999996</v>
+        <v>6172.479999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>2229</v>
+        <v>2231</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.7221269296741</v>
+        <v>63.70645345516848</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/14/2026 15:31</t>
+          <t>10/17/2026 15:35</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/14/2026 18:46</t>
+          <t>10/17/2026 18:50</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/16/2026 12:14</t>
+          <t>10/19/2026 12:16</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/14/2026 09:51</t>
+          <t>10/17/2026 09:55</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/15/2026 14:58</t>
+          <t>10/18/2026 15:02</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/15/2026 17:33</t>
+          <t>10/18/2026 17:36</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/15/2026 17:37</t>
+          <t>10/18/2026 17:39</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/14/2026 17:28</t>
+          <t>10/17/2026 17:32</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/15/2026 08:41</t>
+          <t>10/18/2026 08:52</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/14/2026 18:57</t>
+          <t>10/17/2026 19:01</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/13/2026 16:21</t>
+          <t>10/19/2026 16:24</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/14/2026 17:42</t>
+          <t>10/17/2026 17:47</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/14/2026 19:32</t>
+          <t>10/17/2026 19:37</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/14/2026 18:29</t>
+          <t>10/17/2026 18:33</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/14/2026 18:45</t>
+          <t>10/17/2026 18:49</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/16/2026 01:27</t>
+          <t>10/19/2026 01:30</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/16/2026 11:24</t>
+          <t>10/19/2026 21:52</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>18719.87</v>
+        <v>18908.33</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-6.4</v>
+        <v>-5.46</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>8.6</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3165,7 +3165,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-865.48</v>
+        <v>-836.2700000000001</v>
       </c>
       <c r="P22" t="n">
         <v>15</v>
@@ -3174,25 +3174,25 @@
         <v>37.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.6799331375783082</v>
+        <v>0.6831122276914449</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>7.4</v>
+        <v>7.62</v>
       </c>
       <c r="T22" t="n">
         <v>113</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-1280.13</v>
+        <v>-1091.67</v>
       </c>
       <c r="V22" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>45.13274336283185</v>
+        <v>46.90265486725664</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
       <c r="Y22" s="7" t="n">
         <v>8.609999999999999</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/16/2026 12:51</t>
+          <t>10/19/2026 23:32</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19469.4</v>
+        <v>19500.22</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.8</v>
+        <v>-2.65</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.13</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.35</v>
+        <v>0.41</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-159.8</v>
+        <v>-102.83</v>
       </c>
       <c r="P23" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.4425062796539213</v>
+        <v>0.6620991062039958</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>1.07</v>
+        <v>0.98</v>
       </c>
       <c r="T23" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-530.6</v>
+        <v>-499.7800000000001</v>
       </c>
       <c r="V23" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>28.28282828282828</v>
+        <v>31.68316831683168</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.39</v>
+        <v>0.45</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>2.98</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/14/2026 09:29</t>
+          <t>10/17/2026 09:32</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/14/2026 23:48</t>
+          <t>10/17/2026 23:52</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/16/2026 11:24</t>
+          <t>10/19/2026 21:54</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20502.09</v>
+        <v>20749.59</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-1.99</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>489.35</v>
+        <v>878.8</v>
       </c>
       <c r="P26" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.338713808116395</v>
+        <v>1.96523697072876</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>2.67</v>
+        <v>2.4</v>
       </c>
       <c r="T26" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>502.0899999999999</v>
+        <v>749.5899999999999</v>
       </c>
       <c r="V26" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>43.6241610738255</v>
+        <v>44.37086092715231</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>8.99</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/15/2026 13:53</t>
+          <t>10/18/2026 13:56</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/16/2026 11:24</t>
+          <t>10/19/2026 21:53</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/16/2026 13:28</t>
+          <t>10/19/2026 13:32</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/16/2026 11:53</t>
+          <t>10/19/2026 22:19</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20555.01</v>
+        <v>20563.7</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2.81</v>
+        <v>2.85</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-45.64</v>
+        <v>-26.37</v>
       </c>
       <c r="P30" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>27.5</v>
+        <v>32.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.8297332587203879</v>
+        <v>0.8997185883784606</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>0.64</v>
       </c>
       <c r="T30" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>555.0099999999998</v>
+        <v>563.7</v>
       </c>
       <c r="V30" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>26.89075630252101</v>
+        <v>27.86885245901639</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.83</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/14/2026 18:57</t>
+          <t>10/17/2026 19:00</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/14/2026 19:04</t>
+          <t>10/17/2026 19:07</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/14/2026 20:08</t>
+          <t>10/17/2026 20:12</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>10/14/2026 18:07</t>
+          <t>10/17/2026 18:11</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,11 +4557,11 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/16/2026 14:07</t>
+          <t>10/20/2026 00:41</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20735.74</v>
+        <v>20736.34</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>3.69</v>
@@ -4570,7 +4570,7 @@
         <v>8.84</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4579,28 +4579,37 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>0</v>
+        <v>536.41</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q35" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R35" s="7" t="n">
+        <v>1.307940043514952</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>3.65</v>
       </c>
       <c r="T35" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>735.7399999999999</v>
+        <v>736.3399999999998</v>
       </c>
       <c r="V35" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>52.46913580246913</v>
+        <v>52.4390243902439</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>8.83</v>
@@ -4612,7 +4621,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4657,7 +4666,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>10/14/2026 19:03</t>
+          <t>10/17/2026 19:07</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4775,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>10/14/2026 17:48</t>
+          <t>10/17/2026 17:52</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4884,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>10/13/2026 22:34</t>
+          <t>10/19/2026 22:42</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4993,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10/16/2026 11:55</t>
+          <t>10/19/2026 12:02</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5102,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10/16/2026 10:26</t>
+          <t>10/19/2026 10:29</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5211,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10/15/2026 00:55</t>
+          <t>10/18/2026 00:57</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5320,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>10/15/2026 01:15</t>
+          <t>10/18/2026 01:16</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5429,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>10/15/2026 03:33</t>
+          <t>10/18/2026 03:35</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,20 +5538,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10/16/2026 11:56</t>
+          <t>10/19/2026 16:09</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19685.32</v>
+        <v>19641.71</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-1.55</v>
+        <v>-1.76</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5551,28 +5560,37 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-3.070000000000004</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.9679741289380346</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>0.22</v>
       </c>
       <c r="T44" t="n">
-        <v>874</v>
+        <v>877</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-314.68</v>
+        <v>-358.29</v>
       </c>
       <c r="V44" t="n">
         <v>480</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>54.91990846681922</v>
+        <v>54.73204104903079</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="Y44" s="7" t="n">
         <v>5.13</v>
@@ -5584,7 +5602,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5629,7 +5647,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>10/16/2026 10:55</t>
+          <t>10/19/2026 21:32</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5651,13 +5669,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-18.29</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.7507834854884862</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.16</v>
       </c>
       <c r="T45" t="n">
         <v>61</v>
@@ -5729,20 +5756,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10/16/2026 11:21</t>
+          <t>10/19/2026 21:52</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>18927.2</v>
+        <v>18757.24</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-5.34</v>
+        <v>-6.2</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.76</v>
+        <v>0.73</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5760,19 +5787,19 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-1170.49</v>
+        <v>-1242.76</v>
       </c>
       <c r="V46" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>40.19607843137255</v>
+        <v>40</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>7.43</v>
@@ -5784,7 +5811,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5829,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>10/15/2026 00:14</t>
+          <t>10/18/2026 00:17</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5851,13 +5878,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T47" t="n">
         <v>193</v>
@@ -5929,7 +5965,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>10/15/2026 21:04</t>
+          <t>10/18/2026 21:07</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5951,13 +5987,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T48" t="n">
         <v>410</v>
@@ -6051,13 +6096,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T49" t="n">
         <v>1161</v>
@@ -6129,7 +6183,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>10/15/2026 00:42</t>
+          <t>10/18/2026 00:45</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6229,20 +6283,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10/16/2026 11:06</t>
+          <t>10/19/2026 21:43</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19644.06</v>
+        <v>19463.49</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-1.75</v>
+        <v>-2.65</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6251,28 +6305,19 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>1464.6</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q51" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R51" s="7" t="n">
-        <v>1.450565745190089</v>
-      </c>
-      <c r="S51" s="7" t="n">
-        <v>5.81</v>
+        <v>0</v>
       </c>
       <c r="T51" t="n">
         <v>77</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-355.9400000000001</v>
+        <v>-536.5100000000001</v>
       </c>
       <c r="V51" t="n">
         <v>25</v>
@@ -6281,7 +6326,7 @@
         <v>32.46753246753246</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>10.19</v>
@@ -6293,7 +6338,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6338,17 +6383,17 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10/16/2026 11:34</t>
+          <t>10/19/2026 22:02</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19250.93</v>
+        <v>19209.1</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.72</v>
+        <v>-3.93</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>6.6</v>
+        <v>6.69</v>
       </c>
       <c r="K52" s="7" t="n">
         <v>0.88</v>
@@ -6360,31 +6405,40 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>-808.52</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>0.6364584691615595</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>4.63</v>
       </c>
       <c r="T52" t="n">
         <v>133</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-750.4300000000003</v>
+        <v>-790.9000000000003</v>
       </c>
       <c r="V52" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>38.34586466165413</v>
+        <v>39.09774436090225</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.88</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>6.62</v>
+        <v>6.72</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6393,7 +6447,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6438,20 +6492,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10/16/2026 12:14</t>
+          <t>10/19/2026 22:44</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19574.66</v>
+        <v>19593.06</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-2.16</v>
+        <v>-2.07</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>2.16</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6469,19 +6523,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-425.34</v>
+        <v>-406.9399999999999</v>
       </c>
       <c r="V53" t="n">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.32934131736527</v>
+        <v>36.36363636363637</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>2.13</v>
@@ -6493,7 +6547,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6538,7 +6592,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>10/14/2026 21:51</t>
+          <t>10/17/2026 21:53</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6638,7 +6692,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10/14/2026 19:13</t>
+          <t>10/17/2026 19:17</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6738,7 +6792,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10/16/2026 11:23</t>
+          <t>10/19/2026 11:26</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6838,11 +6892,11 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10/16/2026 04:44</t>
+          <t>10/19/2026 21:50</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19469.35</v>
+        <v>19469.36</v>
       </c>
       <c r="I57" s="7" t="n">
         <v>-2.65</v>
@@ -6869,16 +6923,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1304</v>
+        <v>1322</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-526.53</v>
+        <v>-530.14</v>
       </c>
       <c r="V57" t="n">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.09815950920245</v>
+        <v>42.96520423600605</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.74</v>
@@ -6893,7 +6947,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6938,7 +6992,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>10/16/2026 11:45</t>
+          <t>10/19/2026 18:16</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7038,7 +7092,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>10/16/2026 14:14</t>
+          <t>10/19/2026 14:17</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7138,7 +7192,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>10/16/2026 11:40</t>
+          <t>10/19/2026 22:07</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7238,7 +7292,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10/16/2026 12:35</t>
+          <t>10/19/2026 23:11</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7338,7 +7392,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>10/14/2026 21:40</t>
+          <t>10/17/2026 21:43</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7438,7 +7492,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10/16/2026 12:06</t>
+          <t>10/19/2026 22:35</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7538,7 +7592,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>10/14/2026 19:22</t>
+          <t>10/17/2026 19:25</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7638,7 +7692,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10/16/2026 05:17</t>
+          <t>10/19/2026 22:31</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7738,7 +7792,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>10/14/2026 19:10</t>
+          <t>10/17/2026 19:14</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7838,20 +7892,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>10/16/2026 12:36</t>
+          <t>10/19/2026 23:11</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20398.18</v>
+        <v>20247.71</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>2.04</v>
+        <v>1.29</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>11.35</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7872,7 +7926,7 @@
         <v>104</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>398.1799999999989</v>
+        <v>247.7099999999991</v>
       </c>
       <c r="V67" t="n">
         <v>33</v>
@@ -7881,7 +7935,7 @@
         <v>31.73076923076923</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>11.37</v>
@@ -7893,7 +7947,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7938,7 +7992,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>10/16/2026 14:13</t>
+          <t>10/19/2026 14:16</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8038,7 +8092,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>10/14/2026 17:36</t>
+          <t>10/17/2026 17:40</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8138,7 +8192,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>10/14/2026 17:37</t>
+          <t>10/17/2026 17:40</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8238,7 +8292,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>10/14/2026 17:36</t>
+          <t>10/17/2026 17:40</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8338,7 +8392,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>10/14/2026 19:15</t>
+          <t>10/17/2026 19:19</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8438,7 +8492,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>10/14/2026 19:38</t>
+          <t>10/17/2026 19:42</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8538,7 +8592,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>10/14/2026 19:12</t>
+          <t>10/17/2026 19:16</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8638,7 +8692,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>10/14/2026 21:02</t>
+          <t>10/17/2026 21:04</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8738,7 +8792,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>10/14/2026 20:35</t>
+          <t>10/17/2026 20:40</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8838,7 +8892,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>10/14/2026 20:41</t>
+          <t>10/17/2026 20:45</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8938,7 +8992,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>10/14/2026 20:40</t>
+          <t>10/17/2026 20:44</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9038,7 +9092,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>10/14/2026 20:45</t>
+          <t>10/17/2026 20:48</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9138,7 +9192,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>10/14/2026 20:40</t>
+          <t>10/17/2026 20:44</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9238,7 +9292,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>10/14/2026 20:36</t>
+          <t>10/17/2026 20:40</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9338,7 +9392,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>10/14/2026 20:57</t>
+          <t>10/17/2026 21:00</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9438,7 +9492,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>10/11/2026 20:39</t>
+          <t>10/17/2026 20:46</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9538,7 +9592,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>10/11/2026 18:59</t>
+          <t>10/17/2026 19:14</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9638,7 +9692,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>10/15/2026 02:16</t>
+          <t>10/18/2026 02:20</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9738,7 +9792,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>10/14/2026 20:42</t>
+          <t>10/17/2026 20:46</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9838,20 +9892,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10/16/2026 13:24</t>
+          <t>10/19/2026 10:23</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>19885.27</v>
+        <v>19862.93</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>-0.59</v>
+        <v>-0.7</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>5.56</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9869,19 +9923,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>-114.7299999999998</v>
+        <v>-220.3099999999996</v>
       </c>
       <c r="V87" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>42.57425742574257</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>5.55</v>
@@ -9893,7 +9947,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9938,7 +9992,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>10/16/2026 15:04</t>
+          <t>10/19/2026 15:07</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -10038,20 +10092,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>10/16/2026 12:59</t>
+          <t>10/19/2026 23:37</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>19918.01</v>
+        <v>19977.68</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>-0.4</v>
+        <v>-0.1</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>4.25</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10069,19 +10123,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>-64.80000000000007</v>
+        <v>-22.32000000000008</v>
       </c>
       <c r="V89" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>82.55813953488372</v>
+        <v>82.95454545454545</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>4.27</v>
@@ -10093,7 +10147,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10138,20 +10192,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>10/16/2026 12:54</t>
+          <t>10/19/2026 23:29</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>26510.23</v>
+        <v>26901.92</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>32.61</v>
+        <v>34.57</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.55</v>
+        <v>1.58</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10169,19 +10223,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>6510.23</v>
+        <v>6901.919999999999</v>
       </c>
       <c r="V90" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>66.12903225806451</v>
+        <v>66.14583333333334</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.55</v>
+        <v>1.58</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>5.25</v>
@@ -10193,7 +10247,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10238,7 +10292,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>10/14/2026 20:33</t>
+          <t>10/17/2026 20:37</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -10338,7 +10392,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>10/14/2026 04:39</t>
+          <t>10/17/2026 04:42</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10360,22 +10414,13 @@
         <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="O92" s="7" t="n">
-        <v>20269.59</v>
+        <v>0</v>
       </c>
       <c r="P92" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q92" s="7" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="R92" s="7" t="n">
-        <v>188.9075739315843</v>
-      </c>
-      <c r="S92" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T92" t="n">
         <v>23</v>
@@ -10407,7 +10452,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -10447,7 +10492,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>10/14/2026 19:38</t>
+          <t>10/17/2026 19:42</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10547,7 +10592,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>10/14/2026 19:36</t>
+          <t>10/17/2026 19:40</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10647,7 +10692,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>10/14/2026 19:34</t>
+          <t>10/17/2026 19:38</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10747,7 +10792,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>10/15/2026 00:06</t>
+          <t>10/18/2026 00:08</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10847,7 +10892,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>10/14/2026 20:33</t>
+          <t>10/17/2026 20:38</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10947,7 +10992,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>10/14/2026 20:33</t>
+          <t>10/17/2026 20:38</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11047,7 +11092,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>10/15/2026 00:14</t>
+          <t>10/18/2026 00:17</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11147,7 +11192,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>10/14/2026 05:03</t>
+          <t>10/17/2026 05:06</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11247,7 +11292,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>10/16/2026 13:52</t>
+          <t>10/20/2026 00:30</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11347,7 +11392,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>10/16/2026 10:56</t>
+          <t>10/19/2026 10:59</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11456,7 +11501,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>10/14/2026 17:00</t>
+          <t>10/17/2026 17:04</t>
         </is>
       </c>
       <c r="H103" t="n">
@@ -11565,20 +11610,20 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>10/16/2026 08:45</t>
+          <t>10/19/2026 20:03</t>
         </is>
       </c>
       <c r="H104" s="7" t="n">
-        <v>12645.71</v>
+        <v>12709.55</v>
       </c>
       <c r="I104" s="7" t="n">
-        <v>26.4</v>
+        <v>27.04</v>
       </c>
       <c r="J104" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K104" s="7" t="n">
-        <v>2.28</v>
+        <v>2.31</v>
       </c>
       <c r="L104" t="n">
         <v>10000</v>
@@ -11599,19 +11644,19 @@
         <v>89</v>
       </c>
       <c r="U104" s="7" t="n">
-        <v>2940.380000000001</v>
+        <v>2936.74</v>
       </c>
       <c r="V104" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="W104" s="7" t="n">
-        <v>70.78651685393258</v>
+        <v>73.03370786516854</v>
       </c>
       <c r="X104" s="7" t="n">
-        <v>2.71</v>
+        <v>2.59</v>
       </c>
       <c r="Y104" s="7" t="n">
-        <v>2.97</v>
+        <v>2.96</v>
       </c>
       <c r="Z104" t="inlineStr">
         <is>
@@ -11665,7 +11710,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>10/15/2026 14:58</t>
+          <t>10/18/2026 15:01</t>
         </is>
       </c>
       <c r="H105" s="7" t="n">
@@ -11774,17 +11819,17 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10/16/2026 10:05</t>
+          <t>10/19/2026 21:04</t>
         </is>
       </c>
       <c r="H106" s="7" t="n">
-        <v>24081.8</v>
+        <v>24239.86</v>
       </c>
       <c r="I106" s="7" t="n">
-        <v>-37.28</v>
-      </c>
-      <c r="J106" t="n">
-        <v>43</v>
+        <v>-36.87</v>
+      </c>
+      <c r="J106" s="7" t="n">
+        <v>43.17</v>
       </c>
       <c r="K106" s="7" t="n">
         <v>0.75</v>
@@ -11799,31 +11844,31 @@
         <v>40</v>
       </c>
       <c r="O106" s="7" t="n">
-        <v>-794.13</v>
+        <v>-141.4</v>
       </c>
       <c r="P106" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="Q106" s="7" t="n">
-        <v>40</v>
+        <v>57.49999999999999</v>
       </c>
       <c r="R106" s="7" t="n">
-        <v>0.1336984149494377</v>
+        <v>0.7166559794806028</v>
       </c>
       <c r="S106" s="7" t="n">
-        <v>3.2</v>
+        <v>1.38</v>
       </c>
       <c r="T106" t="n">
-        <v>4035</v>
+        <v>4039</v>
       </c>
       <c r="U106" s="7" t="n">
-        <v>-10133.11</v>
+        <v>-10042.14</v>
       </c>
       <c r="V106" t="n">
-        <v>2447</v>
+        <v>2451</v>
       </c>
       <c r="W106" s="7" t="n">
-        <v>60.64436183395291</v>
+        <v>60.68333745976727</v>
       </c>
       <c r="X106" s="7" t="n">
         <v>0.75</v>
@@ -11838,7 +11883,7 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="AB106" t="inlineStr">
@@ -11883,7 +11928,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 13:18</t>
+          <t>10/18/2026 13:21</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11974,7 +12019,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 07:11</t>
+          <t>10/18/2026 07:13</t>
         </is>
       </c>
       <c r="H108" s="8" t="n">
@@ -12065,7 +12110,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 15:40</t>
+          <t>10/17/2026 15:45</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12156,7 +12201,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 20:15</t>
+          <t>10/17/2026 20:18</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12247,7 +12292,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>10/16/2026 12:27</t>
+          <t>10/19/2026 12:30</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12338,7 +12383,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 21:13</t>
+          <t>10/18/2026 21:16</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12429,7 +12474,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 14:58</t>
+          <t>10/18/2026 15:01</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12520,7 +12565,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>10/13/2026 16:18</t>
+          <t>10/19/2026 16:24</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12611,7 +12656,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 08:07</t>
+          <t>10/18/2026 08:10</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12702,7 +12747,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 08:37</t>
+          <t>10/17/2026 08:39</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12793,7 +12838,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 00:27</t>
+          <t>10/18/2026 00:29</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12906,17 +12951,23 @@
         <v>0</v>
       </c>
       <c r="N118" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O118" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P118" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q118" s="8" t="n"/>
-      <c r="R118" s="8" t="n"/>
-      <c r="S118" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q118" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R118" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S118" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T118" s="8" t="n">
         <v>0</v>
       </c>
@@ -12969,7 +13020,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 21:22</t>
+          <t>10/17/2026 21:25</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12991,17 +13042,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13054,7 +13111,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 19:59</t>
+          <t>10/17/2026 20:02</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13076,17 +13133,23 @@
         <v>0</v>
       </c>
       <c r="N120" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O120" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q120" s="8" t="n"/>
-      <c r="R120" s="8" t="n"/>
-      <c r="S120" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q120" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R120" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S120" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T120" s="8" t="n">
         <v>0</v>
       </c>
@@ -13139,7 +13202,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 17:37</t>
+          <t>10/17/2026 17:41</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13161,17 +13224,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>-58.49</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>0.2666750250752257</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>0.32</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13224,7 +13293,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 05:44</t>
+          <t>10/17/2026 05:48</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13309,7 +13378,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 05:47</t>
+          <t>10/17/2026 05:49</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13394,7 +13463,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 05:47</t>
+          <t>10/17/2026 05:50</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13416,17 +13485,23 @@
         <v>0</v>
       </c>
       <c r="N124" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O124" s="9" t="n">
-        <v>0</v>
+        <v>-1180.45</v>
       </c>
       <c r="P124" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q124" s="8" t="n"/>
-      <c r="R124" s="8" t="n"/>
-      <c r="S124" s="8" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="Q124" s="9" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R124" s="9" t="n">
+        <v>0.2676972896517925</v>
+      </c>
+      <c r="S124" s="9" t="n">
+        <v>1.18</v>
+      </c>
       <c r="T124" s="8" t="n">
         <v>0</v>
       </c>
@@ -13479,7 +13554,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 06:23</t>
+          <t>10/17/2026 06:27</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13564,7 +13639,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 08:03</t>
+          <t>10/17/2026 08:07</t>
         </is>
       </c>
       <c r="H126" s="9" t="n">
@@ -13649,7 +13724,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>10/14/2026 05:35</t>
+          <t>10/17/2026 05:39</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13734,7 +13809,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 10:16</t>
+          <t>10/18/2026 10:19</t>
         </is>
       </c>
       <c r="H128" s="8" t="n">
@@ -13825,7 +13900,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 09:37</t>
+          <t>10/18/2026 09:40</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
@@ -14007,7 +14082,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>10/15/2026 18:20</t>
+          <t>10/18/2026 18:24</t>
         </is>
       </c>
       <c r="H131" s="9" t="n">
@@ -14182,7 +14257,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10/15/2026 13:18</t>
+          <t>10/18/2026 13:21</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -14223,7 +14298,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/15/2026 07:11</t>
+          <t>10/18/2026 07:13</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -14264,7 +14339,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10/14/2026 15:40</t>
+          <t>10/17/2026 15:45</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14305,7 +14380,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10/14/2026 20:15</t>
+          <t>10/17/2026 20:18</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14346,7 +14421,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10/16/2026 12:27</t>
+          <t>10/19/2026 12:30</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14387,7 +14462,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10/15/2026 21:13</t>
+          <t>10/18/2026 21:16</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14428,7 +14503,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10/15/2026 14:58</t>
+          <t>10/18/2026 15:01</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14469,7 +14544,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10/13/2026 16:18</t>
+          <t>10/19/2026 16:24</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14510,7 +14585,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10/15/2026 08:07</t>
+          <t>10/18/2026 08:10</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14551,7 +14626,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10/14/2026 08:37</t>
+          <t>10/17/2026 08:39</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14592,7 +14667,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10/15/2026 00:27</t>
+          <t>10/18/2026 00:29</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14643,7 +14718,7 @@
         <v>2.96</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14674,7 +14749,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>10/14/2026 21:22</t>
+          <t>10/17/2026 21:25</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14684,7 +14759,7 @@
         <v>-33.06</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -14715,7 +14790,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>10/14/2026 19:59</t>
+          <t>10/17/2026 20:02</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14725,7 +14800,7 @@
         <v>-5.87</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14756,7 +14831,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>10/14/2026 17:37</t>
+          <t>10/17/2026 17:41</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14766,7 +14841,7 @@
         <v>-0.16</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20">
@@ -14797,7 +14872,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10/14/2026 05:44</t>
+          <t>10/17/2026 05:48</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14838,7 +14913,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10/14/2026 05:47</t>
+          <t>10/17/2026 05:49</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14879,7 +14954,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>10/14/2026 05:47</t>
+          <t>10/17/2026 05:50</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14889,7 +14964,7 @@
         <v>-2.31</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -14920,7 +14995,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10/14/2026 06:23</t>
+          <t>10/17/2026 06:27</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14961,7 +15036,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10/14/2026 08:03</t>
+          <t>10/17/2026 08:07</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -15002,7 +15077,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>10/14/2026 05:35</t>
+          <t>10/17/2026 05:39</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -15043,7 +15118,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>10/15/2026 10:16</t>
+          <t>10/18/2026 10:19</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -15084,7 +15159,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10/15/2026 09:37</t>
+          <t>10/18/2026 09:40</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -15166,7 +15241,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>10/15/2026 18:20</t>
+          <t>10/18/2026 18:24</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
@@ -15190,7 +15265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -17363,7 +17438,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>58992</t>
+          <t>58990</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -17373,7 +17448,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Golden Fractal</t>
+          <t>Cable Surge</t>
         </is>
       </c>
       <c r="D89" t="b">
@@ -17381,14 +17456,14 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>58993</t>
+          <t>58991</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -17398,7 +17473,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Levels</t>
+          <t>Shiranui</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -17406,24 +17481,24 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>59376</t>
+          <t>58992</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>LIVE XAUUSD: YuHeng Gift EA + fundedtoday copy feed</t>
+          <t>Golden Fractal</t>
         </is>
       </c>
       <c r="D91" t="b">
@@ -17431,49 +17506,49 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>VPS153t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>59377</t>
+          <t>58993</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>UNFUNDED, never traded (earmarked Gold Snap 2HR)</t>
+          <t>Levels</t>
         </is>
       </c>
       <c r="D92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>60490</t>
+          <t>59376</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>KC_A52_DEMO_T1_20k</t>
+          <t>LIVE XAUUSD: YuHeng Gift EA + fundedtoday copy feed</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -17481,39 +17556,39 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS153t2</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>60491</t>
+          <t>59377</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>KC_A52_DEMO_T2_20k</t>
+          <t>UNFUNDED, never traded (earmarked Gold Snap 2HR)</t>
         </is>
       </c>
       <c r="D94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>60492</t>
+          <t>60490</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -17523,7 +17598,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>KC_A52_DEMO_T2_1k</t>
+          <t>KC_A52_DEMO_T1_20k</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -17538,7 +17613,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>60569</t>
+          <t>60491</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -17548,7 +17623,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Demo Dream Catcher Portfolio</t>
+          <t>KC_A52_DEMO_T2_20k</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -17556,14 +17631,14 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>60570</t>
+          <t>60492</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -17573,7 +17648,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>EURO Overnight</t>
+          <t>KC_A52_DEMO_T2_1k</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -17581,14 +17656,14 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>60572</t>
+          <t>60569</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -17598,7 +17673,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Portfolio DC FT Luna</t>
+          <t>Demo Dream Catcher Portfolio</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -17613,7 +17688,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>60575</t>
+          <t>60570</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -17623,7 +17698,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ML_POC</t>
+          <t>EURO Overnight</t>
         </is>
       </c>
       <c r="D99" t="b">
@@ -17631,24 +17706,24 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>60572</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>Portfolio DC FT Luna</t>
         </is>
       </c>
       <c r="D100" t="b">
@@ -17656,39 +17731,39 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>60575</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>ML_POC</t>
         </is>
       </c>
       <c r="D101" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>662436</t>
+          <t>662434</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -17698,7 +17773,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+          <t>LIVE Gold Reaper Conservative</t>
         </is>
       </c>
       <c r="D102" t="b">
@@ -17713,7 +17788,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>663097</t>
+          <t>662435</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -17723,32 +17798,32 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+          <t>Aggv1 Pro Filter 60</t>
         </is>
       </c>
       <c r="D103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>1115442</t>
+          <t>662436</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Gold Snap Internal</t>
+          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
         </is>
       </c>
       <c r="D104" t="b">
@@ -17756,39 +17831,39 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>1115443</t>
+          <t>663097</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta MOL</t>
+          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
         </is>
       </c>
       <c r="D105" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>1115444</t>
+          <t>1115442</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -17798,7 +17873,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Gold Snap Demo</t>
+          <t>Gold Snap Internal</t>
         </is>
       </c>
       <c r="D106" t="b">
@@ -17813,7 +17888,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>14189968</t>
+          <t>1115443</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -17823,7 +17898,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+          <t>T&amp;D19L13 Meta MOL</t>
         </is>
       </c>
       <c r="D107" t="b">
@@ -17831,14 +17906,14 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>600025868</t>
+          <t>1115444</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -17848,13 +17923,63 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>FTMO Manual Trading</t>
+          <t>Gold Snap Demo</t>
         </is>
       </c>
       <c r="D108" t="b">
         <v>1</v>
       </c>
       <c r="E108" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>14189968</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+        </is>
+      </c>
+      <c r="D109" t="b">
+        <v>0</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>600025868</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>FTMO Manual Trading</t>
+        </is>
+      </c>
+      <c r="D110" t="b">
+        <v>1</v>
+      </c>
+      <c r="E110" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -17932,7 +18057,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/15/2026 12:30</t>
+          <t>10/18/2026 12:32</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -17955,7 +18080,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10/13/2026 16:32</t>
+          <t>10/19/2026 16:36</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -17978,7 +18103,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10/15/2026 12:11</t>
+          <t>10/18/2026 12:15</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -18001,7 +18126,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10/15/2026 05:40</t>
+          <t>10/18/2026 05:43</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -18024,7 +18149,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10/14/2026 17:10</t>
+          <t>10/17/2026 17:15</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -18047,7 +18172,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10/16/2026 09:35</t>
+          <t>10/19/2026 09:37</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -18070,7 +18195,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10/15/2026 04:35</t>
+          <t>10/18/2026 04:37</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -18093,7 +18218,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10/16/2026 09:39</t>
+          <t>10/19/2026 09:41</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -18116,7 +18241,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10/14/2026 02:37</t>
+          <t>10/17/2026 02:42</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -18139,7 +18264,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10/15/2026 13:53</t>
+          <t>10/18/2026 13:56</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -18162,7 +18287,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10/14/2026 11:13</t>
+          <t>10/17/2026 11:17</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -18185,7 +18310,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10/15/2026 11:57</t>
+          <t>10/18/2026 12:01</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -18231,7 +18356,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10/14/2026 17:20</t>
+          <t>10/17/2026 17:25</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -18254,7 +18379,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10/14/2026 17:10</t>
+          <t>10/17/2026 17:14</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -18277,7 +18402,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10/15/2026 15:54</t>
+          <t>10/18/2026 15:57</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -18300,7 +18425,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10/15/2026 05:24</t>
+          <t>10/18/2026 05:27</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -18323,7 +18448,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10/15/2026 19:17</t>
+          <t>10/18/2026 19:19</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -18346,7 +18471,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10/15/2026 13:58</t>
+          <t>10/18/2026 14:01</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -18392,7 +18517,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10/15/2026 15:39</t>
+          <t>10/18/2026 15:41</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
@@ -18415,7 +18540,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10/16/2026 08:26</t>
+          <t>10/19/2026 08:36</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -18438,7 +18563,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10/14/2026 06:52</t>
+          <t>10/17/2026 06:54</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -18461,7 +18586,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10/14/2026 06:55</t>
+          <t>10/17/2026 06:58</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -18484,7 +18609,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10/14/2026 23:45</t>
+          <t>10/17/2026 23:49</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -18507,7 +18632,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10/14/2026 23:45</t>
+          <t>10/17/2026 23:49</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -18530,7 +18655,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10/14/2026 06:13</t>
+          <t>10/17/2026 06:15</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -18553,7 +18678,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10/14/2026 09:40</t>
+          <t>10/17/2026 09:43</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -18576,7 +18701,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10/16/2026 09:32</t>
+          <t>10/19/2026 09:35</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -18599,7 +18724,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10/16/2026 09:44</t>
+          <t>10/19/2026 09:46</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -18645,7 +18770,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10/15/2026 12:02</t>
+          <t>10/18/2026 12:06</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -18668,7 +18793,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10/15/2026 12:59</t>
+          <t>10/18/2026 13:02</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -18691,7 +18816,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10/15/2026 18:09</t>
+          <t>10/18/2026 18:12</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
@@ -18714,7 +18839,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/15/2026 01:36</t>
+          <t>10/17/2026 06:46</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-21
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-20 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-21 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/20/2026 23:26</t>
+          <t>10/21/2026 13:17</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>34398.34</v>
+        <v>36894.79</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>37.59</v>
+        <v>47.57</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-6422.84</v>
+        <v>-7353.68</v>
       </c>
       <c r="P2" t="n">
         <v>30</v>
@@ -994,22 +994,22 @@
         <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.8674696408570963</v>
+        <v>0.848262474011187</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>82.08</v>
+        <v>91.06</v>
       </c>
       <c r="T2" t="n">
-        <v>3505</v>
+        <v>3507</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>11021.57</v>
+        <v>11894.79</v>
       </c>
       <c r="V2" t="n">
-        <v>2234</v>
+        <v>2235</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.73751783166905</v>
+        <v>63.72968349016254</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.02</v>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/20/2026 23:54</t>
+          <t>10/21/2026 13:55</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1109,16 +1109,16 @@
         <v>2.49</v>
       </c>
       <c r="T3" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>635.27</v>
+        <v>635.2699999999999</v>
       </c>
       <c r="V3" t="n">
         <v>67</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>44.37086092715231</v>
+        <v>44.07894736842105</v>
       </c>
       <c r="X3" s="7" t="n">
         <v>1.1</v>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -1178,20 +1178,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/20/2026 21:55</t>
+          <t>10/21/2026 11:01</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>20563.85</v>
+        <v>20569.4</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>2.85</v>
+        <v>2.88</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1203,7 +1203,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>-13.03</v>
+        <v>-24.6</v>
       </c>
       <c r="P4" t="n">
         <v>14</v>
@@ -1212,25 +1212,25 @@
         <v>35</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>0.9500594074585106</v>
+        <v>0.9057146142347935</v>
       </c>
       <c r="S4" s="7" t="n">
         <v>0.66</v>
       </c>
       <c r="T4" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>563.8500000000001</v>
+        <v>569.4000000000001</v>
       </c>
       <c r="V4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>28.22580645161291</v>
+        <v>28.8</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="Y4" s="7" t="n">
         <v>1.83</v>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/20/2026 22:51</t>
+          <t>10/21/2026 12:24</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,20 +1505,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/20/2026 22:54</t>
+          <t>10/21/2026 12:28</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>20016.47</v>
+        <v>19806.57</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.08</v>
+        <v>-0.97</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>4.27</v>
+        <v>4.48</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L7" t="n">
         <v>20000</v>
@@ -1530,37 +1530,37 @@
         <v>40</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>-373.64</v>
+        <v>-600.54</v>
       </c>
       <c r="P7" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="Q7" s="7" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="R7" s="7" t="n">
-        <v>0.5070127059941154</v>
+        <v>0.37948564284312</v>
       </c>
       <c r="S7" s="7" t="n">
-        <v>2.95</v>
+        <v>3.17</v>
       </c>
       <c r="T7" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>16.46999999999991</v>
+        <v>-193.4300000000001</v>
       </c>
       <c r="V7" t="n">
         <v>149</v>
       </c>
       <c r="W7" s="7" t="n">
-        <v>83.24022346368714</v>
+        <v>82.32044198895028</v>
       </c>
       <c r="X7" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y7" s="7" t="n">
-        <v>4.27</v>
+        <v>4.49</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1723,20 +1723,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/20/2026 22:39</t>
+          <t>10/21/2026 12:07</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>27525.06</v>
+        <v>27256.68</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>37.69</v>
+        <v>36.35</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1.63</v>
+        <v>1.6</v>
       </c>
       <c r="L9" t="n">
         <v>20000</v>
@@ -1748,7 +1748,7 @@
         <v>40</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>-222.0200000000002</v>
+        <v>-283.8000000000002</v>
       </c>
       <c r="P9" t="n">
         <v>23</v>
@@ -1757,25 +1757,25 @@
         <v>57.49999999999999</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>0.9283732514324058</v>
+        <v>0.9101929996107729</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>6.9</v>
+        <v>6.83</v>
       </c>
       <c r="T9" t="n">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>7529.109999999999</v>
+        <v>7465.48</v>
       </c>
       <c r="V9" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>66.83673469387756</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X9" s="7" t="n">
-        <v>1.63</v>
+        <v>1.61</v>
       </c>
       <c r="Y9" s="7" t="n">
         <v>5.25</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/20/2026 23:30</t>
+          <t>10/21/2026 13:22</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/20/2026 23:29</t>
+          <t>10/21/2026 13:20</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/20/2026 23:40</t>
+          <t>10/21/2026 13:39</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/20/2026 23:36</t>
+          <t>10/21/2026 13:31</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/20/2026 23:36</t>
+          <t>10/21/2026 13:30</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/20/2026 23:33</t>
+          <t>10/21/2026 13:29</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/20/2026 23:41</t>
+          <t>10/21/2026 13:37</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/20/2026 23:30</t>
+          <t>10/21/2026 13:30</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/20/2026 23:38</t>
+          <t>10/21/2026 13:33</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/20/2026 23:43</t>
+          <t>10/21/2026 13:43</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2823,7 +2823,7 @@
         <v>0.05</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -2916,20 +2916,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/20/2026 23:43</t>
+          <t>10/21/2026 13:40</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>20131.92</v>
+        <v>20117.76</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>0.66</v>
+        <v>0.58</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>0.28</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>3.49</v>
+        <v>2.72</v>
       </c>
       <c r="L20" t="n">
         <v>20000</v>
@@ -2938,22 +2938,22 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>20114.04</v>
+        <v>20097.96</v>
       </c>
       <c r="P20" t="n">
         <v>9</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>56.25</v>
+        <v>52.94117647058824</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>320.5748331744518</v>
+        <v>255.3401670463174</v>
       </c>
       <c r="S20" s="7" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="T20" t="n">
         <v>16</v>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/21/2026 01:41</t>
+          <t>10/21/2026 08:01</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3065,22 +3065,22 @@
         <v>3.51</v>
       </c>
       <c r="T21" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>2772.13</v>
+        <v>2500.14</v>
       </c>
       <c r="V21" t="n">
         <v>66</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>71.73913043478261</v>
+        <v>70.96774193548387</v>
       </c>
       <c r="X21" s="7" t="n">
-        <v>2.32</v>
+        <v>2.06</v>
       </c>
       <c r="Y21" s="7" t="n">
-        <v>2.96</v>
+        <v>3.36</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>10/20/2026 23:51</t>
+          <t>10/21/2026 13:50</t>
         </is>
       </c>
       <c r="H22" s="9" t="n">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>10/20/2026 23:49</t>
+          <t>10/21/2026 13:48</t>
         </is>
       </c>
       <c r="H23" s="9" t="n">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10/20/2026 23:51</t>
+          <t>10/21/2026 13:50</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/20/2026 23:49</t>
+          <t>10/21/2026 13:48</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -3595,7 +3595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3982,7 +3982,7 @@
         </is>
       </c>
       <c r="D17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -6778,7 +6778,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>LIVE Dream Catcher multi-market (indices + FX + gold)</t>
+          <t>LIVE Dream Catcher</t>
         </is>
       </c>
       <c r="D129" t="b">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>LIVE Portfolio v4 ph1: Gold Reaper + Gold Snap + Golden Fractal + Range Snap + Dream Catcher x2</t>
+          <t>LIVE Prismatic Spectrum</t>
         </is>
       </c>
       <c r="D163" t="b">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>LIVE XAUUSD: YuHeng Gift EA + fundedtoday copy feed</t>
+          <t>LIVE YuHeng and Smart Gold Hunter</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -8432,7 +8432,7 @@
         </is>
       </c>
       <c r="D195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -8457,7 +8457,7 @@
         </is>
       </c>
       <c r="D196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
         </is>
       </c>
       <c r="D197" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -8893,17 +8893,17 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>52428953</t>
+          <t>26774273</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>prop</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>BTC Dual Breakout Scalper</t>
+          <t>The5ers $200k Challenge</t>
         </is>
       </c>
       <c r="D214" t="b">
@@ -8911,14 +8911,14 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>52441850</t>
+          <t>52428953</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -8928,7 +8928,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>EA Fx RSI MOL</t>
+          <t>BTC Dual Breakout Scalper</t>
         </is>
       </c>
       <c r="D215" t="b">
@@ -8943,7 +8943,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>52441853</t>
+          <t>52441850</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Fx RSI Low DD Prop Firms</t>
+          <t>EA Fx RSI MOL</t>
         </is>
       </c>
       <c r="D216" t="b">
@@ -8968,23 +8968,48 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
+          <t>52441853</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Fx RSI Low DD Prop Firms</t>
+        </is>
+      </c>
+      <c r="D217" t="b">
+        <v>1</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
           <t>600025868</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
         <is>
           <t>FTMO Manual Trading</t>
         </is>
       </c>
-      <c r="D217" t="b">
-        <v>1</v>
-      </c>
-      <c r="E217" t="inlineStr">
+      <c r="D218" t="b">
+        <v>1</v>
+      </c>
+      <c r="E218" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>

</xml_diff>

<commit_message>
Update dashboards — 2026-10-22
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-21 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-22 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/21/2026 20:59</t>
+          <t>10/22/2026 18:37</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>36894.79</v>
+        <v>28380.11</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>47.57</v>
+        <v>13.52</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-7353.68</v>
+        <v>-21065.79</v>
       </c>
       <c r="P2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.848262474011187</v>
+        <v>0.6407922293305123</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>91.06</v>
+        <v>108.79</v>
       </c>
       <c r="T2" t="n">
-        <v>3507</v>
+        <v>3510</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>11894.79</v>
+        <v>3380.110000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>2235</v>
+        <v>2236</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.72968349016254</v>
+        <v>63.70370370370371</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/21/2026 21:36</t>
+          <t>10/22/2026 19:13</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1178,20 +1178,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/21/2026 18:54</t>
+          <t>10/22/2026 23:21</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>20569.4</v>
+        <v>20547.61</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>2.88</v>
+        <v>2.77</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.54</v>
+        <v>1.51</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1203,34 +1203,34 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>-24.6</v>
+        <v>-45.9</v>
       </c>
       <c r="P4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>35</v>
+        <v>32.5</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>0.9057146142347935</v>
+        <v>0.837291740517547</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>0.66</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="T4" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>569.4000000000001</v>
+        <v>547.61</v>
       </c>
       <c r="V4" t="n">
         <v>36</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>28.8</v>
+        <v>28.34645669291339</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>1.54</v>
+        <v>1.51</v>
       </c>
       <c r="Y4" s="7" t="n">
         <v>1.83</v>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1287,20 +1287,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/21/2026 20:14</t>
+          <t>10/22/2026 17:51</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>20082.36</v>
+        <v>19886.06</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.43</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.37</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="L5" t="n">
         <v>20000</v>
@@ -1312,34 +1312,34 @@
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>421.0899999999999</v>
+        <v>-1132.47</v>
       </c>
       <c r="P5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>30</v>
+        <v>27.5</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>1.097421316132853</v>
+        <v>0.7491638573751103</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>9.779999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="T5" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>82.35999999999913</v>
+        <v>-113.9400000000007</v>
       </c>
       <c r="V5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>31.13207547169811</v>
+        <v>31.19266055045872</v>
       </c>
       <c r="X5" s="7" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="Y5" s="7" t="n">
         <v>11.37</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/19/2026 15:07</t>
+          <t>10/22/2026 15:11</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,20 +1505,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/21/2026 20:18</t>
+          <t>10/22/2026 17:54</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>19845.21</v>
+        <v>19888.68</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>-0.78</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="L7" t="n">
         <v>20000</v>
@@ -1530,7 +1530,7 @@
         <v>40</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>-570.3</v>
+        <v>-553.03</v>
       </c>
       <c r="P7" t="n">
         <v>30</v>
@@ -1539,25 +1539,25 @@
         <v>75</v>
       </c>
       <c r="R7" s="7" t="n">
-        <v>0.410731445221686</v>
+        <v>0.4285758568314028</v>
       </c>
       <c r="S7" s="7" t="n">
-        <v>3.17</v>
+        <v>3.18</v>
       </c>
       <c r="T7" t="n">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>-154.7900000000001</v>
+        <v>-111.3200000000001</v>
       </c>
       <c r="V7" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="W7" s="7" t="n">
-        <v>82.41758241758241</v>
+        <v>82.16216216216216</v>
       </c>
       <c r="X7" s="7" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="Y7" s="7" t="n">
         <v>4.49</v>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1654,19 +1654,19 @@
         <v>0.09</v>
       </c>
       <c r="T8" t="n">
+        <v>6</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>475.2</v>
+      </c>
+      <c r="V8" t="n">
         <v>5</v>
       </c>
-      <c r="U8" s="7" t="n">
-        <v>336.6200000000001</v>
-      </c>
-      <c r="V8" t="n">
-        <v>4</v>
-      </c>
       <c r="W8" s="7" t="n">
-        <v>80</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="X8" s="7" t="n">
-        <v>10.73</v>
+        <v>14.73</v>
       </c>
       <c r="Y8" s="7" t="n">
         <v>0.17</v>
@@ -1678,12 +1678,12 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
@@ -1723,20 +1723,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/21/2026 19:58</t>
+          <t>10/23/2026 00:13</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>27465.48</v>
+        <v>28132.05</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>37.39</v>
+        <v>40.73</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1.61</v>
+        <v>1.65</v>
       </c>
       <c r="L9" t="n">
         <v>20000</v>
@@ -1748,34 +1748,34 @@
         <v>40</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>-235.1100000000002</v>
+        <v>1307.94</v>
       </c>
       <c r="P9" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>57.49999999999999</v>
+        <v>65</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>0.9256006911151826</v>
+        <v>1.53896109247645</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>6.88</v>
+        <v>6.09</v>
       </c>
       <c r="T9" t="n">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>7465.48</v>
+        <v>8480.23</v>
       </c>
       <c r="V9" t="n">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>67.15686274509804</v>
       </c>
       <c r="X9" s="7" t="n">
-        <v>1.61</v>
+        <v>1.7</v>
       </c>
       <c r="Y9" s="7" t="n">
         <v>5.25</v>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1832,20 +1832,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/21/2026 21:31</t>
+          <t>10/22/2026 19:07</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>21637.88</v>
+        <v>21244.87</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>8.19</v>
+        <v>6.22</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>3.2</v>
+        <v>4.96</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.7</v>
+        <v>1.46</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1857,37 +1857,37 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>1597.84</v>
+        <v>471.6900000000001</v>
       </c>
       <c r="P10" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>45</v>
+        <v>37.5</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>1.789072376738306</v>
+        <v>1.200636333088045</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>3.21</v>
+        <v>5.14</v>
       </c>
       <c r="T10" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>1637.880000000001</v>
+        <v>1450.490000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>45.83333333333333</v>
+        <v>43.63636363636363</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.7</v>
+        <v>1.53</v>
       </c>
       <c r="Y10" s="7" t="n">
-        <v>3.2</v>
+        <v>4.96</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1941,20 +1941,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/21/2026 21:07</t>
+          <t>10/22/2026 18:46</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>21281.47</v>
+        <v>21195.13</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>6.39</v>
-      </c>
-      <c r="J11" t="n">
-        <v>2</v>
+        <v>5.95</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>2.01</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>2.18</v>
+        <v>1.92</v>
       </c>
       <c r="L11" t="n">
         <v>20000</v>
@@ -1963,37 +1963,37 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>21281.47</v>
+        <v>21195.13</v>
       </c>
       <c r="P11" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>75</v>
+        <v>74.07407407407408</v>
       </c>
       <c r="R11" s="7" t="n">
-        <v>20.59385156472982</v>
+        <v>17.31109794294422</v>
       </c>
       <c r="S11" s="7" t="n">
-        <v>1.01</v>
+        <v>1.04</v>
       </c>
       <c r="T11" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="U11" s="7" t="n">
-        <v>1281.47</v>
+        <v>1195.13</v>
       </c>
       <c r="V11" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W11" s="7" t="n">
-        <v>73.91304347826086</v>
+        <v>73.07692307692307</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>2.18</v>
+        <v>1.92</v>
       </c>
       <c r="Y11" s="7" t="n">
         <v>2</v>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -2050,20 +2050,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/21/2026 21:04</t>
+          <t>10/22/2026 18:45</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>19812.07</v>
+        <v>19777.12</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-1.11</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1.26</v>
+        <v>1.43</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>0.72</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2072,28 +2072,28 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>19760.81</v>
+        <v>19725.13</v>
       </c>
       <c r="P12" t="n">
         <v>10</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>29.02355527192796</v>
+        <v>27.62571710108931</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="T12" t="n">
         <v>31</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>-187.9299999999999</v>
+        <v>-222.8799999999999</v>
       </c>
       <c r="V12" t="n">
         <v>9</v>
@@ -2102,10 +2102,10 @@
         <v>29.03225806451613</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>0.72</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y12" s="7" t="n">
-        <v>1.26</v>
+        <v>1.43</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -2159,20 +2159,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/21/2026 21:29</t>
+          <t>10/22/2026 19:06</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>20450.77</v>
+        <v>20335.86</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>2.26</v>
+        <v>1.69</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>4.44</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1.26</v>
+        <v>1.18</v>
       </c>
       <c r="L13" t="n">
         <v>20000</v>
@@ -2181,37 +2181,37 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>20201.22</v>
+        <v>20086.31</v>
       </c>
       <c r="P13" t="n">
         <v>5</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>20.83333333333334</v>
+        <v>20</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>12.66736166059269</v>
+        <v>11.87898761874844</v>
       </c>
       <c r="S13" s="7" t="n">
         <v>2.22</v>
       </c>
       <c r="T13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>450.77</v>
+        <v>335.86</v>
       </c>
       <c r="V13" t="n">
         <v>4</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>16.66666666666666</v>
+        <v>16</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>1.26</v>
+        <v>1.18</v>
       </c>
       <c r="Y13" s="7" t="n">
         <v>4.44</v>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/21/2026 21:21</t>
+          <t>10/22/2026 18:58</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/21/2026 21:13</t>
+          <t>10/22/2026 18:52</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/21/2026 21:13</t>
+          <t>10/22/2026 18:52</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,20 +2595,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/21/2026 21:10</t>
+          <t>10/22/2026 18:48</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>19954.6</v>
+        <v>19947.8</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-0.23</v>
+        <v>-0.26</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.84</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="L17" t="n">
         <v>20000</v>
@@ -2617,37 +2617,37 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>19954.6</v>
+        <v>19947.8</v>
       </c>
       <c r="P17" t="n">
         <v>3</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>50</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>80.43710191082802</v>
+        <v>78.31705426356589</v>
       </c>
       <c r="S17" s="7" t="n">
         <v>0.42</v>
       </c>
       <c r="T17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-45.39999999999998</v>
+        <v>-52.19999999999998</v>
       </c>
       <c r="V17" t="n">
         <v>2</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="X17" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="Y17" s="7" t="n">
         <v>0.84</v>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/21/2026 21:21</t>
+          <t>10/22/2026 19:00</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2744,19 +2744,19 @@
         <v>0.01</v>
       </c>
       <c r="T18" t="n">
+        <v>5</v>
+      </c>
+      <c r="U18" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="V18" t="n">
         <v>4</v>
       </c>
-      <c r="U18" s="7" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="V18" t="n">
-        <v>3</v>
-      </c>
       <c r="W18" s="7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>6.54</v>
+        <v>8.31</v>
       </c>
       <c r="Y18" s="7" t="n">
         <v>0.01</v>
@@ -2768,12 +2768,12 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/21/2026 21:12</t>
+          <t>10/22/2026 18:53</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,20 +2922,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/21/2026 21:15</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="n">
-        <v>19841.6</v>
+          <t>10/22/2026 18:55</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>19815</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>-0.79</v>
+        <v>-0.92</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>2.41</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.65</v>
       </c>
       <c r="L20" t="n">
         <v>20000</v>
@@ -2944,37 +2944,37 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>19841.6</v>
+        <v>19815</v>
       </c>
       <c r="P20" t="n">
         <v>11</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>68.75</v>
+        <v>61.11111111111111</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>40.44652087475149</v>
+        <v>38.41503021148036</v>
       </c>
       <c r="S20" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="T20" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-158.4</v>
+        <v>-185</v>
       </c>
       <c r="V20" t="n">
         <v>10</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>55.55555555555556</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.65</v>
       </c>
       <c r="Y20" s="7" t="n">
         <v>2.41</v>
@@ -2986,12 +2986,12 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/21/2026 21:22</t>
+          <t>10/22/2026 19:02</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3041,7 +3041,7 @@
         <v>0.05</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.11</v>
+        <v>0.29</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -3134,20 +3134,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/21/2026 21:22</t>
+          <t>10/22/2026 19:04</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>20116.56</v>
+        <v>20087.47</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.58</v>
+        <v>0.43</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>0.28</v>
+        <v>0.33</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>2.72</v>
+        <v>1.89</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3156,40 +3156,40 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>20097.96</v>
+        <v>20064.83</v>
       </c>
       <c r="P22" t="n">
         <v>9</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>52.94117647058824</v>
+        <v>47.36842105263158</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>255.3401670463174</v>
+        <v>179.9106553722693</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="T22" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>114.92</v>
+        <v>144.45</v>
       </c>
       <c r="V22" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>44.44444444444444</v>
+        <v>61.53846153846154</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>2.61</v>
+        <v>2.46</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>0.19</v>
+        <v>0.32</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>EURO Overnight | AUDCAD, EURO Overnight | AUDUSD, EURO Overnight | EURAUD, EURO Overnight | EURGBP, EURO Overnight | EURUSD, EURO Overnight | GBPUSD, EURO Overnight | NZDUSD, EURO Overnight | USDCAD</t>
+          <t>EURO Overnight | AUDCAD, EURO Overnight | AUDUSD, EURO Overnight | EURAUD, EURO Overnight | EURGBP, EURO Overnight | EURUSD, EURO Overnight | GBPUSD, EURO Overnight | NZDUSD, EURO Overnight | USDCAD, EURO Overnight | USDCHF</t>
         </is>
       </c>
     </row>
@@ -3243,20 +3243,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/21/2026 15:58</t>
+          <t>10/22/2026 21:04</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>12544.94</v>
+        <v>12624.48</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>25.39</v>
+        <v>26.18</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>2.1</v>
+        <v>2.07</v>
       </c>
       <c r="L23" t="n">
         <v>10000</v>
@@ -3268,34 +3268,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>950.17</v>
+        <v>886.41</v>
       </c>
       <c r="P23" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>72.5</v>
+        <v>70</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.672448690728946</v>
+        <v>1.574941300089509</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>3.51</v>
+        <v>3.84</v>
       </c>
       <c r="T23" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>2374.27</v>
+        <v>2579.68</v>
       </c>
       <c r="V23" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>70.21276595744681</v>
+        <v>70.52631578947368</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>1.95</v>
+        <v>2.03</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>3.36</v>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3549,7 +3549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E221"/>
+  <dimension ref="A1:E232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8597,117 +8597,117 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>639884</t>
+          <t>60898</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Manual Trading (Diego)</t>
+          <t>BlackDog</t>
         </is>
       </c>
       <c r="D204" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>647832</t>
+          <t>60899</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Axis Rotation AUDUSD</t>
+          <t>AMStocktastic</t>
         </is>
       </c>
       <c r="D205" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>657902</t>
+          <t>60900</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>T&amp;D19</t>
+          <t>Finex</t>
         </is>
       </c>
       <c r="D206" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>658071</t>
+          <t>60901</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>T&amp;D V1</t>
+          <t>USAPattern5</t>
         </is>
       </c>
       <c r="D207" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>60902</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>CyberZ</t>
         </is>
       </c>
       <c r="D208" t="b">
@@ -8715,49 +8715,49 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>60903</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>SniperBot EURUSD</t>
         </is>
       </c>
       <c r="D209" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>662436</t>
+          <t>60904</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+          <t>TokioDrifter</t>
         </is>
       </c>
       <c r="D210" t="b">
@@ -8765,39 +8765,39 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>662437</t>
+          <t>60905</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Gold Talon V1.2</t>
+          <t>Tokyo Drive</t>
         </is>
       </c>
       <c r="D211" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>663097</t>
+          <t>60907</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -8807,7 +8807,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+          <t>October Demos (live mirror, all strategies)</t>
         </is>
       </c>
       <c r="D212" t="b">
@@ -8815,14 +8815,14 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>1115442</t>
+          <t>60908</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -8832,7 +8832,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Gold Snap Internal</t>
+          <t>SK Stochastic</t>
         </is>
       </c>
       <c r="D213" t="b">
@@ -8840,14 +8840,14 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>1115443</t>
+          <t>60909</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -8857,57 +8857,57 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta MOL</t>
+          <t>SK Stochastic (MasterLive demo)</t>
         </is>
       </c>
       <c r="D214" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS242t3</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>1115444</t>
+          <t>639884</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Gold Snap Demo</t>
+          <t>Manual Trading (Diego)</t>
         </is>
       </c>
       <c r="D215" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>VPS204</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14189968</t>
+          <t>647832</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+          <t>Axis Rotation AUDUSD</t>
         </is>
       </c>
       <c r="D216" t="b">
@@ -8915,53 +8915,53 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>26774273</t>
+          <t>657902</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>The5ers $200k Challenge</t>
+          <t>T&amp;D19</t>
         </is>
       </c>
       <c r="D217" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>52428953</t>
+          <t>658071</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>BTC Dual Breakout Scalper</t>
+          <t>T&amp;D V1</t>
         </is>
       </c>
       <c r="D218" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -8972,17 +8972,17 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>52441850</t>
+          <t>662434</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>EA Fx RSI MOL</t>
+          <t>LIVE Gold Reaper Conservative</t>
         </is>
       </c>
       <c r="D219" t="b">
@@ -8990,55 +8990,330 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>52441853</t>
+          <t>662435</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Fx RSI Low DD Prop Firms</t>
+          <t>Aggv1 Pro Filter 60</t>
         </is>
       </c>
       <c r="D220" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
+          <t>662436</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
+        </is>
+      </c>
+      <c r="D221" t="b">
+        <v>1</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>662437</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Gold Talon V1.2</t>
+        </is>
+      </c>
+      <c r="D222" t="b">
+        <v>0</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>663097</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
+        </is>
+      </c>
+      <c r="D223" t="b">
+        <v>1</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>VPS149</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>1115442</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Gold Snap Internal</t>
+        </is>
+      </c>
+      <c r="D224" t="b">
+        <v>1</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>1115443</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta MOL</t>
+        </is>
+      </c>
+      <c r="D225" t="b">
+        <v>0</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>1115444</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Gold Snap Demo</t>
+        </is>
+      </c>
+      <c r="D226" t="b">
+        <v>1</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>14189968</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
+        </is>
+      </c>
+      <c r="D227" t="b">
+        <v>0</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>26774273</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>The5ers $200k Challenge</t>
+        </is>
+      </c>
+      <c r="D228" t="b">
+        <v>1</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>52428953</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>BTC Dual Breakout Scalper</t>
+        </is>
+      </c>
+      <c r="D229" t="b">
+        <v>1</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>52441850</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>EA Fx RSI MOL</t>
+        </is>
+      </c>
+      <c r="D230" t="b">
+        <v>1</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>52441853</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Fx RSI Low DD Prop Firms</t>
+        </is>
+      </c>
+      <c r="D231" t="b">
+        <v>1</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
           <t>600025868</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
+      <c r="B232" t="inlineStr">
         <is>
           <t>prop</t>
         </is>
       </c>
-      <c r="C221" t="inlineStr">
+      <c r="C232" t="inlineStr">
         <is>
           <t>FTMO Manual Trading</t>
         </is>
       </c>
-      <c r="D221" t="b">
-        <v>1</v>
-      </c>
-      <c r="E221" t="inlineStr">
+      <c r="D232" t="b">
+        <v>1</v>
+      </c>
+      <c r="E232" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>

</xml_diff>

<commit_message>
Update dashboards — 2026-10-23
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-22 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-23 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/22/2026 18:37</t>
+          <t>10/24/2026 00:02</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>28380.11</v>
+        <v>23884.83</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>13.52</v>
+        <v>-4.46</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
-      <c r="K2" s="7" t="n">
-        <v>1.01</v>
+      <c r="K2" t="n">
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-21065.79</v>
+        <v>-26819.04</v>
       </c>
       <c r="P2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>70</v>
+        <v>67.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.6407922293305123</v>
+        <v>0.5779481502860518</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>108.79</v>
+        <v>114.13</v>
       </c>
       <c r="T2" t="n">
-        <v>3510</v>
+        <v>3511</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>3380.110000000002</v>
+        <v>-1115.169999999996</v>
       </c>
       <c r="V2" t="n">
-        <v>2236</v>
+        <v>2237</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.70370370370371</v>
+        <v>63.71404158359442</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/22/2026 19:13</t>
+          <t>10/23/2026 13:19</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1178,20 +1178,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/22/2026 23:21</t>
+          <t>10/23/2026 22:31</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>20547.61</v>
+        <v>20534.05</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>2.77</v>
+        <v>2.7</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1203,7 +1203,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>-45.9</v>
+        <v>-55.27</v>
       </c>
       <c r="P4" t="n">
         <v>13</v>
@@ -1212,25 +1212,25 @@
         <v>32.5</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>0.837291740517547</v>
+        <v>0.8103749957113939</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.75</v>
       </c>
       <c r="T4" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>547.61</v>
+        <v>534.05</v>
       </c>
       <c r="V4" t="n">
         <v>36</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>28.34645669291339</v>
+        <v>28.125</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="Y4" s="7" t="n">
         <v>1.83</v>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1287,20 +1287,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/22/2026 17:51</t>
+          <t>10/23/2026 23:28</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>19886.06</v>
+        <v>20047.72</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.24</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.37</v>
       </c>
-      <c r="K5" s="7" t="n">
-        <v>0.99</v>
+      <c r="K5" t="n">
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>20000</v>
@@ -1312,34 +1312,34 @@
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>-1132.47</v>
+        <v>-359.0700000000001</v>
       </c>
       <c r="P5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>27.5</v>
+        <v>32.5</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>0.7491638573751103</v>
+        <v>0.9098855594037042</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>11.5</v>
+        <v>11.18</v>
       </c>
       <c r="T5" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>-113.9400000000007</v>
+        <v>47.71999999999927</v>
       </c>
       <c r="V5" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>31.19266055045872</v>
+        <v>32.43243243243244</v>
       </c>
       <c r="X5" s="7" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="Y5" s="7" t="n">
         <v>11.37</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1505,20 +1505,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/22/2026 17:54</t>
+          <t>10/23/2026 23:31</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>19888.68</v>
+        <v>19919.01</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.41</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="L7" t="n">
         <v>20000</v>
@@ -1530,34 +1530,34 @@
         <v>40</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>-553.03</v>
+        <v>-165</v>
       </c>
       <c r="P7" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q7" s="7" t="n">
-        <v>75</v>
+        <v>82.5</v>
       </c>
       <c r="R7" s="7" t="n">
-        <v>0.4285758568314028</v>
+        <v>0.7295569651374343</v>
       </c>
       <c r="S7" s="7" t="n">
-        <v>3.18</v>
+        <v>1.55</v>
       </c>
       <c r="T7" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>-111.3200000000001</v>
+        <v>-80.99000000000007</v>
       </c>
       <c r="V7" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="W7" s="7" t="n">
-        <v>82.16216216216216</v>
+        <v>82.88770053475936</v>
       </c>
       <c r="X7" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="Y7" s="7" t="n">
         <v>4.49</v>
@@ -1723,20 +1723,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/23/2026 00:13</t>
+          <t>10/23/2026 23:17</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>28132.05</v>
+        <v>28140.15</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>40.73</v>
+        <v>40.77</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1.65</v>
+        <v>1.64</v>
       </c>
       <c r="L9" t="n">
         <v>20000</v>
@@ -1748,34 +1748,34 @@
         <v>40</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>1307.94</v>
+        <v>1114.02</v>
       </c>
       <c r="P9" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>1.53896109247645</v>
+        <v>1.423955732813737</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>6.09</v>
+        <v>6.15</v>
       </c>
       <c r="T9" t="n">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>8480.23</v>
+        <v>8140.149999999999</v>
       </c>
       <c r="V9" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>67.15686274509804</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X9" s="7" t="n">
-        <v>1.7</v>
+        <v>1.64</v>
       </c>
       <c r="Y9" s="7" t="n">
         <v>5.25</v>
@@ -1832,20 +1832,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/22/2026 19:07</t>
+          <t>10/23/2026 13:15</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>21244.87</v>
+        <v>21450.49</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>6.22</v>
+        <v>7.25</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>4.96</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.46</v>
+        <v>1.53</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1857,37 +1857,37 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>471.6900000000001</v>
+        <v>716.45</v>
       </c>
       <c r="P10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>1.200636333088045</v>
+        <v>1.309906005199344</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>5.14</v>
+        <v>5.13</v>
       </c>
       <c r="T10" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>1450.490000000001</v>
+        <v>1103.56</v>
       </c>
       <c r="V10" t="n">
         <v>24</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>43.63636363636363</v>
+        <v>42.10526315789473</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.53</v>
+        <v>1.36</v>
       </c>
       <c r="Y10" s="7" t="n">
-        <v>4.96</v>
+        <v>5.59</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/22/2026 18:46</t>
+          <t>10/23/2026 12:57</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/22/2026 18:45</t>
+          <t>10/23/2026 12:56</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2093,7 +2093,7 @@
         <v>31</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>-222.8799999999999</v>
+        <v>-237.1099999999999</v>
       </c>
       <c r="V12" t="n">
         <v>9</v>
@@ -2102,10 +2102,10 @@
         <v>29.03225806451613</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="Y12" s="7" t="n">
-        <v>1.43</v>
+        <v>1.5</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -2159,20 +2159,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/22/2026 19:06</t>
+          <t>10/23/2026 13:16</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>20335.86</v>
+        <v>20592.45</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1.69</v>
+        <v>2.97</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>4.44</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1.18</v>
+        <v>1.3</v>
       </c>
       <c r="L13" t="n">
         <v>20000</v>
@@ -2181,37 +2181,37 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>20086.31</v>
+        <v>20346.15</v>
       </c>
       <c r="P13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>20</v>
+        <v>22.22222222222222</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>11.87898761874844</v>
+        <v>11.37899424583741</v>
       </c>
       <c r="S13" s="7" t="n">
         <v>2.22</v>
       </c>
       <c r="T13" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>335.86</v>
+        <v>460.04</v>
       </c>
       <c r="V13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>16</v>
+        <v>17.85714285714286</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>1.18</v>
+        <v>1.22</v>
       </c>
       <c r="Y13" s="7" t="n">
         <v>4.44</v>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/22/2026 18:58</t>
+          <t>10/23/2026 13:06</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/22/2026 18:52</t>
+          <t>10/23/2026 13:02</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/22/2026 18:52</t>
+          <t>10/23/2026 13:02</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/22/2026 18:48</t>
+          <t>10/23/2026 12:59</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,20 +2704,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/22/2026 19:00</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="n">
-        <v>20014.4</v>
+          <t>10/23/2026 07:12</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>20019</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>0.02</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>6.54</v>
+        <v>8.31</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2726,19 +2726,19 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
+        <v>6</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>20019</v>
+      </c>
+      <c r="P18" t="n">
         <v>5</v>
       </c>
-      <c r="O18" s="7" t="n">
-        <v>20014.4</v>
-      </c>
-      <c r="P18" t="n">
-        <v>4</v>
-      </c>
       <c r="Q18" s="7" t="n">
-        <v>80</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>7698.846153846153</v>
+        <v>7700.615384615384</v>
       </c>
       <c r="S18" s="7" t="n">
         <v>0.01</v>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/22/2026 18:53</t>
+          <t>10/23/2026 13:04</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,20 +2922,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/22/2026 18:55</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>19815</v>
+          <t>10/23/2026 13:04</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>19832.4</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>-0.92</v>
+        <v>-0.83</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>2.41</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="L20" t="n">
         <v>20000</v>
@@ -2944,19 +2944,19 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>19815</v>
+        <v>19832.4</v>
       </c>
       <c r="P20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>61.11111111111111</v>
+        <v>63.1578947368421</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>38.41503021148036</v>
+        <v>38.44788519637462</v>
       </c>
       <c r="S20" s="7" t="n">
         <v>1.2</v>
@@ -2965,16 +2965,16 @@
         <v>18</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-185</v>
+        <v>-167.6</v>
       </c>
       <c r="V20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>55.55555555555556</v>
+        <v>61.11111111111111</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="Y20" s="7" t="n">
         <v>2.41</v>
@@ -2986,12 +2986,12 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/22/2026 19:02</t>
+          <t>10/23/2026 13:10</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3041,7 +3041,7 @@
         <v>0.05</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.29</v>
+        <v>0.36</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -3134,20 +3134,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/22/2026 19:04</t>
+          <t>10/23/2026 13:13</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>20087.47</v>
+        <v>20144.45</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.43</v>
+        <v>0.71</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>0.33</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>1.89</v>
+        <v>2.46</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3156,37 +3156,37 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>20064.83</v>
+        <v>20111.97</v>
       </c>
       <c r="P22" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>47.36842105263158</v>
+        <v>59.25925925925925</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>179.9106553722693</v>
+        <v>178.5264365786919</v>
       </c>
       <c r="S22" s="7" t="n">
         <v>0.18</v>
       </c>
       <c r="T22" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>144.45</v>
+        <v>153.85</v>
       </c>
       <c r="V22" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>61.53846153846154</v>
+        <v>60</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>2.46</v>
+        <v>2.54</v>
       </c>
       <c r="Y22" s="7" t="n">
         <v>0.32</v>
@@ -3243,20 +3243,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/22/2026 21:04</t>
+          <t>10/23/2026 16:01</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>12624.48</v>
+        <v>12799.62</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>26.18</v>
+        <v>27.93</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>2.07</v>
+        <v>2.14</v>
       </c>
       <c r="L23" t="n">
         <v>10000</v>
@@ -3268,7 +3268,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>886.41</v>
+        <v>954.4899999999999</v>
       </c>
       <c r="P23" t="n">
         <v>28</v>
@@ -3277,25 +3277,25 @@
         <v>70</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.574941300089509</v>
+        <v>1.61909919960564</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>3.84</v>
+        <v>3.87</v>
       </c>
       <c r="T23" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>2579.68</v>
+        <v>2754.82</v>
       </c>
       <c r="V23" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>70.52631578947368</v>
+        <v>70.83333333333334</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>2.03</v>
+        <v>2.1</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>3.36</v>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards — 2026-10-26
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-23 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-26 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -748,12 +748,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/24/2026 00:02</t>
+          <t>10/27/2026 00:38</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>23884.83</v>
+        <v>22079.79</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>-4.46</v>
+        <v>-11.68</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-26819.04</v>
+        <v>-12843.87</v>
       </c>
       <c r="P2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>67.5</v>
+        <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.5779481502860518</v>
+        <v>0.7557693514435502</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>114.13</v>
+        <v>66.78</v>
       </c>
       <c r="T2" t="n">
-        <v>3511</v>
+        <v>3514</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>-1115.169999999996</v>
+        <v>-2920.209999999994</v>
       </c>
       <c r="V2" t="n">
-        <v>2237</v>
+        <v>2239</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.71404158359442</v>
+        <v>63.71656232214001</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/23/2026 13:19</t>
+          <t>10/27/2026 01:03</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/23/2026 22:31</t>
+          <t>10/26/2026 23:13</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,14 +1287,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/23/2026 23:28</t>
+          <t>10/27/2026 00:07</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>20047.72</v>
+        <v>19967.72</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.24</v>
+        <v>-0.16</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.37</v>
@@ -1312,31 +1312,31 @@
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>-359.0700000000001</v>
+        <v>-1035.12</v>
       </c>
       <c r="P5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>0.9098855594037042</v>
+        <v>0.7453328740835506</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>11.18</v>
+        <v>11.5</v>
       </c>
       <c r="T5" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>47.71999999999927</v>
+        <v>-32.2800000000002</v>
       </c>
       <c r="V5" t="n">
         <v>36</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>32.43243243243244</v>
+        <v>32.14285714285715</v>
       </c>
       <c r="X5" s="7" t="n">
         <v>1</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/22/2026 15:11</t>
+          <t>10/25/2026 15:14</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/23/2026 23:31</t>
+          <t>10/27/2026 00:08</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>19919.01</v>
+        <v>19937.1</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>-0.41</v>
+        <v>-0.32</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>4.48</v>
@@ -1530,31 +1530,31 @@
         <v>40</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>-165</v>
+        <v>-55.69</v>
       </c>
       <c r="P7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q7" s="7" t="n">
-        <v>82.5</v>
+        <v>85</v>
       </c>
       <c r="R7" s="7" t="n">
-        <v>0.7295569651374343</v>
+        <v>0.8907417943536521</v>
       </c>
       <c r="S7" s="7" t="n">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="T7" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>-80.99000000000007</v>
+        <v>-62.90000000000003</v>
       </c>
       <c r="V7" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="W7" s="7" t="n">
-        <v>82.88770053475936</v>
+        <v>83.06878306878306</v>
       </c>
       <c r="X7" s="7" t="n">
         <v>0.98</v>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1723,20 +1723,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/23/2026 23:17</t>
+          <t>10/26/2026 23:56</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>28140.15</v>
+        <v>28178.43</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>40.77</v>
+        <v>40.96</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1.64</v>
+        <v>1.63</v>
       </c>
       <c r="L9" t="n">
         <v>20000</v>
@@ -1748,7 +1748,7 @@
         <v>40</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>1114.02</v>
+        <v>840.8099999999999</v>
       </c>
       <c r="P9" t="n">
         <v>24</v>
@@ -1757,25 +1757,25 @@
         <v>60</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>1.423955732813737</v>
+        <v>1.312410825753522</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>6.15</v>
+        <v>6.24</v>
       </c>
       <c r="T9" t="n">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>8140.149999999999</v>
+        <v>7864.549999999999</v>
       </c>
       <c r="V9" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>66.35071090047393</v>
       </c>
       <c r="X9" s="7" t="n">
-        <v>1.64</v>
+        <v>1.59</v>
       </c>
       <c r="Y9" s="7" t="n">
         <v>5.25</v>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1832,20 +1832,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/23/2026 13:15</t>
+          <t>10/26/2026 14:17</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>21450.49</v>
+        <v>21103.56</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>7.25</v>
+        <v>5.52</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>4.96</v>
+        <v>5.6</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.53</v>
+        <v>1.36</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1857,37 +1857,37 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>716.45</v>
+        <v>337.83</v>
       </c>
       <c r="P10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>1.309906005199344</v>
+        <v>1.129336186797242</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>5.13</v>
+        <v>5.79</v>
       </c>
       <c r="T10" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>1103.56</v>
+        <v>1015.59</v>
       </c>
       <c r="V10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>42.10526315789473</v>
+        <v>42.3728813559322</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.36</v>
+        <v>1.32</v>
       </c>
       <c r="Y10" s="7" t="n">
-        <v>5.59</v>
+        <v>6.01</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/23/2026 12:57</t>
+          <t>10/27/2026 00:42</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,20 +2050,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/23/2026 12:56</t>
+          <t>10/27/2026 00:39</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>19777.12</v>
+        <v>19762.89</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>-1.11</v>
+        <v>-1.18</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1.43</v>
+        <v>1.5</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2072,22 +2072,22 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>19725.13</v>
+        <v>19710.67</v>
       </c>
       <c r="P12" t="n">
         <v>10</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>32.25806451612903</v>
+        <v>31.25</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>27.62571710108931</v>
+        <v>27.096823736578</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="T12" t="n">
         <v>31</v>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
@@ -2159,20 +2159,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/23/2026 13:16</t>
+          <t>10/27/2026 01:02</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>20592.45</v>
+        <v>20326.83</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>2.97</v>
+        <v>1.64</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>4.44</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1.3</v>
+        <v>1.15</v>
       </c>
       <c r="L13" t="n">
         <v>20000</v>
@@ -2181,37 +2181,37 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>20346.15</v>
+        <v>20080.53</v>
       </c>
       <c r="P13" t="n">
         <v>6</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>22.22222222222222</v>
+        <v>20.68965517241379</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>11.37899424583741</v>
+        <v>10.021146122537</v>
       </c>
       <c r="S13" s="7" t="n">
         <v>2.22</v>
       </c>
       <c r="T13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>460.04</v>
+        <v>326.8299999999999</v>
       </c>
       <c r="V13" t="n">
         <v>5</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>17.85714285714286</v>
+        <v>17.24137931034483</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>1.22</v>
+        <v>1.15</v>
       </c>
       <c r="Y13" s="7" t="n">
         <v>4.44</v>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/23/2026 13:06</t>
+          <t>10/27/2026 00:50</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/23/2026 13:02</t>
+          <t>10/27/2026 00:47</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/23/2026 13:02</t>
+          <t>10/27/2026 00:47</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,20 +2595,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/23/2026 12:59</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>19947.8</v>
+          <t>10/27/2026 00:44</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>19844</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-0.26</v>
+        <v>-0.78</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.84</v>
+        <v>1.21</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>0.8</v>
+        <v>0.57</v>
       </c>
       <c r="L17" t="n">
         <v>20000</v>
@@ -2617,28 +2617,28 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>19947.8</v>
+        <v>19844</v>
       </c>
       <c r="P17" t="n">
         <v>3</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>37.5</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>78.31705426356589</v>
+        <v>55.84798231066888</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>0.42</v>
+        <v>0.61</v>
       </c>
       <c r="T17" t="n">
         <v>7</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-52.19999999999998</v>
+        <v>-156</v>
       </c>
       <c r="V17" t="n">
         <v>2</v>
@@ -2647,10 +2647,10 @@
         <v>28.57142857142857</v>
       </c>
       <c r="X17" s="7" t="n">
-        <v>0.8</v>
+        <v>0.57</v>
       </c>
       <c r="Y17" s="7" t="n">
-        <v>0.84</v>
+        <v>1.21</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2659,12 +2659,12 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2704,20 +2704,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/23/2026 07:12</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>20019</v>
+          <t>10/27/2026 00:53</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>20024.4</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>0.02</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>8.31</v>
+        <v>10.38</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2726,37 +2726,37 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
+        <v>7</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>20024.4</v>
+      </c>
+      <c r="P18" t="n">
         <v>6</v>
       </c>
-      <c r="O18" s="7" t="n">
-        <v>20019</v>
-      </c>
-      <c r="P18" t="n">
-        <v>5</v>
-      </c>
       <c r="Q18" s="7" t="n">
-        <v>83.33333333333334</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>7700.615384615384</v>
+        <v>7702.692307692308</v>
       </c>
       <c r="S18" s="7" t="n">
         <v>0.01</v>
       </c>
       <c r="T18" t="n">
+        <v>6</v>
+      </c>
+      <c r="U18" s="7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="V18" t="n">
         <v>5</v>
       </c>
-      <c r="U18" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="V18" t="n">
-        <v>4</v>
-      </c>
       <c r="W18" s="7" t="n">
-        <v>80</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>8.31</v>
+        <v>10.38</v>
       </c>
       <c r="Y18" s="7" t="n">
         <v>0.01</v>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/23/2026 13:04</t>
+          <t>10/26/2026 14:05</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,20 +2922,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/23/2026 13:04</t>
+          <t>10/27/2026 00:46</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>19832.4</v>
+        <v>19848.6</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>-0.83</v>
+        <v>-0.75</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>2.41</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="L20" t="n">
         <v>20000</v>
@@ -2944,37 +2944,37 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>19832.4</v>
+        <v>19848.6</v>
       </c>
       <c r="P20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>63.1578947368421</v>
+        <v>65</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>38.44788519637462</v>
+        <v>38.47847432024169</v>
       </c>
       <c r="S20" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="T20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-167.6</v>
+        <v>-151.4</v>
       </c>
       <c r="V20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>61.11111111111111</v>
+        <v>63.1578947368421</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="Y20" s="7" t="n">
         <v>2.41</v>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/23/2026 13:10</t>
+          <t>10/27/2026 00:54</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3106,7 +3106,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>60570</t>
+          <t>60569</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EURO Overnight</t>
+          <t>Demo Dream Catcher Portfolio</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS92t2</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -3134,20 +3134,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/23/2026 13:13</t>
+          <t>10/26/2026 15:41</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>20144.45</v>
+        <v>19996.67</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.71</v>
+        <v>0</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="K22" s="7" t="n">
-        <v>2.46</v>
+        <v>6.97</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3156,49 +3156,49 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>20111.97</v>
+        <v>19958.47</v>
       </c>
       <c r="P22" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>59.25925925925925</v>
+        <v>50</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>178.5264365786919</v>
+        <v>8.528486718520139</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>0.18</v>
+        <v>3.56</v>
       </c>
       <c r="T22" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>153.85</v>
+        <v>-341.03</v>
       </c>
       <c r="V22" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>60</v>
+        <v>41.93548387096774</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>2.54</v>
+        <v>0.88</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>0.32</v>
+        <v>6.97</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3208,207 +3208,1454 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>EURO Overnight | AUDCAD, EURO Overnight | AUDUSD, EURO Overnight | EURAUD, EURO Overnight | EURGBP, EURO Overnight | EURUSD, EURO Overnight | GBPUSD, EURO Overnight | NZDUSD, EURO Overnight | USDCAD, EURO Overnight | USDCHF</t>
+          <t>Demo Dream Catcher Portfolio | AUDJPY, Demo Dream Catcher Portfolio | USDJPY, Demo Dream Catcher Portfolio | USTECH</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>60570</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EURO Overnight</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TradeSmart-Server01</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+      <c r="F23" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10/27/2026 00:59</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>20089.17</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="L23" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>32</v>
+      </c>
+      <c r="O23" s="7" t="n">
+        <v>20053.09</v>
+      </c>
+      <c r="P23" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q23" s="7" t="n">
+        <v>56.25</v>
+      </c>
+      <c r="R23" s="7" t="n">
+        <v>111.6865927029861</v>
+      </c>
+      <c r="S23" s="7" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="T23" t="n">
+        <v>31</v>
+      </c>
+      <c r="U23" s="7" t="n">
+        <v>89.16999999999999</v>
+      </c>
+      <c r="V23" t="n">
+        <v>18</v>
+      </c>
+      <c r="W23" s="7" t="n">
+        <v>58.06451612903226</v>
+      </c>
+      <c r="X23" s="7" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="Y23" s="7" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>EURO Overnight | AUDCAD, EURO Overnight | AUDUSD, EURO Overnight | EURAUD, EURO Overnight | EURGBP, EURO Overnight | EURUSD, EURO Overnight | GBPUSD, EURO Overnight | NZDUSD, EURO Overnight | USDCAD, EURO Overnight | USDCHF</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>60898</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BlackDog</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:51</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>20006.2</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" s="7" t="n">
+        <v>20005.4</v>
+      </c>
+      <c r="P24" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q24" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1</v>
+      </c>
+      <c r="U24" s="7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="V24" t="n">
+        <v>1</v>
+      </c>
+      <c r="W24" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>BlackDog | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>60899</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AMStocktastic</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:50</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" s="7" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>AMStocktastic | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>60900</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Finex</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:53</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>20013.43</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>2</v>
+      </c>
+      <c r="O26" s="7" t="n">
+        <v>20013.43</v>
+      </c>
+      <c r="P26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q26" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>2</v>
+      </c>
+      <c r="U26" s="7" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="V26" t="n">
+        <v>2</v>
+      </c>
+      <c r="W26" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Finex | EURCHF, Finex | EURGBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>60901</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>USAPattern5</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:55</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>19997.2</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>1</v>
+      </c>
+      <c r="U27" s="7" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>USAPattern5 | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>60902</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CyberZ</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F28" t="b">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:58</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>19921.43</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2</v>
+      </c>
+      <c r="O28" s="7" t="n">
+        <v>19921.43</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R28" s="7" t="n">
+        <v>254.5500827287769</v>
+      </c>
+      <c r="S28" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="T28" t="n">
+        <v>2</v>
+      </c>
+      <c r="U28" s="7" t="n">
+        <v>-78.56999999999999</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="7" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>CyberZ | USDJPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>60903</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SniperBot EURUSD</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:58</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>19993.4</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>2</v>
+      </c>
+      <c r="O29" s="7" t="n">
+        <v>19992.6</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R29" s="7" t="n">
+        <v>2702.702702702703</v>
+      </c>
+      <c r="S29" s="7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T29" t="n">
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="n">
+        <v>-6.6</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>SniperBot EURUSD | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>60905</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Tokyo Drive</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>10/26/2026 15:04</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>19981.75</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K30" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L30" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>3</v>
+      </c>
+      <c r="O30" s="7" t="n">
+        <v>19980.95</v>
+      </c>
+      <c r="P30" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q30" s="7" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="R30" s="7" t="n">
+        <v>559.5951915012581</v>
+      </c>
+      <c r="S30" s="7" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="T30" t="n">
+        <v>3</v>
+      </c>
+      <c r="U30" s="7" t="n">
+        <v>7.030000000000001</v>
+      </c>
+      <c r="V30" t="n">
+        <v>2</v>
+      </c>
+      <c r="W30" s="7" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="X30" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="Y30" s="7" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Tokyo Drive | USDJPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>60907</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>October Demos (live mirror, all strategies)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>10/26/2026 15:02</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>996.65</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>7</v>
+      </c>
+      <c r="O31" s="7" t="n">
+        <v>996.21</v>
+      </c>
+      <c r="P31" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q31" s="7" t="n">
+        <v>57.14285714285714</v>
+      </c>
+      <c r="R31" s="7" t="n">
+        <v>132.7738095238095</v>
+      </c>
+      <c r="S31" s="7" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="T31" t="n">
+        <v>12</v>
+      </c>
+      <c r="U31" s="7" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="V31" t="n">
+        <v>5</v>
+      </c>
+      <c r="W31" s="7" t="n">
+        <v>41.66666666666667</v>
+      </c>
+      <c r="X31" s="7" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="Y31" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>October Demos (live mirror, all strategies) | EURCHF, October Demos (live mirror, all strategies) | EURGBP, October Demos (live mirror, all strategies) | EURUSD, October Demos (live mirror, all strategies) | USDJPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>60909</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SK Stochastic (MasterLive demo)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>10/26/2026 15:00</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>1</v>
+      </c>
+      <c r="U32" s="7" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>SK Stochastic (MasterLive demo) | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>1115445</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>licensed</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Smart Gold Hunter</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>OX Securities</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>VPS242t2</t>
         </is>
       </c>
-      <c r="F23" t="b">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>10/23/2026 16:01</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="n">
-        <v>12799.62</v>
-      </c>
-      <c r="I23" s="7" t="n">
-        <v>27.93</v>
-      </c>
-      <c r="J23" s="7" t="n">
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>10/26/2026 21:11</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>12885.3</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>28.79</v>
+      </c>
+      <c r="J33" s="7" t="n">
         <v>3.38</v>
       </c>
-      <c r="K23" s="7" t="n">
+      <c r="K33" s="7" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="L33" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>40</v>
+      </c>
+      <c r="O33" s="7" t="n">
+        <v>994.3299999999999</v>
+      </c>
+      <c r="P33" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q33" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="R33" s="7" t="n">
+        <v>1.644940132577478</v>
+      </c>
+      <c r="S33" s="7" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="T33" t="n">
+        <v>97</v>
+      </c>
+      <c r="U33" s="7" t="n">
+        <v>2840.5</v>
+      </c>
+      <c r="V33" t="n">
+        <v>69</v>
+      </c>
+      <c r="W33" s="7" t="n">
+        <v>71.1340206185567</v>
+      </c>
+      <c r="X33" s="7" t="n">
         <v>2.14</v>
       </c>
-      <c r="L23" t="n">
-        <v>10000</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>40</v>
-      </c>
-      <c r="O23" s="7" t="n">
-        <v>954.4899999999999</v>
-      </c>
-      <c r="P23" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q23" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="R23" s="7" t="n">
-        <v>1.61909919960564</v>
-      </c>
-      <c r="S23" s="7" t="n">
-        <v>3.87</v>
-      </c>
-      <c r="T23" t="n">
-        <v>96</v>
-      </c>
-      <c r="U23" s="7" t="n">
-        <v>2754.82</v>
-      </c>
-      <c r="V23" t="n">
-        <v>68</v>
-      </c>
-      <c r="W23" s="7" t="n">
-        <v>70.83333333333334</v>
-      </c>
-      <c r="X23" s="7" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="Y23" s="7" t="n">
+      <c r="Y33" s="7" t="n">
         <v>3.36</v>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="Z33" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
         <is>
           <t>RECONCILE</t>
         </is>
       </c>
-      <c r="AC23" t="inlineStr">
+      <c r="AC33" t="inlineStr">
         <is>
           <t>Smart Gold Hunter | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>58989</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>TSma4f AUDCAD</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>TradeSmart</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>VPS92</t>
         </is>
       </c>
-      <c r="F24" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="F34" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>10/20/2026 23:29</t>
         </is>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H34" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="I24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="8" t="n">
+      <c r="I34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="M24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" s="9" t="n">
+      <c r="M34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="P24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="9" t="n">
+      <c r="P34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="R24" s="8" t="n"/>
-      <c r="S24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" s="8" t="n"/>
-      <c r="X24" s="8" t="n"/>
-      <c r="Y24" s="8" t="n"/>
-      <c r="Z24" s="8" t="n"/>
-      <c r="AA24" s="8" t="n"/>
-      <c r="AB24" s="8" t="inlineStr">
+      <c r="R34" s="8" t="n"/>
+      <c r="S34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="8" t="n"/>
+      <c r="X34" s="8" t="n"/>
+      <c r="Y34" s="8" t="n"/>
+      <c r="Z34" s="8" t="n"/>
+      <c r="AA34" s="8" t="n"/>
+      <c r="AB34" s="8" t="inlineStr">
         <is>
           <t>DATA GAP - Bach missing</t>
         </is>
       </c>
-      <c r="AC24" s="8" t="inlineStr"/>
+      <c r="AC34" s="8" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>60904</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>TokioDrifter</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:57</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="R35" s="8" t="n"/>
+      <c r="S35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="8" t="n"/>
+      <c r="X35" s="8" t="n"/>
+      <c r="Y35" s="8" t="n"/>
+      <c r="Z35" s="8" t="n"/>
+      <c r="AA35" s="8" t="n"/>
+      <c r="AB35" s="8" t="inlineStr">
+        <is>
+          <t>DATA GAP - Bach missing</t>
+        </is>
+      </c>
+      <c r="AC35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>60908</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>SK Stochastic</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>10/26/2026 15:00</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="R36" s="8" t="n"/>
+      <c r="S36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="8" t="n"/>
+      <c r="X36" s="8" t="n"/>
+      <c r="Y36" s="8" t="n"/>
+      <c r="Z36" s="8" t="n"/>
+      <c r="AA36" s="8" t="n"/>
+      <c r="AB36" s="8" t="inlineStr">
+        <is>
+          <t>DATA GAP - Bach missing</t>
+        </is>
+      </c>
+      <c r="AC36" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3421,7 +4668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3538,6 +4785,88 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>60904</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TokioDrifter</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10/26/2026 14:57</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>60908</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SK Stochastic</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>10/26/2026 15:00</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3549,7 +4878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:E220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8522,7 +9851,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>60569</t>
+          <t>60572</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -8532,7 +9861,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Demo Dream Catcher Portfolio</t>
+          <t>Portfolio DC FT Luna</t>
         </is>
       </c>
       <c r="D201" t="b">
@@ -8547,7 +9876,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>60572</t>
+          <t>60575</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -8557,7 +9886,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Portfolio DC FT Luna</t>
+          <t>ML_POC</t>
         </is>
       </c>
       <c r="D202" t="b">
@@ -8565,124 +9894,124 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>60575</t>
+          <t>639884</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>ML_POC</t>
+          <t>Manual Trading (Diego)</t>
         </is>
       </c>
       <c r="D203" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>60898</t>
+          <t>647832</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>BlackDog</t>
+          <t>Axis Rotation AUDUSD</t>
         </is>
       </c>
       <c r="D204" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS242</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>60899</t>
+          <t>657902</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>AMStocktastic</t>
+          <t>T&amp;D19</t>
         </is>
       </c>
       <c r="D205" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS153</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>60900</t>
+          <t>658071</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Finex</t>
+          <t>T&amp;D V1</t>
         </is>
       </c>
       <c r="D206" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>60901</t>
+          <t>662434</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>USAPattern5</t>
+          <t>LIVE Gold Reaper Conservative</t>
         </is>
       </c>
       <c r="D207" t="b">
@@ -8690,49 +10019,49 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>60902</t>
+          <t>662435</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>CyberZ</t>
+          <t>Aggv1 Pro Filter 60</t>
         </is>
       </c>
       <c r="D208" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>60903</t>
+          <t>662436</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>SniperBot EURUSD</t>
+          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
         </is>
       </c>
       <c r="D209" t="b">
@@ -8740,49 +10069,49 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>60904</t>
+          <t>662437</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>TokioDrifter</t>
+          <t>Gold Talon V1.2</t>
         </is>
       </c>
       <c r="D210" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>60905</t>
+          <t>663097</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Tokyo Drive</t>
+          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
         </is>
       </c>
       <c r="D211" t="b">
@@ -8790,24 +10119,24 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS149</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>60907</t>
+          <t>1115442</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>October Demos (live mirror, all strategies)</t>
+          <t>Gold Snap Internal</t>
         </is>
       </c>
       <c r="D212" t="b">
@@ -8815,14 +10144,14 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>60908</t>
+          <t>1115443</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -8832,22 +10161,22 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>SK Stochastic</t>
+          <t>T&amp;D19L13 Meta MOL</t>
         </is>
       </c>
       <c r="D213" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>60909</t>
+          <t>1115444</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -8857,7 +10186,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>SK Stochastic (MasterLive demo)</t>
+          <t>Gold Snap Demo</t>
         </is>
       </c>
       <c r="D214" t="b">
@@ -8865,24 +10194,24 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>639884</t>
+          <t>14189968</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Manual Trading (Diego)</t>
+          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
         </is>
       </c>
       <c r="D215" t="b">
@@ -8890,78 +10219,78 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>647832</t>
+          <t>26774273</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>prop</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Axis Rotation AUDUSD</t>
+          <t>The5ers $200k Challenge</t>
         </is>
       </c>
       <c r="D216" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92t2</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>657902</t>
+          <t>52428953</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>T&amp;D19</t>
+          <t>BTC Dual Breakout Scalper</t>
         </is>
       </c>
       <c r="D217" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>658071</t>
+          <t>52441850</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>T&amp;D V1</t>
+          <t>EA Fx RSI MOL</t>
         </is>
       </c>
       <c r="D218" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -8972,17 +10301,17 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>52441853</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>LIVE Gold Reaper Conservative</t>
+          <t>Fx RSI Low DD Prop Firms</t>
         </is>
       </c>
       <c r="D219" t="b">
@@ -8990,330 +10319,30 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS92</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>600025868</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>prop</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>FTMO Manual Trading</t>
         </is>
       </c>
       <c r="D220" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E220" t="inlineStr">
-        <is>
-          <t>VPS92t2</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>662436</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>LIVE Talon v2 multi-market (JPY crosses + XAUUSD)</t>
-        </is>
-      </c>
-      <c r="D221" t="b">
-        <v>1</v>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>VPS149</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>662437</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>Gold Talon V1.2</t>
-        </is>
-      </c>
-      <c r="D222" t="b">
-        <v>0</v>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>VPS92t2</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>663097</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>LIVE Gold Talon V2 (JPY crosses + XAGUSD)</t>
-        </is>
-      </c>
-      <c r="D223" t="b">
-        <v>1</v>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>VPS149</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>1115442</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>Gold Snap Internal</t>
-        </is>
-      </c>
-      <c r="D224" t="b">
-        <v>1</v>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>VPS204</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>1115443</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>T&amp;D19L13 Meta MOL</t>
-        </is>
-      </c>
-      <c r="D225" t="b">
-        <v>0</v>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>VPS204</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>1115444</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>Gold Snap Demo</t>
-        </is>
-      </c>
-      <c r="D226" t="b">
-        <v>1</v>
-      </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>VPS204</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>14189968</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>Prop Challenge - Gold Reaper (FundedNext)</t>
-        </is>
-      </c>
-      <c r="D227" t="b">
-        <v>0</v>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>VPS92t2</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>26774273</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>prop</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>The5ers $200k Challenge</t>
-        </is>
-      </c>
-      <c r="D228" t="b">
-        <v>1</v>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>VPS92t2</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>52428953</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>BTC Dual Breakout Scalper</t>
-        </is>
-      </c>
-      <c r="D229" t="b">
-        <v>1</v>
-      </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>52441850</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>EA Fx RSI MOL</t>
-        </is>
-      </c>
-      <c r="D230" t="b">
-        <v>1</v>
-      </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>52441853</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>Fx RSI Low DD Prop Firms</t>
-        </is>
-      </c>
-      <c r="D231" t="b">
-        <v>1</v>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>600025868</t>
-        </is>
-      </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>prop</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>FTMO Manual Trading</t>
-        </is>
-      </c>
-      <c r="D232" t="b">
-        <v>1</v>
-      </c>
-      <c r="E232" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -9330,13 +10359,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -9373,6 +10402,29 @@
         <is>
           <t>Balance</t>
         </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>60574</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>60574 Demo Yen Cross</t>
+        </is>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10/26/2026 18:23</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>50000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboards — 2026-10-28
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-27 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-28 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/27/2026 22:20</t>
+          <t>10/28/2026 22:20</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>27278.25</v>
+        <v>35934.69</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>9.109999999999999</v>
+        <v>43.74</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
+      <c r="K2" s="7" t="n">
+        <v>1.02</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>54.71999999999963</v>
+        <v>4512.919999999999</v>
       </c>
       <c r="P2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>77.5</v>
+        <v>80</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.001290732249955</v>
+        <v>1.120886329745073</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>51.62</v>
+        <v>58.55</v>
       </c>
       <c r="T2" t="n">
-        <v>3519</v>
+        <v>3526</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>2278.250000000002</v>
+        <v>10934.68999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2243</v>
+        <v>2250</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.73969877806195</v>
+        <v>63.8116846284742</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1069,14 +1069,14 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/27/2026 22:46</t>
+          <t>10/28/2026 22:47</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>20492.47</v>
+        <v>20471.49</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>2.47</v>
+        <v>2.36</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8.99</v>
@@ -1094,31 +1094,31 @@
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>-83.18999999999997</v>
+        <v>-251.18</v>
       </c>
       <c r="P3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.9221665013753486</v>
+        <v>0.7746173034474094</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>2.48</v>
+        <v>2.5</v>
       </c>
       <c r="T3" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>492.4699999999997</v>
+        <v>471.4899999999997</v>
       </c>
       <c r="V3" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>43.2258064516129</v>
+        <v>44.23076923076923</v>
       </c>
       <c r="X3" s="7" t="n">
         <v>1.07</v>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/27/2026 20:20</t>
+          <t>10/28/2026 20:40</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,20 +1287,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/27/2026 22:04</t>
+          <t>10/28/2026 22:07</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>19686.53</v>
+        <v>19695.65</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>-1.57</v>
+        <v>-1.52</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>5.13</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="L5" t="n">
         <v>20000</v>
@@ -1312,34 +1312,34 @@
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>-21.72000000000002</v>
+        <v>1.379999999999976</v>
       </c>
       <c r="P5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>52.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>0.9049369747899159</v>
+        <v>1.006588370094529</v>
       </c>
       <c r="S5" s="7" t="n">
         <v>0.87</v>
       </c>
       <c r="T5" t="n">
-        <v>922</v>
+        <v>924</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>-313.47</v>
+        <v>-304.35</v>
       </c>
       <c r="V5" t="n">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>54.55531453362256</v>
+        <v>54.65367965367965</v>
       </c>
       <c r="X5" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="Y5" s="7" t="n">
         <v>5.13</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1396,20 +1396,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/27/2026 21:34</t>
+          <t>10/28/2026 21:42</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
-        <v>19967.72</v>
+        <v>20589.36</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>-0.16</v>
+        <v>2.95</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>11.37</v>
       </c>
-      <c r="K6" t="n">
-        <v>1</v>
+      <c r="K6" s="7" t="n">
+        <v>1.05</v>
       </c>
       <c r="L6" t="n">
         <v>20000</v>
@@ -1421,34 +1421,34 @@
         <v>40</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>-1035.12</v>
+        <v>-1706.31</v>
       </c>
       <c r="P6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>30</v>
+        <v>27.5</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>0.7453328740835506</v>
+        <v>0.5884145017729213</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>11.5</v>
+        <v>12.24</v>
       </c>
       <c r="T6" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>-32.2800000000002</v>
+        <v>589.3599999999998</v>
       </c>
       <c r="V6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W6" s="7" t="n">
-        <v>31.85840707964602</v>
+        <v>32.17391304347826</v>
       </c>
       <c r="X6" s="7" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="Y6" s="7" t="n">
         <v>11.37</v>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/25/2026 15:14</t>
+          <t>10/28/2026 15:16</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,20 +1614,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/27/2026 21:35</t>
+          <t>10/28/2026 21:42</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
-        <v>19981.29</v>
+        <v>20017.16</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>-0.1</v>
+        <v>0.08</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>0.99</v>
+        <v>1.01</v>
       </c>
       <c r="L8" t="n">
         <v>20000</v>
@@ -1639,7 +1639,7 @@
         <v>40</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>-60.08</v>
+        <v>-64.00999999999999</v>
       </c>
       <c r="P8" t="n">
         <v>34</v>
@@ -1648,25 +1648,25 @@
         <v>85</v>
       </c>
       <c r="R8" s="7" t="n">
-        <v>0.8821290537756764</v>
+        <v>0.8744187871534794</v>
       </c>
       <c r="S8" s="7" t="n">
-        <v>1.54</v>
+        <v>1.55</v>
       </c>
       <c r="T8" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>-3.140000000000157</v>
+        <v>17.15999999999985</v>
       </c>
       <c r="V8" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="W8" s="7" t="n">
-        <v>83.50515463917526</v>
+        <v>83.67346938775511</v>
       </c>
       <c r="X8" s="7" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="Y8" s="7" t="n">
         <v>4.49</v>
@@ -1832,20 +1832,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/27/2026 21:16</t>
+          <t>10/28/2026 21:30</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>27906.27</v>
+        <v>28184.02</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>39.6</v>
+        <v>40.99</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.6</v>
+        <v>1.62</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1857,7 +1857,7 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>398.85</v>
+        <v>466.17</v>
       </c>
       <c r="P10" t="n">
         <v>25</v>
@@ -1866,25 +1866,25 @@
         <v>62.5</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>1.14593425732141</v>
+        <v>1.170565808538352</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>6.29</v>
+        <v>6.36</v>
       </c>
       <c r="T10" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>7908.16</v>
+        <v>8510.08</v>
       </c>
       <c r="V10" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>66.97674418604652</v>
+        <v>67.2811059907834</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.6</v>
+        <v>1.64</v>
       </c>
       <c r="Y10" s="7" t="n">
         <v>5.25</v>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1941,20 +1941,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/27/2026 22:43</t>
+          <t>10/28/2026 22:44</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>21015.59</v>
+        <v>20911.99</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>5.08</v>
+        <v>4.56</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>6.01</v>
+        <v>6.45</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1.32</v>
+        <v>1.28</v>
       </c>
       <c r="L11" t="n">
         <v>20000</v>
@@ -1966,7 +1966,7 @@
         <v>40</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>225.0300000000001</v>
+        <v>248.39</v>
       </c>
       <c r="P11" t="n">
         <v>15</v>
@@ -1975,28 +1975,28 @@
         <v>37.5</v>
       </c>
       <c r="R11" s="7" t="n">
-        <v>1.084354827826635</v>
+        <v>1.093934122452067</v>
       </c>
       <c r="S11" s="7" t="n">
-        <v>6.23</v>
+        <v>6.65</v>
       </c>
       <c r="T11" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="U11" s="7" t="n">
-        <v>1015.59</v>
+        <v>911.9900000000001</v>
       </c>
       <c r="V11" t="n">
         <v>25</v>
       </c>
       <c r="W11" s="7" t="n">
-        <v>42.3728813559322</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>1.32</v>
+        <v>1.28</v>
       </c>
       <c r="Y11" s="7" t="n">
-        <v>6.01</v>
+        <v>6.45</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -2050,20 +2050,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/27/2026 22:26</t>
+          <t>10/28/2026 22:26</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>20876.26</v>
+        <v>21045.82</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>4.36</v>
+        <v>5.21</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3.42</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1.51</v>
+        <v>1.61</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2072,37 +2072,37 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>20876.26</v>
+        <v>21045.82</v>
       </c>
       <c r="P12" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>70</v>
+        <v>70.96774193548387</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>13.07984075824996</v>
+        <v>13.17795497022897</v>
       </c>
       <c r="S12" s="7" t="n">
         <v>1.77</v>
       </c>
       <c r="T12" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>876.2599999999999</v>
+        <v>1045.82</v>
       </c>
       <c r="V12" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W12" s="7" t="n">
-        <v>68.96551724137932</v>
+        <v>70</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>1.51</v>
+        <v>1.61</v>
       </c>
       <c r="Y12" s="7" t="n">
         <v>3.41</v>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/27/2026 22:22</t>
+          <t>10/28/2026 22:21</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2199,16 +2199,16 @@
         <v>0.85</v>
       </c>
       <c r="T13" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-237.1099999999999</v>
+        <v>-237.11</v>
       </c>
       <c r="V13" t="n">
         <v>9</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>29.03225806451613</v>
+        <v>26.47058823529412</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>0.67</v>
@@ -2223,12 +2223,12 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -2268,20 +2268,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/27/2026 22:46</t>
+          <t>10/28/2026 22:48</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>20326.83</v>
+        <v>20093.17</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>1.64</v>
+        <v>0.47</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>4.44</v>
+        <v>4.65</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1.15</v>
+        <v>1.04</v>
       </c>
       <c r="L14" t="n">
         <v>20000</v>
@@ -2290,40 +2290,40 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>20080.53</v>
+        <v>19848.17</v>
       </c>
       <c r="P14" t="n">
         <v>6</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>20.68965517241379</v>
+        <v>20</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>10.021146122537</v>
+        <v>9.073941341577513</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>2.22</v>
+        <v>2.39</v>
       </c>
       <c r="T14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>326.8299999999999</v>
+        <v>93.16999999999993</v>
       </c>
       <c r="V14" t="n">
         <v>5</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>17.24137931034483</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="X14" s="7" t="n">
-        <v>1.15</v>
+        <v>1.04</v>
       </c>
       <c r="Y14" s="7" t="n">
-        <v>4.44</v>
+        <v>4.66</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>3EMA Core5 (DD ERC) | US30, 3EMA Core5 (DD ERC) | USDJPY.pro, 3EMA Core5 (DD ERC) | XAUUSD</t>
+          <t>3EMA Core5 (DD ERC) | JP225, 3EMA Core5 (DD ERC) | US30, 3EMA Core5 (DD ERC) | USDJPY.pro, 3EMA Core5 (DD ERC) | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/27/2026 22:35</t>
+          <t>10/28/2026 22:33</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2417,7 +2417,7 @@
         <v>0.1</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" s="7" t="n">
         <v>-9.780000000000001</v>
@@ -2426,7 +2426,7 @@
         <v>1</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>50</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>0.76</v>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/27/2026 22:32</t>
+          <t>10/28/2026 22:32</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/27/2026 22:33</t>
+          <t>10/28/2026 22:30</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/27/2026 22:29</t>
+          <t>10/28/2026 22:27</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/27/2026 22:39</t>
+          <t>10/28/2026 22:37</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2823,7 +2823,7 @@
         <v>0.09</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.46</v>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/27/2026 22:35</t>
+          <t>10/28/2026 22:36</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/27/2026 22:31</t>
+          <t>10/28/2026 22:29</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3071,7 +3071,7 @@
         <v>1.2</v>
       </c>
       <c r="T21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="U21" s="7" t="n">
         <v>-151.4</v>
@@ -3080,7 +3080,7 @@
         <v>12</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>63.1578947368421</v>
+        <v>60</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>0.71</v>
@@ -3095,12 +3095,12 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/27/2026 22:40</t>
+          <t>10/28/2026 22:39</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3243,20 +3243,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/27/2026 23:21</t>
+          <t>10/28/2026 23:28</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19751.82</v>
+        <v>20277.25</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-1.25</v>
+        <v>1.39</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.97</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.92</v>
+        <v>1.09</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3265,37 +3265,37 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>19701.18</v>
+        <v>20229.93</v>
       </c>
       <c r="P23" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>46.875</v>
+        <v>51.42857142857142</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>7.164439883101685</v>
+        <v>7.329884165535022</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>3.56</v>
       </c>
       <c r="T23" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-248.1800000000001</v>
+        <v>277.2500000000001</v>
       </c>
       <c r="V23" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>45.16129032258064</v>
+        <v>48.57142857142857</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.92</v>
+        <v>1.09</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.97</v>
@@ -3307,12 +3307,12 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -3352,20 +3352,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/27/2026 22:43</t>
+          <t>10/28/2026 22:44</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>20045.7</v>
+        <v>20057.94</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0.22</v>
+        <v>0.28</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>0.54</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3374,37 +3374,37 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>20001.14</v>
+        <v>9.499999999999996</v>
       </c>
       <c r="P24" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>51.28205128205128</v>
+        <v>52.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>85.5249545704264</v>
+        <v>1.040147065038245</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>0.34</v>
+        <v>0.67</v>
       </c>
       <c r="T24" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>52.81000000000001</v>
+        <v>57.94</v>
       </c>
       <c r="V24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>53.84615384615385</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
       <c r="Y24" s="7" t="n">
         <v>0.54</v>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/27/2026 23:11</t>
+          <t>10/28/2026 23:15</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/27/2026 23:10</t>
+          <t>10/28/2026 23:13</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3574,7 +3574,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -3670,17 +3670,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/27/2026 23:12</t>
+          <t>10/28/2026 23:18</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20029.35</v>
+        <v>20029.15</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>0.15</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -3707,19 +3707,19 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>29.35</v>
+        <v>29.15</v>
       </c>
       <c r="V27" t="n">
         <v>3</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>147.75</v>
+        <v>73.88</v>
       </c>
       <c r="Y27" s="7" t="n">
         <v>0</v>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>Finex | EURCHF, Finex | EURGBP, Finex | USDCAD</t>
+          <t>Finex | EURCHF, Finex | EURGBP, Finex | EURUSD, Finex | USDCAD</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/27/2026 23:13</t>
+          <t>10/28/2026 23:18</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3786,7 +3786,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>3.62</v>
+        <v>3.92</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/27/2026 23:13</t>
+          <t>10/28/2026 16:59</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -3991,20 +3991,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/27/2026 23:13</t>
-        </is>
-      </c>
-      <c r="H30" s="7" t="n">
-        <v>19992.2</v>
+          <t>10/28/2026 23:18</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>20001</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>-0.04</v>
+        <v>0</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>0.04</v>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
+      <c r="K30" s="7" t="n">
+        <v>1.13</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4013,37 +4013,37 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>19990.6</v>
+        <v>19998.6</v>
       </c>
       <c r="P30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>50</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>2127.659574468085</v>
+        <v>2128.510638297872</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>0.02</v>
       </c>
       <c r="T30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>-7.8</v>
+        <v>0.9999999999999991</v>
       </c>
       <c r="V30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>0</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>0.04</v>
@@ -4072,7 +4072,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>60905</t>
+          <t>60904</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tokyo Drive</t>
+          <t>TokioDrifter</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4100,20 +4100,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/27/2026 23:14</t>
+          <t>10/28/2026 23:17</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20007.03</v>
+        <v>19999.2</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="K31" s="7" t="n">
-        <v>1.2</v>
+        <v>0.11</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4122,76 +4122,73 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>20004.63</v>
+        <v>20000</v>
       </c>
       <c r="P31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>75</v>
-      </c>
-      <c r="R31" s="7" t="n">
-        <v>560.257198769919</v>
+        <v>100</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>7.030000000000001</v>
+        <v>-4.85</v>
       </c>
       <c r="V31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>0</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="Y31" s="7" t="n">
-        <v>0.17</v>
+        <v>0.02</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>Tokyo Drive | USDJPY</t>
+          <t>TokioDrifter | USDJPY</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>60907</t>
+          <t>60905</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>October Demos (live mirror, all strategies)</t>
+          <t>Tokyo Drive</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4209,62 +4206,62 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/27/2026 23:15</t>
+          <t>10/28/2026 23:20</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>1000.41</v>
+        <v>19970.93</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.06</v>
+        <v>-0.15</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>0.68</v>
+        <v>0.24</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>1.08</v>
+        <v>0.59</v>
       </c>
       <c r="L32" t="n">
-        <v>1000</v>
+        <v>20000</v>
       </c>
       <c r="M32" t="n">
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>999.49</v>
+        <v>19967.73</v>
       </c>
       <c r="P32" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>63.63636363636363</v>
+        <v>60</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>117.7628504672897</v>
+        <v>275.7726709783956</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>0.36</v>
+        <v>0.12</v>
       </c>
       <c r="T32" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>0.4099999999999999</v>
+        <v>-29.06999999999999</v>
       </c>
       <c r="V32" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>1.05</v>
+        <v>0.59</v>
       </c>
       <c r="Y32" s="7" t="n">
-        <v>0.68</v>
+        <v>0.23</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4278,29 +4275,29 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>October Demos (live mirror, all strategies) | EURCHF, October Demos (live mirror, all strategies) | EURGBP, October Demos (live mirror, all strategies) | EURUSD, October Demos (live mirror, all strategies) | USDCAD, October Demos (live mirror, all strategies) | USDJPY</t>
+          <t>Tokyo Drive | USDJPY</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>60909</t>
+          <t>60907</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SK Stochastic (MasterLive demo)</t>
+          <t>October Demos (live mirror, all strategies)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4318,68 +4315,71 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/27/2026 23:16</t>
+          <t>10/28/2026 23:21</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>19999.96</v>
+        <v>1002.62</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0</v>
+        <v>0.29</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
+        <v>0.68</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>1.31</v>
       </c>
       <c r="L33" t="n">
-        <v>20000</v>
+        <v>1000</v>
       </c>
       <c r="M33" t="n">
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>20000</v>
+        <v>1001.34</v>
       </c>
       <c r="P33" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>100</v>
+        <v>61.53846153846154</v>
+      </c>
+      <c r="R33" s="7" t="n">
+        <v>97.19020172910663</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="T33" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-0.04</v>
+        <v>2.42</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>0</v>
+        <v>36.84210526315789</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="Y33" s="7" t="n">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4389,212 +4389,229 @@
       </c>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>SK Stochastic (MasterLive demo) | EURUSD</t>
+          <t>October Demos (live mirror, all strategies) | EURCHF, October Demos (live mirror, all strategies) | EURGBP, October Demos (live mirror, all strategies) | EURUSD, October Demos (live mirror, all strategies) | USDCAD, October Demos (live mirror, all strategies) | USDJPY</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>60909</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SK Stochastic (MasterLive demo)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+      <c r="F34" t="b">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>10/28/2026 23:23</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>19999.96</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>1</v>
+      </c>
+      <c r="U34" s="7" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="V34" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>SK Stochastic (MasterLive demo) | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>1115445</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>licensed</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Smart Gold Hunter</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>OX Securities</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>VPS242t2</t>
         </is>
       </c>
-      <c r="F34" t="b">
-        <v>1</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>10/28/2026 00:15</t>
-        </is>
-      </c>
-      <c r="H34" s="7" t="n">
-        <v>12843.3</v>
-      </c>
-      <c r="I34" s="7" t="n">
-        <v>28.37</v>
-      </c>
-      <c r="J34" s="7" t="n">
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>10/29/2026 00:33</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>12585.42</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="J35" s="7" t="n">
         <v>3.38</v>
       </c>
-      <c r="K34" s="7" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="L34" t="n">
+      <c r="K35" s="7" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="L35" t="n">
         <v>10000</v>
       </c>
-      <c r="M34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" t="n">
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
         <v>40</v>
       </c>
-      <c r="O34" s="7" t="n">
-        <v>754.3599999999999</v>
-      </c>
-      <c r="P34" t="n">
+      <c r="O35" s="7" t="n">
+        <v>735.52</v>
+      </c>
+      <c r="P35" t="n">
         <v>27</v>
       </c>
-      <c r="Q34" s="7" t="n">
+      <c r="Q35" s="7" t="n">
         <v>67.5</v>
       </c>
-      <c r="R34" s="7" t="n">
-        <v>1.450735531363153</v>
-      </c>
-      <c r="S34" s="7" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="T34" t="n">
-        <v>100</v>
-      </c>
-      <c r="U34" s="7" t="n">
-        <v>2798.5</v>
-      </c>
-      <c r="V34" t="n">
+      <c r="R35" s="7" t="n">
+        <v>1.434586341774695</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="T35" t="n">
+        <v>103</v>
+      </c>
+      <c r="U35" s="7" t="n">
+        <v>2414.75</v>
+      </c>
+      <c r="V35" t="n">
         <v>71</v>
       </c>
-      <c r="W34" s="7" t="n">
-        <v>71</v>
-      </c>
-      <c r="X34" s="7" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="Y34" s="7" t="n">
+      <c r="W35" s="7" t="n">
+        <v>68.93203883495146</v>
+      </c>
+      <c r="X35" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="Y35" s="7" t="n">
         <v>3.36</v>
       </c>
-      <c r="Z34" t="inlineStr">
+      <c r="Z35" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr">
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
         <is>
           <t>RECONCILE</t>
         </is>
       </c>
-      <c r="AC34" t="inlineStr">
+      <c r="AC35" t="inlineStr">
         <is>
           <t>Smart Gold Hunter | XAUUSD.PRO</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>58989</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>TSma4f AUDCAD</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>TradeSmart</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>10/20/2026 23:29</t>
-        </is>
-      </c>
-      <c r="H35" s="8" t="n">
-        <v>20000</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="8" t="n">
-        <v>20000</v>
-      </c>
-      <c r="M35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O35" s="9" t="n">
-        <v>20000</v>
-      </c>
-      <c r="P35" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="R35" s="8" t="n"/>
-      <c r="S35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W35" s="8" t="n"/>
-      <c r="X35" s="8" t="n"/>
-      <c r="Y35" s="8" t="n"/>
-      <c r="Z35" s="8" t="n"/>
-      <c r="AA35" s="8" t="n"/>
-      <c r="AB35" s="8" t="inlineStr">
-        <is>
-          <t>DATA GAP - Bach missing</t>
-        </is>
-      </c>
-      <c r="AC35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>60904</t>
+          <t>58989</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -4604,7 +4621,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>TokioDrifter</t>
+          <t>TSma4f AUDCAD</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -4614,7 +4631,7 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>VPS242t3</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F36" s="8" t="b">
@@ -4622,7 +4639,7 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>10/27/2026 23:12</t>
+          <t>10/20/2026 23:29</t>
         </is>
       </c>
       <c r="H36" s="8" t="n">
@@ -4711,7 +4728,7 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>10/27/2026 23:13</t>
+          <t>10/28/2026 23:18</t>
         </is>
       </c>
       <c r="H37" s="8" t="n">
@@ -4780,7 +4797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4900,7 +4917,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>60904</t>
+          <t>60908</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4910,7 +4927,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TokioDrifter</t>
+          <t>SK Stochastic</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4925,7 +4942,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/27/2026 23:12</t>
+          <t>10/28/2026 23:18</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -4935,47 +4952,6 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>60908</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SK Stochastic</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>TradeSmart</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>VPS242t3</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>10/27/2026 23:13</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10507,11 +10483,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/27/2026 23:45</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>50000</v>
+          <t>10/28/2026 23:57</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>49231.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboards — 2026-10-29
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-28 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-29 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/28/2026 22:20</t>
+          <t>10/29/2026 22:59</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>35934.69</v>
+        <v>30007.31</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>43.74</v>
+        <v>20.03</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>4512.919999999999</v>
+        <v>-1944.680000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>80</v>
+        <v>77.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.120886329745073</v>
+        <v>0.9533638920051358</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>58.55</v>
+        <v>59.41</v>
       </c>
       <c r="T2" t="n">
-        <v>3526</v>
+        <v>3531</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>10934.68999999999</v>
+        <v>6435.889999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>2250</v>
+        <v>2254</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.8116846284742</v>
+        <v>63.8346077598414</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,14 +1069,14 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/28/2026 22:47</t>
+          <t>10/29/2026 23:25</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>20471.49</v>
+        <v>20459.08</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>2.36</v>
+        <v>2.3</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8.99</v>
@@ -1094,7 +1094,7 @@
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>-251.18</v>
+        <v>-220.61</v>
       </c>
       <c r="P3" t="n">
         <v>15</v>
@@ -1103,22 +1103,22 @@
         <v>37.5</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.7746173034474094</v>
+        <v>0.7964645858897121</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>2.5</v>
+        <v>2.29</v>
       </c>
       <c r="T3" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>471.4899999999997</v>
+        <v>459.0799999999997</v>
       </c>
       <c r="V3" t="n">
         <v>69</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>44.23076923076923</v>
+        <v>43.67088607594937</v>
       </c>
       <c r="X3" s="7" t="n">
         <v>1.07</v>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/28/2026 20:40</t>
+          <t>10/29/2026 21:31</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,14 +1287,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/28/2026 22:07</t>
+          <t>10/29/2026 22:47</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>19695.65</v>
+        <v>19709.68</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>-1.52</v>
+        <v>-1.45</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>5.13</v>
@@ -1312,31 +1312,31 @@
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>1.379999999999976</v>
+        <v>-116.54</v>
       </c>
       <c r="P5" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>1.006588370094529</v>
+        <v>0.4612112806287563</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="T5" t="n">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>-304.35</v>
+        <v>-290.3199999999999</v>
       </c>
       <c r="V5" t="n">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>54.65367965367965</v>
+        <v>54.73118279569893</v>
       </c>
       <c r="X5" s="7" t="n">
         <v>0.95</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1396,20 +1396,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/28/2026 21:42</t>
+          <t>10/29/2026 22:28</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
-        <v>20589.36</v>
+        <v>20328.7</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>2.95</v>
+        <v>1.65</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>11.37</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1.05</v>
+        <v>1.03</v>
       </c>
       <c r="L6" t="n">
         <v>20000</v>
@@ -1421,7 +1421,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>-1706.31</v>
+        <v>-1729.82</v>
       </c>
       <c r="P6" t="n">
         <v>11</v>
@@ -1430,25 +1430,25 @@
         <v>27.5</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>0.5884145017729213</v>
+        <v>0.5850964571225723</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>12.24</v>
+        <v>11.05</v>
       </c>
       <c r="T6" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>589.3599999999998</v>
+        <v>328.6999999999998</v>
       </c>
       <c r="V6" t="n">
         <v>37</v>
       </c>
       <c r="W6" s="7" t="n">
-        <v>32.17391304347826</v>
+        <v>31.89655172413793</v>
       </c>
       <c r="X6" s="7" t="n">
-        <v>1.05</v>
+        <v>1.03</v>
       </c>
       <c r="Y6" s="7" t="n">
         <v>11.37</v>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1614,20 +1614,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/28/2026 21:42</t>
+          <t>10/29/2026 22:27</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
-        <v>20017.16</v>
+        <v>20082.46</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.08</v>
+        <v>0.41</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="L8" t="n">
         <v>20000</v>
@@ -1639,34 +1639,34 @@
         <v>40</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>-64.00999999999999</v>
+        <v>66.48999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>85</v>
+        <v>87.5</v>
       </c>
       <c r="R8" s="7" t="n">
-        <v>0.8744187871534794</v>
+        <v>1.162523526679866</v>
       </c>
       <c r="S8" s="7" t="n">
-        <v>1.55</v>
+        <v>1.05</v>
       </c>
       <c r="T8" t="n">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>17.15999999999985</v>
+        <v>90.95999999999989</v>
       </c>
       <c r="V8" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="W8" s="7" t="n">
-        <v>83.67346938775511</v>
+        <v>84.07960199004975</v>
       </c>
       <c r="X8" s="7" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="Y8" s="7" t="n">
         <v>4.49</v>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1832,20 +1832,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/28/2026 21:30</t>
+          <t>10/29/2026 22:15</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>28184.02</v>
+        <v>27362.65</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>40.99</v>
+        <v>36.88</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>5.24</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.62</v>
+        <v>1.51</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1857,7 +1857,7 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>466.17</v>
+        <v>140.9599999999999</v>
       </c>
       <c r="P10" t="n">
         <v>25</v>
@@ -1866,28 +1866,28 @@
         <v>62.5</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>1.170565808538352</v>
+        <v>1.042507636960173</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>6.36</v>
+        <v>5.39</v>
       </c>
       <c r="T10" t="n">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>8510.08</v>
+        <v>6786.120000000001</v>
       </c>
       <c r="V10" t="n">
         <v>146</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>67.2811059907834</v>
+        <v>65.76576576576578</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.64</v>
+        <v>1.45</v>
       </c>
       <c r="Y10" s="7" t="n">
-        <v>5.25</v>
+        <v>6.05</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1941,20 +1941,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/28/2026 22:44</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="n">
-        <v>20911.99</v>
+          <t>10/29/2026 23:23</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>21072</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>4.56</v>
+        <v>5.36</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>6.45</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1.28</v>
+        <v>1.33</v>
       </c>
       <c r="L11" t="n">
         <v>20000</v>
@@ -1966,34 +1966,34 @@
         <v>40</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>248.39</v>
+        <v>571.0200000000001</v>
       </c>
       <c r="P11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="R11" s="7" t="n">
-        <v>1.093934122452067</v>
+        <v>1.23009412978305</v>
       </c>
       <c r="S11" s="7" t="n">
-        <v>6.65</v>
+        <v>6.6</v>
       </c>
       <c r="T11" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="U11" s="7" t="n">
-        <v>911.9900000000001</v>
+        <v>1072</v>
       </c>
       <c r="V11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W11" s="7" t="n">
-        <v>41.66666666666667</v>
+        <v>42.62295081967213</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>1.28</v>
+        <v>1.33</v>
       </c>
       <c r="Y11" s="7" t="n">
         <v>6.45</v>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/28/2026 22:26</t>
+          <t>10/29/2026 23:04</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,20 +2159,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/28/2026 22:21</t>
+          <t>10/29/2026 22:59</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>19762.89</v>
+        <v>19749.26</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-1.18</v>
+        <v>-1.25</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1.5</v>
+        <v>1.56</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="L13" t="n">
         <v>20000</v>
@@ -2181,28 +2181,28 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>19710.67</v>
+        <v>19696.31</v>
       </c>
       <c r="P13" t="n">
         <v>10</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>31.25</v>
+        <v>30.3030303030303</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>27.096823736578</v>
+        <v>26.59125576560774</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
       <c r="T13" t="n">
         <v>34</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-237.11</v>
+        <v>-251.3399999999999</v>
       </c>
       <c r="V13" t="n">
         <v>9</v>
@@ -2211,10 +2211,10 @@
         <v>26.47058823529412</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="Y13" s="7" t="n">
-        <v>1.5</v>
+        <v>1.57</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2268,20 +2268,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/28/2026 22:48</t>
+          <t>10/29/2026 23:26</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>20093.17</v>
+        <v>19958.41</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>0.47</v>
+        <v>-0.2</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>4.65</v>
+        <v>5.29</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1.04</v>
+        <v>0.98</v>
       </c>
       <c r="L14" t="n">
         <v>20000</v>
@@ -2290,40 +2290,40 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>19848.17</v>
+        <v>19711.39</v>
       </c>
       <c r="P14" t="n">
         <v>6</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>20</v>
+        <v>19.35483870967742</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>9.073941341577513</v>
+        <v>8.595677204556315</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>2.39</v>
+        <v>2.72</v>
       </c>
       <c r="T14" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>93.16999999999993</v>
+        <v>-41.59000000000003</v>
       </c>
       <c r="V14" t="n">
         <v>5</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>16.66666666666666</v>
+        <v>15.625</v>
       </c>
       <c r="X14" s="7" t="n">
-        <v>1.04</v>
+        <v>0.98</v>
       </c>
       <c r="Y14" s="7" t="n">
-        <v>4.66</v>
+        <v>5.3</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -2377,20 +2377,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/28/2026 22:33</t>
+          <t>10/29/2026 23:11</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>19990.22</v>
+        <v>19986.29</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-0.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.76</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L15" t="n">
         <v>20000</v>
@@ -2399,28 +2399,28 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>19990.22</v>
+        <v>19986.29</v>
       </c>
       <c r="P15" t="n">
         <v>2</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>50</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>500.3809642767924</v>
+        <v>455.6471792538671</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="T15" t="n">
         <v>3</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-9.780000000000001</v>
+        <v>-13.71</v>
       </c>
       <c r="V15" t="n">
         <v>1</v>
@@ -2429,10 +2429,10 @@
         <v>33.33333333333333</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>0.76</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y15" s="7" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/28/2026 22:32</t>
+          <t>10/29/2026 23:13</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/28/2026 22:30</t>
+          <t>10/29/2026 23:08</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/28/2026 22:27</t>
+          <t>10/29/2026 11:16</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/28/2026 22:37</t>
+          <t>10/29/2026 23:14</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2823,7 +2823,7 @@
         <v>0.09</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.46</v>
@@ -2853,22 +2853,22 @@
         <v>0.01</v>
       </c>
       <c r="T19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U19" s="7" t="n">
-        <v>19.2</v>
+        <v>-4.999999999999998</v>
       </c>
       <c r="V19" t="n">
         <v>5</v>
       </c>
       <c r="W19" s="7" t="n">
-        <v>71.42857142857143</v>
+        <v>62.5</v>
       </c>
       <c r="X19" s="7" t="n">
-        <v>3.46</v>
+        <v>0.84</v>
       </c>
       <c r="Y19" s="7" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2877,12 +2877,12 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/28/2026 22:36</t>
+          <t>10/29/2026 23:13</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,20 +3031,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/28/2026 22:29</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>19848.6</v>
+          <t>10/29/2026 23:07</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>19856</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>-0.75</v>
+        <v>-0.71</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>2.41</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="L21" t="n">
         <v>20000</v>
@@ -3053,37 +3053,37 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>19848.6</v>
+        <v>19856</v>
       </c>
       <c r="P21" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="7" t="n">
-        <v>65</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>38.47847432024169</v>
+        <v>37.63468634686347</v>
       </c>
       <c r="S21" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="T21" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>-151.4</v>
+        <v>-144</v>
       </c>
       <c r="V21" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>60</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="X21" s="7" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="Y21" s="7" t="n">
         <v>2.41</v>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/28/2026 22:39</t>
+          <t>10/29/2026 23:16</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3243,20 +3243,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/28/2026 23:28</t>
+          <t>10/30/2026 00:01</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>20277.25</v>
+        <v>20048.57</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1.39</v>
+        <v>0.25</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.97</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1.09</v>
+        <v>1.02</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3265,37 +3265,37 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>20229.93</v>
+        <v>20001.25</v>
       </c>
       <c r="P23" t="n">
         <v>18</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>51.42857142857142</v>
+        <v>50</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>7.329884165535022</v>
+        <v>6.840429011101961</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>3.56</v>
       </c>
       <c r="T23" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>277.2500000000001</v>
+        <v>-158.5399999999999</v>
       </c>
       <c r="V23" t="n">
         <v>17</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>48.57142857142857</v>
+        <v>45.94594594594595</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>1.09</v>
+        <v>0.96</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.97</v>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3352,20 +3352,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/28/2026 22:44</t>
+          <t>10/29/2026 23:22</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>20057.94</v>
+        <v>19983.06</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0.28</v>
+        <v>-0.08</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>0.54</v>
+        <v>0.87</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>1.27</v>
+        <v>0.96</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3377,7 +3377,7 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>9.499999999999996</v>
+        <v>-82.55000000000001</v>
       </c>
       <c r="P24" t="n">
         <v>21</v>
@@ -3386,28 +3386,28 @@
         <v>52.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>1.040147065038245</v>
+        <v>0.7505363996252756</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>0.67</v>
+        <v>1.05</v>
       </c>
       <c r="T24" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>57.94</v>
+        <v>-134.66</v>
       </c>
       <c r="V24" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>52.08333333333334</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>1.27</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y24" s="7" t="n">
-        <v>0.54</v>
+        <v>1.44</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/28/2026 23:15</t>
+          <t>10/29/2026 23:53</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/28/2026 23:13</t>
+          <t>10/29/2026 23:53</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3670,17 +3670,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/28/2026 23:18</t>
+          <t>10/29/2026 23:54</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20029.15</v>
+        <v>20043.15</v>
       </c>
       <c r="I27" s="7" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="J27" s="7" t="n">
         <v>0.15</v>
-      </c>
-      <c r="J27" s="7" t="n">
-        <v>0.07000000000000001</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -3692,13 +3692,13 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>20028.95</v>
+        <v>20042.75</v>
       </c>
       <c r="P27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q27" s="7" t="n">
         <v>100</v>
@@ -3707,19 +3707,19 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>29.15</v>
+        <v>43.15</v>
       </c>
       <c r="V27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>60</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>73.88</v>
+        <v>108.87</v>
       </c>
       <c r="Y27" s="7" t="n">
         <v>0</v>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/28/2026 23:18</t>
+          <t>10/29/2026 23:55</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/28/2026 16:59</t>
+          <t>10/29/2026 23:53</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -3991,20 +3991,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/28/2026 23:18</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>20001</v>
+          <t>10/29/2026 23:53</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>20008.2</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>0.04</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.13</v>
+        <v>2.05</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4013,37 +4013,37 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>19998.6</v>
+        <v>20005</v>
       </c>
       <c r="P30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>2128.510638297872</v>
+        <v>2129.191489361703</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>0.02</v>
       </c>
       <c r="T30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>0.9999999999999991</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>50</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>1.13</v>
+        <v>2.05</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>0.04</v>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4100,14 +4100,14 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/28/2026 23:17</t>
+          <t>10/29/2026 23:53</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>19999.2</v>
+        <v>19995.15</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0.11</v>
@@ -4122,19 +4122,22 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>20000</v>
+        <v>19994.35</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>100</v>
+        <v>50</v>
+      </c>
+      <c r="R31" s="7" t="n">
+        <v>3539.823008849558</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -4166,7 +4169,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -4206,7 +4209,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/28/2026 23:20</t>
+          <t>10/29/2026 23:54</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4315,20 +4318,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/28/2026 23:21</t>
+          <t>10/29/2026 23:55</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>1002.62</v>
+        <v>1008.06</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.29</v>
+        <v>0.83</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.68</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>1.31</v>
+        <v>1.85</v>
       </c>
       <c r="L33" t="n">
         <v>1000</v>
@@ -4337,37 +4340,37 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>1001.34</v>
+        <v>1006.26</v>
       </c>
       <c r="P33" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>61.53846153846154</v>
+        <v>62.5</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>97.19020172910663</v>
+        <v>95.1309635173059</v>
       </c>
       <c r="S33" s="7" t="n">
         <v>0.36</v>
       </c>
       <c r="T33" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>2.42</v>
+        <v>8.06</v>
       </c>
       <c r="V33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>36.84210526315789</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>1.24</v>
+        <v>1.81</v>
       </c>
       <c r="Y33" s="7" t="n">
         <v>0.68</v>
@@ -4379,7 +4382,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4424,7 +4427,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>10/28/2026 23:23</t>
+          <t>10/29/2026 23:57</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4530,20 +4533,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10/29/2026 00:33</t>
+          <t>10/30/2026 00:58</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>12585.42</v>
+        <v>12312.61</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>25.79</v>
+        <v>23.06</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>3.38</v>
+        <v>5.26</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.91</v>
+        <v>1.72</v>
       </c>
       <c r="L35" t="n">
         <v>10000</v>
@@ -4555,37 +4558,37 @@
         <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>735.52</v>
+        <v>395.92</v>
       </c>
       <c r="P35" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>67.5</v>
+        <v>62.5</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>1.434586341774695</v>
+        <v>1.202390324196665</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>3.87</v>
+        <v>6.37</v>
       </c>
       <c r="T35" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>2414.75</v>
+        <v>2267.81</v>
       </c>
       <c r="V35" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>68.93203883495146</v>
+        <v>67.9245283018868</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="Y35" s="7" t="n">
-        <v>3.36</v>
+        <v>5.28</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -4594,7 +4597,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4728,7 +4731,7 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>10/28/2026 23:18</t>
+          <t>10/29/2026 23:53</t>
         </is>
       </c>
       <c r="H37" s="8" t="n">
@@ -4942,7 +4945,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/28/2026 23:18</t>
+          <t>10/29/2026 23:53</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -10422,11 +10425,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -10483,11 +10486,264 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/28/2026 23:57</t>
+          <t>10/30/2026 00:25</t>
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>49231.23</v>
+        <v>49229.99</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>61199</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>61199 Demo BroadStreet GBPUSD</t>
+        </is>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>10/29/2026 19:22</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>61200</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>61200 Demo BroadStreet EURUSD</t>
+        </is>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>10/29/2026 20:11</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>61201</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>61201 Demo BroadStreet EURUSD &amp; GBPUSD</t>
+        </is>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:50</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>61202</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>61202 Demo DarkNebula</t>
+        </is>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:50</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>19999.76</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>61203</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>61203 Demo QuartzGrid Cruise</t>
+        </is>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:52</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>19999.84</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>61204</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>61204 Demo GoldLadder</t>
+        </is>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:55</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>61205</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>61205 Demo QuartzGrid Steady</t>
+        </is>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:55</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>19999.84</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>61206</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>61206 Demo QuartzGrid Drive</t>
+        </is>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:57</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>20009.49</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>61207</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>61207 Demo Gold Bolt</t>
+        </is>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>10/29/2026 21:57</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>61220</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>61220 Demo Swing Break</t>
+        </is>
+      </c>
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>10/29/2026 22:17</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>61221</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>61221 Demo Dream Catcher Book</t>
+        </is>
+      </c>
+      <c r="C15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10/29/2026 22:29</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>20000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboards — 2026-10-30
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-10-29 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-10-30 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC37"/>
+  <dimension ref="A1:AC47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10/29/2026 22:59</t>
+          <t>10/30/2026 20:54</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>30007.31</v>
+        <v>25309.54</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>20.03</v>
+        <v>1.24</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
-      <c r="K2" s="7" t="n">
-        <v>1.01</v>
+      <c r="K2" t="n">
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-1944.680000000001</v>
+        <v>-6961.97</v>
       </c>
       <c r="P2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>77.5</v>
+        <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.9533638920051358</v>
+        <v>0.8476588664256594</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>59.41</v>
+        <v>59.98</v>
       </c>
       <c r="T2" t="n">
-        <v>3531</v>
+        <v>3536</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>6435.889999999998</v>
+        <v>309.5399999999918</v>
       </c>
       <c r="V2" t="n">
-        <v>2254</v>
+        <v>2256</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.8346077598414</v>
+        <v>63.80090497737556</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10/29/2026 23:25</t>
+          <t>10/30/2026 21:29</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/29/2026 21:31</t>
+          <t>10/30/2026 18:45</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,14 +1287,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/29/2026 22:47</t>
+          <t>10/30/2026 20:39</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>19709.68</v>
+        <v>19695.51</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>-1.45</v>
+        <v>-1.53</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>5.13</v>
@@ -1312,31 +1312,31 @@
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>-116.54</v>
+        <v>-167.69</v>
       </c>
       <c r="P5" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>0.4612112806287563</v>
+        <v>0.2703420067879209</v>
       </c>
       <c r="S5" s="7" t="n">
         <v>0.88</v>
       </c>
       <c r="T5" t="n">
-        <v>930</v>
+        <v>944</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>-290.3199999999999</v>
+        <v>-304.4900000000002</v>
       </c>
       <c r="V5" t="n">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>54.73118279569893</v>
+        <v>54.13135593220338</v>
       </c>
       <c r="X5" s="7" t="n">
         <v>0.95</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1396,20 +1396,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/29/2026 22:28</t>
+          <t>10/30/2026 20:10</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
-        <v>20328.7</v>
+        <v>19816.88</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>1.65</v>
+        <v>-0.92</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>11.37</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1.03</v>
+        <v>0.99</v>
       </c>
       <c r="L6" t="n">
         <v>20000</v>
@@ -1421,34 +1421,34 @@
         <v>40</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>-1729.82</v>
+        <v>-1945.9</v>
       </c>
       <c r="P6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>0.5850964571225723</v>
+        <v>0.5663722927516274</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>11.05</v>
+        <v>10.69</v>
       </c>
       <c r="T6" t="n">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>328.6999999999998</v>
+        <v>-183.1200000000006</v>
       </c>
       <c r="V6" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="W6" s="7" t="n">
-        <v>31.89655172413793</v>
+        <v>32.78688524590164</v>
       </c>
       <c r="X6" s="7" t="n">
-        <v>1.03</v>
+        <v>0.99</v>
       </c>
       <c r="Y6" s="7" t="n">
         <v>11.37</v>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1614,20 +1614,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10/29/2026 22:27</t>
+          <t>10/30/2026 20:08</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
-        <v>20082.46</v>
+        <v>20170.94</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.41</v>
+        <v>0.86</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="L8" t="n">
         <v>20000</v>
@@ -1639,34 +1639,34 @@
         <v>40</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>66.48999999999999</v>
+        <v>320.28</v>
       </c>
       <c r="P8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>87.5</v>
+        <v>92.5</v>
       </c>
       <c r="R8" s="7" t="n">
-        <v>1.162523526679866</v>
+        <v>2.476080744769103</v>
       </c>
       <c r="S8" s="7" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="T8" t="n">
+        <v>205</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>170.9399999999999</v>
+      </c>
+      <c r="V8" t="n">
+        <v>173</v>
+      </c>
+      <c r="W8" s="7" t="n">
+        <v>84.39024390243902</v>
+      </c>
+      <c r="X8" s="7" t="n">
         <v>1.05</v>
-      </c>
-      <c r="T8" t="n">
-        <v>201</v>
-      </c>
-      <c r="U8" s="7" t="n">
-        <v>90.95999999999989</v>
-      </c>
-      <c r="V8" t="n">
-        <v>169</v>
-      </c>
-      <c r="W8" s="7" t="n">
-        <v>84.07960199004975</v>
-      </c>
-      <c r="X8" s="7" t="n">
-        <v>1.03</v>
       </c>
       <c r="Y8" s="7" t="n">
         <v>4.49</v>
@@ -1832,20 +1832,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/29/2026 22:15</t>
+          <t>10/30/2026 19:57</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>27362.65</v>
+        <v>26703.95</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>36.88</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>5.24</v>
+        <v>33.59</v>
+      </c>
+      <c r="J10" t="n">
+        <v>7</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.51</v>
+        <v>1.44</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1857,37 +1857,37 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>140.9599999999999</v>
+        <v>-98.00000000000006</v>
       </c>
       <c r="P10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>62.5</v>
+        <v>60</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>1.042507636960173</v>
+        <v>0.9736093756732302</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>5.39</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="T10" t="n">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>6786.120000000001</v>
+        <v>6703.950000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>65.76576576576578</v>
+        <v>65.33333333333333</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
       <c r="Y10" s="7" t="n">
-        <v>6.05</v>
+        <v>7</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1941,20 +1941,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10/29/2026 23:23</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>21072</v>
+          <t>10/30/2026 21:24</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>21519.27</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>5.36</v>
+        <v>7.6</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>6.45</v>
+        <v>8.15</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1.33</v>
+        <v>1.4</v>
       </c>
       <c r="L11" t="n">
         <v>20000</v>
@@ -1966,7 +1966,7 @@
         <v>40</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>571.0200000000001</v>
+        <v>1046.53</v>
       </c>
       <c r="P11" t="n">
         <v>16</v>
@@ -1975,28 +1975,28 @@
         <v>40</v>
       </c>
       <c r="R11" s="7" t="n">
-        <v>1.23009412978305</v>
+        <v>1.390614327464644</v>
       </c>
       <c r="S11" s="7" t="n">
-        <v>6.6</v>
+        <v>8.33</v>
       </c>
       <c r="T11" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="U11" s="7" t="n">
-        <v>1072</v>
+        <v>1519.27</v>
       </c>
       <c r="V11" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="W11" s="7" t="n">
-        <v>42.62295081967213</v>
+        <v>43.28358208955223</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>1.33</v>
+        <v>1.4</v>
       </c>
       <c r="Y11" s="7" t="n">
-        <v>6.45</v>
+        <v>8.15</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -2050,20 +2050,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10/29/2026 23:04</t>
+          <t>10/30/2026 21:00</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>21045.82</v>
+        <v>21242.11</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>5.21</v>
+        <v>6.19</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3.42</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1.61</v>
+        <v>1.72</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2072,37 +2072,37 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>21045.82</v>
+        <v>21242.11</v>
       </c>
       <c r="P12" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>70.96774193548387</v>
+        <v>71.875</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>13.17795497022897</v>
+        <v>13.29153623154861</v>
       </c>
       <c r="S12" s="7" t="n">
         <v>1.77</v>
       </c>
       <c r="T12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>1045.82</v>
+        <v>1242.11</v>
       </c>
       <c r="V12" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W12" s="7" t="n">
-        <v>70</v>
+        <v>70.96774193548387</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>1.61</v>
+        <v>1.72</v>
       </c>
       <c r="Y12" s="7" t="n">
         <v>3.41</v>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -2159,17 +2159,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/29/2026 22:59</t>
+          <t>10/30/2026 20:56</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>19749.26</v>
+        <v>19749.93</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-1.25</v>
+        <v>-1.24</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1.56</v>
+        <v>1.57</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>0.66</v>
@@ -2181,19 +2181,19 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>19696.31</v>
+        <v>19695.06</v>
       </c>
       <c r="P13" t="n">
         <v>10</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>30.3030303030303</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>26.59125576560774</v>
+        <v>26.54813853936957</v>
       </c>
       <c r="S13" s="7" t="n">
         <v>0.88</v>
@@ -2202,13 +2202,13 @@
         <v>34</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-251.3399999999999</v>
+        <v>-250.07</v>
       </c>
       <c r="V13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>26.47058823529412</v>
+        <v>29.41176470588236</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>0.66</v>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -2268,11 +2268,11 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10/29/2026 23:26</t>
+          <t>10/30/2026 21:29</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>19958.41</v>
+        <v>19958.1</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>-0.2</v>
@@ -2290,34 +2290,34 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>19711.39</v>
+        <v>19711.08</v>
       </c>
       <c r="P14" t="n">
         <v>6</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>19.35483870967742</v>
+        <v>18.75</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>8.595677204556315</v>
+        <v>8.59465051495151</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>2.72</v>
+        <v>2.73</v>
       </c>
       <c r="T14" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>-41.59000000000003</v>
+        <v>-41.90000000000009</v>
       </c>
       <c r="V14" t="n">
         <v>5</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>15.625</v>
+        <v>15.15151515151515</v>
       </c>
       <c r="X14" s="7" t="n">
         <v>0.98</v>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/29/2026 23:11</t>
+          <t>10/30/2026 21:15</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10/29/2026 23:13</t>
+          <t>10/30/2026 21:13</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10/29/2026 23:08</t>
+          <t>10/30/2026 21:06</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,20 +2704,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10/29/2026 11:16</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>19844</v>
+          <t>10/30/2026 21:09</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>19822.2</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>-0.78</v>
+        <v>-0.89</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1.21</v>
+        <v>1.32</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2726,40 +2726,40 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>19844</v>
+        <v>19822.2</v>
       </c>
       <c r="P18" t="n">
         <v>3</v>
       </c>
       <c r="Q18" s="7" t="n">
-        <v>37.5</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>55.84798231066888</v>
+        <v>52.67413972888426</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>0.61</v>
+        <v>0.66</v>
       </c>
       <c r="T18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-156</v>
+        <v>-177.8</v>
       </c>
       <c r="V18" t="n">
         <v>2</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>25</v>
+        <v>22.22222222222222</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="Y18" s="7" t="n">
-        <v>1.21</v>
+        <v>1.32</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -2813,20 +2813,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10/29/2026 23:14</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="n">
-        <v>20019.2</v>
+          <t>10/30/2026 21:15</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>19995</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.09</v>
+        <v>-0.03</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.46</v>
+        <v>0.84</v>
       </c>
       <c r="L19" t="n">
         <v>20000</v>
@@ -2835,22 +2835,22 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O19" s="7" t="n">
-        <v>20019.2</v>
+        <v>19995</v>
       </c>
       <c r="P19" t="n">
         <v>6</v>
       </c>
       <c r="Q19" s="7" t="n">
-        <v>75</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>2567.564102564103</v>
+        <v>625.84375</v>
       </c>
       <c r="S19" s="7" t="n">
-        <v>0.01</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T19" t="n">
         <v>8</v>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10/29/2026 23:13</t>
+          <t>10/30/2026 21:13</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,20 +3031,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10/29/2026 23:07</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>19856</v>
+          <t>10/30/2026 21:05</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>19824.8</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>-0.71</v>
+        <v>-0.87</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>2.41</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L21" t="n">
         <v>20000</v>
@@ -3053,37 +3053,37 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>19856</v>
+        <v>19824.8</v>
       </c>
       <c r="P21" t="n">
         <v>14</v>
       </c>
       <c r="Q21" s="7" t="n">
-        <v>63.63636363636363</v>
+        <v>60.86956521739131</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>37.63468634686347</v>
+        <v>35.58618283321703</v>
       </c>
       <c r="S21" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="T21" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>-144</v>
+        <v>-175.2</v>
       </c>
       <c r="V21" t="n">
         <v>13</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>59.09090909090909</v>
+        <v>54.16666666666666</v>
       </c>
       <c r="X21" s="7" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y21" s="7" t="n">
         <v>2.41</v>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10/29/2026 23:16</t>
+          <t>10/30/2026 21:17</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3243,20 +3243,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10/30/2026 00:01</t>
+          <t>10/30/2026 22:15</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>20048.57</v>
+        <v>19631.78</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.25</v>
+        <v>-1.85</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.97</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1.02</v>
+        <v>0.9</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3265,19 +3265,19 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>20001.25</v>
+        <v>19571.94</v>
       </c>
       <c r="P23" t="n">
         <v>18</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>50</v>
+        <v>47.36842105263158</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>6.840429011101961</v>
+        <v>6.078436816444513</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>3.56</v>
@@ -3286,7 +3286,7 @@
         <v>37</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-158.5399999999999</v>
+        <v>-368.2199999999999</v>
       </c>
       <c r="V23" t="n">
         <v>17</v>
@@ -3295,7 +3295,7 @@
         <v>45.94594594594595</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.97</v>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -3352,20 +3352,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>10/29/2026 23:22</t>
+          <t>10/30/2026 21:24</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>19983.06</v>
+        <v>19874.84</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.63</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>0.87</v>
+        <v>1.43</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>0.96</v>
+        <v>0.72</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3377,7 +3377,7 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>-82.55000000000001</v>
+        <v>-198.86</v>
       </c>
       <c r="P24" t="n">
         <v>21</v>
@@ -3386,25 +3386,25 @@
         <v>52.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0.7505363996252756</v>
+        <v>0.5434068835671481</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>1.05</v>
+        <v>1.64</v>
       </c>
       <c r="T24" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-134.66</v>
+        <v>-125.16</v>
       </c>
       <c r="V24" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>52.08333333333334</v>
+        <v>50</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="Y24" s="7" t="n">
         <v>1.44</v>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10/29/2026 23:53</t>
+          <t>10/30/2026 22:05</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3564,14 +3564,14 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10/29/2026 23:53</t>
+          <t>10/30/2026 22:03</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>19999.88</v>
+        <v>20008.88</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>0.09</v>
@@ -3586,13 +3586,13 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>20000</v>
+        <v>20008.76</v>
       </c>
       <c r="P26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q26" s="7" t="n">
         <v>100</v>
@@ -3604,33 +3604,30 @@
         <v>1</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>-0.12</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="V26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X26" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>0</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3670,17 +3667,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10/29/2026 23:54</t>
+          <t>10/30/2026 22:07</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20043.15</v>
+        <v>20064.37</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -3692,13 +3689,13 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>20042.75</v>
+        <v>20063.57</v>
       </c>
       <c r="P27" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q27" s="7" t="n">
         <v>100</v>
@@ -3707,19 +3704,19 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
+        <v>8</v>
+      </c>
+      <c r="U27" s="7" t="n">
+        <v>64.37</v>
+      </c>
+      <c r="V27" t="n">
         <v>6</v>
       </c>
-      <c r="U27" s="7" t="n">
-        <v>43.15</v>
-      </c>
-      <c r="V27" t="n">
-        <v>4</v>
-      </c>
       <c r="W27" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>75</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>108.87</v>
+        <v>161.92</v>
       </c>
       <c r="Y27" s="7" t="n">
         <v>0</v>
@@ -3731,7 +3728,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3776,7 +3773,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>10/29/2026 23:55</t>
+          <t>10/30/2026 22:07</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3882,11 +3879,11 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10/29/2026 23:53</t>
+          <t>10/30/2026 22:05</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19921.43</v>
+        <v>19921.32</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>-0.39</v>
@@ -3904,19 +3901,19 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>19921.43</v>
+        <v>19920.6</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>50</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>254.5500827287769</v>
+        <v>251.8891687657431</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>0.2</v>
@@ -3925,7 +3922,7 @@
         <v>2</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-78.56999999999999</v>
+        <v>-78.67999999999999</v>
       </c>
       <c r="V29" t="n">
         <v>0</v>
@@ -3946,12 +3943,12 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -3991,7 +3988,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10/29/2026 23:53</t>
+          <t>10/30/2026 22:05</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4100,7 +4097,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10/29/2026 23:53</t>
+          <t>10/30/2026 22:06</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4209,20 +4206,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10/29/2026 23:54</t>
+          <t>10/30/2026 22:05</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>19970.93</v>
+        <v>19935.44</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>-0.15</v>
+        <v>-0.33</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>0.24</v>
+        <v>0.42</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>0.59</v>
+        <v>0.39</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4231,40 +4228,40 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>19967.73</v>
+        <v>19931.44</v>
       </c>
       <c r="P32" t="n">
         <v>3</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>275.7726709783956</v>
+        <v>183.924375917768</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="T32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>-29.06999999999999</v>
+        <v>-64.55999999999999</v>
       </c>
       <c r="V32" t="n">
         <v>2</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>0.59</v>
+        <v>0.39</v>
       </c>
       <c r="Y32" s="7" t="n">
-        <v>0.23</v>
+        <v>0.41</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4273,7 +4270,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -4318,20 +4315,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10/29/2026 23:55</t>
+          <t>10/30/2026 22:07</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>1008.06</v>
+        <v>1016.51</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.83</v>
+        <v>1.66</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.68</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>1.85</v>
+        <v>2.44</v>
       </c>
       <c r="L33" t="n">
         <v>1000</v>
@@ -4340,37 +4337,37 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>1006.26</v>
+        <v>1014.35</v>
       </c>
       <c r="P33" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>62.5</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>95.1309635173059</v>
+        <v>81.56791104050835</v>
       </c>
       <c r="S33" s="7" t="n">
         <v>0.36</v>
       </c>
       <c r="T33" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>8.06</v>
+        <v>16.51</v>
       </c>
       <c r="V33" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>54.16666666666666</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>1.81</v>
+        <v>2.41</v>
       </c>
       <c r="Y33" s="7" t="n">
         <v>0.68</v>
@@ -4427,14 +4424,14 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>10/29/2026 23:57</t>
+          <t>10/30/2026 22:10</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>19999.96</v>
+        <v>20002.97</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>0.03</v>
@@ -4449,13 +4446,13 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>20000</v>
+        <v>20002.93</v>
       </c>
       <c r="P34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q34" s="7" t="n">
         <v>100</v>
@@ -4467,33 +4464,30 @@
         <v>1</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>-0.04</v>
+        <v>2.97</v>
       </c>
       <c r="V34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X34" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>0</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -4505,289 +4499,1361 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>61199</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BroadStreet GBPUSD</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>10/31/2026 00:44</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>19999.88</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>1</v>
+      </c>
+      <c r="U35" s="7" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>BroadStreet GBPUSD | GBPUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>61200</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BroadStreet EURUSD</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F36" t="b">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>10/31/2026 00:47</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>20000.18</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>2</v>
+      </c>
+      <c r="O36" s="7" t="n">
+        <v>19999.94</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R36" s="7" t="n">
+        <v>333333.3333333334</v>
+      </c>
+      <c r="S36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>1</v>
+      </c>
+      <c r="U36" s="7" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="V36" t="n">
+        <v>1</v>
+      </c>
+      <c r="W36" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>BroadStreet EURUSD | EURUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>61201</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BroadStreet EURUSD &amp; GBPUSD</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F37" t="b">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:21</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>20000.18</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>2</v>
+      </c>
+      <c r="O37" s="7" t="n">
+        <v>19999.94</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R37" s="7" t="n">
+        <v>333333.3333333334</v>
+      </c>
+      <c r="S37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U37" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="V37" t="n">
+        <v>1</v>
+      </c>
+      <c r="W37" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="X37" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Y37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>BroadStreet EURUSD &amp; GBPUSD | EURUSD, BroadStreet EURUSD &amp; GBPUSD | GBPUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>61202</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DarkNebula</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F38" t="b">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:19</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>19999.28</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="n">
+        <v>1</v>
+      </c>
+      <c r="O38" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>2</v>
+      </c>
+      <c r="U38" s="7" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="V38" t="n">
+        <v>0</v>
+      </c>
+      <c r="W38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>DarkNebula | AUDCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>61203</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>QuartzGrid Cruise</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F39" t="b">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:21</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>19999.84</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" s="7" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>QuartzGrid Cruise | AUDCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>61204</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GoldLadder</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F40" t="b">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:24</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>20785.7</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="J40" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K40" s="7" t="n">
+        <v>20.91</v>
+      </c>
+      <c r="L40" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="n">
+        <v>14</v>
+      </c>
+      <c r="O40" s="7" t="n">
+        <v>20785.7</v>
+      </c>
+      <c r="P40" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q40" s="7" t="n">
+        <v>64.28571428571429</v>
+      </c>
+      <c r="R40" s="7" t="n">
+        <v>527.7536746071971</v>
+      </c>
+      <c r="S40" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="T40" t="n">
+        <v>13</v>
+      </c>
+      <c r="U40" s="7" t="n">
+        <v>785.7</v>
+      </c>
+      <c r="V40" t="n">
+        <v>8</v>
+      </c>
+      <c r="W40" s="7" t="n">
+        <v>61.53846153846154</v>
+      </c>
+      <c r="X40" s="7" t="n">
+        <v>20.91</v>
+      </c>
+      <c r="Y40" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>GoldLadder | XAUUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>61205</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>QuartzGrid Steady</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F41" t="b">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:24</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>19999.84</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="n">
+        <v>1</v>
+      </c>
+      <c r="O41" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1</v>
+      </c>
+      <c r="U41" s="7" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="V41" t="n">
+        <v>0</v>
+      </c>
+      <c r="W41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>QuartzGrid Steady | AUDCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>61206</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>QuartzGrid Drive</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F42" t="b">
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:28</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="n">
+        <v>20021.54</v>
+      </c>
+      <c r="I42" s="7" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="J42" s="7" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>12</v>
+      </c>
+      <c r="O42" s="7" t="n">
+        <v>20020.26</v>
+      </c>
+      <c r="P42" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T42" t="n">
+        <v>14</v>
+      </c>
+      <c r="U42" s="7" t="n">
+        <v>21.54</v>
+      </c>
+      <c r="V42" t="n">
+        <v>11</v>
+      </c>
+      <c r="W42" s="7" t="n">
+        <v>78.57142857142857</v>
+      </c>
+      <c r="X42" s="7" t="n">
+        <v>45.88</v>
+      </c>
+      <c r="Y42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>QuartzGrid Drive | AUDCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>61207</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Gold Bolt</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>VPS153</t>
+        </is>
+      </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:28</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="n">
+        <v>20369.03</v>
+      </c>
+      <c r="I43" s="7" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K43" s="7" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="L43" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>5</v>
+      </c>
+      <c r="O43" s="7" t="n">
+        <v>20369.03</v>
+      </c>
+      <c r="P43" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>382.8715785526809</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="T43" t="n">
+        <v>4</v>
+      </c>
+      <c r="U43" s="7" t="n">
+        <v>369.03</v>
+      </c>
+      <c r="V43" t="n">
+        <v>3</v>
+      </c>
+      <c r="W43" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="X43" s="7" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="Y43" s="7" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>Gold Bolt | XAUUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>61220</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Prismatic Swing Break</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TradeSmart</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>VPS242t2</t>
+        </is>
+      </c>
+      <c r="F44" t="b">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>10/30/2026 19:58</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>20445.2</v>
+      </c>
+      <c r="I44" s="7" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K44" s="7" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="L44" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="n">
+        <v>8</v>
+      </c>
+      <c r="O44" s="7" t="n">
+        <v>20445.2</v>
+      </c>
+      <c r="P44" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>509.3341621084037</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="T44" t="n">
+        <v>7</v>
+      </c>
+      <c r="U44" s="7" t="n">
+        <v>445.2</v>
+      </c>
+      <c r="V44" t="n">
+        <v>6</v>
+      </c>
+      <c r="W44" s="7" t="n">
+        <v>85.71428571428571</v>
+      </c>
+      <c r="X44" s="7" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="Y44" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>OK (small account, full sample)</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>Prismatic Swing Break | XAUUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>1115445</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>licensed</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Smart Gold Hunter</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>OX Securities</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>VPS242t2</t>
         </is>
       </c>
-      <c r="F35" t="b">
-        <v>1</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>10/30/2026 00:58</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="n">
+      <c r="F45" t="b">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>10/30/2026 23:15</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="n">
         <v>12312.61</v>
       </c>
-      <c r="I35" s="7" t="n">
+      <c r="I45" s="7" t="n">
         <v>23.06</v>
       </c>
-      <c r="J35" s="7" t="n">
+      <c r="J45" s="7" t="n">
         <v>5.26</v>
       </c>
-      <c r="K35" s="7" t="n">
+      <c r="K45" s="7" t="n">
         <v>1.72</v>
       </c>
-      <c r="L35" t="n">
+      <c r="L45" t="n">
         <v>10000</v>
       </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" t="n">
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
         <v>40</v>
       </c>
-      <c r="O35" s="7" t="n">
+      <c r="O45" s="7" t="n">
         <v>395.92</v>
       </c>
-      <c r="P35" t="n">
+      <c r="P45" t="n">
         <v>25</v>
       </c>
-      <c r="Q35" s="7" t="n">
+      <c r="Q45" s="7" t="n">
         <v>62.5</v>
       </c>
-      <c r="R35" s="7" t="n">
+      <c r="R45" s="7" t="n">
         <v>1.202390324196665</v>
       </c>
-      <c r="S35" s="7" t="n">
+      <c r="S45" s="7" t="n">
         <v>6.37</v>
       </c>
-      <c r="T35" t="n">
+      <c r="T45" t="n">
         <v>106</v>
       </c>
-      <c r="U35" s="7" t="n">
+      <c r="U45" s="7" t="n">
         <v>2267.81</v>
       </c>
-      <c r="V35" t="n">
+      <c r="V45" t="n">
         <v>72</v>
       </c>
-      <c r="W35" s="7" t="n">
+      <c r="W45" s="7" t="n">
         <v>67.9245283018868</v>
       </c>
-      <c r="X35" s="7" t="n">
+      <c r="X45" s="7" t="n">
         <v>1.7</v>
       </c>
-      <c r="Y35" s="7" t="n">
+      <c r="Y45" s="7" t="n">
         <v>5.28</v>
       </c>
-      <c r="Z35" t="inlineStr">
+      <c r="Z45" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="AA35" t="inlineStr">
+      <c r="AA45" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="AB35" t="inlineStr">
+      <c r="AB45" t="inlineStr">
         <is>
           <t>RECONCILE</t>
         </is>
       </c>
-      <c r="AC35" t="inlineStr">
+      <c r="AC45" t="inlineStr">
         <is>
           <t>Smart Gold Hunter | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>58989</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>TSma4f AUDCAD</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D46" s="8" t="inlineStr">
         <is>
           <t>TradeSmart</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t>VPS92</t>
         </is>
       </c>
-      <c r="F36" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
+      <c r="F46" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
         <is>
           <t>10/20/2026 23:29</t>
         </is>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H46" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="I36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" s="8" t="n">
+      <c r="I46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="M36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O36" s="9" t="n">
+      <c r="M46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O46" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="P36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q36" s="9" t="n">
+      <c r="P46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q46" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="R36" s="8" t="n"/>
-      <c r="S36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W36" s="8" t="n"/>
-      <c r="X36" s="8" t="n"/>
-      <c r="Y36" s="8" t="n"/>
-      <c r="Z36" s="8" t="n"/>
-      <c r="AA36" s="8" t="n"/>
-      <c r="AB36" s="8" t="inlineStr">
+      <c r="R46" s="8" t="n"/>
+      <c r="S46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" s="8" t="n"/>
+      <c r="X46" s="8" t="n"/>
+      <c r="Y46" s="8" t="n"/>
+      <c r="Z46" s="8" t="n"/>
+      <c r="AA46" s="8" t="n"/>
+      <c r="AB46" s="8" t="inlineStr">
         <is>
           <t>DATA GAP - Bach missing</t>
         </is>
       </c>
-      <c r="AC36" s="8" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="AC46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>60908</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>SK Stochastic</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>TradeSmart</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>VPS242t3</t>
         </is>
       </c>
-      <c r="F37" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>10/29/2026 23:53</t>
-        </is>
-      </c>
-      <c r="H37" s="8" t="n">
+      <c r="F47" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>10/30/2026 22:04</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="I37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" s="8" t="n">
+      <c r="I47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="M37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O37" s="9" t="n">
+      <c r="M47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="P37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q37" s="9" t="n">
+      <c r="P47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q47" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="R37" s="8" t="n"/>
-      <c r="S37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W37" s="8" t="n"/>
-      <c r="X37" s="8" t="n"/>
-      <c r="Y37" s="8" t="n"/>
-      <c r="Z37" s="8" t="n"/>
-      <c r="AA37" s="8" t="n"/>
-      <c r="AB37" s="8" t="inlineStr">
+      <c r="R47" s="8" t="n"/>
+      <c r="S47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W47" s="8" t="n"/>
+      <c r="X47" s="8" t="n"/>
+      <c r="Y47" s="8" t="n"/>
+      <c r="Z47" s="8" t="n"/>
+      <c r="AA47" s="8" t="n"/>
+      <c r="AB47" s="8" t="inlineStr">
         <is>
           <t>DATA GAP - Bach missing</t>
         </is>
       </c>
-      <c r="AC37" s="8" t="inlineStr"/>
+      <c r="AC47" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4945,7 +6011,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/29/2026 23:53</t>
+          <t>10/30/2026 22:04</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -10425,11 +11491,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -10486,22 +11552,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10/30/2026 00:25</t>
+          <t>10/30/2026 22:45</t>
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>49229.99</v>
+        <v>49151.86</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>61199</t>
+          <t>61221</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>61199 Demo BroadStreet GBPUSD</t>
+          <t>61221 Demo Dream Catcher Book</t>
         </is>
       </c>
       <c r="C5" t="b">
@@ -10509,241 +11575,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10/29/2026 19:22</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>61200</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>61200 Demo BroadStreet EURUSD</t>
-        </is>
-      </c>
-      <c r="C6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>10/29/2026 20:11</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>61201</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>61201 Demo BroadStreet EURUSD &amp; GBPUSD</t>
-        </is>
-      </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:50</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>61202</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>61202 Demo DarkNebula</t>
-        </is>
-      </c>
-      <c r="C8" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:50</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>19999.76</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>61203</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>61203 Demo QuartzGrid Cruise</t>
-        </is>
-      </c>
-      <c r="C9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:52</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>19999.84</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>61204</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>61204 Demo GoldLadder</t>
-        </is>
-      </c>
-      <c r="C10" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:55</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>61205</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>61205 Demo QuartzGrid Steady</t>
-        </is>
-      </c>
-      <c r="C11" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:55</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>19999.84</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>61206</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>61206 Demo QuartzGrid Drive</t>
-        </is>
-      </c>
-      <c r="C12" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:57</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>20009.49</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>61207</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>61207 Demo Gold Bolt</t>
-        </is>
-      </c>
-      <c r="C13" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>10/29/2026 21:57</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>61220</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>61220 Demo Swing Break</t>
-        </is>
-      </c>
-      <c r="C14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>10/29/2026 22:17</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>61221</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>61221 Demo Dream Catcher Book</t>
-        </is>
-      </c>
-      <c r="C15" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>10/29/2026 22:29</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>20000</v>
+          <t>10/30/2026 20:14</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>20007.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>